<commit_message>
Lisää Roolit-exceliin uusi osio Urakkatilanne
Halutaan viedä urakoiden tilannetietoa tietyille käyttäjärooleilla omassa osiossaan. Viedään sen oikeuksien hallintaa varten uusi osio Roolit-exceliin.
</commit_message>
<xml_diff>
--- a/resources/roolit.xlsx
+++ b/resources/roolit.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10908"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samumi/Desktop/projektit/harjaroot/harja/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jarno.vayrynen/harja/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:81_{81F20872-FECA-8649-900B-F40E0B104EC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:81_{0FBD2778-313A-6A48-AE06-97A9D546ED0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10600" yWindow="-28300" windowWidth="51200" windowHeight="28300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="960" yWindow="500" windowWidth="50240" windowHeight="26600" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Oikeudet" sheetId="1" r:id="rId1"/>
@@ -107,7 +107,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1880" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1886" uniqueCount="266">
   <si>
     <t xml:space="preserve">Roolimääritysten selitykset: </t>
   </si>
@@ -974,6 +974,9 @@
   </si>
   <si>
     <t>Lupaukset</t>
+  </si>
+  <si>
+    <t>Urakkatilanne</t>
   </si>
 </sst>
 </file>
@@ -1352,7 +1355,7 @@
 </file>
 
 <file path=xl/revisions/revisionHeaders.xml><?xml version="1.0" encoding="utf-8"?>
-<headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" guid="{E4DF9D60-182D-0E4C-8CE9-DE4AF3C25295}" diskRevisions="1" revisionId="103" version="6">
+<headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" guid="{57942C57-C2FE-6C48-BE4D-8BEB0F10ABDA}" diskRevisions="1" revisionId="110" version="8">
   <header guid="{8EBC2E30-8A6E-AD43-9F6F-B4500CF04203}" dateTime="2024-06-11T12:49:05" maxSheetId="3" userName="Jarno Väyrynen" r:id="rId9" minRId="87" maxRId="97">
     <sheetIdMap count="2">
       <sheetId val="1"/>
@@ -1360,6 +1363,18 @@
     </sheetIdMap>
   </header>
   <header guid="{E4DF9D60-182D-0E4C-8CE9-DE4AF3C25295}" dateTime="2024-09-11T15:51:57" maxSheetId="3" userName="Microsoft Office User" r:id="rId10" minRId="99" maxRId="102">
+    <sheetIdMap count="2">
+      <sheetId val="1"/>
+      <sheetId val="2"/>
+    </sheetIdMap>
+  </header>
+  <header guid="{B2ACF18C-7218-464D-B445-888C770C7207}" dateTime="2024-11-18T11:43:33" maxSheetId="3" userName="Jarno Väyrynen" r:id="rId11" minRId="104" maxRId="108">
+    <sheetIdMap count="2">
+      <sheetId val="1"/>
+      <sheetId val="2"/>
+    </sheetIdMap>
+  </header>
+  <header guid="{57942C57-C2FE-6C48-BE4D-8BEB0F10ABDA}" dateTime="2024-11-18T11:58:37" maxSheetId="3" userName="Jarno Väyrynen" r:id="rId12" minRId="109" maxRId="110">
     <sheetIdMap count="2">
       <sheetId val="1"/>
       <sheetId val="2"/>
@@ -1396,6 +1411,813 @@
     <formula>Oikeudet!$A$5:$Y$128</formula>
   </rdn>
   <rcv guid="{843152D8-333A-1941-83E9-0CB5262068A2}" action="add"/>
+</revisions>
+</file>
+
+<file path=xl/revisions/revisionLog2.xml><?xml version="1.0" encoding="utf-8"?>
+<revisions xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <rfmt sheetId="1" xfDxf="1" sqref="A130" start="0" length="0">
+    <dxf/>
+  </rfmt>
+  <rfmt sheetId="1" xfDxf="1" sqref="B130" start="0" length="0">
+    <dxf/>
+  </rfmt>
+  <rfmt sheetId="1" xfDxf="1" sqref="C130" start="0" length="0">
+    <dxf/>
+  </rfmt>
+  <rfmt sheetId="1" xfDxf="1" sqref="D130" start="0" length="0">
+    <dxf/>
+  </rfmt>
+  <rfmt sheetId="1" xfDxf="1" sqref="E130" start="0" length="0">
+    <dxf/>
+  </rfmt>
+  <rfmt sheetId="1" xfDxf="1" sqref="F130" start="0" length="0">
+    <dxf/>
+  </rfmt>
+  <rfmt sheetId="1" xfDxf="1" sqref="G130" start="0" length="0">
+    <dxf/>
+  </rfmt>
+  <rfmt sheetId="1" xfDxf="1" sqref="H130" start="0" length="0">
+    <dxf/>
+  </rfmt>
+  <rfmt sheetId="1" xfDxf="1" sqref="I130" start="0" length="0">
+    <dxf/>
+  </rfmt>
+  <rfmt sheetId="1" xfDxf="1" sqref="J130" start="0" length="0">
+    <dxf/>
+  </rfmt>
+  <rfmt sheetId="1" xfDxf="1" sqref="K130" start="0" length="0">
+    <dxf/>
+  </rfmt>
+  <rfmt sheetId="1" xfDxf="1" sqref="L130" start="0" length="0">
+    <dxf/>
+  </rfmt>
+  <rfmt sheetId="1" xfDxf="1" sqref="M130" start="0" length="0">
+    <dxf/>
+  </rfmt>
+  <rfmt sheetId="1" xfDxf="1" sqref="N130" start="0" length="0">
+    <dxf/>
+  </rfmt>
+  <rfmt sheetId="1" xfDxf="1" sqref="O130" start="0" length="0">
+    <dxf/>
+  </rfmt>
+  <rfmt sheetId="1" xfDxf="1" sqref="P130" start="0" length="0">
+    <dxf/>
+  </rfmt>
+  <rfmt sheetId="1" xfDxf="1" sqref="Q130" start="0" length="0">
+    <dxf/>
+  </rfmt>
+  <rfmt sheetId="1" xfDxf="1" sqref="R130" start="0" length="0">
+    <dxf/>
+  </rfmt>
+  <rfmt sheetId="1" xfDxf="1" sqref="S130" start="0" length="0">
+    <dxf/>
+  </rfmt>
+  <rfmt sheetId="1" xfDxf="1" sqref="T130" start="0" length="0">
+    <dxf/>
+  </rfmt>
+  <rfmt sheetId="1" xfDxf="1" sqref="U130" start="0" length="0">
+    <dxf/>
+  </rfmt>
+  <rfmt sheetId="1" xfDxf="1" sqref="V130" start="0" length="0">
+    <dxf/>
+  </rfmt>
+  <rfmt sheetId="1" xfDxf="1" sqref="W130" start="0" length="0">
+    <dxf/>
+  </rfmt>
+  <rfmt sheetId="1" xfDxf="1" sqref="X130" start="0" length="0">
+    <dxf/>
+  </rfmt>
+  <rfmt sheetId="1" sqref="A130" start="0" length="0">
+    <dxf>
+      <font>
+        <color auto="1"/>
+        <family val="2"/>
+      </font>
+      <alignment vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rfmt sheetId="1" sqref="B130" start="0" length="0">
+    <dxf>
+      <font>
+        <color auto="1"/>
+        <family val="2"/>
+      </font>
+      <alignment vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rfmt sheetId="1" sqref="C130" start="0" length="0">
+    <dxf>
+      <alignment vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rfmt sheetId="1" sqref="D130" start="0" length="0">
+    <dxf>
+      <font>
+        <color auto="1"/>
+        <family val="2"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rfmt sheetId="1" sqref="E130" start="0" length="0">
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rfmt sheetId="1" sqref="F130" start="0" length="0">
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rfmt sheetId="1" sqref="G130" start="0" length="0">
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rfmt sheetId="1" sqref="H130" start="0" length="0">
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rfmt sheetId="1" sqref="I130" start="0" length="0">
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rfmt sheetId="1" sqref="J130" start="0" length="0">
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rfmt sheetId="1" sqref="K130" start="0" length="0">
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rfmt sheetId="1" sqref="L130" start="0" length="0">
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rfmt sheetId="1" sqref="M130" start="0" length="0">
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rfmt sheetId="1" sqref="N130" start="0" length="0">
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rfmt sheetId="1" sqref="O130" start="0" length="0">
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rfmt sheetId="1" sqref="P130" start="0" length="0">
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rfmt sheetId="1" sqref="Q130" start="0" length="0">
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rfmt sheetId="1" sqref="R130" start="0" length="0">
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rfmt sheetId="1" sqref="S130" start="0" length="0">
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rfmt sheetId="1" sqref="T130" start="0" length="0">
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rfmt sheetId="1" sqref="U130" start="0" length="0">
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rfmt sheetId="1" sqref="V130" start="0" length="0">
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rfmt sheetId="1" sqref="W130" start="0" length="0">
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rfmt sheetId="1" sqref="X130" start="0" length="0">
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rfmt sheetId="1" sqref="Y130" start="0" length="0">
+    <dxf>
+      <alignment vertical="top"/>
+    </dxf>
+  </rfmt>
+  <rfmt sheetId="1" sqref="E130" start="0" length="0">
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+  </rfmt>
+  <rfmt sheetId="1" sqref="D130" start="0" length="0">
+    <dxf>
+      <font>
+        <color auto="1"/>
+        <family val="2"/>
+      </font>
+      <alignment horizontal="general"/>
+    </dxf>
+  </rfmt>
+  <rcc rId="104" sId="1">
+    <nc r="A130" t="inlineStr">
+      <is>
+        <t>Urakoiden tilanne</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="105" sId="1" odxf="1" dxf="1">
+    <nc r="D130" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+    <ndxf>
+      <font>
+        <color auto="1"/>
+        <family val="2"/>
+      </font>
+      <alignment horizontal="center"/>
+    </ndxf>
+  </rcc>
+  <rcc rId="106" sId="1" odxf="1" dxf="1">
+    <nc r="E130" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+    <ndxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+    </ndxf>
+  </rcc>
+  <rcc rId="107" sId="1">
+    <nc r="K130" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="108" sId="1">
+    <nc r="L130" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+</revisions>
+</file>
+
+<file path=xl/revisions/revisionLog3.xml><?xml version="1.0" encoding="utf-8"?>
+<revisions xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <rcc rId="109" sId="1">
+    <oc r="A130" t="inlineStr">
+      <is>
+        <t>Urakoiden tilanne</t>
+      </is>
+    </oc>
+    <nc r="A130" t="inlineStr">
+      <is>
+        <t>Urakkatilanne</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="110" sId="1">
+    <nc r="B130" t="inlineStr">
+      <is>
+        <t>Urakkatilanne</t>
+      </is>
+    </nc>
+  </rcc>
 </revisions>
 </file>
 
@@ -1679,10 +2501,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y129"/>
+  <dimension ref="A1:Y130"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="10.1640625" customWidth="1"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="31.6640625" customWidth="1"/>
     <col min="3" max="3" width="14.1640625" customWidth="1"/>
     <col min="4" max="4" width="30.33203125" customWidth="1"/>
@@ -8693,6 +9515,45 @@
       <c r="W129" s="31"/>
       <c r="X129" s="31"/>
       <c r="Y129" s="7"/>
+    </row>
+    <row r="130" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A130" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="B130" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="C130" s="16"/>
+      <c r="D130" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="E130" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="F130" s="31"/>
+      <c r="G130" s="31"/>
+      <c r="H130" s="31"/>
+      <c r="I130" s="31"/>
+      <c r="J130" s="31"/>
+      <c r="K130" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="L130" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="M130" s="31"/>
+      <c r="N130" s="31"/>
+      <c r="O130" s="31"/>
+      <c r="P130" s="31"/>
+      <c r="Q130" s="31"/>
+      <c r="R130" s="31"/>
+      <c r="S130" s="31"/>
+      <c r="T130" s="31"/>
+      <c r="U130" s="31"/>
+      <c r="V130" s="31"/>
+      <c r="W130" s="31"/>
+      <c r="X130" s="31"/>
+      <c r="Y130" s="7"/>
     </row>
   </sheetData>
   <customSheetViews>

</xml_diff>

<commit_message>
Lisää roolit exceliin päällystystysilmoitusten hallinta osioon
</commit_message>
<xml_diff>
--- a/resources/roolit.xlsx
+++ b/resources/roolit.xlsx
@@ -1,46 +1,46 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10908"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/markusva/repos/GitHub/harja/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samumi/Desktop/projektit/harjaroot/harja/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:81_{52E623A0-1020-5F4D-958D-4B687C79E8A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:81_{7CD2B2E3-7BBD-904C-AB1F-9E8264DCD3CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28800" yWindow="-10300" windowWidth="41120" windowHeight="27320" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-10000" yWindow="-28300" windowWidth="51200" windowHeight="28300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Oikeudet" sheetId="1" r:id="rId1"/>
     <sheet name="Roolit" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Oikeudet!$A$5:$Y$132</definedName>
-    <definedName name="Z_1CE83972_B6A5_C44D_86E5_E9D9B38739F4_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$132</definedName>
-    <definedName name="Z_1DD617EE_F308_3E45_A8EF_4713F47FA0DD_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$132</definedName>
-    <definedName name="Z_2064F962_35EF_41F3_8A86_D37B72D177C7_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$132</definedName>
-    <definedName name="Z_3EBD3306_FC69_2148_8542_F6313DC2056F_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$132</definedName>
-    <definedName name="Z_47348D7B_5AFC_4A25_B239_A26E1359728E_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$132</definedName>
-    <definedName name="Z_476C495F_6E55_F04C_8145_4E8EBD6B3DE3_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$132</definedName>
-    <definedName name="Z_5327B0A1_A5FC_7747_93A1_427B210F3DF4_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$132</definedName>
-    <definedName name="Z_56F6E422_2CD8_6B4D_9E39_69A269028D26_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$132</definedName>
-    <definedName name="Z_6AA8E519_028C_D745_9E2E_8FB60E5B789F_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$132</definedName>
-    <definedName name="Z_7A9649F2_657F_9445_B6E6_FE94C6A09957_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$132</definedName>
-    <definedName name="Z_8411E1B5_4691_4435_A9A2_147FF80D0D98_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$132</definedName>
-    <definedName name="Z_843152D8_333A_1941_83E9_0CB5262068A2_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$132</definedName>
-    <definedName name="Z_87BEAE97_700C_BF40_B102_636C54D81F08_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$132</definedName>
-    <definedName name="Z_D01EF3E4_E485_4912_A9DA_396AAE5B8752_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$132</definedName>
-    <definedName name="Z_D57E2FB1_FF7F_8446_9C97_237A4D57F6BE_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$132</definedName>
-    <definedName name="Z_E3BBF62E_A283_4D48_98B7_21A2A94F634F_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$132</definedName>
-    <definedName name="Z_F86DF6F3_8AE5_3A44_B2D2_D623E01AE54F_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$132</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Oikeudet!$A$5:$Y$133</definedName>
+    <definedName name="Z_1CE83972_B6A5_C44D_86E5_E9D9B38739F4_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$133</definedName>
+    <definedName name="Z_1DD617EE_F308_3E45_A8EF_4713F47FA0DD_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$133</definedName>
+    <definedName name="Z_2064F962_35EF_41F3_8A86_D37B72D177C7_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$133</definedName>
+    <definedName name="Z_3EBD3306_FC69_2148_8542_F6313DC2056F_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$133</definedName>
+    <definedName name="Z_47348D7B_5AFC_4A25_B239_A26E1359728E_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$133</definedName>
+    <definedName name="Z_476C495F_6E55_F04C_8145_4E8EBD6B3DE3_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$133</definedName>
+    <definedName name="Z_5327B0A1_A5FC_7747_93A1_427B210F3DF4_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$133</definedName>
+    <definedName name="Z_56F6E422_2CD8_6B4D_9E39_69A269028D26_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$133</definedName>
+    <definedName name="Z_6AA8E519_028C_D745_9E2E_8FB60E5B789F_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$133</definedName>
+    <definedName name="Z_7A9649F2_657F_9445_B6E6_FE94C6A09957_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$133</definedName>
+    <definedName name="Z_8411E1B5_4691_4435_A9A2_147FF80D0D98_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$133</definedName>
+    <definedName name="Z_843152D8_333A_1941_83E9_0CB5262068A2_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$133</definedName>
+    <definedName name="Z_87BEAE97_700C_BF40_B102_636C54D81F08_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$133</definedName>
+    <definedName name="Z_D01EF3E4_E485_4912_A9DA_396AAE5B8752_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$133</definedName>
+    <definedName name="Z_D57E2FB1_FF7F_8446_9C97_237A4D57F6BE_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$133</definedName>
+    <definedName name="Z_E3BBF62E_A283_4D48_98B7_21A2A94F634F_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$133</definedName>
+    <definedName name="Z_F86DF6F3_8AE5_3A44_B2D2_D623E01AE54F_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$133</definedName>
   </definedNames>
   <calcPr calcId="0"/>
   <customWorkbookViews>
+    <customWorkbookView name="Microsoft Office User - Personal View" guid="{843152D8-333A-1941-83E9-0CB5262068A2}" mergeInterval="0" personalView="1" maximized="1" xWindow="-530" yWindow="-1415" windowWidth="2560" windowHeight="1415" tabRatio="500" activeSheetId="1"/>
+    <customWorkbookView name="Jarno Väyrynen - Personal View" guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" mergeInterval="0" personalView="1" xWindow="48" yWindow="25" windowWidth="2512" windowHeight="1336" tabRatio="500" activeSheetId="1"/>
     <customWorkbookView name="Microsoft Office User - Oma näkymä" guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" mergeInterval="0" personalView="1" xWindow="1440" yWindow="-515" windowWidth="2056" windowHeight="1366" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Jarno Väyrynen - Personal View" guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" mergeInterval="0" personalView="1" xWindow="48" yWindow="25" windowWidth="2512" windowHeight="1336" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Microsoft Office User - Personal View" guid="{843152D8-333A-1941-83E9-0CB5262068A2}" mergeInterval="0" personalView="1" maximized="1" xWindow="-530" yWindow="-1415" windowWidth="2560" windowHeight="1415" tabRatio="500" activeSheetId="1"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -109,7 +109,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1948" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1951" uniqueCount="271">
   <si>
     <t xml:space="preserve">Roolimääritysten selitykset: </t>
   </si>
@@ -991,6 +991,9 @@
   </si>
   <si>
     <t>KokonaisurakanPaikkaustenyhteenveto</t>
+  </si>
+  <si>
+    <t>Paallystysilmoitukset</t>
   </si>
 </sst>
 </file>
@@ -1285,7 +1288,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normaali" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1369,7 +1372,7 @@
 </file>
 
 <file path=xl/revisions/revisionHeaders.xml><?xml version="1.0" encoding="utf-8"?>
-<headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" guid="{CFB45395-62D4-124C-9898-DEF874662F1B}" diskRevisions="1" revisionId="183" version="9">
+<headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" guid="{CF3F0B66-D3D6-2C4C-93DF-DEE3169712D4}" diskRevisions="1" revisionId="188" version="11">
   <header guid="{8EBC2E30-8A6E-AD43-9F6F-B4500CF04203}" dateTime="2024-06-11T12:49:05" maxSheetId="3" userName="Jarno Väyrynen" r:id="rId9" minRId="87" maxRId="97">
     <sheetIdMap count="2">
       <sheetId val="1"/>
@@ -1395,6 +1398,18 @@
     </sheetIdMap>
   </header>
   <header guid="{CFB45395-62D4-124C-9898-DEF874662F1B}" dateTime="2024-11-20T15:11:13" maxSheetId="3" userName="Microsoft Office User" r:id="rId13" minRId="111" maxRId="182">
+    <sheetIdMap count="2">
+      <sheetId val="1"/>
+      <sheetId val="2"/>
+    </sheetIdMap>
+  </header>
+  <header guid="{914F1AF8-08B4-0D4C-9E3F-19E7ECD50FAF}" dateTime="2024-12-13T10:42:57" maxSheetId="3" userName="Microsoft Office User" r:id="rId14" minRId="184" maxRId="187">
+    <sheetIdMap count="2">
+      <sheetId val="1"/>
+      <sheetId val="2"/>
+    </sheetIdMap>
+  </header>
+  <header guid="{CF3F0B66-D3D6-2C4C-93DF-DEE3169712D4}" dateTime="2024-12-13T12:53:42" maxSheetId="3" userName="Microsoft Office User" r:id="rId15" minRId="188">
     <sheetIdMap count="2">
       <sheetId val="1"/>
       <sheetId val="2"/>
@@ -4680,6 +4695,50 @@
 </revisions>
 </file>
 
+<file path=xl/revisions/revisionLog5.xml><?xml version="1.0" encoding="utf-8"?>
+<revisions xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <rrc rId="184" sId="1" ref="A131:XFD131" action="insertRow"/>
+  <rcc rId="185" sId="1">
+    <nc r="A131" t="inlineStr">
+      <is>
+        <t>Hallinta</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="186" sId="1">
+    <nc r="D131" t="inlineStr">
+      <is>
+        <t>R*,W*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="187" sId="1">
+    <nc r="B131" t="inlineStr">
+      <is>
+        <t>Paallystysilmoitukset</t>
+      </is>
+    </nc>
+  </rcc>
+</revisions>
+</file>
+
+<file path=xl/revisions/revisionLog6.xml><?xml version="1.0" encoding="utf-8"?>
+<revisions xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <rcc rId="188" sId="1">
+    <oc r="D131" t="inlineStr">
+      <is>
+        <t>R*,W*</t>
+      </is>
+    </oc>
+    <nc r="D131" t="inlineStr">
+      <is>
+        <t>R*,W*,sido*</t>
+      </is>
+    </nc>
+  </rcc>
+</revisions>
+</file>
+
 <file path=xl/revisions/revisionLog9.xml><?xml version="1.0" encoding="utf-8"?>
 <revisions xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <rcc rId="87" sId="1">
@@ -4779,9 +4838,10 @@
 </file>
 
 <file path=xl/revisions/userNames.xml><?xml version="1.0" encoding="utf-8"?>
-<users xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" count="2">
+<users xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" count="3">
   <userInfo guid="{8EBC2E30-8A6E-AD43-9F6F-B4500CF04203}" name="Jarno Väyrynen" id="-589133089" dateTime="2024-06-10T14:55:26"/>
   <userInfo guid="{CFB45395-62D4-124C-9898-DEF874662F1B}" name="Microsoft Office User" id="-296973103" dateTime="2024-11-20T15:04:38"/>
+  <userInfo guid="{CF3F0B66-D3D6-2C4C-93DF-DEE3169712D4}" name="Microsoft Office User" id="-296992802" dateTime="2024-12-13T10:34:14"/>
 </users>
 </file>
 
@@ -4961,7 +5021,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y134"/>
+  <dimension ref="A1:Y135"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -12092,11 +12152,11 @@
         <v>209</v>
       </c>
       <c r="B131" s="11" t="s">
-        <v>229</v>
+        <v>270</v>
       </c>
       <c r="C131" s="12"/>
       <c r="D131" s="12" t="s">
-        <v>41</v>
+        <v>100</v>
       </c>
       <c r="E131" s="12"/>
       <c r="F131" s="12"/>
@@ -12122,136 +12182,169 @@
     </row>
     <row r="132" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A132" s="11" t="s">
-        <v>230</v>
+        <v>209</v>
       </c>
       <c r="B132" s="11" t="s">
-        <v>231</v>
-      </c>
-      <c r="C132" s="16"/>
+        <v>229</v>
+      </c>
+      <c r="C132" s="12"/>
       <c r="D132" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E132" s="16"/>
-      <c r="F132" s="16"/>
-      <c r="G132" s="16"/>
-      <c r="H132" s="16"/>
-      <c r="I132" s="16"/>
-      <c r="J132" s="16"/>
-      <c r="K132" s="16"/>
-      <c r="L132" s="16"/>
-      <c r="M132" s="16"/>
-      <c r="N132" s="16"/>
-      <c r="O132" s="16"/>
-      <c r="P132" s="16"/>
-      <c r="Q132" s="16"/>
-      <c r="R132" s="16"/>
-      <c r="S132" s="16"/>
-      <c r="T132" s="16"/>
-      <c r="U132" s="16"/>
-      <c r="V132" s="16"/>
-      <c r="W132" s="16"/>
-      <c r="X132" s="16"/>
+      <c r="E132" s="12"/>
+      <c r="F132" s="12"/>
+      <c r="G132" s="12"/>
+      <c r="H132" s="12"/>
+      <c r="I132" s="12"/>
+      <c r="J132" s="12"/>
+      <c r="K132" s="12"/>
+      <c r="L132" s="12"/>
+      <c r="M132" s="12"/>
+      <c r="N132" s="12"/>
+      <c r="O132" s="12"/>
+      <c r="P132" s="12"/>
+      <c r="Q132" s="12"/>
+      <c r="R132" s="12"/>
+      <c r="S132" s="12"/>
+      <c r="T132" s="12"/>
+      <c r="U132" s="12"/>
+      <c r="V132" s="12"/>
+      <c r="W132" s="12"/>
+      <c r="X132" s="12"/>
       <c r="Y132" s="7"/>
     </row>
     <row r="133" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A133" s="11" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B133" s="11" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C133" s="16"/>
       <c r="D133" s="12" t="s">
-        <v>234</v>
-      </c>
-      <c r="E133" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="F133" s="31"/>
-      <c r="G133" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="H133" s="31"/>
-      <c r="I133" s="31"/>
-      <c r="J133" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="K133" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="L133" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="M133" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="N133" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="O133" s="31"/>
-      <c r="P133" s="31"/>
-      <c r="Q133" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="R133" s="31" t="s">
-        <v>236</v>
-      </c>
-      <c r="S133" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="T133" s="31"/>
-      <c r="U133" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="V133" s="31"/>
-      <c r="W133" s="31"/>
-      <c r="X133" s="31"/>
+        <v>41</v>
+      </c>
+      <c r="E133" s="16"/>
+      <c r="F133" s="16"/>
+      <c r="G133" s="16"/>
+      <c r="H133" s="16"/>
+      <c r="I133" s="16"/>
+      <c r="J133" s="16"/>
+      <c r="K133" s="16"/>
+      <c r="L133" s="16"/>
+      <c r="M133" s="16"/>
+      <c r="N133" s="16"/>
+      <c r="O133" s="16"/>
+      <c r="P133" s="16"/>
+      <c r="Q133" s="16"/>
+      <c r="R133" s="16"/>
+      <c r="S133" s="16"/>
+      <c r="T133" s="16"/>
+      <c r="U133" s="16"/>
+      <c r="V133" s="16"/>
+      <c r="W133" s="16"/>
+      <c r="X133" s="16"/>
       <c r="Y133" s="7"/>
     </row>
     <row r="134" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A134" s="11" t="s">
-        <v>265</v>
+        <v>232</v>
       </c>
       <c r="B134" s="11" t="s">
-        <v>265</v>
+        <v>233</v>
       </c>
       <c r="C134" s="16"/>
       <c r="D134" s="12" t="s">
-        <v>38</v>
+        <v>234</v>
       </c>
       <c r="E134" s="31" t="s">
-        <v>38</v>
+        <v>234</v>
       </c>
       <c r="F134" s="31"/>
-      <c r="G134" s="31"/>
+      <c r="G134" s="31" t="s">
+        <v>234</v>
+      </c>
       <c r="H134" s="31"/>
       <c r="I134" s="31"/>
-      <c r="J134" s="31"/>
+      <c r="J134" s="31" t="s">
+        <v>235</v>
+      </c>
       <c r="K134" s="31" t="s">
-        <v>38</v>
+        <v>234</v>
       </c>
       <c r="L134" s="31" t="s">
-        <v>38</v>
-      </c>
-      <c r="M134" s="31"/>
-      <c r="N134" s="31"/>
+        <v>234</v>
+      </c>
+      <c r="M134" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="N134" s="31" t="s">
+        <v>234</v>
+      </c>
       <c r="O134" s="31"/>
       <c r="P134" s="31"/>
-      <c r="Q134" s="31"/>
-      <c r="R134" s="31"/>
-      <c r="S134" s="31"/>
+      <c r="Q134" s="31" t="s">
+        <v>235</v>
+      </c>
+      <c r="R134" s="31" t="s">
+        <v>236</v>
+      </c>
+      <c r="S134" s="31" t="s">
+        <v>235</v>
+      </c>
       <c r="T134" s="31"/>
-      <c r="U134" s="31"/>
+      <c r="U134" s="31" t="s">
+        <v>235</v>
+      </c>
       <c r="V134" s="31"/>
       <c r="W134" s="31"/>
       <c r="X134" s="31"/>
       <c r="Y134" s="7"/>
     </row>
+    <row r="135" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A135" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="B135" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="C135" s="16"/>
+      <c r="D135" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="E135" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="F135" s="31"/>
+      <c r="G135" s="31"/>
+      <c r="H135" s="31"/>
+      <c r="I135" s="31"/>
+      <c r="J135" s="31"/>
+      <c r="K135" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="L135" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="M135" s="31"/>
+      <c r="N135" s="31"/>
+      <c r="O135" s="31"/>
+      <c r="P135" s="31"/>
+      <c r="Q135" s="31"/>
+      <c r="R135" s="31"/>
+      <c r="S135" s="31"/>
+      <c r="T135" s="31"/>
+      <c r="U135" s="31"/>
+      <c r="V135" s="31"/>
+      <c r="W135" s="31"/>
+      <c r="X135" s="31"/>
+      <c r="Y135" s="7"/>
+    </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="130">
-      <pane xSplit="2" ySplit="6" topLeftCell="C53" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="B71" sqref="B71"/>
+    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="115">
+      <pane xSplit="2" ySplit="6" topLeftCell="C86" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="B126" sqref="B126"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
@@ -12261,9 +12354,9 @@
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
-    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="115">
-      <pane xSplit="2" ySplit="6" topLeftCell="C86" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="B126" sqref="B126"/>
+    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="130">
+      <pane xSplit="2" ySplit="6" topLeftCell="C53" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="B71" sqref="B71"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
@@ -12615,7 +12708,7 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="150">
+    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="150">
       <selection activeCell="A22" sqref="A22"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -12625,7 +12718,7 @@
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
-    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="150">
+    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="150">
       <selection activeCell="A22" sqref="A22"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Piilota pohjavesirapsa muilta kuin JVH:lta
</commit_message>
<xml_diff>
--- a/resources/roolit.xlsx
+++ b/resources/roolit.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10908"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samumi/Desktop/projektit/harjaroot/harja/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jarno.vayrynen/harja/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:81_{7CD2B2E3-7BBD-904C-AB1F-9E8264DCD3CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:81_{3E2764DF-46E8-2941-BD8D-D71DB856DE8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10000" yWindow="-28300" windowWidth="51200" windowHeight="28300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="960" yWindow="500" windowWidth="50240" windowHeight="26600" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Oikeudet" sheetId="1" r:id="rId1"/>
@@ -38,9 +38,9 @@
   </definedNames>
   <calcPr calcId="0"/>
   <customWorkbookViews>
+    <customWorkbookView name="Microsoft Office User - Oma näkymä" guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" mergeInterval="0" personalView="1" xWindow="1440" yWindow="-515" windowWidth="2056" windowHeight="1366" tabRatio="500" activeSheetId="1"/>
+    <customWorkbookView name="Jarno Väyrynen - Personal View" guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" mergeInterval="0" personalView="1" xWindow="48" yWindow="25" windowWidth="2512" windowHeight="1336" tabRatio="500" activeSheetId="1"/>
     <customWorkbookView name="Microsoft Office User - Personal View" guid="{843152D8-333A-1941-83E9-0CB5262068A2}" mergeInterval="0" personalView="1" maximized="1" xWindow="-530" yWindow="-1415" windowWidth="2560" windowHeight="1415" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Jarno Väyrynen - Personal View" guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" mergeInterval="0" personalView="1" xWindow="48" yWindow="25" windowWidth="2512" windowHeight="1336" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Microsoft Office User - Oma näkymä" guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" mergeInterval="0" personalView="1" xWindow="1440" yWindow="-515" windowWidth="2056" windowHeight="1366" tabRatio="500" activeSheetId="1"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -109,7 +109,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1951" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1932" uniqueCount="271">
   <si>
     <t xml:space="preserve">Roolimääritysten selitykset: </t>
   </si>
@@ -1372,7 +1372,7 @@
 </file>
 
 <file path=xl/revisions/revisionHeaders.xml><?xml version="1.0" encoding="utf-8"?>
-<headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" guid="{CF3F0B66-D3D6-2C4C-93DF-DEE3169712D4}" diskRevisions="1" revisionId="188" version="11">
+<headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" guid="{64AC07D8-8D49-4F46-96EF-A9E3AD0E8431}" diskRevisions="1" revisionId="207" version="12">
   <header guid="{8EBC2E30-8A6E-AD43-9F6F-B4500CF04203}" dateTime="2024-06-11T12:49:05" maxSheetId="3" userName="Jarno Väyrynen" r:id="rId9" minRId="87" maxRId="97">
     <sheetIdMap count="2">
       <sheetId val="1"/>
@@ -1410,6 +1410,12 @@
     </sheetIdMap>
   </header>
   <header guid="{CF3F0B66-D3D6-2C4C-93DF-DEE3169712D4}" dateTime="2024-12-13T12:53:42" maxSheetId="3" userName="Microsoft Office User" r:id="rId15" minRId="188">
+    <sheetIdMap count="2">
+      <sheetId val="1"/>
+      <sheetId val="2"/>
+    </sheetIdMap>
+  </header>
+  <header guid="{64AC07D8-8D49-4F46-96EF-A9E3AD0E8431}" dateTime="2025-02-12T12:59:07" maxSheetId="3" userName="Jarno Väyrynen" r:id="rId16" minRId="189" maxRId="207">
     <sheetIdMap count="2">
       <sheetId val="1"/>
       <sheetId val="2"/>
@@ -4739,6 +4745,163 @@
 </revisions>
 </file>
 
+<file path=xl/revisions/revisionLog7.xml><?xml version="1.0" encoding="utf-8"?>
+<revisions xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <rcc rId="189" sId="1">
+    <oc r="E102" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </oc>
+    <nc r="E102"/>
+  </rcc>
+  <rcc rId="190" sId="1">
+    <oc r="F102" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </oc>
+    <nc r="F102"/>
+  </rcc>
+  <rcc rId="191" sId="1">
+    <oc r="G102" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </oc>
+    <nc r="G102"/>
+  </rcc>
+  <rcc rId="192" sId="1">
+    <oc r="H102" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </oc>
+    <nc r="H102"/>
+  </rcc>
+  <rcc rId="193" sId="1">
+    <oc r="I102" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </oc>
+    <nc r="I102"/>
+  </rcc>
+  <rcc rId="194" sId="1">
+    <oc r="J102" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </oc>
+    <nc r="J102"/>
+  </rcc>
+  <rcc rId="195" sId="1">
+    <oc r="K102" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </oc>
+    <nc r="K102"/>
+  </rcc>
+  <rcc rId="196" sId="1">
+    <oc r="L102" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </oc>
+    <nc r="L102"/>
+  </rcc>
+  <rcc rId="197" sId="1">
+    <oc r="M102" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </oc>
+    <nc r="M102"/>
+  </rcc>
+  <rcc rId="198" sId="1">
+    <oc r="N102" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </oc>
+    <nc r="N102"/>
+  </rcc>
+  <rcc rId="199" sId="1">
+    <oc r="O102" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </oc>
+    <nc r="O102"/>
+  </rcc>
+  <rcc rId="200" sId="1">
+    <oc r="P102" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </oc>
+    <nc r="P102"/>
+  </rcc>
+  <rcc rId="201" sId="1">
+    <oc r="Q102" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </oc>
+    <nc r="Q102"/>
+  </rcc>
+  <rcc rId="202" sId="1">
+    <oc r="R102" t="inlineStr">
+      <is>
+        <t>R+</t>
+      </is>
+    </oc>
+    <nc r="R102"/>
+  </rcc>
+  <rcc rId="203" sId="1">
+    <oc r="S102" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </oc>
+    <nc r="S102"/>
+  </rcc>
+  <rcc rId="204" sId="1">
+    <oc r="T102" t="inlineStr">
+      <is>
+        <t>R+</t>
+      </is>
+    </oc>
+    <nc r="T102"/>
+  </rcc>
+  <rcc rId="205" sId="1">
+    <oc r="U102" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </oc>
+    <nc r="U102"/>
+  </rcc>
+  <rcc rId="206" sId="1">
+    <oc r="V102" t="inlineStr">
+      <is>
+        <t>R+</t>
+      </is>
+    </oc>
+    <nc r="V102"/>
+  </rcc>
+  <rcc rId="207" sId="1">
+    <oc r="X102" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </oc>
+    <nc r="X102"/>
+  </rcc>
+</revisions>
+</file>
+
 <file path=xl/revisions/revisionLog9.xml><?xml version="1.0" encoding="utf-8"?>
 <revisions xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <rcc rId="87" sId="1">
@@ -4837,11 +5000,12 @@
 </revisions>
 </file>
 
-<file path=xl/revisions/userNames.xml><?xml version="1.0" encoding="utf-8"?>
-<users xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" count="3">
+<file path=xl/revisions/userNames1.xml><?xml version="1.0" encoding="utf-8"?>
+<users xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" count="4">
   <userInfo guid="{8EBC2E30-8A6E-AD43-9F6F-B4500CF04203}" name="Jarno Väyrynen" id="-589133089" dateTime="2024-06-10T14:55:26"/>
   <userInfo guid="{CFB45395-62D4-124C-9898-DEF874662F1B}" name="Microsoft Office User" id="-296973103" dateTime="2024-11-20T15:04:38"/>
   <userInfo guid="{CF3F0B66-D3D6-2C4C-93DF-DEE3169712D4}" name="Microsoft Office User" id="-296992802" dateTime="2024-12-13T10:34:14"/>
+  <userInfo guid="{64AC07D8-8D49-4F46-96EF-A9E3AD0E8431}" name="Jarno Väyrynen" id="-589128654" dateTime="2025-02-12T12:58:37"/>
 </users>
 </file>
 
@@ -10845,64 +11009,26 @@
       <c r="D102" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="E102" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="F102" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="G102" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="H102" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="I102" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="J102" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="K102" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="L102" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="M102" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="N102" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="O102" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="P102" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q102" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="R102" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="S102" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="T102" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="U102" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="V102" s="12" t="s">
-        <v>44</v>
-      </c>
+      <c r="E102" s="12"/>
+      <c r="F102" s="12"/>
+      <c r="G102" s="12"/>
+      <c r="H102" s="12"/>
+      <c r="I102" s="12"/>
+      <c r="J102" s="12"/>
+      <c r="K102" s="12"/>
+      <c r="L102" s="12"/>
+      <c r="M102" s="12"/>
+      <c r="N102" s="12"/>
+      <c r="O102" s="12"/>
+      <c r="P102" s="12"/>
+      <c r="Q102" s="12"/>
+      <c r="R102" s="12"/>
+      <c r="S102" s="12"/>
+      <c r="T102" s="12"/>
+      <c r="U102" s="12"/>
+      <c r="V102" s="12"/>
       <c r="W102" s="12"/>
-      <c r="X102" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="X102" s="12"/>
       <c r="Y102" s="13"/>
     </row>
     <row r="103" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -12342,9 +12468,9 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="115">
-      <pane xSplit="2" ySplit="6" topLeftCell="C86" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="B126" sqref="B126"/>
+    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="130">
+      <pane xSplit="2" ySplit="6" topLeftCell="C53" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="B71" sqref="B71"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
@@ -12354,9 +12480,9 @@
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
-    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="130">
-      <pane xSplit="2" ySplit="6" topLeftCell="C53" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="B71" sqref="B71"/>
+    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="115">
+      <pane xSplit="2" ySplit="6" topLeftCell="C86" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="B126" sqref="B126"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
@@ -12708,7 +12834,7 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="150">
+    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="150">
       <selection activeCell="A22" sqref="A22"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -12718,7 +12844,7 @@
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
-    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="150">
+    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="150">
       <selection activeCell="A22" sqref="A22"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Harja-1210: Tiemerkintöjen korjauskustannukset. Testit puuttuu
</commit_message>
<xml_diff>
--- a/resources/roolit.xlsx
+++ b/resources/roolit.xlsx
@@ -1,46 +1,46 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jarno.vayrynen/harja/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lauri.nayha/Projects/harja/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:81_{3E2764DF-46E8-2941-BD8D-D71DB856DE8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:81_{A8790524-4076-984A-9AA0-56B44D9CB46B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="960" yWindow="500" windowWidth="50240" windowHeight="26600" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="98860" yWindow="2380" windowWidth="34560" windowHeight="14920" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Oikeudet" sheetId="1" r:id="rId1"/>
     <sheet name="Roolit" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Oikeudet!$A$5:$Y$133</definedName>
-    <definedName name="Z_1CE83972_B6A5_C44D_86E5_E9D9B38739F4_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$133</definedName>
-    <definedName name="Z_1DD617EE_F308_3E45_A8EF_4713F47FA0DD_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$133</definedName>
-    <definedName name="Z_2064F962_35EF_41F3_8A86_D37B72D177C7_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$133</definedName>
-    <definedName name="Z_3EBD3306_FC69_2148_8542_F6313DC2056F_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$133</definedName>
-    <definedName name="Z_47348D7B_5AFC_4A25_B239_A26E1359728E_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$133</definedName>
-    <definedName name="Z_476C495F_6E55_F04C_8145_4E8EBD6B3DE3_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$133</definedName>
-    <definedName name="Z_5327B0A1_A5FC_7747_93A1_427B210F3DF4_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$133</definedName>
-    <definedName name="Z_56F6E422_2CD8_6B4D_9E39_69A269028D26_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$133</definedName>
-    <definedName name="Z_6AA8E519_028C_D745_9E2E_8FB60E5B789F_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$133</definedName>
-    <definedName name="Z_7A9649F2_657F_9445_B6E6_FE94C6A09957_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$133</definedName>
-    <definedName name="Z_8411E1B5_4691_4435_A9A2_147FF80D0D98_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$133</definedName>
-    <definedName name="Z_843152D8_333A_1941_83E9_0CB5262068A2_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$133</definedName>
-    <definedName name="Z_87BEAE97_700C_BF40_B102_636C54D81F08_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$133</definedName>
-    <definedName name="Z_D01EF3E4_E485_4912_A9DA_396AAE5B8752_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$133</definedName>
-    <definedName name="Z_D57E2FB1_FF7F_8446_9C97_237A4D57F6BE_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$133</definedName>
-    <definedName name="Z_E3BBF62E_A283_4D48_98B7_21A2A94F634F_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$133</definedName>
-    <definedName name="Z_F86DF6F3_8AE5_3A44_B2D2_D623E01AE54F_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$133</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_1CE83972_B6A5_C44D_86E5_E9D9B38739F4_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_1DD617EE_F308_3E45_A8EF_4713F47FA0DD_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_2064F962_35EF_41F3_8A86_D37B72D177C7_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_3EBD3306_FC69_2148_8542_F6313DC2056F_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_47348D7B_5AFC_4A25_B239_A26E1359728E_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_476C495F_6E55_F04C_8145_4E8EBD6B3DE3_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_5327B0A1_A5FC_7747_93A1_427B210F3DF4_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_56F6E422_2CD8_6B4D_9E39_69A269028D26_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_6AA8E519_028C_D745_9E2E_8FB60E5B789F_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_7A9649F2_657F_9445_B6E6_FE94C6A09957_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_8411E1B5_4691_4435_A9A2_147FF80D0D98_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_843152D8_333A_1941_83E9_0CB5262068A2_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_87BEAE97_700C_BF40_B102_636C54D81F08_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_D01EF3E4_E485_4912_A9DA_396AAE5B8752_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_D57E2FB1_FF7F_8446_9C97_237A4D57F6BE_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_E3BBF62E_A283_4D48_98B7_21A2A94F634F_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_F86DF6F3_8AE5_3A44_B2D2_D623E01AE54F_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
   </definedNames>
   <calcPr calcId="0"/>
   <customWorkbookViews>
+    <customWorkbookView name="Microsoft Office User - Personal View" guid="{843152D8-333A-1941-83E9-0CB5262068A2}" mergeInterval="0" personalView="1" xWindow="4943" yWindow="119" windowWidth="1728" windowHeight="746" tabRatio="500" activeSheetId="1"/>
+    <customWorkbookView name="Jarno Väyrynen - Personal View" guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" mergeInterval="0" personalView="1" xWindow="48" yWindow="25" windowWidth="2512" windowHeight="1336" tabRatio="500" activeSheetId="1"/>
     <customWorkbookView name="Microsoft Office User - Oma näkymä" guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" mergeInterval="0" personalView="1" xWindow="1440" yWindow="-515" windowWidth="2056" windowHeight="1366" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Jarno Väyrynen - Personal View" guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" mergeInterval="0" personalView="1" xWindow="48" yWindow="25" windowWidth="2512" windowHeight="1336" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Microsoft Office User - Personal View" guid="{843152D8-333A-1941-83E9-0CB5262068A2}" mergeInterval="0" personalView="1" maximized="1" xWindow="-530" yWindow="-1415" windowWidth="2560" windowHeight="1415" tabRatio="500" activeSheetId="1"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -85,6 +85,7 @@
         <r>
           <rPr>
             <sz val="10"/>
+            <color rgb="FF000000"/>
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
@@ -109,7 +110,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1932" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1947" uniqueCount="273">
   <si>
     <t xml:space="preserve">Roolimääritysten selitykset: </t>
   </si>
@@ -995,12 +996,18 @@
   <si>
     <t>Paallystysilmoitukset</t>
   </si>
+  <si>
+    <t>Tiemerkinnän kustannukset</t>
+  </si>
+  <si>
+    <t>Koitetaan pärjätä yhdellä rivillä kaikkien välilehtien osalta</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1066,6 +1073,12 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="7">
@@ -1372,7 +1385,7 @@
 </file>
 
 <file path=xl/revisions/revisionHeaders.xml><?xml version="1.0" encoding="utf-8"?>
-<headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" guid="{64AC07D8-8D49-4F46-96EF-A9E3AD0E8431}" diskRevisions="1" revisionId="207" version="12">
+<headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" guid="{16592C61-0221-A548-A820-56B21F0EE301}" diskRevisions="1" revisionId="224" version="13">
   <header guid="{8EBC2E30-8A6E-AD43-9F6F-B4500CF04203}" dateTime="2024-06-11T12:49:05" maxSheetId="3" userName="Jarno Väyrynen" r:id="rId9" minRId="87" maxRId="97">
     <sheetIdMap count="2">
       <sheetId val="1"/>
@@ -1416,6 +1429,12 @@
     </sheetIdMap>
   </header>
   <header guid="{64AC07D8-8D49-4F46-96EF-A9E3AD0E8431}" dateTime="2025-02-12T12:59:07" maxSheetId="3" userName="Jarno Väyrynen" r:id="rId16" minRId="189" maxRId="207">
+    <sheetIdMap count="2">
+      <sheetId val="1"/>
+      <sheetId val="2"/>
+    </sheetIdMap>
+  </header>
+  <header guid="{16592C61-0221-A548-A820-56B21F0EE301}" dateTime="2025-02-19T11:57:01" maxSheetId="3" userName="Microsoft Office User" r:id="rId17" minRId="208" maxRId="223">
     <sheetIdMap count="2">
       <sheetId val="1"/>
       <sheetId val="2"/>
@@ -4902,6 +4921,123 @@
 </revisions>
 </file>
 
+<file path=xl/revisions/revisionLog8.xml><?xml version="1.0" encoding="utf-8"?>
+<revisions xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <rrc rId="208" sId="1" ref="A37:XFD37" action="insertRow"/>
+  <rcc rId="209" sId="1">
+    <nc r="A37" t="inlineStr">
+      <is>
+        <t>Urakat</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="210" sId="1">
+    <nc r="B37" t="inlineStr">
+      <is>
+        <t>Tiemerkinnän kustannukset</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="211" sId="1">
+    <nc r="D37" t="inlineStr">
+      <is>
+        <t>R*,W*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="212" sId="1">
+    <nc r="E37" t="inlineStr">
+      <is>
+        <t>R*,W*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="213" sId="1">
+    <nc r="F37" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="214" sId="1">
+    <nc r="J37" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="215" sId="1">
+    <nc r="K37" t="inlineStr">
+      <is>
+        <t>R*,W*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="216" sId="1">
+    <nc r="L37" t="inlineStr">
+      <is>
+        <t>R*,W</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="217" sId="1">
+    <nc r="M37" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="218" sId="1">
+    <nc r="N37" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="219" sId="1">
+    <nc r="R37" t="inlineStr">
+      <is>
+        <t>R+,W+</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="220" sId="1">
+    <nc r="S37" t="inlineStr">
+      <is>
+        <t>R,W</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="221" sId="1">
+    <nc r="U37" t="inlineStr">
+      <is>
+        <t>R,W</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="222" sId="1">
+    <nc r="V37" t="inlineStr">
+      <is>
+        <t>R+</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="223" sId="1">
+    <nc r="Y37" t="inlineStr">
+      <is>
+        <t>Koitetaan pärjätä yhdellä rivillä kaikkien välilehtien osalta</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcv guid="{843152D8-333A-1941-83E9-0CB5262068A2}" action="delete"/>
+  <rdn rId="0" localSheetId="1" customView="1" name="Z_843152D8_333A_1941_83E9_0CB5262068A2_.wvu.FilterData" hidden="1" oldHidden="1">
+    <formula>Oikeudet!$A$5:$Y$134</formula>
+    <oldFormula>Oikeudet!$A$5:$Y$134</oldFormula>
+  </rdn>
+  <rcv guid="{843152D8-333A-1941-83E9-0CB5262068A2}" action="add"/>
+</revisions>
+</file>
+
 <file path=xl/revisions/revisionLog9.xml><?xml version="1.0" encoding="utf-8"?>
 <revisions xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <rcc rId="87" sId="1">
@@ -5000,7 +5136,7 @@
 </revisions>
 </file>
 
-<file path=xl/revisions/userNames1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/revisions/userNames.xml><?xml version="1.0" encoding="utf-8"?>
 <users xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" count="4">
   <userInfo guid="{8EBC2E30-8A6E-AD43-9F6F-B4500CF04203}" name="Jarno Väyrynen" id="-589133089" dateTime="2024-06-10T14:55:26"/>
   <userInfo guid="{CFB45395-62D4-124C-9898-DEF874662F1B}" name="Microsoft Office User" id="-296973103" dateTime="2024-11-20T15:04:38"/>
@@ -5185,7 +5321,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y135"/>
+  <dimension ref="A1:Y136"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -7179,15 +7315,15 @@
       <c r="A37" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B37" s="11" t="s">
-        <v>91</v>
+      <c r="B37" s="16" t="s">
+        <v>271</v>
       </c>
       <c r="C37" s="12"/>
       <c r="D37" s="12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E37" s="12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F37" s="12" t="s">
         <v>38</v>
@@ -7199,138 +7335,130 @@
         <v>39</v>
       </c>
       <c r="K37" s="12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="L37" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="M37" s="12"/>
+        <v>37</v>
+      </c>
+      <c r="M37" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="N37" s="12" t="s">
         <v>38</v>
       </c>
       <c r="O37" s="12"/>
       <c r="P37" s="12"/>
-      <c r="Q37" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="Q37" s="12"/>
       <c r="R37" s="12" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="S37" s="12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="T37" s="12"/>
-      <c r="U37" s="12"/>
+      <c r="U37" s="12" t="s">
+        <v>40</v>
+      </c>
       <c r="V37" s="12" t="s">
         <v>44</v>
       </c>
       <c r="W37" s="12"/>
       <c r="X37" s="12"/>
-      <c r="Y37" s="13"/>
+      <c r="Y37" s="13" t="s">
+        <v>272</v>
+      </c>
     </row>
     <row r="38" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A38" s="11" t="s">
         <v>34</v>
       </c>
       <c r="B38" s="11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C38" s="12"/>
       <c r="D38" s="12" t="s">
-        <v>93</v>
+        <v>38</v>
       </c>
       <c r="E38" s="12" t="s">
-        <v>94</v>
+        <v>38</v>
       </c>
       <c r="F38" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G38" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="H38" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="I38" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="J38" s="20" t="s">
-        <v>95</v>
+      <c r="G38" s="12"/>
+      <c r="H38" s="12"/>
+      <c r="I38" s="12"/>
+      <c r="J38" s="12" t="s">
+        <v>39</v>
       </c>
       <c r="K38" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="L38" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="M38" s="12" t="s">
-        <v>40</v>
-      </c>
+        <v>38</v>
+      </c>
+      <c r="M38" s="12"/>
       <c r="N38" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="O38" s="12" t="s">
-        <v>38</v>
-      </c>
+      <c r="O38" s="12"/>
       <c r="P38" s="12"/>
-      <c r="Q38" s="20" t="s">
-        <v>95</v>
+      <c r="Q38" s="12" t="s">
+        <v>39</v>
       </c>
       <c r="R38" s="12" t="s">
-        <v>96</v>
+        <v>44</v>
       </c>
       <c r="S38" s="12" t="s">
-        <v>97</v>
-      </c>
-      <c r="T38" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="U38" s="12" t="s">
-        <v>39</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="T38" s="12"/>
+      <c r="U38" s="12"/>
       <c r="V38" s="12" t="s">
         <v>44</v>
       </c>
       <c r="W38" s="12"/>
       <c r="X38" s="12"/>
-      <c r="Y38" s="13" t="s">
-        <v>98</v>
-      </c>
+      <c r="Y38" s="13"/>
     </row>
     <row r="39" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A39" s="11" t="s">
         <v>34</v>
       </c>
       <c r="B39" s="11" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="C39" s="12"/>
       <c r="D39" s="12" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="E39" s="12" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="F39" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G39" s="12"/>
+      <c r="G39" s="12" t="s">
+        <v>37</v>
+      </c>
       <c r="H39" s="12" t="s">
         <v>38</v>
       </c>
       <c r="I39" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="J39" s="12" t="s">
+      <c r="J39" s="20" t="s">
+        <v>95</v>
+      </c>
+      <c r="K39" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="L39" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="M39" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="K39" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="L39" s="12" t="s">
-        <v>101</v>
-      </c>
-      <c r="M39" s="12"/>
       <c r="N39" s="12" t="s">
         <v>38</v>
       </c>
@@ -7338,14 +7466,14 @@
         <v>38</v>
       </c>
       <c r="P39" s="12"/>
-      <c r="Q39" s="12" t="s">
-        <v>103</v>
+      <c r="Q39" s="20" t="s">
+        <v>95</v>
       </c>
       <c r="R39" s="12" t="s">
-        <v>42</v>
+        <v>96</v>
       </c>
       <c r="S39" s="12" t="s">
-        <v>40</v>
+        <v>97</v>
       </c>
       <c r="T39" s="12" t="s">
         <v>44</v>
@@ -7358,28 +7486,28 @@
       </c>
       <c r="W39" s="12"/>
       <c r="X39" s="12"/>
-      <c r="Y39" s="13"/>
+      <c r="Y39" s="13" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="40" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A40" s="11" t="s">
         <v>34</v>
       </c>
       <c r="B40" s="11" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="C40" s="12"/>
       <c r="D40" s="12" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="E40" s="12" t="s">
-        <v>37</v>
+        <v>101</v>
       </c>
       <c r="F40" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G40" s="12" t="s">
-        <v>106</v>
-      </c>
+      <c r="G40" s="12"/>
       <c r="H40" s="12" t="s">
         <v>38</v>
       </c>
@@ -7387,13 +7515,13 @@
         <v>39</v>
       </c>
       <c r="J40" s="12" t="s">
-        <v>71</v>
+        <v>40</v>
       </c>
       <c r="K40" s="12" t="s">
-        <v>41</v>
+        <v>102</v>
       </c>
       <c r="L40" s="12" t="s">
-        <v>72</v>
+        <v>101</v>
       </c>
       <c r="M40" s="12"/>
       <c r="N40" s="12" t="s">
@@ -7404,7 +7532,7 @@
       </c>
       <c r="P40" s="12"/>
       <c r="Q40" s="12" t="s">
-        <v>71</v>
+        <v>103</v>
       </c>
       <c r="R40" s="12" t="s">
         <v>42</v>
@@ -7430,19 +7558,21 @@
         <v>34</v>
       </c>
       <c r="B41" s="11" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C41" s="12"/>
       <c r="D41" s="12" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="E41" s="12" t="s">
-        <v>101</v>
+        <v>37</v>
       </c>
       <c r="F41" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G41" s="12"/>
+      <c r="G41" s="12" t="s">
+        <v>106</v>
+      </c>
       <c r="H41" s="12" t="s">
         <v>38</v>
       </c>
@@ -7450,13 +7580,13 @@
         <v>39</v>
       </c>
       <c r="J41" s="12" t="s">
-        <v>40</v>
+        <v>71</v>
       </c>
       <c r="K41" s="12" t="s">
-        <v>102</v>
+        <v>41</v>
       </c>
       <c r="L41" s="12" t="s">
-        <v>101</v>
+        <v>72</v>
       </c>
       <c r="M41" s="12"/>
       <c r="N41" s="12" t="s">
@@ -7467,7 +7597,7 @@
       </c>
       <c r="P41" s="12"/>
       <c r="Q41" s="12" t="s">
-        <v>103</v>
+        <v>71</v>
       </c>
       <c r="R41" s="12" t="s">
         <v>42</v>
@@ -7493,14 +7623,14 @@
         <v>34</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C42" s="12"/>
       <c r="D42" s="12" t="s">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="E42" s="12" t="s">
-        <v>37</v>
+        <v>101</v>
       </c>
       <c r="F42" s="12" t="s">
         <v>38</v>
@@ -7516,10 +7646,10 @@
         <v>40</v>
       </c>
       <c r="K42" s="12" t="s">
-        <v>41</v>
+        <v>102</v>
       </c>
       <c r="L42" s="12" t="s">
-        <v>37</v>
+        <v>101</v>
       </c>
       <c r="M42" s="12"/>
       <c r="N42" s="12" t="s">
@@ -7530,7 +7660,7 @@
       </c>
       <c r="P42" s="12"/>
       <c r="Q42" s="12" t="s">
-        <v>40</v>
+        <v>103</v>
       </c>
       <c r="R42" s="12" t="s">
         <v>42</v>
@@ -7556,14 +7686,14 @@
         <v>34</v>
       </c>
       <c r="B43" s="11" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C43" s="12"/>
       <c r="D43" s="12" t="s">
-        <v>110</v>
+        <v>70</v>
       </c>
       <c r="E43" s="12" t="s">
-        <v>111</v>
+        <v>37</v>
       </c>
       <c r="F43" s="12" t="s">
         <v>38</v>
@@ -7579,10 +7709,10 @@
         <v>40</v>
       </c>
       <c r="K43" s="12" t="s">
-        <v>112</v>
+        <v>41</v>
       </c>
       <c r="L43" s="12" t="s">
-        <v>111</v>
+        <v>37</v>
       </c>
       <c r="M43" s="12"/>
       <c r="N43" s="12" t="s">
@@ -7596,10 +7726,10 @@
         <v>40</v>
       </c>
       <c r="R43" s="12" t="s">
-        <v>113</v>
+        <v>42</v>
       </c>
       <c r="S43" s="12" t="s">
-        <v>114</v>
+        <v>40</v>
       </c>
       <c r="T43" s="12" t="s">
         <v>44</v>
@@ -7619,14 +7749,14 @@
         <v>34</v>
       </c>
       <c r="B44" s="11" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="C44" s="12"/>
       <c r="D44" s="12" t="s">
-        <v>41</v>
+        <v>110</v>
       </c>
       <c r="E44" s="12" t="s">
-        <v>37</v>
+        <v>111</v>
       </c>
       <c r="F44" s="12" t="s">
         <v>38</v>
@@ -7642,10 +7772,10 @@
         <v>40</v>
       </c>
       <c r="K44" s="12" t="s">
-        <v>41</v>
+        <v>112</v>
       </c>
       <c r="L44" s="12" t="s">
-        <v>37</v>
+        <v>111</v>
       </c>
       <c r="M44" s="12"/>
       <c r="N44" s="12" t="s">
@@ -7659,10 +7789,10 @@
         <v>40</v>
       </c>
       <c r="R44" s="12" t="s">
-        <v>42</v>
+        <v>113</v>
       </c>
       <c r="S44" s="12" t="s">
-        <v>40</v>
+        <v>114</v>
       </c>
       <c r="T44" s="12" t="s">
         <v>44</v>
@@ -7675,14 +7805,14 @@
       </c>
       <c r="W44" s="12"/>
       <c r="X44" s="12"/>
-      <c r="Y44" s="7"/>
+      <c r="Y44" s="13"/>
     </row>
     <row r="45" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A45" s="11" t="s">
         <v>34</v>
       </c>
       <c r="B45" s="11" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C45" s="12"/>
       <c r="D45" s="12" t="s">
@@ -7745,7 +7875,7 @@
         <v>34</v>
       </c>
       <c r="B46" s="11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C46" s="12"/>
       <c r="D46" s="12" t="s">
@@ -7808,7 +7938,7 @@
         <v>34</v>
       </c>
       <c r="B47" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C47" s="12"/>
       <c r="D47" s="12" t="s">
@@ -7820,14 +7950,12 @@
       <c r="F47" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G47" s="12" t="s">
-        <v>68</v>
-      </c>
+      <c r="G47" s="12"/>
       <c r="H47" s="12" t="s">
         <v>38</v>
       </c>
       <c r="I47" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J47" s="12" t="s">
         <v>40</v>
@@ -7836,20 +7964,16 @@
         <v>41</v>
       </c>
       <c r="L47" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="M47" s="12" t="s">
-        <v>40</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="M47" s="12"/>
       <c r="N47" s="12" t="s">
         <v>38</v>
       </c>
       <c r="O47" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="P47" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="P47" s="12"/>
       <c r="Q47" s="12" t="s">
         <v>40</v>
       </c>
@@ -7863,85 +7987,101 @@
         <v>44</v>
       </c>
       <c r="U47" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="V47" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="W47" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="X47" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y47" s="13"/>
-    </row>
-    <row r="48" spans="1:25" ht="28" x14ac:dyDescent="0.15">
+      <c r="W47" s="12"/>
+      <c r="X47" s="12"/>
+      <c r="Y47" s="7"/>
+    </row>
+    <row r="48" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A48" s="11" t="s">
         <v>34</v>
       </c>
       <c r="B48" s="11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C48" s="12"/>
-      <c r="D48" s="21" t="s">
-        <v>120</v>
-      </c>
-      <c r="E48" s="21" t="s">
-        <v>121</v>
+      <c r="D48" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="E48" s="12" t="s">
+        <v>37</v>
       </c>
       <c r="F48" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G48" s="12"/>
+      <c r="G48" s="12" t="s">
+        <v>68</v>
+      </c>
       <c r="H48" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="I48" s="12"/>
-      <c r="J48" s="21" t="s">
-        <v>122</v>
-      </c>
-      <c r="K48" s="12"/>
-      <c r="L48" s="12"/>
-      <c r="M48" s="12"/>
-      <c r="N48" s="12"/>
-      <c r="O48" s="12"/>
-      <c r="P48" s="12"/>
-      <c r="Q48" s="12"/>
-      <c r="R48" s="21" t="s">
-        <v>123</v>
-      </c>
-      <c r="S48" s="21" t="s">
-        <v>122</v>
+      <c r="I48" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="J48" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="K48" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="L48" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="M48" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="N48" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="O48" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="P48" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q48" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="R48" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="S48" s="12" t="s">
+        <v>40</v>
       </c>
       <c r="T48" s="12" t="s">
         <v>44</v>
       </c>
       <c r="U48" s="12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="V48" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="W48" s="12"/>
-      <c r="X48" s="12"/>
-      <c r="Y48" s="13" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="49" spans="1:25" ht="70" x14ac:dyDescent="0.15">
+      <c r="W48" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="X48" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y48" s="13"/>
+    </row>
+    <row r="49" spans="1:25" ht="28" x14ac:dyDescent="0.15">
       <c r="A49" s="11" t="s">
         <v>34</v>
       </c>
       <c r="B49" s="11" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="C49" s="12"/>
       <c r="D49" s="21" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="F49" s="12" t="s">
         <v>38</v>
@@ -7952,20 +8092,20 @@
       </c>
       <c r="I49" s="12"/>
       <c r="J49" s="21" t="s">
-        <v>128</v>
-      </c>
-      <c r="K49" s="21"/>
-      <c r="L49" s="21"/>
+        <v>122</v>
+      </c>
+      <c r="K49" s="12"/>
+      <c r="L49" s="12"/>
       <c r="M49" s="12"/>
       <c r="N49" s="12"/>
       <c r="O49" s="12"/>
       <c r="P49" s="12"/>
       <c r="Q49" s="12"/>
       <c r="R49" s="21" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="S49" s="21" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="T49" s="12" t="s">
         <v>44</v>
@@ -7979,82 +8119,84 @@
       <c r="W49" s="12"/>
       <c r="X49" s="12"/>
       <c r="Y49" s="13" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="50" spans="1:25" x14ac:dyDescent="0.15">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="50" spans="1:25" ht="70" x14ac:dyDescent="0.15">
       <c r="A50" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B50" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="C50" s="15"/>
-      <c r="D50" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="E50" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="F50" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="G50" s="15"/>
-      <c r="H50" s="15"/>
-      <c r="I50" s="15"/>
-      <c r="J50" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="K50" s="15"/>
-      <c r="L50" s="15"/>
-      <c r="M50" s="15"/>
-      <c r="N50" s="15"/>
-      <c r="O50" s="15"/>
-      <c r="P50" s="15"/>
-      <c r="Q50" s="15"/>
-      <c r="R50" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="S50" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="T50" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="U50" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="V50" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="W50" s="15"/>
-      <c r="X50" s="15"/>
-      <c r="Y50" s="7" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="51" spans="1:25" ht="14" x14ac:dyDescent="0.15">
+      <c r="B50" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="C50" s="12"/>
+      <c r="D50" s="21" t="s">
+        <v>126</v>
+      </c>
+      <c r="E50" s="21" t="s">
+        <v>127</v>
+      </c>
+      <c r="F50" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="G50" s="12"/>
+      <c r="H50" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I50" s="12"/>
+      <c r="J50" s="21" t="s">
+        <v>128</v>
+      </c>
+      <c r="K50" s="21"/>
+      <c r="L50" s="21"/>
+      <c r="M50" s="12"/>
+      <c r="N50" s="12"/>
+      <c r="O50" s="12"/>
+      <c r="P50" s="12"/>
+      <c r="Q50" s="12"/>
+      <c r="R50" s="21" t="s">
+        <v>129</v>
+      </c>
+      <c r="S50" s="21" t="s">
+        <v>130</v>
+      </c>
+      <c r="T50" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="U50" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="V50" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="W50" s="12"/>
+      <c r="X50" s="12"/>
+      <c r="Y50" s="13" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="51" spans="1:25" x14ac:dyDescent="0.15">
       <c r="A51" s="11" t="s">
         <v>34</v>
       </c>
       <c r="B51" s="14" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C51" s="15"/>
-      <c r="D51" s="21" t="s">
-        <v>135</v>
-      </c>
-      <c r="E51" s="21" t="s">
-        <v>136</v>
-      </c>
-      <c r="F51" s="21" t="s">
-        <v>38</v>
-      </c>
-      <c r="G51" s="21"/>
-      <c r="H51" s="21"/>
-      <c r="I51" s="21"/>
-      <c r="J51" s="21" t="s">
-        <v>137</v>
+      <c r="D51" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="E51" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="F51" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="G51" s="15"/>
+      <c r="H51" s="15"/>
+      <c r="I51" s="15"/>
+      <c r="J51" s="15" t="s">
+        <v>39</v>
       </c>
       <c r="K51" s="15"/>
       <c r="L51" s="15"/>
@@ -8063,156 +8205,174 @@
       <c r="O51" s="15"/>
       <c r="P51" s="15"/>
       <c r="Q51" s="15"/>
-      <c r="R51" s="21" t="s">
-        <v>138</v>
-      </c>
-      <c r="S51" s="21" t="s">
-        <v>137</v>
-      </c>
-      <c r="T51" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="U51" s="21" t="s">
-        <v>40</v>
-      </c>
-      <c r="V51" s="12" t="s">
+      <c r="R51" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="S51" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="T51" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="U51" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="V51" s="15" t="s">
         <v>44</v>
       </c>
       <c r="W51" s="15"/>
       <c r="X51" s="15"/>
-      <c r="Y51" s="7"/>
-    </row>
-    <row r="52" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A52" s="17" t="s">
+      <c r="Y51" s="7" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="52" spans="1:25" ht="14" x14ac:dyDescent="0.15">
+      <c r="A52" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B52" s="17" t="s">
+      <c r="B52" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="C52" s="15"/>
+      <c r="D52" s="21" t="s">
+        <v>135</v>
+      </c>
+      <c r="E52" s="21" t="s">
+        <v>136</v>
+      </c>
+      <c r="F52" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="G52" s="21"/>
+      <c r="H52" s="21"/>
+      <c r="I52" s="21"/>
+      <c r="J52" s="21" t="s">
+        <v>137</v>
+      </c>
+      <c r="K52" s="15"/>
+      <c r="L52" s="15"/>
+      <c r="M52" s="15"/>
+      <c r="N52" s="15"/>
+      <c r="O52" s="15"/>
+      <c r="P52" s="15"/>
+      <c r="Q52" s="15"/>
+      <c r="R52" s="21" t="s">
+        <v>138</v>
+      </c>
+      <c r="S52" s="21" t="s">
+        <v>137</v>
+      </c>
+      <c r="T52" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="U52" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="V52" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="W52" s="15"/>
+      <c r="X52" s="15"/>
+      <c r="Y52" s="7"/>
+    </row>
+    <row r="53" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A53" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="B53" s="17" t="s">
         <v>139</v>
       </c>
-      <c r="D52" s="12" t="s">
+      <c r="D53" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E52" s="12" t="s">
+      <c r="E53" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="F52" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="G52" s="22"/>
-      <c r="H52" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="I52" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="J52" s="12" t="s">
+      <c r="F53" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="G53" s="22"/>
+      <c r="H53" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I53" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="J53" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="K52" s="22"/>
-      <c r="L52" s="22"/>
-      <c r="M52" s="22"/>
-      <c r="N52" s="22"/>
-      <c r="O52" s="22"/>
-      <c r="P52" s="22"/>
-      <c r="Q52" s="22"/>
-      <c r="R52" s="12" t="s">
+      <c r="K53" s="22"/>
+      <c r="L53" s="22"/>
+      <c r="M53" s="22"/>
+      <c r="N53" s="22"/>
+      <c r="O53" s="22"/>
+      <c r="P53" s="22"/>
+      <c r="Q53" s="22"/>
+      <c r="R53" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="S52" s="12" t="s">
+      <c r="S53" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="T52" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="U52" s="12" t="s">
+      <c r="T53" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="U53" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="V52" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="W52" s="22"/>
-      <c r="X52" s="22"/>
-    </row>
-    <row r="53" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A53" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="B53" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="C53" s="15"/>
-      <c r="D53" s="15" t="s">
-        <v>141</v>
-      </c>
-      <c r="E53" s="15" t="s">
-        <v>142</v>
-      </c>
-      <c r="F53" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="G53" s="15"/>
-      <c r="H53" s="15"/>
-      <c r="I53" s="15"/>
-      <c r="J53" s="15" t="s">
-        <v>143</v>
-      </c>
-      <c r="K53" s="15"/>
-      <c r="L53" s="15"/>
-      <c r="M53" s="15"/>
-      <c r="N53" s="15"/>
-      <c r="O53" s="15"/>
-      <c r="P53" s="15"/>
-      <c r="Q53" s="15"/>
-      <c r="R53" s="15" t="s">
-        <v>144</v>
-      </c>
-      <c r="S53" s="15" t="s">
-        <v>143</v>
-      </c>
-      <c r="T53" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="U53" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="V53" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="W53" s="15"/>
-      <c r="X53" s="15"/>
-      <c r="Y53" s="13"/>
+      <c r="V53" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="W53" s="22"/>
+      <c r="X53" s="22"/>
     </row>
     <row r="54" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A54" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B54" s="11" t="s">
-        <v>145</v>
-      </c>
-      <c r="C54" s="12"/>
-      <c r="D54" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="E54" s="12"/>
-      <c r="F54" s="12"/>
-      <c r="G54" s="12"/>
-      <c r="H54" s="12"/>
-      <c r="I54" s="12"/>
-      <c r="J54" s="12"/>
-      <c r="K54" s="12"/>
-      <c r="L54" s="12"/>
-      <c r="M54" s="12"/>
-      <c r="N54" s="12"/>
-      <c r="O54" s="12"/>
-      <c r="P54" s="12"/>
-      <c r="Q54" s="12"/>
-      <c r="R54" s="12"/>
-      <c r="S54" s="12"/>
-      <c r="T54" s="12"/>
-      <c r="U54" s="12"/>
-      <c r="V54" s="12"/>
-      <c r="W54" s="12"/>
-      <c r="X54" s="12"/>
+      <c r="B54" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="C54" s="15"/>
+      <c r="D54" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="E54" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="F54" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="G54" s="15"/>
+      <c r="H54" s="15"/>
+      <c r="I54" s="15"/>
+      <c r="J54" s="15" t="s">
+        <v>143</v>
+      </c>
+      <c r="K54" s="15"/>
+      <c r="L54" s="15"/>
+      <c r="M54" s="15"/>
+      <c r="N54" s="15"/>
+      <c r="O54" s="15"/>
+      <c r="P54" s="15"/>
+      <c r="Q54" s="15"/>
+      <c r="R54" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="S54" s="15" t="s">
+        <v>143</v>
+      </c>
+      <c r="T54" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="U54" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="V54" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="W54" s="15"/>
+      <c r="X54" s="15"/>
       <c r="Y54" s="13"/>
     </row>
     <row r="55" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -8220,26 +8380,18 @@
         <v>34</v>
       </c>
       <c r="B55" s="11" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C55" s="12"/>
       <c r="D55" s="12" t="s">
-        <v>147</v>
-      </c>
-      <c r="E55" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="F55" s="12" t="s">
-        <v>38</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="E55" s="12"/>
+      <c r="F55" s="12"/>
       <c r="G55" s="12"/>
-      <c r="H55" s="12" t="s">
-        <v>38</v>
-      </c>
+      <c r="H55" s="12"/>
       <c r="I55" s="12"/>
-      <c r="J55" s="12" t="s">
-        <v>149</v>
-      </c>
+      <c r="J55" s="12"/>
       <c r="K55" s="12"/>
       <c r="L55" s="12"/>
       <c r="M55" s="12"/>
@@ -8247,44 +8399,40 @@
       <c r="O55" s="12"/>
       <c r="P55" s="12"/>
       <c r="Q55" s="12"/>
-      <c r="R55" s="12" t="s">
-        <v>150</v>
-      </c>
-      <c r="S55" s="12" t="s">
-        <v>151</v>
-      </c>
-      <c r="T55" s="12" t="s">
-        <v>150</v>
-      </c>
-      <c r="U55" s="12" t="s">
-        <v>151</v>
-      </c>
-      <c r="V55" s="12" t="s">
-        <v>150</v>
-      </c>
+      <c r="R55" s="12"/>
+      <c r="S55" s="12"/>
+      <c r="T55" s="12"/>
+      <c r="U55" s="12"/>
+      <c r="V55" s="12"/>
       <c r="W55" s="12"/>
       <c r="X55" s="12"/>
-      <c r="Y55" s="13" t="s">
-        <v>152</v>
-      </c>
+      <c r="Y55" s="13"/>
     </row>
     <row r="56" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A56" s="11" t="s">
         <v>34</v>
       </c>
       <c r="B56" s="11" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="C56" s="12"/>
       <c r="D56" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="E56" s="12"/>
-      <c r="F56" s="12"/>
+        <v>147</v>
+      </c>
+      <c r="E56" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="F56" s="12" t="s">
+        <v>38</v>
+      </c>
       <c r="G56" s="12"/>
-      <c r="H56" s="12"/>
+      <c r="H56" s="12" t="s">
+        <v>38</v>
+      </c>
       <c r="I56" s="12"/>
-      <c r="J56" s="12"/>
+      <c r="J56" s="12" t="s">
+        <v>149</v>
+      </c>
       <c r="K56" s="12"/>
       <c r="L56" s="12"/>
       <c r="M56" s="12"/>
@@ -8292,40 +8440,44 @@
       <c r="O56" s="12"/>
       <c r="P56" s="12"/>
       <c r="Q56" s="12"/>
-      <c r="R56" s="12"/>
-      <c r="S56" s="12"/>
-      <c r="T56" s="12"/>
-      <c r="U56" s="12"/>
-      <c r="V56" s="12"/>
+      <c r="R56" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="S56" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="T56" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="U56" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="V56" s="12" t="s">
+        <v>150</v>
+      </c>
       <c r="W56" s="12"/>
       <c r="X56" s="12"/>
-      <c r="Y56" s="13"/>
+      <c r="Y56" s="13" t="s">
+        <v>152</v>
+      </c>
     </row>
     <row r="57" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A57" s="11" t="s">
         <v>34</v>
       </c>
       <c r="B57" s="11" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C57" s="12"/>
       <c r="D57" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E57" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="F57" s="12" t="s">
-        <v>38</v>
-      </c>
+      <c r="E57" s="12"/>
+      <c r="F57" s="12"/>
       <c r="G57" s="12"/>
-      <c r="H57" s="12" t="s">
-        <v>38</v>
-      </c>
+      <c r="H57" s="12"/>
       <c r="I57" s="12"/>
-      <c r="J57" s="12" t="s">
-        <v>40</v>
-      </c>
+      <c r="J57" s="12"/>
       <c r="K57" s="12"/>
       <c r="L57" s="12"/>
       <c r="M57" s="12"/>
@@ -8333,21 +8485,11 @@
       <c r="O57" s="12"/>
       <c r="P57" s="12"/>
       <c r="Q57" s="12"/>
-      <c r="R57" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="S57" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="T57" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="U57" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="V57" s="12" t="s">
-        <v>44</v>
-      </c>
+      <c r="R57" s="12"/>
+      <c r="S57" s="12"/>
+      <c r="T57" s="12"/>
+      <c r="U57" s="12"/>
+      <c r="V57" s="12"/>
       <c r="W57" s="12"/>
       <c r="X57" s="12"/>
       <c r="Y57" s="13"/>
@@ -8356,10 +8498,10 @@
       <c r="A58" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B58" s="14" t="s">
-        <v>155</v>
-      </c>
-      <c r="C58" s="15"/>
+      <c r="B58" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="C58" s="12"/>
       <c r="D58" s="12" t="s">
         <v>41</v>
       </c>
@@ -8373,29 +8515,17 @@
       <c r="H58" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="I58" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="I58" s="12"/>
       <c r="J58" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="K58" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="L58" s="12" t="s">
-        <v>37</v>
-      </c>
+      <c r="K58" s="12"/>
+      <c r="L58" s="12"/>
       <c r="M58" s="12"/>
-      <c r="N58" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="O58" s="12" t="s">
-        <v>38</v>
-      </c>
+      <c r="N58" s="12"/>
+      <c r="O58" s="12"/>
       <c r="P58" s="12"/>
-      <c r="Q58" s="12" t="s">
-        <v>40</v>
-      </c>
+      <c r="Q58" s="12"/>
       <c r="R58" s="12" t="s">
         <v>42</v>
       </c>
@@ -8416,13 +8546,13 @@
       <c r="Y58" s="13"/>
     </row>
     <row r="59" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A59" s="23" t="s">
+      <c r="A59" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B59" s="24" t="s">
-        <v>156</v>
-      </c>
-      <c r="C59" s="25"/>
+      <c r="B59" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="C59" s="15"/>
       <c r="D59" s="12" t="s">
         <v>41</v>
       </c>
@@ -8465,8 +8595,12 @@
       <c r="S59" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="T59" s="12"/>
-      <c r="U59" s="12"/>
+      <c r="T59" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="U59" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="V59" s="12" t="s">
         <v>44</v>
       </c>
@@ -8474,12 +8608,12 @@
       <c r="X59" s="12"/>
       <c r="Y59" s="13"/>
     </row>
-    <row r="60" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="60" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A60" s="23" t="s">
         <v>34</v>
       </c>
       <c r="B60" s="24" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C60" s="25"/>
       <c r="D60" s="12" t="s">
@@ -8499,7 +8633,7 @@
         <v>39</v>
       </c>
       <c r="J60" s="12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K60" s="12" t="s">
         <v>41</v>
@@ -8525,9 +8659,7 @@
         <v>40</v>
       </c>
       <c r="T60" s="12"/>
-      <c r="U60" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="U60" s="12"/>
       <c r="V60" s="12" t="s">
         <v>44</v>
       </c>
@@ -8535,12 +8667,12 @@
       <c r="X60" s="12"/>
       <c r="Y60" s="13"/>
     </row>
-    <row r="61" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="61" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A61" s="23" t="s">
         <v>34</v>
       </c>
       <c r="B61" s="24" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C61" s="25"/>
       <c r="D61" s="12" t="s">
@@ -8559,12 +8691,14 @@
       <c r="I61" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="J61" s="12"/>
+      <c r="J61" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="K61" s="12" t="s">
         <v>41</v>
       </c>
       <c r="L61" s="12" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="M61" s="12"/>
       <c r="N61" s="12" t="s">
@@ -8584,95 +8718,81 @@
         <v>40</v>
       </c>
       <c r="T61" s="12"/>
-      <c r="U61" s="12"/>
-      <c r="V61" s="12"/>
+      <c r="U61" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="V61" s="12" t="s">
+        <v>44</v>
+      </c>
       <c r="W61" s="12"/>
       <c r="X61" s="12"/>
       <c r="Y61" s="13"/>
     </row>
     <row r="62" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A62" s="11" t="s">
+      <c r="A62" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="B62" s="11" t="s">
-        <v>159</v>
-      </c>
-      <c r="C62" s="12"/>
+      <c r="B62" s="24" t="s">
+        <v>158</v>
+      </c>
+      <c r="C62" s="25"/>
       <c r="D62" s="12" t="s">
         <v>41</v>
       </c>
       <c r="E62" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F62" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G62" s="12" t="s">
-        <v>38</v>
-      </c>
+      <c r="G62" s="12"/>
       <c r="H62" s="12" t="s">
         <v>38</v>
       </c>
       <c r="I62" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="J62" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="J62" s="12"/>
       <c r="K62" s="12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="L62" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="M62" s="12" t="s">
-        <v>39</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="M62" s="12"/>
       <c r="N62" s="12" t="s">
         <v>38</v>
       </c>
       <c r="O62" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="P62" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="P62" s="12"/>
       <c r="Q62" s="12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="R62" s="12" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="S62" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="T62" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="U62" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="V62" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="W62" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="X62" s="12" t="s">
-        <v>39</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="T62" s="12"/>
+      <c r="U62" s="12"/>
+      <c r="V62" s="12"/>
+      <c r="W62" s="12"/>
+      <c r="X62" s="12"/>
       <c r="Y62" s="13"/>
     </row>
     <row r="63" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A63" s="11" t="s">
-        <v>160</v>
-      </c>
-      <c r="B63" s="24" t="s">
-        <v>161</v>
+        <v>34</v>
+      </c>
+      <c r="B63" s="11" t="s">
+        <v>159</v>
       </c>
       <c r="C63" s="12"/>
       <c r="D63" s="12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E63" s="12" t="s">
         <v>38</v>
@@ -8680,9 +8800,15 @@
       <c r="F63" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G63" s="12"/>
-      <c r="H63" s="12"/>
-      <c r="I63" s="12"/>
+      <c r="G63" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="H63" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I63" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="J63" s="12" t="s">
         <v>39</v>
       </c>
@@ -8692,12 +8818,18 @@
       <c r="L63" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="M63" s="12"/>
+      <c r="M63" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="N63" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="O63" s="12"/>
-      <c r="P63" s="12"/>
+      <c r="O63" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="P63" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="Q63" s="12" t="s">
         <v>39</v>
       </c>
@@ -8707,13 +8839,21 @@
       <c r="S63" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="T63" s="12"/>
-      <c r="U63" s="12"/>
+      <c r="T63" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="U63" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="V63" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="W63" s="12"/>
-      <c r="X63" s="12"/>
+      <c r="W63" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="X63" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="Y63" s="13"/>
     </row>
     <row r="64" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -8721,7 +8861,7 @@
         <v>160</v>
       </c>
       <c r="B64" s="24" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C64" s="12"/>
       <c r="D64" s="12" t="s">
@@ -8774,7 +8914,7 @@
         <v>160</v>
       </c>
       <c r="B65" s="24" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C65" s="12"/>
       <c r="D65" s="12" t="s">
@@ -8826,8 +8966,8 @@
       <c r="A66" s="11" t="s">
         <v>160</v>
       </c>
-      <c r="B66" s="11" t="s">
-        <v>164</v>
+      <c r="B66" s="24" t="s">
+        <v>163</v>
       </c>
       <c r="C66" s="12"/>
       <c r="D66" s="12" t="s">
@@ -8880,7 +9020,7 @@
         <v>160</v>
       </c>
       <c r="B67" s="11" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C67" s="12"/>
       <c r="D67" s="12" t="s">
@@ -8901,12 +9041,18 @@
       <c r="K67" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="L67" s="12"/>
+      <c r="L67" s="12" t="s">
+        <v>38</v>
+      </c>
       <c r="M67" s="12"/>
-      <c r="N67" s="12"/>
+      <c r="N67" s="12" t="s">
+        <v>38</v>
+      </c>
       <c r="O67" s="12"/>
       <c r="P67" s="12"/>
-      <c r="Q67" s="12"/>
+      <c r="Q67" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="R67" s="12" t="s">
         <v>44</v>
       </c>
@@ -8927,7 +9073,7 @@
         <v>160</v>
       </c>
       <c r="B68" s="11" t="s">
-        <v>267</v>
+        <v>165</v>
       </c>
       <c r="C68" s="12"/>
       <c r="D68" s="12" t="s">
@@ -8948,18 +9094,12 @@
       <c r="K68" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="L68" s="12" t="s">
-        <v>38</v>
-      </c>
+      <c r="L68" s="12"/>
       <c r="M68" s="12"/>
-      <c r="N68" s="12" t="s">
-        <v>38</v>
-      </c>
+      <c r="N68" s="12"/>
       <c r="O68" s="12"/>
       <c r="P68" s="12"/>
-      <c r="Q68" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="Q68" s="12"/>
       <c r="R68" s="12" t="s">
         <v>44</v>
       </c>
@@ -8980,7 +9120,7 @@
         <v>160</v>
       </c>
       <c r="B69" s="11" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C69" s="12"/>
       <c r="D69" s="12" t="s">
@@ -9033,7 +9173,7 @@
         <v>160</v>
       </c>
       <c r="B70" s="11" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C70" s="12"/>
       <c r="D70" s="12" t="s">
@@ -9086,7 +9226,7 @@
         <v>160</v>
       </c>
       <c r="B71" s="11" t="s">
-        <v>166</v>
+        <v>269</v>
       </c>
       <c r="C71" s="12"/>
       <c r="D71" s="12" t="s">
@@ -9139,32 +9279,50 @@
         <v>160</v>
       </c>
       <c r="B72" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C72" s="12"/>
       <c r="D72" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="E72" s="12"/>
-      <c r="F72" s="12"/>
-      <c r="G72" s="12" t="s">
-        <v>46</v>
-      </c>
+      <c r="E72" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F72" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="G72" s="12"/>
       <c r="H72" s="12"/>
       <c r="I72" s="12"/>
-      <c r="J72" s="12"/>
-      <c r="K72" s="12"/>
-      <c r="L72" s="12"/>
+      <c r="J72" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="K72" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="L72" s="12" t="s">
+        <v>38</v>
+      </c>
       <c r="M72" s="12"/>
-      <c r="N72" s="12"/>
+      <c r="N72" s="12" t="s">
+        <v>38</v>
+      </c>
       <c r="O72" s="12"/>
       <c r="P72" s="12"/>
-      <c r="Q72" s="12"/>
-      <c r="R72" s="12"/>
-      <c r="S72" s="12"/>
+      <c r="Q72" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="R72" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="S72" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="T72" s="12"/>
       <c r="U72" s="12"/>
-      <c r="V72" s="12"/>
+      <c r="V72" s="12" t="s">
+        <v>44</v>
+      </c>
       <c r="W72" s="12"/>
       <c r="X72" s="12"/>
       <c r="Y72" s="13"/>
@@ -9174,70 +9332,34 @@
         <v>160</v>
       </c>
       <c r="B73" s="11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C73" s="12"/>
       <c r="D73" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="E73" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="F73" s="12" t="s">
-        <v>38</v>
-      </c>
+      <c r="E73" s="12"/>
+      <c r="F73" s="12"/>
       <c r="G73" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="H73" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="I73" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="J73" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="K73" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="L73" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="M73" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="N73" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="O73" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="P73" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q73" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="R73" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="S73" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="T73" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="U73" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="V73" s="12" t="s">
-        <v>44</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="H73" s="12"/>
+      <c r="I73" s="12"/>
+      <c r="J73" s="12"/>
+      <c r="K73" s="12"/>
+      <c r="L73" s="12"/>
+      <c r="M73" s="12"/>
+      <c r="N73" s="12"/>
+      <c r="O73" s="12"/>
+      <c r="P73" s="12"/>
+      <c r="Q73" s="12"/>
+      <c r="R73" s="12"/>
+      <c r="S73" s="12"/>
+      <c r="T73" s="12"/>
+      <c r="U73" s="12"/>
+      <c r="V73" s="12"/>
       <c r="W73" s="12"/>
-      <c r="X73" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="X73" s="12"/>
       <c r="Y73" s="13"/>
     </row>
     <row r="74" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -9245,7 +9367,7 @@
         <v>160</v>
       </c>
       <c r="B74" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C74" s="12"/>
       <c r="D74" s="12" t="s">
@@ -9305,9 +9427,7 @@
       <c r="V74" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="W74" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="W74" s="12"/>
       <c r="X74" s="12" t="s">
         <v>39</v>
       </c>
@@ -9318,7 +9438,7 @@
         <v>160</v>
       </c>
       <c r="B75" s="11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C75" s="12"/>
       <c r="D75" s="12" t="s">
@@ -9378,7 +9498,9 @@
       <c r="V75" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="W75" s="12"/>
+      <c r="W75" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="X75" s="12" t="s">
         <v>39</v>
       </c>
@@ -9389,7 +9511,7 @@
         <v>160</v>
       </c>
       <c r="B76" s="11" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C76" s="12"/>
       <c r="D76" s="12" t="s">
@@ -9460,34 +9582,70 @@
         <v>160</v>
       </c>
       <c r="B77" s="11" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C77" s="12"/>
       <c r="D77" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="E77" s="12"/>
-      <c r="F77" s="12"/>
+      <c r="E77" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F77" s="12" t="s">
+        <v>38</v>
+      </c>
       <c r="G77" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="H77" s="12"/>
-      <c r="I77" s="12"/>
-      <c r="J77" s="12"/>
-      <c r="K77" s="12"/>
-      <c r="L77" s="12"/>
-      <c r="M77" s="12"/>
-      <c r="N77" s="12"/>
-      <c r="O77" s="12"/>
-      <c r="P77" s="12"/>
-      <c r="Q77" s="12"/>
-      <c r="R77" s="12"/>
-      <c r="S77" s="12"/>
-      <c r="T77" s="12"/>
-      <c r="U77" s="12"/>
-      <c r="V77" s="12"/>
+        <v>38</v>
+      </c>
+      <c r="H77" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I77" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="J77" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="K77" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="L77" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="M77" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="N77" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="O77" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="P77" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q77" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="R77" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="S77" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="T77" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="U77" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="V77" s="12" t="s">
+        <v>44</v>
+      </c>
       <c r="W77" s="12"/>
-      <c r="X77" s="12"/>
+      <c r="X77" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="Y77" s="13"/>
     </row>
     <row r="78" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -9495,70 +9653,34 @@
         <v>160</v>
       </c>
       <c r="B78" s="11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C78" s="12"/>
       <c r="D78" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="E78" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="F78" s="12" t="s">
-        <v>38</v>
-      </c>
+      <c r="E78" s="12"/>
+      <c r="F78" s="12"/>
       <c r="G78" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="H78" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="I78" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="J78" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="K78" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="L78" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="M78" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="N78" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="O78" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="P78" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q78" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="R78" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="S78" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="T78" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="U78" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="V78" s="12" t="s">
-        <v>44</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="H78" s="12"/>
+      <c r="I78" s="12"/>
+      <c r="J78" s="12"/>
+      <c r="K78" s="12"/>
+      <c r="L78" s="12"/>
+      <c r="M78" s="12"/>
+      <c r="N78" s="12"/>
+      <c r="O78" s="12"/>
+      <c r="P78" s="12"/>
+      <c r="Q78" s="12"/>
+      <c r="R78" s="12"/>
+      <c r="S78" s="12"/>
+      <c r="T78" s="12"/>
+      <c r="U78" s="12"/>
+      <c r="V78" s="12"/>
       <c r="W78" s="12"/>
-      <c r="X78" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="X78" s="12"/>
       <c r="Y78" s="13"/>
     </row>
     <row r="79" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -9566,7 +9688,7 @@
         <v>160</v>
       </c>
       <c r="B79" s="11" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C79" s="12"/>
       <c r="D79" s="12" t="s">
@@ -9637,7 +9759,7 @@
         <v>160</v>
       </c>
       <c r="B80" s="11" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C80" s="12"/>
       <c r="D80" s="12" t="s">
@@ -9673,7 +9795,9 @@
       <c r="N80" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="O80" s="12"/>
+      <c r="O80" s="12" t="s">
+        <v>38</v>
+      </c>
       <c r="P80" s="12" t="s">
         <v>39</v>
       </c>
@@ -9706,7 +9830,7 @@
         <v>160</v>
       </c>
       <c r="B81" s="11" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C81" s="12"/>
       <c r="D81" s="12" t="s">
@@ -9742,9 +9866,7 @@
       <c r="N81" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="O81" s="12" t="s">
-        <v>38</v>
-      </c>
+      <c r="O81" s="12"/>
       <c r="P81" s="12" t="s">
         <v>39</v>
       </c>
@@ -9777,7 +9899,7 @@
         <v>160</v>
       </c>
       <c r="B82" s="11" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C82" s="12"/>
       <c r="D82" s="12" t="s">
@@ -9789,8 +9911,12 @@
       <c r="F82" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G82" s="12"/>
-      <c r="H82" s="12"/>
+      <c r="G82" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="H82" s="12" t="s">
+        <v>38</v>
+      </c>
       <c r="I82" s="12" t="s">
         <v>39</v>
       </c>
@@ -9803,11 +9929,15 @@
       <c r="L82" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="M82" s="12"/>
+      <c r="M82" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="N82" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="O82" s="12"/>
+      <c r="O82" s="12" t="s">
+        <v>38</v>
+      </c>
       <c r="P82" s="12" t="s">
         <v>39</v>
       </c>
@@ -9840,7 +9970,7 @@
         <v>160</v>
       </c>
       <c r="B83" s="11" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C83" s="12"/>
       <c r="D83" s="12" t="s">
@@ -9853,10 +9983,10 @@
         <v>38</v>
       </c>
       <c r="G83" s="12"/>
-      <c r="H83" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="I83" s="12"/>
+      <c r="H83" s="12"/>
+      <c r="I83" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="J83" s="12" t="s">
         <v>39</v>
       </c>
@@ -9870,10 +10000,10 @@
       <c r="N83" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="O83" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="P83" s="12"/>
+      <c r="O83" s="12"/>
+      <c r="P83" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="Q83" s="12" t="s">
         <v>39</v>
       </c>
@@ -9883,13 +10013,19 @@
       <c r="S83" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="T83" s="12"/>
-      <c r="U83" s="12"/>
+      <c r="T83" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="U83" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="V83" s="12" t="s">
         <v>44</v>
       </c>
       <c r="W83" s="12"/>
-      <c r="X83" s="12"/>
+      <c r="X83" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="Y83" s="13"/>
     </row>
     <row r="84" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -9897,32 +10033,54 @@
         <v>160</v>
       </c>
       <c r="B84" s="11" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C84" s="12"/>
       <c r="D84" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="E84" s="12"/>
-      <c r="F84" s="12"/>
-      <c r="G84" s="12" t="s">
+      <c r="E84" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F84" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="G84" s="12"/>
+      <c r="H84" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="H84" s="12"/>
       <c r="I84" s="12"/>
-      <c r="J84" s="12"/>
-      <c r="K84" s="12"/>
-      <c r="L84" s="12"/>
+      <c r="J84" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="K84" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="L84" s="12" t="s">
+        <v>38</v>
+      </c>
       <c r="M84" s="12"/>
-      <c r="N84" s="12"/>
-      <c r="O84" s="12"/>
+      <c r="N84" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="O84" s="12" t="s">
+        <v>46</v>
+      </c>
       <c r="P84" s="12"/>
-      <c r="Q84" s="12"/>
-      <c r="R84" s="12"/>
-      <c r="S84" s="12"/>
+      <c r="Q84" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="R84" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="S84" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="T84" s="12"/>
       <c r="U84" s="12"/>
-      <c r="V84" s="12"/>
+      <c r="V84" s="12" t="s">
+        <v>44</v>
+      </c>
       <c r="W84" s="12"/>
       <c r="X84" s="12"/>
       <c r="Y84" s="13"/>
@@ -9932,7 +10090,7 @@
         <v>160</v>
       </c>
       <c r="B85" s="11" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C85" s="12"/>
       <c r="D85" s="12" t="s">
@@ -9967,7 +10125,7 @@
         <v>160</v>
       </c>
       <c r="B86" s="11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C86" s="12"/>
       <c r="D86" s="12" t="s">
@@ -10002,68 +10160,34 @@
         <v>160</v>
       </c>
       <c r="B87" s="11" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C87" s="12"/>
       <c r="D87" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="E87" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="F87" s="12" t="s">
-        <v>38</v>
-      </c>
+      <c r="E87" s="12"/>
+      <c r="F87" s="12"/>
       <c r="G87" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="H87" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="I87" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="J87" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="K87" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="L87" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="M87" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="N87" s="12" t="s">
-        <v>38</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="H87" s="12"/>
+      <c r="I87" s="12"/>
+      <c r="J87" s="12"/>
+      <c r="K87" s="12"/>
+      <c r="L87" s="12"/>
+      <c r="M87" s="12"/>
+      <c r="N87" s="12"/>
       <c r="O87" s="12"/>
-      <c r="P87" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q87" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="R87" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="S87" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="T87" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="U87" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="V87" s="12" t="s">
-        <v>44</v>
-      </c>
+      <c r="P87" s="12"/>
+      <c r="Q87" s="12"/>
+      <c r="R87" s="12"/>
+      <c r="S87" s="12"/>
+      <c r="T87" s="12"/>
+      <c r="U87" s="12"/>
+      <c r="V87" s="12"/>
       <c r="W87" s="12"/>
-      <c r="X87" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="X87" s="12"/>
       <c r="Y87" s="13"/>
     </row>
     <row r="88" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -10071,7 +10195,7 @@
         <v>160</v>
       </c>
       <c r="B88" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C88" s="12"/>
       <c r="D88" s="12" t="s">
@@ -10140,7 +10264,7 @@
         <v>160</v>
       </c>
       <c r="B89" s="11" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C89" s="12"/>
       <c r="D89" s="12" t="s">
@@ -10176,9 +10300,7 @@
       <c r="N89" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="O89" s="12" t="s">
-        <v>38</v>
-      </c>
+      <c r="O89" s="12"/>
       <c r="P89" s="12" t="s">
         <v>39</v>
       </c>
@@ -10211,7 +10333,7 @@
         <v>160</v>
       </c>
       <c r="B90" s="11" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C90" s="12"/>
       <c r="D90" s="12" t="s">
@@ -10272,7 +10394,9 @@
         <v>44</v>
       </c>
       <c r="W90" s="12"/>
-      <c r="X90" s="12"/>
+      <c r="X90" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="Y90" s="13"/>
     </row>
     <row r="91" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -10280,7 +10404,7 @@
         <v>160</v>
       </c>
       <c r="B91" s="11" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C91" s="12"/>
       <c r="D91" s="12" t="s">
@@ -10349,7 +10473,7 @@
         <v>160</v>
       </c>
       <c r="B92" s="11" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C92" s="12"/>
       <c r="D92" s="12" t="s">
@@ -10418,7 +10542,7 @@
         <v>160</v>
       </c>
       <c r="B93" s="11" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C93" s="12"/>
       <c r="D93" s="12" t="s">
@@ -10487,7 +10611,7 @@
         <v>160</v>
       </c>
       <c r="B94" s="11" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C94" s="12"/>
       <c r="D94" s="12" t="s">
@@ -10556,32 +10680,66 @@
         <v>160</v>
       </c>
       <c r="B95" s="11" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C95" s="12"/>
       <c r="D95" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="E95" s="12"/>
-      <c r="F95" s="12"/>
+      <c r="E95" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F95" s="12" t="s">
+        <v>38</v>
+      </c>
       <c r="G95" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="H95" s="12"/>
-      <c r="I95" s="12"/>
-      <c r="J95" s="12"/>
-      <c r="K95" s="12"/>
-      <c r="L95" s="12"/>
-      <c r="M95" s="12"/>
-      <c r="N95" s="12"/>
-      <c r="O95" s="12"/>
-      <c r="P95" s="12"/>
-      <c r="Q95" s="12"/>
-      <c r="R95" s="12"/>
-      <c r="S95" s="12"/>
-      <c r="T95" s="12"/>
-      <c r="U95" s="12"/>
-      <c r="V95" s="12"/>
+        <v>38</v>
+      </c>
+      <c r="H95" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I95" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="J95" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="K95" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="L95" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="M95" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="N95" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="O95" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="P95" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q95" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="R95" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="S95" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="T95" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="U95" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="V95" s="12" t="s">
+        <v>44</v>
+      </c>
       <c r="W95" s="12"/>
       <c r="X95" s="12"/>
       <c r="Y95" s="13"/>
@@ -10591,66 +10749,32 @@
         <v>160</v>
       </c>
       <c r="B96" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C96" s="12"/>
       <c r="D96" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="E96" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="F96" s="12" t="s">
-        <v>38</v>
-      </c>
+      <c r="E96" s="12"/>
+      <c r="F96" s="12"/>
       <c r="G96" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="H96" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="I96" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="J96" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="K96" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="L96" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="M96" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="N96" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="O96" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="P96" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q96" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="R96" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="S96" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="T96" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="U96" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="V96" s="12" t="s">
-        <v>44</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="H96" s="12"/>
+      <c r="I96" s="12"/>
+      <c r="J96" s="12"/>
+      <c r="K96" s="12"/>
+      <c r="L96" s="12"/>
+      <c r="M96" s="12"/>
+      <c r="N96" s="12"/>
+      <c r="O96" s="12"/>
+      <c r="P96" s="12"/>
+      <c r="Q96" s="12"/>
+      <c r="R96" s="12"/>
+      <c r="S96" s="12"/>
+      <c r="T96" s="12"/>
+      <c r="U96" s="12"/>
+      <c r="V96" s="12"/>
       <c r="W96" s="12"/>
       <c r="X96" s="12"/>
       <c r="Y96" s="13"/>
@@ -10660,7 +10784,7 @@
         <v>160</v>
       </c>
       <c r="B97" s="11" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C97" s="12"/>
       <c r="D97" s="12" t="s">
@@ -10672,9 +10796,15 @@
       <c r="F97" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G97" s="12"/>
-      <c r="H97" s="12"/>
-      <c r="I97" s="12"/>
+      <c r="G97" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="H97" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I97" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="J97" s="12" t="s">
         <v>39</v>
       </c>
@@ -10684,12 +10814,18 @@
       <c r="L97" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="M97" s="12"/>
+      <c r="M97" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="N97" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="O97" s="12"/>
-      <c r="P97" s="12"/>
+      <c r="O97" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="P97" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="Q97" s="12" t="s">
         <v>39</v>
       </c>
@@ -10699,8 +10835,12 @@
       <c r="S97" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="T97" s="12"/>
-      <c r="U97" s="12"/>
+      <c r="T97" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="U97" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="V97" s="12" t="s">
         <v>44</v>
       </c>
@@ -10713,7 +10853,7 @@
         <v>160</v>
       </c>
       <c r="B98" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C98" s="12"/>
       <c r="D98" s="12" t="s">
@@ -10725,17 +10865,11 @@
       <c r="F98" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G98" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="H98" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="I98" s="12" t="s">
-        <v>38</v>
-      </c>
+      <c r="G98" s="12"/>
+      <c r="H98" s="12"/>
+      <c r="I98" s="12"/>
       <c r="J98" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="K98" s="12" t="s">
         <v>38</v>
@@ -10743,18 +10877,12 @@
       <c r="L98" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="M98" s="26" t="s">
-        <v>38</v>
-      </c>
+      <c r="M98" s="12"/>
       <c r="N98" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="O98" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="P98" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="O98" s="12"/>
+      <c r="P98" s="12"/>
       <c r="Q98" s="12" t="s">
         <v>39</v>
       </c>
@@ -10764,21 +10892,13 @@
       <c r="S98" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="T98" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="U98" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="T98" s="12"/>
+      <c r="U98" s="12"/>
       <c r="V98" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="W98" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="X98" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="W98" s="12"/>
+      <c r="X98" s="12"/>
       <c r="Y98" s="13"/>
     </row>
     <row r="99" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -10786,7 +10906,7 @@
         <v>160</v>
       </c>
       <c r="B99" s="11" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C99" s="12"/>
       <c r="D99" s="12" t="s">
@@ -10859,7 +10979,7 @@
         <v>160</v>
       </c>
       <c r="B100" s="11" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C100" s="12"/>
       <c r="D100" s="12" t="s">
@@ -10932,7 +11052,7 @@
         <v>160</v>
       </c>
       <c r="B101" s="11" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C101" s="12"/>
       <c r="D101" s="12" t="s">
@@ -10951,10 +11071,10 @@
         <v>38</v>
       </c>
       <c r="I101" s="12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J101" s="12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="K101" s="12" t="s">
         <v>38</v>
@@ -10962,8 +11082,8 @@
       <c r="L101" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="M101" s="12" t="s">
-        <v>39</v>
+      <c r="M101" s="26" t="s">
+        <v>38</v>
       </c>
       <c r="N101" s="12" t="s">
         <v>38</v>
@@ -10992,7 +11112,9 @@
       <c r="V101" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="W101" s="12"/>
+      <c r="W101" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="X101" s="12" t="s">
         <v>39</v>
       </c>
@@ -11003,32 +11125,70 @@
         <v>160</v>
       </c>
       <c r="B102" s="11" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C102" s="12"/>
       <c r="D102" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="E102" s="12"/>
-      <c r="F102" s="12"/>
-      <c r="G102" s="12"/>
-      <c r="H102" s="12"/>
-      <c r="I102" s="12"/>
-      <c r="J102" s="12"/>
-      <c r="K102" s="12"/>
-      <c r="L102" s="12"/>
-      <c r="M102" s="12"/>
-      <c r="N102" s="12"/>
-      <c r="O102" s="12"/>
-      <c r="P102" s="12"/>
-      <c r="Q102" s="12"/>
-      <c r="R102" s="12"/>
-      <c r="S102" s="12"/>
-      <c r="T102" s="12"/>
-      <c r="U102" s="12"/>
-      <c r="V102" s="12"/>
+      <c r="E102" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F102" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="G102" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="H102" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I102" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="J102" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="K102" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="L102" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="M102" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="N102" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="O102" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="P102" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q102" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="R102" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="S102" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="T102" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="U102" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="V102" s="12" t="s">
+        <v>44</v>
+      </c>
       <c r="W102" s="12"/>
-      <c r="X102" s="12"/>
+      <c r="X102" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="Y102" s="13"/>
     </row>
     <row r="103" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -11036,82 +11196,44 @@
         <v>160</v>
       </c>
       <c r="B103" s="11" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C103" s="12"/>
       <c r="D103" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="E103" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="F103" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="G103" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="H103" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="I103" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="J103" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="K103" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="L103" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="M103" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="N103" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="O103" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="P103" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q103" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="R103" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="S103" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="T103" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="U103" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="V103" s="12" t="s">
-        <v>44</v>
-      </c>
+      <c r="E103" s="12"/>
+      <c r="F103" s="12"/>
+      <c r="G103" s="12"/>
+      <c r="H103" s="12"/>
+      <c r="I103" s="12"/>
+      <c r="J103" s="12"/>
+      <c r="K103" s="12"/>
+      <c r="L103" s="12"/>
+      <c r="M103" s="12"/>
+      <c r="N103" s="12"/>
+      <c r="O103" s="12"/>
+      <c r="P103" s="12"/>
+      <c r="Q103" s="12"/>
+      <c r="R103" s="12"/>
+      <c r="S103" s="12"/>
+      <c r="T103" s="12"/>
+      <c r="U103" s="12"/>
+      <c r="V103" s="12"/>
       <c r="W103" s="12"/>
-      <c r="X103" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="X103" s="12"/>
       <c r="Y103" s="13"/>
     </row>
-    <row r="104" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="104" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A104" s="11" t="s">
         <v>160</v>
       </c>
       <c r="B104" s="11" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C104" s="12"/>
       <c r="D104" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E104" s="12" t="s">
         <v>38</v>
@@ -11132,7 +11254,7 @@
         <v>39</v>
       </c>
       <c r="K104" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="L104" s="12" t="s">
         <v>38</v>
@@ -11153,34 +11275,32 @@
         <v>39</v>
       </c>
       <c r="R104" s="12" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="S104" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="T104" s="12" t="s">
         <v>44</v>
       </c>
       <c r="U104" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="V104" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="W104" s="12" t="s">
-        <v>40</v>
-      </c>
+      <c r="W104" s="12"/>
       <c r="X104" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="Y104" s="13"/>
     </row>
-    <row r="105" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="105" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A105" s="11" t="s">
         <v>160</v>
       </c>
       <c r="B105" s="11" t="s">
-        <v>159</v>
+        <v>199</v>
       </c>
       <c r="C105" s="12"/>
       <c r="D105" s="12" t="s">
@@ -11205,7 +11325,7 @@
         <v>39</v>
       </c>
       <c r="K105" s="12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="L105" s="12" t="s">
         <v>38</v>
@@ -11226,25 +11346,25 @@
         <v>39</v>
       </c>
       <c r="R105" s="12" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="S105" s="12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="T105" s="12" t="s">
         <v>44</v>
       </c>
       <c r="U105" s="12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="V105" s="12" t="s">
         <v>44</v>
       </c>
       <c r="W105" s="12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="X105" s="12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="Y105" s="13"/>
     </row>
@@ -11253,29 +11373,35 @@
         <v>160</v>
       </c>
       <c r="B106" s="11" t="s">
-        <v>200</v>
+        <v>159</v>
       </c>
       <c r="C106" s="12"/>
       <c r="D106" s="12" t="s">
         <v>41</v>
       </c>
       <c r="E106" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F106" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G106" s="12"/>
-      <c r="H106" s="12"/>
-      <c r="I106" s="12"/>
+      <c r="G106" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="H106" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I106" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="J106" s="12" t="s">
         <v>39</v>
       </c>
       <c r="K106" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="L106" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="M106" s="12" t="s">
         <v>39</v>
@@ -11283,62 +11409,66 @@
       <c r="N106" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="O106" s="12"/>
-      <c r="P106" s="12"/>
+      <c r="O106" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="P106" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="Q106" s="12" t="s">
         <v>39</v>
       </c>
       <c r="R106" s="12" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="S106" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="T106" s="12"/>
+        <v>39</v>
+      </c>
+      <c r="T106" s="12" t="s">
+        <v>44</v>
+      </c>
       <c r="U106" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="V106" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="W106" s="12"/>
-      <c r="X106" s="12"/>
+      <c r="W106" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="X106" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="Y106" s="13"/>
     </row>
     <row r="107" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A107" s="11" t="s">
-        <v>201</v>
+        <v>160</v>
       </c>
       <c r="B107" s="11" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C107" s="12"/>
       <c r="D107" s="12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E107" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F107" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G107" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="H107" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="I107" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="G107" s="12"/>
+      <c r="H107" s="12"/>
+      <c r="I107" s="12"/>
       <c r="J107" s="12" t="s">
-        <v>203</v>
+        <v>39</v>
       </c>
       <c r="K107" s="12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="L107" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="M107" s="12" t="s">
         <v>39</v>
@@ -11346,46 +11476,34 @@
       <c r="N107" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="O107" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="P107" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="O107" s="12"/>
+      <c r="P107" s="12"/>
       <c r="Q107" s="12" t="s">
-        <v>203</v>
+        <v>39</v>
       </c>
       <c r="R107" s="12" t="s">
-        <v>204</v>
+        <v>42</v>
       </c>
       <c r="S107" s="12" t="s">
-        <v>203</v>
-      </c>
-      <c r="T107" s="12" t="s">
-        <v>44</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="T107" s="12"/>
       <c r="U107" s="12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="V107" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="W107" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="X107" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y107" s="35" t="s">
-        <v>205</v>
-      </c>
+      <c r="W107" s="12"/>
+      <c r="X107" s="12"/>
+      <c r="Y107" s="13"/>
     </row>
     <row r="108" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A108" s="11" t="s">
         <v>201</v>
       </c>
       <c r="B108" s="11" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="C108" s="12"/>
       <c r="D108" s="12" t="s">
@@ -11451,18 +11569,20 @@
       <c r="X108" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="Y108" s="35"/>
+      <c r="Y108" s="35" t="s">
+        <v>205</v>
+      </c>
     </row>
     <row r="109" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A109" s="11" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="B109" s="11" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C109" s="12"/>
       <c r="D109" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E109" s="12" t="s">
         <v>38</v>
@@ -11480,10 +11600,10 @@
         <v>39</v>
       </c>
       <c r="J109" s="12" t="s">
-        <v>39</v>
+        <v>203</v>
       </c>
       <c r="K109" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="L109" s="12" t="s">
         <v>38</v>
@@ -11501,37 +11621,37 @@
         <v>39</v>
       </c>
       <c r="Q109" s="12" t="s">
-        <v>39</v>
+        <v>203</v>
       </c>
       <c r="R109" s="12" t="s">
-        <v>42</v>
+        <v>204</v>
       </c>
       <c r="S109" s="12" t="s">
-        <v>40</v>
+        <v>203</v>
       </c>
       <c r="T109" s="12" t="s">
         <v>44</v>
       </c>
       <c r="U109" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="V109" s="12" t="s">
         <v>44</v>
       </c>
       <c r="W109" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="X109" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y109" s="7"/>
+        <v>39</v>
+      </c>
+      <c r="Y109" s="35"/>
     </row>
     <row r="110" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A110" s="11" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="B110" s="11" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="C110" s="12"/>
       <c r="D110" s="12" t="s">
@@ -11597,110 +11717,150 @@
       <c r="X110" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="Y110" s="13"/>
-    </row>
-    <row r="111" spans="1:25" s="30" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A111" s="27" t="s">
-        <v>209</v>
-      </c>
-      <c r="B111" s="27" t="s">
-        <v>210</v>
-      </c>
-      <c r="C111" s="28"/>
+      <c r="Y110" s="7"/>
+    </row>
+    <row r="111" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A111" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="B111" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="C111" s="12"/>
       <c r="D111" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E111" s="28"/>
-      <c r="F111" s="28"/>
-      <c r="G111" s="28"/>
-      <c r="H111" s="28"/>
-      <c r="I111" s="28"/>
-      <c r="J111" s="28"/>
-      <c r="K111" s="28"/>
-      <c r="L111" s="28"/>
-      <c r="M111" s="28"/>
-      <c r="N111" s="28"/>
-      <c r="O111" s="28"/>
-      <c r="P111" s="28"/>
-      <c r="Q111" s="28"/>
-      <c r="R111" s="28"/>
-      <c r="S111" s="28"/>
-      <c r="T111" s="28"/>
-      <c r="U111" s="28"/>
-      <c r="V111" s="28"/>
-      <c r="W111" s="28"/>
-      <c r="X111" s="28"/>
-      <c r="Y111" s="29" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="112" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A112" s="11" t="s">
+      <c r="E111" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F111" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="G111" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="H111" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I111" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="J111" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="K111" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="L111" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="M111" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="N111" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="O111" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="P111" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q111" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="R111" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="S111" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="T111" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="U111" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="V111" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="W111" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="X111" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="Y111" s="13"/>
+    </row>
+    <row r="112" spans="1:25" s="30" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A112" s="27" t="s">
         <v>209</v>
       </c>
-      <c r="B112" s="11" t="s">
-        <v>212</v>
-      </c>
-      <c r="C112" s="12"/>
+      <c r="B112" s="27" t="s">
+        <v>210</v>
+      </c>
+      <c r="C112" s="28"/>
       <c r="D112" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E112" s="12"/>
-      <c r="F112" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="G112" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="H112" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="I112" s="12"/>
-      <c r="J112" s="12"/>
-      <c r="K112" s="12"/>
-      <c r="L112" s="12"/>
-      <c r="M112" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="N112" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="O112" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="P112" s="12"/>
-      <c r="Q112" s="12"/>
-      <c r="R112" s="12"/>
-      <c r="S112" s="12"/>
-      <c r="T112" s="12"/>
-      <c r="U112" s="12"/>
-      <c r="V112" s="12"/>
-      <c r="W112" s="12"/>
-      <c r="X112" s="12"/>
-      <c r="Y112" s="7"/>
+      <c r="E112" s="28"/>
+      <c r="F112" s="28"/>
+      <c r="G112" s="28"/>
+      <c r="H112" s="28"/>
+      <c r="I112" s="28"/>
+      <c r="J112" s="28"/>
+      <c r="K112" s="28"/>
+      <c r="L112" s="28"/>
+      <c r="M112" s="28"/>
+      <c r="N112" s="28"/>
+      <c r="O112" s="28"/>
+      <c r="P112" s="28"/>
+      <c r="Q112" s="28"/>
+      <c r="R112" s="28"/>
+      <c r="S112" s="28"/>
+      <c r="T112" s="28"/>
+      <c r="U112" s="28"/>
+      <c r="V112" s="28"/>
+      <c r="W112" s="28"/>
+      <c r="X112" s="28"/>
+      <c r="Y112" s="29" t="s">
+        <v>211</v>
+      </c>
     </row>
     <row r="113" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A113" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B113" s="11" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C113" s="12"/>
       <c r="D113" s="12" t="s">
         <v>41</v>
       </c>
       <c r="E113" s="12"/>
-      <c r="F113" s="12"/>
-      <c r="G113" s="12"/>
-      <c r="H113" s="12"/>
+      <c r="F113" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="G113" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="H113" s="12" t="s">
+        <v>46</v>
+      </c>
       <c r="I113" s="12"/>
       <c r="J113" s="12"/>
       <c r="K113" s="12"/>
       <c r="L113" s="12"/>
-      <c r="M113" s="12"/>
-      <c r="N113" s="12"/>
-      <c r="O113" s="12"/>
+      <c r="M113" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="N113" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="O113" s="12" t="s">
+        <v>46</v>
+      </c>
       <c r="P113" s="12"/>
       <c r="Q113" s="12"/>
       <c r="R113" s="12"/>
@@ -11717,7 +11877,7 @@
         <v>209</v>
       </c>
       <c r="B114" s="11" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C114" s="12"/>
       <c r="D114" s="12" t="s">
@@ -11750,7 +11910,7 @@
         <v>209</v>
       </c>
       <c r="B115" s="11" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C115" s="12"/>
       <c r="D115" s="12" t="s">
@@ -11783,7 +11943,7 @@
         <v>209</v>
       </c>
       <c r="B116" s="11" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C116" s="12"/>
       <c r="D116" s="12" t="s">
@@ -11816,7 +11976,7 @@
         <v>209</v>
       </c>
       <c r="B117" s="11" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C117" s="12"/>
       <c r="D117" s="12" t="s">
@@ -11849,7 +12009,7 @@
         <v>209</v>
       </c>
       <c r="B118" s="11" t="s">
-        <v>76</v>
+        <v>217</v>
       </c>
       <c r="C118" s="12"/>
       <c r="D118" s="12" t="s">
@@ -11882,7 +12042,7 @@
         <v>209</v>
       </c>
       <c r="B119" s="11" t="s">
-        <v>218</v>
+        <v>76</v>
       </c>
       <c r="C119" s="12"/>
       <c r="D119" s="12" t="s">
@@ -11914,74 +12074,74 @@
       <c r="A120" s="11" t="s">
         <v>209</v>
       </c>
-      <c r="B120" s="14" t="s">
-        <v>219</v>
-      </c>
-      <c r="C120" s="15"/>
-      <c r="D120" s="15" t="s">
+      <c r="B120" s="11" t="s">
+        <v>218</v>
+      </c>
+      <c r="C120" s="12"/>
+      <c r="D120" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E120" s="15"/>
-      <c r="F120" s="15"/>
-      <c r="G120" s="15"/>
-      <c r="H120" s="15"/>
-      <c r="I120" s="15"/>
-      <c r="J120" s="15"/>
-      <c r="K120" s="15"/>
-      <c r="L120" s="15"/>
-      <c r="M120" s="15"/>
-      <c r="N120" s="15"/>
-      <c r="O120" s="15"/>
-      <c r="P120" s="15"/>
-      <c r="Q120" s="15"/>
-      <c r="R120" s="15"/>
-      <c r="S120" s="15"/>
-      <c r="T120" s="15"/>
-      <c r="U120" s="15"/>
-      <c r="V120" s="15"/>
-      <c r="W120" s="15"/>
-      <c r="X120" s="15"/>
-      <c r="Y120" s="13"/>
+      <c r="E120" s="12"/>
+      <c r="F120" s="12"/>
+      <c r="G120" s="12"/>
+      <c r="H120" s="12"/>
+      <c r="I120" s="12"/>
+      <c r="J120" s="12"/>
+      <c r="K120" s="12"/>
+      <c r="L120" s="12"/>
+      <c r="M120" s="12"/>
+      <c r="N120" s="12"/>
+      <c r="O120" s="12"/>
+      <c r="P120" s="12"/>
+      <c r="Q120" s="12"/>
+      <c r="R120" s="12"/>
+      <c r="S120" s="12"/>
+      <c r="T120" s="12"/>
+      <c r="U120" s="12"/>
+      <c r="V120" s="12"/>
+      <c r="W120" s="12"/>
+      <c r="X120" s="12"/>
+      <c r="Y120" s="7"/>
     </row>
     <row r="121" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A121" s="11" t="s">
         <v>209</v>
       </c>
-      <c r="B121" s="11" t="s">
-        <v>220</v>
-      </c>
-      <c r="C121" s="12"/>
-      <c r="D121" s="12" t="s">
+      <c r="B121" s="14" t="s">
+        <v>219</v>
+      </c>
+      <c r="C121" s="15"/>
+      <c r="D121" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="E121" s="12"/>
-      <c r="F121" s="12"/>
-      <c r="G121" s="12"/>
-      <c r="H121" s="12"/>
-      <c r="I121" s="12"/>
-      <c r="J121" s="12"/>
-      <c r="K121" s="12"/>
-      <c r="L121" s="12"/>
-      <c r="M121" s="12"/>
-      <c r="N121" s="12"/>
-      <c r="O121" s="12"/>
-      <c r="P121" s="12"/>
-      <c r="Q121" s="12"/>
-      <c r="R121" s="12"/>
-      <c r="S121" s="12"/>
-      <c r="T121" s="12"/>
-      <c r="U121" s="12"/>
-      <c r="V121" s="12"/>
-      <c r="W121" s="12"/>
-      <c r="X121" s="12"/>
-      <c r="Y121" s="7"/>
+      <c r="E121" s="15"/>
+      <c r="F121" s="15"/>
+      <c r="G121" s="15"/>
+      <c r="H121" s="15"/>
+      <c r="I121" s="15"/>
+      <c r="J121" s="15"/>
+      <c r="K121" s="15"/>
+      <c r="L121" s="15"/>
+      <c r="M121" s="15"/>
+      <c r="N121" s="15"/>
+      <c r="O121" s="15"/>
+      <c r="P121" s="15"/>
+      <c r="Q121" s="15"/>
+      <c r="R121" s="15"/>
+      <c r="S121" s="15"/>
+      <c r="T121" s="15"/>
+      <c r="U121" s="15"/>
+      <c r="V121" s="15"/>
+      <c r="W121" s="15"/>
+      <c r="X121" s="15"/>
+      <c r="Y121" s="13"/>
     </row>
     <row r="122" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A122" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B122" s="11" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C122" s="12"/>
       <c r="D122" s="12" t="s">
@@ -12014,7 +12174,7 @@
         <v>209</v>
       </c>
       <c r="B123" s="11" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C123" s="12"/>
       <c r="D123" s="12" t="s">
@@ -12047,7 +12207,7 @@
         <v>209</v>
       </c>
       <c r="B124" s="11" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C124" s="12"/>
       <c r="D124" s="12" t="s">
@@ -12075,12 +12235,12 @@
       <c r="X124" s="12"/>
       <c r="Y124" s="7"/>
     </row>
-    <row r="125" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="125" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A125" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B125" s="11" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C125" s="12"/>
       <c r="D125" s="12" t="s">
@@ -12113,7 +12273,7 @@
         <v>209</v>
       </c>
       <c r="B126" s="11" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C126" s="12"/>
       <c r="D126" s="12" t="s">
@@ -12146,7 +12306,7 @@
         <v>209</v>
       </c>
       <c r="B127" s="11" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C127" s="12"/>
       <c r="D127" s="12" t="s">
@@ -12179,7 +12339,7 @@
         <v>209</v>
       </c>
       <c r="B128" s="11" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C128" s="12"/>
       <c r="D128" s="12" t="s">
@@ -12212,7 +12372,7 @@
         <v>209</v>
       </c>
       <c r="B129" s="11" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C129" s="12"/>
       <c r="D129" s="12" t="s">
@@ -12245,7 +12405,7 @@
         <v>209</v>
       </c>
       <c r="B130" s="11" t="s">
-        <v>264</v>
+        <v>228</v>
       </c>
       <c r="C130" s="12"/>
       <c r="D130" s="12" t="s">
@@ -12278,11 +12438,11 @@
         <v>209</v>
       </c>
       <c r="B131" s="11" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="C131" s="12"/>
       <c r="D131" s="12" t="s">
-        <v>100</v>
+        <v>41</v>
       </c>
       <c r="E131" s="12"/>
       <c r="F131" s="12"/>
@@ -12311,11 +12471,11 @@
         <v>209</v>
       </c>
       <c r="B132" s="11" t="s">
-        <v>229</v>
+        <v>270</v>
       </c>
       <c r="C132" s="12"/>
       <c r="D132" s="12" t="s">
-        <v>41</v>
+        <v>100</v>
       </c>
       <c r="E132" s="12"/>
       <c r="F132" s="12"/>
@@ -12341,136 +12501,169 @@
     </row>
     <row r="133" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A133" s="11" t="s">
-        <v>230</v>
+        <v>209</v>
       </c>
       <c r="B133" s="11" t="s">
-        <v>231</v>
-      </c>
-      <c r="C133" s="16"/>
+        <v>229</v>
+      </c>
+      <c r="C133" s="12"/>
       <c r="D133" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E133" s="16"/>
-      <c r="F133" s="16"/>
-      <c r="G133" s="16"/>
-      <c r="H133" s="16"/>
-      <c r="I133" s="16"/>
-      <c r="J133" s="16"/>
-      <c r="K133" s="16"/>
-      <c r="L133" s="16"/>
-      <c r="M133" s="16"/>
-      <c r="N133" s="16"/>
-      <c r="O133" s="16"/>
-      <c r="P133" s="16"/>
-      <c r="Q133" s="16"/>
-      <c r="R133" s="16"/>
-      <c r="S133" s="16"/>
-      <c r="T133" s="16"/>
-      <c r="U133" s="16"/>
-      <c r="V133" s="16"/>
-      <c r="W133" s="16"/>
-      <c r="X133" s="16"/>
+      <c r="E133" s="12"/>
+      <c r="F133" s="12"/>
+      <c r="G133" s="12"/>
+      <c r="H133" s="12"/>
+      <c r="I133" s="12"/>
+      <c r="J133" s="12"/>
+      <c r="K133" s="12"/>
+      <c r="L133" s="12"/>
+      <c r="M133" s="12"/>
+      <c r="N133" s="12"/>
+      <c r="O133" s="12"/>
+      <c r="P133" s="12"/>
+      <c r="Q133" s="12"/>
+      <c r="R133" s="12"/>
+      <c r="S133" s="12"/>
+      <c r="T133" s="12"/>
+      <c r="U133" s="12"/>
+      <c r="V133" s="12"/>
+      <c r="W133" s="12"/>
+      <c r="X133" s="12"/>
       <c r="Y133" s="7"/>
     </row>
     <row r="134" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A134" s="11" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B134" s="11" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C134" s="16"/>
       <c r="D134" s="12" t="s">
-        <v>234</v>
-      </c>
-      <c r="E134" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="F134" s="31"/>
-      <c r="G134" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="H134" s="31"/>
-      <c r="I134" s="31"/>
-      <c r="J134" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="K134" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="L134" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="M134" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="N134" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="O134" s="31"/>
-      <c r="P134" s="31"/>
-      <c r="Q134" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="R134" s="31" t="s">
-        <v>236</v>
-      </c>
-      <c r="S134" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="T134" s="31"/>
-      <c r="U134" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="V134" s="31"/>
-      <c r="W134" s="31"/>
-      <c r="X134" s="31"/>
+        <v>41</v>
+      </c>
+      <c r="E134" s="16"/>
+      <c r="F134" s="16"/>
+      <c r="G134" s="16"/>
+      <c r="H134" s="16"/>
+      <c r="I134" s="16"/>
+      <c r="J134" s="16"/>
+      <c r="K134" s="16"/>
+      <c r="L134" s="16"/>
+      <c r="M134" s="16"/>
+      <c r="N134" s="16"/>
+      <c r="O134" s="16"/>
+      <c r="P134" s="16"/>
+      <c r="Q134" s="16"/>
+      <c r="R134" s="16"/>
+      <c r="S134" s="16"/>
+      <c r="T134" s="16"/>
+      <c r="U134" s="16"/>
+      <c r="V134" s="16"/>
+      <c r="W134" s="16"/>
+      <c r="X134" s="16"/>
       <c r="Y134" s="7"/>
     </row>
     <row r="135" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A135" s="11" t="s">
-        <v>265</v>
+        <v>232</v>
       </c>
       <c r="B135" s="11" t="s">
-        <v>265</v>
+        <v>233</v>
       </c>
       <c r="C135" s="16"/>
       <c r="D135" s="12" t="s">
-        <v>38</v>
+        <v>234</v>
       </c>
       <c r="E135" s="31" t="s">
-        <v>38</v>
+        <v>234</v>
       </c>
       <c r="F135" s="31"/>
-      <c r="G135" s="31"/>
+      <c r="G135" s="31" t="s">
+        <v>234</v>
+      </c>
       <c r="H135" s="31"/>
       <c r="I135" s="31"/>
-      <c r="J135" s="31"/>
+      <c r="J135" s="31" t="s">
+        <v>235</v>
+      </c>
       <c r="K135" s="31" t="s">
-        <v>38</v>
+        <v>234</v>
       </c>
       <c r="L135" s="31" t="s">
-        <v>38</v>
-      </c>
-      <c r="M135" s="31"/>
-      <c r="N135" s="31"/>
+        <v>234</v>
+      </c>
+      <c r="M135" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="N135" s="31" t="s">
+        <v>234</v>
+      </c>
       <c r="O135" s="31"/>
       <c r="P135" s="31"/>
-      <c r="Q135" s="31"/>
-      <c r="R135" s="31"/>
-      <c r="S135" s="31"/>
+      <c r="Q135" s="31" t="s">
+        <v>235</v>
+      </c>
+      <c r="R135" s="31" t="s">
+        <v>236</v>
+      </c>
+      <c r="S135" s="31" t="s">
+        <v>235</v>
+      </c>
       <c r="T135" s="31"/>
-      <c r="U135" s="31"/>
+      <c r="U135" s="31" t="s">
+        <v>235</v>
+      </c>
       <c r="V135" s="31"/>
       <c r="W135" s="31"/>
       <c r="X135" s="31"/>
       <c r="Y135" s="7"/>
     </row>
+    <row r="136" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A136" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="B136" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="C136" s="16"/>
+      <c r="D136" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="E136" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="F136" s="31"/>
+      <c r="G136" s="31"/>
+      <c r="H136" s="31"/>
+      <c r="I136" s="31"/>
+      <c r="J136" s="31"/>
+      <c r="K136" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="L136" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="M136" s="31"/>
+      <c r="N136" s="31"/>
+      <c r="O136" s="31"/>
+      <c r="P136" s="31"/>
+      <c r="Q136" s="31"/>
+      <c r="R136" s="31"/>
+      <c r="S136" s="31"/>
+      <c r="T136" s="31"/>
+      <c r="U136" s="31"/>
+      <c r="V136" s="31"/>
+      <c r="W136" s="31"/>
+      <c r="X136" s="31"/>
+      <c r="Y136" s="7"/>
+    </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="130">
-      <pane xSplit="2" ySplit="6" topLeftCell="C53" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="B71" sqref="B71"/>
+    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="115">
+      <pane xSplit="2" ySplit="6" topLeftCell="Q19" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="Y37" sqref="Y37"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
@@ -12480,15 +12673,15 @@
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
-    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="115">
-      <pane xSplit="2" ySplit="6" topLeftCell="C86" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="B126" sqref="B126"/>
+    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="130">
+      <pane xSplit="2" ySplit="6" topLeftCell="C53" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="B71" sqref="B71"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
   </customSheetViews>
   <mergeCells count="6">
-    <mergeCell ref="Y107:Y108"/>
+    <mergeCell ref="Y108:Y109"/>
     <mergeCell ref="C1:O1"/>
     <mergeCell ref="C2:O2"/>
     <mergeCell ref="C5:H5"/>
@@ -12834,7 +13027,7 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="150">
+    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="150">
       <selection activeCell="A22" sqref="A22"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -12844,7 +13037,7 @@
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
-    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="150">
+    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="150">
       <selection activeCell="A22" sqref="A22"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Muuta roolit.xlsx testiympäristöä varten
</commit_message>
<xml_diff>
--- a/resources/roolit.xlsx
+++ b/resources/roolit.xlsx
@@ -1,46 +1,48 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lauri.nayha/Projects/harja/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\samuli\dev\harjaroot\harja\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:81_{A8790524-4076-984A-9AA0-56B44D9CB46B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:81_{C33009BB-AF4A-4311-9633-F3E6F0CC09C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="98860" yWindow="2380" windowWidth="34560" windowHeight="14920" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="23748" yWindow="156" windowWidth="25476" windowHeight="14232" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Oikeudet" sheetId="1" r:id="rId1"/>
     <sheet name="Roolit" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_1CE83972_B6A5_C44D_86E5_E9D9B38739F4_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_1DD617EE_F308_3E45_A8EF_4713F47FA0DD_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_2064F962_35EF_41F3_8A86_D37B72D177C7_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_3EBD3306_FC69_2148_8542_F6313DC2056F_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_47348D7B_5AFC_4A25_B239_A26E1359728E_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_476C495F_6E55_F04C_8145_4E8EBD6B3DE3_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_5327B0A1_A5FC_7747_93A1_427B210F3DF4_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_56F6E422_2CD8_6B4D_9E39_69A269028D26_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_6AA8E519_028C_D745_9E2E_8FB60E5B789F_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_7A9649F2_657F_9445_B6E6_FE94C6A09957_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_8411E1B5_4691_4435_A9A2_147FF80D0D98_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_843152D8_333A_1941_83E9_0CB5262068A2_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_87BEAE97_700C_BF40_B102_636C54D81F08_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_D01EF3E4_E485_4912_A9DA_396AAE5B8752_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_D57E2FB1_FF7F_8446_9C97_237A4D57F6BE_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_E3BBF62E_A283_4D48_98B7_21A2A94F634F_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_F86DF6F3_8AE5_3A44_B2D2_D623E01AE54F_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_1CE83972_B6A5_C44D_86E5_E9D9B38739F4_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_1DD617EE_F308_3E45_A8EF_4713F47FA0DD_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_2064F962_35EF_41F3_8A86_D37B72D177C7_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_3EBD3306_FC69_2148_8542_F6313DC2056F_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_47348D7B_5AFC_4A25_B239_A26E1359728E_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_476C495F_6E55_F04C_8145_4E8EBD6B3DE3_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_5327B0A1_A5FC_7747_93A1_427B210F3DF4_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_56F6E422_2CD8_6B4D_9E39_69A269028D26_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_6AA8E519_028C_D745_9E2E_8FB60E5B789F_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_7A9649F2_657F_9445_B6E6_FE94C6A09957_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_810C905A_C0DA_4100_B6A9_F2260D80EA70_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_8411E1B5_4691_4435_A9A2_147FF80D0D98_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_843152D8_333A_1941_83E9_0CB5262068A2_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_87BEAE97_700C_BF40_B102_636C54D81F08_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_D01EF3E4_E485_4912_A9DA_396AAE5B8752_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_D57E2FB1_FF7F_8446_9C97_237A4D57F6BE_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_E3BBF62E_A283_4D48_98B7_21A2A94F634F_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_F86DF6F3_8AE5_3A44_B2D2_D623E01AE54F_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
   </definedNames>
   <calcPr calcId="0"/>
   <customWorkbookViews>
+    <customWorkbookView name="Samuli Taskila - Personal View" guid="{810C905A-C0DA-4100-B6A9-F2260D80EA70}" mergeInterval="0" personalView="1" xWindow="1979" yWindow="13" windowWidth="2123" windowHeight="1186" tabRatio="500" activeSheetId="1"/>
+    <customWorkbookView name="Microsoft Office User - Oma näkymä" guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" mergeInterval="0" personalView="1" xWindow="1440" yWindow="-515" windowWidth="2056" windowHeight="1366" tabRatio="500" activeSheetId="1"/>
+    <customWorkbookView name="Jarno Väyrynen - Personal View" guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" mergeInterval="0" personalView="1" xWindow="48" yWindow="25" windowWidth="2512" windowHeight="1336" tabRatio="500" activeSheetId="1"/>
     <customWorkbookView name="Microsoft Office User - Personal View" guid="{843152D8-333A-1941-83E9-0CB5262068A2}" mergeInterval="0" personalView="1" xWindow="4943" yWindow="119" windowWidth="1728" windowHeight="746" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Jarno Väyrynen - Personal View" guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" mergeInterval="0" personalView="1" xWindow="48" yWindow="25" windowWidth="2512" windowHeight="1336" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Microsoft Office User - Oma näkymä" guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" mergeInterval="0" personalView="1" xWindow="1440" yWindow="-515" windowWidth="2056" windowHeight="1366" tabRatio="500" activeSheetId="1"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -110,7 +112,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1947" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1989" uniqueCount="275">
   <si>
     <t xml:space="preserve">Roolimääritysten selitykset: </t>
   </si>
@@ -1001,6 +1003,12 @@
   </si>
   <si>
     <t>Koitetaan pärjätä yhdellä rivillä kaikkien välilehtien osalta</t>
+  </si>
+  <si>
+    <t>Tiemerkintä - Muut kustannukset</t>
+  </si>
+  <si>
+    <t>Tiemerkintä - Sakot ja bonukset</t>
   </si>
 </sst>
 </file>
@@ -1385,7 +1393,7 @@
 </file>
 
 <file path=xl/revisions/revisionHeaders.xml><?xml version="1.0" encoding="utf-8"?>
-<headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" guid="{16592C61-0221-A548-A820-56B21F0EE301}" diskRevisions="1" revisionId="224" version="13">
+<headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" guid="{4A6ED1B0-9135-4362-95CD-B6A2DDFC57B0}" diskRevisions="1" revisionId="269" version="14">
   <header guid="{8EBC2E30-8A6E-AD43-9F6F-B4500CF04203}" dateTime="2024-06-11T12:49:05" maxSheetId="3" userName="Jarno Väyrynen" r:id="rId9" minRId="87" maxRId="97">
     <sheetIdMap count="2">
       <sheetId val="1"/>
@@ -1440,6 +1448,12 @@
       <sheetId val="2"/>
     </sheetIdMap>
   </header>
+  <header guid="{4A6ED1B0-9135-4362-95CD-B6A2DDFC57B0}" dateTime="2025-04-02T11:13:06" maxSheetId="3" userName="Samuli Taskila" r:id="rId18" minRId="225" maxRId="268">
+    <sheetIdMap count="2">
+      <sheetId val="1"/>
+      <sheetId val="2"/>
+    </sheetIdMap>
+  </header>
 </headers>
 </file>
 
@@ -1471,6 +1485,335 @@
     <formula>Oikeudet!$A$5:$Y$128</formula>
   </rdn>
   <rcv guid="{843152D8-333A-1941-83E9-0CB5262068A2}" action="add"/>
+</revisions>
+</file>
+
+<file path=xl/revisions/revisionLog10.xml><?xml version="1.0" encoding="utf-8"?>
+<revisions xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <rrc rId="225" sId="1" ref="A107:XFD107" action="insertRow"/>
+  <rfmt sheetId="1" sqref="Y107" start="0" length="0">
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+  </rfmt>
+  <rcc rId="226" sId="1">
+    <nc r="A107" t="inlineStr">
+      <is>
+        <t>Raportit</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="227" sId="1">
+    <nc r="D107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="228" sId="1">
+    <nc r="E107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="229" sId="1">
+    <nc r="F107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="230" sId="1">
+    <nc r="G107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="231" sId="1">
+    <nc r="H107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="232" sId="1">
+    <nc r="I107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="233" sId="1">
+    <nc r="J107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="234" sId="1">
+    <nc r="K107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="235" sId="1">
+    <nc r="L107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="236" sId="1">
+    <nc r="M107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="237" sId="1">
+    <nc r="N107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="238" sId="1">
+    <nc r="P107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="239" sId="1">
+    <nc r="Q107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="240" sId="1">
+    <nc r="R107" t="inlineStr">
+      <is>
+        <t>R+</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="241" sId="1">
+    <nc r="S107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="242" sId="1">
+    <nc r="T107" t="inlineStr">
+      <is>
+        <t>R+</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="243" sId="1">
+    <nc r="U107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="244" sId="1">
+    <nc r="V107" t="inlineStr">
+      <is>
+        <t>R+</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="245" sId="1">
+    <nc r="X107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rfmt sheetId="1" sqref="Y107" start="0" length="0">
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+  </rfmt>
+  <rcc rId="246" sId="1">
+    <nc r="B107" t="inlineStr">
+      <is>
+        <t>Tiemerkintä - Muut kustannukset</t>
+      </is>
+    </nc>
+  </rcc>
+  <rrc rId="247" sId="1" ref="A107:XFD107" action="insertRow"/>
+  <rcc rId="248" sId="1">
+    <nc r="A107" t="inlineStr">
+      <is>
+        <t>Raportit</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="249" sId="1">
+    <nc r="D107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="250" sId="1">
+    <nc r="E107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="251" sId="1">
+    <nc r="F107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="252" sId="1">
+    <nc r="G107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="253" sId="1">
+    <nc r="H107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="254" sId="1">
+    <nc r="I107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="255" sId="1">
+    <nc r="J107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="256" sId="1">
+    <nc r="K107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="257" sId="1">
+    <nc r="L107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="258" sId="1">
+    <nc r="M107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="259" sId="1">
+    <nc r="N107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="260" sId="1">
+    <nc r="P107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="261" sId="1">
+    <nc r="Q107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="262" sId="1">
+    <nc r="R107" t="inlineStr">
+      <is>
+        <t>R+</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="263" sId="1">
+    <nc r="S107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="264" sId="1">
+    <nc r="T107" t="inlineStr">
+      <is>
+        <t>R+</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="265" sId="1">
+    <nc r="U107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="266" sId="1">
+    <nc r="V107" t="inlineStr">
+      <is>
+        <t>R+</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="267" sId="1">
+    <nc r="X107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="268" sId="1">
+    <nc r="B107" t="inlineStr">
+      <is>
+        <t>Tiemerkintä - Sakot ja bonukset</t>
+      </is>
+    </nc>
+  </rcc>
+  <rdn rId="0" localSheetId="1" customView="1" name="Z_810C905A_C0DA_4100_B6A9_F2260D80EA70_.wvu.FilterData" hidden="1" oldHidden="1">
+    <formula>Oikeudet!$A$5:$Y$136</formula>
+  </rdn>
+  <rcv guid="{810C905A-C0DA-4100-B6A9-F2260D80EA70}" action="add"/>
 </revisions>
 </file>
 
@@ -5137,11 +5480,12 @@
 </file>
 
 <file path=xl/revisions/userNames.xml><?xml version="1.0" encoding="utf-8"?>
-<users xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" count="4">
+<users xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" count="5">
   <userInfo guid="{8EBC2E30-8A6E-AD43-9F6F-B4500CF04203}" name="Jarno Väyrynen" id="-589133089" dateTime="2024-06-10T14:55:26"/>
   <userInfo guid="{CFB45395-62D4-124C-9898-DEF874662F1B}" name="Microsoft Office User" id="-296973103" dateTime="2024-11-20T15:04:38"/>
   <userInfo guid="{CF3F0B66-D3D6-2C4C-93DF-DEE3169712D4}" name="Microsoft Office User" id="-296992802" dateTime="2024-12-13T10:34:14"/>
   <userInfo guid="{64AC07D8-8D49-4F46-96EF-A9E3AD0E8431}" name="Jarno Väyrynen" id="-589128654" dateTime="2025-02-12T12:58:37"/>
+  <userInfo guid="{4A6ED1B0-9135-4362-95CD-B6A2DDFC57B0}" name="Samuli Taskila" id="-1631752395" dateTime="2025-04-02T11:10:08"/>
 </users>
 </file>
 
@@ -5321,12 +5665,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y136"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <dimension ref="A1:Y138"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="31.6640625" customWidth="1"/>
-    <col min="3" max="3" width="14.1640625" customWidth="1"/>
+    <col min="3" max="3" width="14.109375" customWidth="1"/>
     <col min="4" max="4" width="30.33203125" customWidth="1"/>
     <col min="5" max="5" width="26.33203125" customWidth="1"/>
     <col min="6" max="6" width="12.6640625" customWidth="1"/>
@@ -5335,22 +5679,22 @@
     <col min="9" max="9" width="18.33203125" customWidth="1"/>
     <col min="10" max="10" width="25.33203125" customWidth="1"/>
     <col min="11" max="11" width="40.6640625" customWidth="1"/>
-    <col min="12" max="12" width="38.1640625" customWidth="1"/>
+    <col min="12" max="12" width="38.109375" customWidth="1"/>
     <col min="13" max="13" width="12.33203125" customWidth="1"/>
     <col min="14" max="14" width="10.6640625" customWidth="1"/>
-    <col min="15" max="16" width="12.5" customWidth="1"/>
+    <col min="15" max="16" width="12.44140625" customWidth="1"/>
     <col min="17" max="17" width="21.6640625" customWidth="1"/>
     <col min="18" max="18" width="36" customWidth="1"/>
     <col min="19" max="19" width="29.6640625" customWidth="1"/>
     <col min="20" max="20" width="15" customWidth="1"/>
     <col min="21" max="21" width="17.6640625" customWidth="1"/>
-    <col min="22" max="22" width="11.5" customWidth="1"/>
+    <col min="22" max="22" width="11.44140625" customWidth="1"/>
     <col min="23" max="23" width="11.6640625" customWidth="1"/>
     <col min="24" max="24" width="11.33203125" customWidth="1"/>
     <col min="25" max="25" width="59" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="24" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:25" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -5371,7 +5715,7 @@
       <c r="N1" s="36"/>
       <c r="O1" s="36"/>
     </row>
-    <row r="2" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="37" t="s">
@@ -5390,7 +5734,7 @@
       <c r="N2" s="37"/>
       <c r="O2" s="37"/>
     </row>
-    <row r="3" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3" s="2" t="s">
         <v>3</v>
@@ -5405,10 +5749,10 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C4" s="6"/>
     </row>
-    <row r="5" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7"/>
       <c r="B5" s="7"/>
       <c r="C5" s="38" t="s">
@@ -5443,7 +5787,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>11</v>
       </c>
@@ -5516,7 +5860,7 @@
       </c>
       <c r="Y6" s="7"/>
     </row>
-    <row r="7" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>34</v>
       </c>
@@ -5589,7 +5933,7 @@
       </c>
       <c r="Y7" s="13"/>
     </row>
-    <row r="8" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>34</v>
       </c>
@@ -5648,7 +5992,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>34</v>
       </c>
@@ -5701,7 +6045,7 @@
       <c r="X9" s="12"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>34</v>
       </c>
@@ -5754,7 +6098,7 @@
       <c r="X10" s="12"/>
       <c r="Y10" s="13"/>
     </row>
-    <row r="11" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
         <v>34</v>
       </c>
@@ -5813,7 +6157,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>34</v>
       </c>
@@ -5866,7 +6210,7 @@
       <c r="X12" s="12"/>
       <c r="Y12" s="13"/>
     </row>
-    <row r="13" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
         <v>34</v>
       </c>
@@ -5933,7 +6277,7 @@
       <c r="X13" s="12"/>
       <c r="Y13" s="13"/>
     </row>
-    <row r="14" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
         <v>34</v>
       </c>
@@ -6000,7 +6344,7 @@
       <c r="X14" s="12"/>
       <c r="Y14" s="13"/>
     </row>
-    <row r="15" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
         <v>34</v>
       </c>
@@ -6057,7 +6401,7 @@
       <c r="X15" s="12"/>
       <c r="Y15" s="13"/>
     </row>
-    <row r="16" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
         <v>34</v>
       </c>
@@ -6114,7 +6458,7 @@
       <c r="X16" s="12"/>
       <c r="Y16" s="13"/>
     </row>
-    <row r="17" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
         <v>34</v>
       </c>
@@ -6171,7 +6515,7 @@
       <c r="X17" s="12"/>
       <c r="Y17" s="13"/>
     </row>
-    <row r="18" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
         <v>34</v>
       </c>
@@ -6238,7 +6582,7 @@
       <c r="X18" s="12"/>
       <c r="Y18" s="13"/>
     </row>
-    <row r="19" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
         <v>34</v>
       </c>
@@ -6305,7 +6649,7 @@
       <c r="X19" s="12"/>
       <c r="Y19" s="13"/>
     </row>
-    <row r="20" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
         <v>34</v>
       </c>
@@ -6360,7 +6704,7 @@
       <c r="X20" s="12"/>
       <c r="Y20" s="13"/>
     </row>
-    <row r="21" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
         <v>34</v>
       </c>
@@ -6421,7 +6765,7 @@
       <c r="X21" s="12"/>
       <c r="Y21" s="13"/>
     </row>
-    <row r="22" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
         <v>34</v>
       </c>
@@ -6488,7 +6832,7 @@
       <c r="X22" s="12"/>
       <c r="Y22" s="13"/>
     </row>
-    <row r="23" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
         <v>34</v>
       </c>
@@ -6561,7 +6905,7 @@
       </c>
       <c r="Y23" s="13"/>
     </row>
-    <row r="24" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
         <v>34</v>
       </c>
@@ -6634,7 +6978,7 @@
       </c>
       <c r="Y24" s="13"/>
     </row>
-    <row r="25" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
         <v>34</v>
       </c>
@@ -6707,7 +7051,7 @@
       </c>
       <c r="Y25" s="13"/>
     </row>
-    <row r="26" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
         <v>34</v>
       </c>
@@ -6778,7 +7122,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="27" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
         <v>34</v>
       </c>
@@ -6847,7 +7191,7 @@
       <c r="X27" s="12"/>
       <c r="Y27" s="13"/>
     </row>
-    <row r="28" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
         <v>34</v>
       </c>
@@ -6893,7 +7237,7 @@
       </c>
       <c r="Y28" s="13"/>
     </row>
-    <row r="29" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
         <v>34</v>
       </c>
@@ -6962,7 +7306,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="30" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
         <v>34</v>
       </c>
@@ -7023,7 +7367,7 @@
       <c r="X30" s="12"/>
       <c r="Y30" s="13"/>
     </row>
-    <row r="31" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="11" t="s">
         <v>34</v>
       </c>
@@ -7080,7 +7424,7 @@
       <c r="X31" s="12"/>
       <c r="Y31" s="13"/>
     </row>
-    <row r="32" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
         <v>34</v>
       </c>
@@ -7133,7 +7477,7 @@
       <c r="X32" s="12"/>
       <c r="Y32" s="13"/>
     </row>
-    <row r="33" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="11" t="s">
         <v>34</v>
       </c>
@@ -7178,7 +7522,7 @@
       <c r="X33" s="12"/>
       <c r="Y33" s="13"/>
     </row>
-    <row r="34" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="34" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="17" t="s">
         <v>34</v>
       </c>
@@ -7207,7 +7551,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="35" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="11" t="s">
         <v>34</v>
       </c>
@@ -7254,7 +7598,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="36" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
         <v>34</v>
       </c>
@@ -7311,7 +7655,7 @@
       </c>
       <c r="Y36" s="13"/>
     </row>
-    <row r="37" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="11" t="s">
         <v>34</v>
       </c>
@@ -7368,7 +7712,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="38" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="38" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="11" t="s">
         <v>34</v>
       </c>
@@ -7421,7 +7765,7 @@
       <c r="X38" s="12"/>
       <c r="Y38" s="13"/>
     </row>
-    <row r="39" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="11" t="s">
         <v>34</v>
       </c>
@@ -7490,7 +7834,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="40" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="40" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
         <v>34</v>
       </c>
@@ -7553,7 +7897,7 @@
       <c r="X40" s="12"/>
       <c r="Y40" s="13"/>
     </row>
-    <row r="41" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="41" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="11" t="s">
         <v>34</v>
       </c>
@@ -7618,7 +7962,7 @@
       <c r="X41" s="12"/>
       <c r="Y41" s="13"/>
     </row>
-    <row r="42" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="42" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="11" t="s">
         <v>34</v>
       </c>
@@ -7681,7 +8025,7 @@
       <c r="X42" s="12"/>
       <c r="Y42" s="13"/>
     </row>
-    <row r="43" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="43" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="11" t="s">
         <v>34</v>
       </c>
@@ -7744,7 +8088,7 @@
       <c r="X43" s="12"/>
       <c r="Y43" s="13"/>
     </row>
-    <row r="44" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="44" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="11" t="s">
         <v>34</v>
       </c>
@@ -7807,7 +8151,7 @@
       <c r="X44" s="12"/>
       <c r="Y44" s="13"/>
     </row>
-    <row r="45" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="45" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="11" t="s">
         <v>34</v>
       </c>
@@ -7870,7 +8214,7 @@
       <c r="X45" s="12"/>
       <c r="Y45" s="7"/>
     </row>
-    <row r="46" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="46" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="11" t="s">
         <v>34</v>
       </c>
@@ -7933,7 +8277,7 @@
       <c r="X46" s="12"/>
       <c r="Y46" s="7"/>
     </row>
-    <row r="47" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="47" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="11" t="s">
         <v>34</v>
       </c>
@@ -7996,7 +8340,7 @@
       <c r="X47" s="12"/>
       <c r="Y47" s="7"/>
     </row>
-    <row r="48" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="48" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="11" t="s">
         <v>34</v>
       </c>
@@ -8069,7 +8413,7 @@
       </c>
       <c r="Y48" s="13"/>
     </row>
-    <row r="49" spans="1:25" ht="28" x14ac:dyDescent="0.15">
+    <row r="49" spans="1:25" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A49" s="11" t="s">
         <v>34</v>
       </c>
@@ -8122,7 +8466,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="50" spans="1:25" ht="70" x14ac:dyDescent="0.15">
+    <row r="50" spans="1:25" ht="66" x14ac:dyDescent="0.25">
       <c r="A50" s="11" t="s">
         <v>34</v>
       </c>
@@ -8175,7 +8519,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="51" spans="1:25" x14ac:dyDescent="0.15">
+    <row r="51" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A51" s="11" t="s">
         <v>34</v>
       </c>
@@ -8226,7 +8570,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="52" spans="1:25" ht="14" x14ac:dyDescent="0.15">
+    <row r="52" spans="1:25" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A52" s="11" t="s">
         <v>34</v>
       </c>
@@ -8275,7 +8619,7 @@
       <c r="X52" s="15"/>
       <c r="Y52" s="7"/>
     </row>
-    <row r="53" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="53" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="17" t="s">
         <v>34</v>
       </c>
@@ -8326,7 +8670,7 @@
       <c r="W53" s="22"/>
       <c r="X53" s="22"/>
     </row>
-    <row r="54" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="54" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11" t="s">
         <v>34</v>
       </c>
@@ -8375,7 +8719,7 @@
       <c r="X54" s="15"/>
       <c r="Y54" s="13"/>
     </row>
-    <row r="55" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="55" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="11" t="s">
         <v>34</v>
       </c>
@@ -8408,7 +8752,7 @@
       <c r="X55" s="12"/>
       <c r="Y55" s="13"/>
     </row>
-    <row r="56" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="56" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="11" t="s">
         <v>34</v>
       </c>
@@ -8461,7 +8805,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="57" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="57" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="11" t="s">
         <v>34</v>
       </c>
@@ -8494,7 +8838,7 @@
       <c r="X57" s="12"/>
       <c r="Y57" s="13"/>
     </row>
-    <row r="58" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="58" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="11" t="s">
         <v>34</v>
       </c>
@@ -8545,7 +8889,7 @@
       <c r="X58" s="12"/>
       <c r="Y58" s="13"/>
     </row>
-    <row r="59" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="59" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="11" t="s">
         <v>34</v>
       </c>
@@ -8608,7 +8952,7 @@
       <c r="X59" s="12"/>
       <c r="Y59" s="13"/>
     </row>
-    <row r="60" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="60" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="23" t="s">
         <v>34</v>
       </c>
@@ -8667,7 +9011,7 @@
       <c r="X60" s="12"/>
       <c r="Y60" s="13"/>
     </row>
-    <row r="61" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="61" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="23" t="s">
         <v>34</v>
       </c>
@@ -8728,7 +9072,7 @@
       <c r="X61" s="12"/>
       <c r="Y61" s="13"/>
     </row>
-    <row r="62" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="62" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="23" t="s">
         <v>34</v>
       </c>
@@ -8783,7 +9127,7 @@
       <c r="X62" s="12"/>
       <c r="Y62" s="13"/>
     </row>
-    <row r="63" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="63" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="11" t="s">
         <v>34</v>
       </c>
@@ -8856,7 +9200,7 @@
       </c>
       <c r="Y63" s="13"/>
     </row>
-    <row r="64" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="64" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="11" t="s">
         <v>160</v>
       </c>
@@ -8909,7 +9253,7 @@
       <c r="X64" s="12"/>
       <c r="Y64" s="13"/>
     </row>
-    <row r="65" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="65" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="11" t="s">
         <v>160</v>
       </c>
@@ -8962,7 +9306,7 @@
       <c r="X65" s="12"/>
       <c r="Y65" s="13"/>
     </row>
-    <row r="66" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="66" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="11" t="s">
         <v>160</v>
       </c>
@@ -9015,7 +9359,7 @@
       <c r="X66" s="12"/>
       <c r="Y66" s="13"/>
     </row>
-    <row r="67" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="67" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="11" t="s">
         <v>160</v>
       </c>
@@ -9068,7 +9412,7 @@
       <c r="X67" s="12"/>
       <c r="Y67" s="13"/>
     </row>
-    <row r="68" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="68" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="11" t="s">
         <v>160</v>
       </c>
@@ -9115,7 +9459,7 @@
       <c r="X68" s="12"/>
       <c r="Y68" s="13"/>
     </row>
-    <row r="69" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="69" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="11" t="s">
         <v>160</v>
       </c>
@@ -9168,7 +9512,7 @@
       <c r="X69" s="12"/>
       <c r="Y69" s="13"/>
     </row>
-    <row r="70" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="70" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="11" t="s">
         <v>160</v>
       </c>
@@ -9221,7 +9565,7 @@
       <c r="X70" s="12"/>
       <c r="Y70" s="13"/>
     </row>
-    <row r="71" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="71" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="11" t="s">
         <v>160</v>
       </c>
@@ -9274,7 +9618,7 @@
       <c r="X71" s="12"/>
       <c r="Y71" s="13"/>
     </row>
-    <row r="72" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="72" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="11" t="s">
         <v>160</v>
       </c>
@@ -9327,7 +9671,7 @@
       <c r="X72" s="12"/>
       <c r="Y72" s="13"/>
     </row>
-    <row r="73" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="73" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="11" t="s">
         <v>160</v>
       </c>
@@ -9362,7 +9706,7 @@
       <c r="X73" s="12"/>
       <c r="Y73" s="13"/>
     </row>
-    <row r="74" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="74" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="11" t="s">
         <v>160</v>
       </c>
@@ -9433,7 +9777,7 @@
       </c>
       <c r="Y74" s="13"/>
     </row>
-    <row r="75" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="75" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="11" t="s">
         <v>160</v>
       </c>
@@ -9506,7 +9850,7 @@
       </c>
       <c r="Y75" s="13"/>
     </row>
-    <row r="76" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="76" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="11" t="s">
         <v>160</v>
       </c>
@@ -9577,7 +9921,7 @@
       </c>
       <c r="Y76" s="13"/>
     </row>
-    <row r="77" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="77" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="11" t="s">
         <v>160</v>
       </c>
@@ -9648,7 +9992,7 @@
       </c>
       <c r="Y77" s="13"/>
     </row>
-    <row r="78" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="78" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="11" t="s">
         <v>160</v>
       </c>
@@ -9683,7 +10027,7 @@
       <c r="X78" s="12"/>
       <c r="Y78" s="13"/>
     </row>
-    <row r="79" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="79" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="11" t="s">
         <v>160</v>
       </c>
@@ -9754,7 +10098,7 @@
       </c>
       <c r="Y79" s="13"/>
     </row>
-    <row r="80" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="80" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="11" t="s">
         <v>160</v>
       </c>
@@ -9825,7 +10169,7 @@
       </c>
       <c r="Y80" s="13"/>
     </row>
-    <row r="81" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="81" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="11" t="s">
         <v>160</v>
       </c>
@@ -9894,7 +10238,7 @@
       </c>
       <c r="Y81" s="13"/>
     </row>
-    <row r="82" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="82" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="11" t="s">
         <v>160</v>
       </c>
@@ -9965,7 +10309,7 @@
       </c>
       <c r="Y82" s="13"/>
     </row>
-    <row r="83" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="83" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="11" t="s">
         <v>160</v>
       </c>
@@ -10028,7 +10372,7 @@
       </c>
       <c r="Y83" s="13"/>
     </row>
-    <row r="84" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="84" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="11" t="s">
         <v>160</v>
       </c>
@@ -10085,7 +10429,7 @@
       <c r="X84" s="12"/>
       <c r="Y84" s="13"/>
     </row>
-    <row r="85" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="85" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="11" t="s">
         <v>160</v>
       </c>
@@ -10120,7 +10464,7 @@
       <c r="X85" s="12"/>
       <c r="Y85" s="13"/>
     </row>
-    <row r="86" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="86" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="11" t="s">
         <v>160</v>
       </c>
@@ -10155,7 +10499,7 @@
       <c r="X86" s="12"/>
       <c r="Y86" s="13"/>
     </row>
-    <row r="87" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="87" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="11" t="s">
         <v>160</v>
       </c>
@@ -10190,7 +10534,7 @@
       <c r="X87" s="12"/>
       <c r="Y87" s="13"/>
     </row>
-    <row r="88" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="88" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="11" t="s">
         <v>160</v>
       </c>
@@ -10259,7 +10603,7 @@
       </c>
       <c r="Y88" s="13"/>
     </row>
-    <row r="89" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="89" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="11" t="s">
         <v>160</v>
       </c>
@@ -10328,7 +10672,7 @@
       </c>
       <c r="Y89" s="13"/>
     </row>
-    <row r="90" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="90" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="11" t="s">
         <v>160</v>
       </c>
@@ -10399,7 +10743,7 @@
       </c>
       <c r="Y90" s="13"/>
     </row>
-    <row r="91" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="91" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="11" t="s">
         <v>160</v>
       </c>
@@ -10468,7 +10812,7 @@
       <c r="X91" s="12"/>
       <c r="Y91" s="13"/>
     </row>
-    <row r="92" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="92" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="11" t="s">
         <v>160</v>
       </c>
@@ -10537,7 +10881,7 @@
       <c r="X92" s="12"/>
       <c r="Y92" s="13"/>
     </row>
-    <row r="93" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="93" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="11" t="s">
         <v>160</v>
       </c>
@@ -10606,7 +10950,7 @@
       <c r="X93" s="12"/>
       <c r="Y93" s="13"/>
     </row>
-    <row r="94" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="94" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="11" t="s">
         <v>160</v>
       </c>
@@ -10675,7 +11019,7 @@
       <c r="X94" s="12"/>
       <c r="Y94" s="13"/>
     </row>
-    <row r="95" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="95" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="11" t="s">
         <v>160</v>
       </c>
@@ -10744,7 +11088,7 @@
       <c r="X95" s="12"/>
       <c r="Y95" s="13"/>
     </row>
-    <row r="96" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="96" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="11" t="s">
         <v>160</v>
       </c>
@@ -10779,7 +11123,7 @@
       <c r="X96" s="12"/>
       <c r="Y96" s="13"/>
     </row>
-    <row r="97" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="97" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="11" t="s">
         <v>160</v>
       </c>
@@ -10848,7 +11192,7 @@
       <c r="X97" s="12"/>
       <c r="Y97" s="13"/>
     </row>
-    <row r="98" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="98" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="11" t="s">
         <v>160</v>
       </c>
@@ -10901,7 +11245,7 @@
       <c r="X98" s="12"/>
       <c r="Y98" s="13"/>
     </row>
-    <row r="99" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="99" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="11" t="s">
         <v>160</v>
       </c>
@@ -10974,7 +11318,7 @@
       </c>
       <c r="Y99" s="13"/>
     </row>
-    <row r="100" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="100" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="11" t="s">
         <v>160</v>
       </c>
@@ -11047,7 +11391,7 @@
       </c>
       <c r="Y100" s="13"/>
     </row>
-    <row r="101" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="101" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="11" t="s">
         <v>160</v>
       </c>
@@ -11120,7 +11464,7 @@
       </c>
       <c r="Y101" s="13"/>
     </row>
-    <row r="102" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="102" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="11" t="s">
         <v>160</v>
       </c>
@@ -11191,7 +11535,7 @@
       </c>
       <c r="Y102" s="13"/>
     </row>
-    <row r="103" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="103" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="11" t="s">
         <v>160</v>
       </c>
@@ -11224,7 +11568,7 @@
       <c r="X103" s="12"/>
       <c r="Y103" s="13"/>
     </row>
-    <row r="104" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="104" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="11" t="s">
         <v>160</v>
       </c>
@@ -11295,7 +11639,7 @@
       </c>
       <c r="Y104" s="13"/>
     </row>
-    <row r="105" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="105" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="11" t="s">
         <v>160</v>
       </c>
@@ -11368,7 +11712,7 @@
       </c>
       <c r="Y105" s="13"/>
     </row>
-    <row r="106" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="106" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="11" t="s">
         <v>160</v>
       </c>
@@ -11441,34 +11785,40 @@
       </c>
       <c r="Y106" s="13"/>
     </row>
-    <row r="107" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="107" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="11" t="s">
         <v>160</v>
       </c>
       <c r="B107" s="11" t="s">
-        <v>200</v>
+        <v>274</v>
       </c>
       <c r="C107" s="12"/>
       <c r="D107" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E107" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F107" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G107" s="12"/>
-      <c r="H107" s="12"/>
-      <c r="I107" s="12"/>
+      <c r="G107" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="H107" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I107" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="J107" s="12" t="s">
         <v>39</v>
       </c>
       <c r="K107" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="L107" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="M107" s="12" t="s">
         <v>39</v>
@@ -11477,33 +11827,39 @@
         <v>38</v>
       </c>
       <c r="O107" s="12"/>
-      <c r="P107" s="12"/>
+      <c r="P107" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="Q107" s="12" t="s">
         <v>39</v>
       </c>
       <c r="R107" s="12" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="S107" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="T107" s="12"/>
+        <v>39</v>
+      </c>
+      <c r="T107" s="12" t="s">
+        <v>44</v>
+      </c>
       <c r="U107" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="V107" s="12" t="s">
         <v>44</v>
       </c>
       <c r="W107" s="12"/>
-      <c r="X107" s="12"/>
+      <c r="X107" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="Y107" s="13"/>
     </row>
-    <row r="108" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="108" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="11" t="s">
-        <v>201</v>
+        <v>160</v>
       </c>
       <c r="B108" s="11" t="s">
-        <v>202</v>
+        <v>273</v>
       </c>
       <c r="C108" s="12"/>
       <c r="D108" s="12" t="s">
@@ -11525,7 +11881,7 @@
         <v>39</v>
       </c>
       <c r="J108" s="12" t="s">
-        <v>203</v>
+        <v>39</v>
       </c>
       <c r="K108" s="12" t="s">
         <v>38</v>
@@ -11539,20 +11895,18 @@
       <c r="N108" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="O108" s="12" t="s">
-        <v>38</v>
-      </c>
+      <c r="O108" s="12"/>
       <c r="P108" s="12" t="s">
         <v>39</v>
       </c>
       <c r="Q108" s="12" t="s">
-        <v>203</v>
+        <v>39</v>
       </c>
       <c r="R108" s="12" t="s">
-        <v>204</v>
+        <v>44</v>
       </c>
       <c r="S108" s="12" t="s">
-        <v>203</v>
+        <v>39</v>
       </c>
       <c r="T108" s="12" t="s">
         <v>44</v>
@@ -11563,50 +11917,40 @@
       <c r="V108" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="W108" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="W108" s="12"/>
       <c r="X108" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="Y108" s="35" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="109" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="Y108" s="13"/>
+    </row>
+    <row r="109" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="11" t="s">
-        <v>201</v>
+        <v>160</v>
       </c>
       <c r="B109" s="11" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="C109" s="12"/>
       <c r="D109" s="12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E109" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F109" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G109" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="H109" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="I109" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="G109" s="12"/>
+      <c r="H109" s="12"/>
+      <c r="I109" s="12"/>
       <c r="J109" s="12" t="s">
-        <v>203</v>
+        <v>39</v>
       </c>
       <c r="K109" s="12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="L109" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="M109" s="12" t="s">
         <v>39</v>
@@ -11614,48 +11958,38 @@
       <c r="N109" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="O109" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="P109" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="O109" s="12"/>
+      <c r="P109" s="12"/>
       <c r="Q109" s="12" t="s">
-        <v>203</v>
+        <v>39</v>
       </c>
       <c r="R109" s="12" t="s">
-        <v>204</v>
+        <v>42</v>
       </c>
       <c r="S109" s="12" t="s">
-        <v>203</v>
-      </c>
-      <c r="T109" s="12" t="s">
-        <v>44</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="T109" s="12"/>
       <c r="U109" s="12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="V109" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="W109" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="X109" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y109" s="35"/>
-    </row>
-    <row r="110" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="W109" s="12"/>
+      <c r="X109" s="12"/>
+      <c r="Y109" s="13"/>
+    </row>
+    <row r="110" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="11" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="B110" s="11" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="C110" s="12"/>
       <c r="D110" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E110" s="12" t="s">
         <v>38</v>
@@ -11673,10 +12007,10 @@
         <v>39</v>
       </c>
       <c r="J110" s="12" t="s">
-        <v>39</v>
+        <v>203</v>
       </c>
       <c r="K110" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="L110" s="12" t="s">
         <v>38</v>
@@ -11694,41 +12028,43 @@
         <v>39</v>
       </c>
       <c r="Q110" s="12" t="s">
-        <v>39</v>
+        <v>203</v>
       </c>
       <c r="R110" s="12" t="s">
-        <v>42</v>
+        <v>204</v>
       </c>
       <c r="S110" s="12" t="s">
-        <v>40</v>
+        <v>203</v>
       </c>
       <c r="T110" s="12" t="s">
         <v>44</v>
       </c>
       <c r="U110" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="V110" s="12" t="s">
         <v>44</v>
       </c>
       <c r="W110" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="X110" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y110" s="7"/>
-    </row>
-    <row r="111" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>39</v>
+      </c>
+      <c r="Y110" s="35" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="111" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="11" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B111" s="11" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="C111" s="12"/>
       <c r="D111" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E111" s="12" t="s">
         <v>38</v>
@@ -11746,10 +12082,10 @@
         <v>39</v>
       </c>
       <c r="J111" s="12" t="s">
-        <v>39</v>
+        <v>203</v>
       </c>
       <c r="K111" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="L111" s="12" t="s">
         <v>38</v>
@@ -11767,166 +12103,246 @@
         <v>39</v>
       </c>
       <c r="Q111" s="12" t="s">
-        <v>39</v>
+        <v>203</v>
       </c>
       <c r="R111" s="12" t="s">
-        <v>42</v>
+        <v>204</v>
       </c>
       <c r="S111" s="12" t="s">
-        <v>40</v>
+        <v>203</v>
       </c>
       <c r="T111" s="12" t="s">
         <v>44</v>
       </c>
       <c r="U111" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="V111" s="12" t="s">
         <v>44</v>
       </c>
       <c r="W111" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="X111" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y111" s="13"/>
-    </row>
-    <row r="112" spans="1:25" s="30" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A112" s="27" t="s">
-        <v>209</v>
-      </c>
-      <c r="B112" s="27" t="s">
-        <v>210</v>
-      </c>
-      <c r="C112" s="28"/>
+        <v>39</v>
+      </c>
+      <c r="Y111" s="35"/>
+    </row>
+    <row r="112" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A112" s="11" t="s">
+        <v>207</v>
+      </c>
+      <c r="B112" s="11" t="s">
+        <v>208</v>
+      </c>
+      <c r="C112" s="12"/>
       <c r="D112" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E112" s="28"/>
-      <c r="F112" s="28"/>
-      <c r="G112" s="28"/>
-      <c r="H112" s="28"/>
-      <c r="I112" s="28"/>
-      <c r="J112" s="28"/>
-      <c r="K112" s="28"/>
-      <c r="L112" s="28"/>
-      <c r="M112" s="28"/>
-      <c r="N112" s="28"/>
-      <c r="O112" s="28"/>
-      <c r="P112" s="28"/>
-      <c r="Q112" s="28"/>
-      <c r="R112" s="28"/>
-      <c r="S112" s="28"/>
-      <c r="T112" s="28"/>
-      <c r="U112" s="28"/>
-      <c r="V112" s="28"/>
-      <c r="W112" s="28"/>
-      <c r="X112" s="28"/>
-      <c r="Y112" s="29" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="113" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E112" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F112" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="G112" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="H112" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I112" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="J112" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="K112" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="L112" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="M112" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="N112" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="O112" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="P112" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q112" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="R112" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="S112" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="T112" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="U112" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="V112" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="W112" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="X112" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="Y112" s="7"/>
+    </row>
+    <row r="113" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="11" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="B113" s="11" t="s">
-        <v>212</v>
+        <v>199</v>
       </c>
       <c r="C113" s="12"/>
       <c r="D113" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E113" s="12"/>
+      <c r="E113" s="12" t="s">
+        <v>38</v>
+      </c>
       <c r="F113" s="12" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="G113" s="12" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="H113" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="I113" s="12"/>
-      <c r="J113" s="12"/>
-      <c r="K113" s="12"/>
-      <c r="L113" s="12"/>
+        <v>38</v>
+      </c>
+      <c r="I113" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="J113" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="K113" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="L113" s="12" t="s">
+        <v>38</v>
+      </c>
       <c r="M113" s="12" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="N113" s="12" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="O113" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="P113" s="12"/>
-      <c r="Q113" s="12"/>
-      <c r="R113" s="12"/>
-      <c r="S113" s="12"/>
-      <c r="T113" s="12"/>
-      <c r="U113" s="12"/>
-      <c r="V113" s="12"/>
-      <c r="W113" s="12"/>
-      <c r="X113" s="12"/>
-      <c r="Y113" s="7"/>
-    </row>
-    <row r="114" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A114" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="P113" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q113" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="R113" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="S113" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="T113" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="U113" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="V113" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="W113" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="X113" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="Y113" s="13"/>
+    </row>
+    <row r="114" spans="1:25" s="30" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A114" s="27" t="s">
         <v>209</v>
       </c>
-      <c r="B114" s="11" t="s">
-        <v>213</v>
-      </c>
-      <c r="C114" s="12"/>
+      <c r="B114" s="27" t="s">
+        <v>210</v>
+      </c>
+      <c r="C114" s="28"/>
       <c r="D114" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E114" s="12"/>
-      <c r="F114" s="12"/>
-      <c r="G114" s="12"/>
-      <c r="H114" s="12"/>
-      <c r="I114" s="12"/>
-      <c r="J114" s="12"/>
-      <c r="K114" s="12"/>
-      <c r="L114" s="12"/>
-      <c r="M114" s="12"/>
-      <c r="N114" s="12"/>
-      <c r="O114" s="12"/>
-      <c r="P114" s="12"/>
-      <c r="Q114" s="12"/>
-      <c r="R114" s="12"/>
-      <c r="S114" s="12"/>
-      <c r="T114" s="12"/>
-      <c r="U114" s="12"/>
-      <c r="V114" s="12"/>
-      <c r="W114" s="12"/>
-      <c r="X114" s="12"/>
-      <c r="Y114" s="7"/>
-    </row>
-    <row r="115" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E114" s="28"/>
+      <c r="F114" s="28"/>
+      <c r="G114" s="28"/>
+      <c r="H114" s="28"/>
+      <c r="I114" s="28"/>
+      <c r="J114" s="28"/>
+      <c r="K114" s="28"/>
+      <c r="L114" s="28"/>
+      <c r="M114" s="28"/>
+      <c r="N114" s="28"/>
+      <c r="O114" s="28"/>
+      <c r="P114" s="28"/>
+      <c r="Q114" s="28"/>
+      <c r="R114" s="28"/>
+      <c r="S114" s="28"/>
+      <c r="T114" s="28"/>
+      <c r="U114" s="28"/>
+      <c r="V114" s="28"/>
+      <c r="W114" s="28"/>
+      <c r="X114" s="28"/>
+      <c r="Y114" s="29" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="115" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B115" s="11" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C115" s="12"/>
       <c r="D115" s="12" t="s">
         <v>41</v>
       </c>
       <c r="E115" s="12"/>
-      <c r="F115" s="12"/>
-      <c r="G115" s="12"/>
-      <c r="H115" s="12"/>
+      <c r="F115" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="G115" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="H115" s="12" t="s">
+        <v>46</v>
+      </c>
       <c r="I115" s="12"/>
       <c r="J115" s="12"/>
       <c r="K115" s="12"/>
       <c r="L115" s="12"/>
-      <c r="M115" s="12"/>
-      <c r="N115" s="12"/>
-      <c r="O115" s="12"/>
+      <c r="M115" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="N115" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="O115" s="12" t="s">
+        <v>46</v>
+      </c>
       <c r="P115" s="12"/>
       <c r="Q115" s="12"/>
       <c r="R115" s="12"/>
@@ -11938,12 +12354,12 @@
       <c r="X115" s="12"/>
       <c r="Y115" s="7"/>
     </row>
-    <row r="116" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="116" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B116" s="11" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C116" s="12"/>
       <c r="D116" s="12" t="s">
@@ -11971,12 +12387,12 @@
       <c r="X116" s="12"/>
       <c r="Y116" s="7"/>
     </row>
-    <row r="117" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="117" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B117" s="11" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C117" s="12"/>
       <c r="D117" s="12" t="s">
@@ -12004,12 +12420,12 @@
       <c r="X117" s="12"/>
       <c r="Y117" s="7"/>
     </row>
-    <row r="118" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="118" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B118" s="11" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C118" s="12"/>
       <c r="D118" s="12" t="s">
@@ -12037,12 +12453,12 @@
       <c r="X118" s="12"/>
       <c r="Y118" s="7"/>
     </row>
-    <row r="119" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="119" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B119" s="11" t="s">
-        <v>76</v>
+        <v>216</v>
       </c>
       <c r="C119" s="12"/>
       <c r="D119" s="12" t="s">
@@ -12070,12 +12486,12 @@
       <c r="X119" s="12"/>
       <c r="Y119" s="7"/>
     </row>
-    <row r="120" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="120" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B120" s="11" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C120" s="12"/>
       <c r="D120" s="12" t="s">
@@ -12103,45 +12519,45 @@
       <c r="X120" s="12"/>
       <c r="Y120" s="7"/>
     </row>
-    <row r="121" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="121" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="11" t="s">
         <v>209</v>
       </c>
-      <c r="B121" s="14" t="s">
-        <v>219</v>
-      </c>
-      <c r="C121" s="15"/>
-      <c r="D121" s="15" t="s">
+      <c r="B121" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="C121" s="12"/>
+      <c r="D121" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E121" s="15"/>
-      <c r="F121" s="15"/>
-      <c r="G121" s="15"/>
-      <c r="H121" s="15"/>
-      <c r="I121" s="15"/>
-      <c r="J121" s="15"/>
-      <c r="K121" s="15"/>
-      <c r="L121" s="15"/>
-      <c r="M121" s="15"/>
-      <c r="N121" s="15"/>
-      <c r="O121" s="15"/>
-      <c r="P121" s="15"/>
-      <c r="Q121" s="15"/>
-      <c r="R121" s="15"/>
-      <c r="S121" s="15"/>
-      <c r="T121" s="15"/>
-      <c r="U121" s="15"/>
-      <c r="V121" s="15"/>
-      <c r="W121" s="15"/>
-      <c r="X121" s="15"/>
-      <c r="Y121" s="13"/>
-    </row>
-    <row r="122" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E121" s="12"/>
+      <c r="F121" s="12"/>
+      <c r="G121" s="12"/>
+      <c r="H121" s="12"/>
+      <c r="I121" s="12"/>
+      <c r="J121" s="12"/>
+      <c r="K121" s="12"/>
+      <c r="L121" s="12"/>
+      <c r="M121" s="12"/>
+      <c r="N121" s="12"/>
+      <c r="O121" s="12"/>
+      <c r="P121" s="12"/>
+      <c r="Q121" s="12"/>
+      <c r="R121" s="12"/>
+      <c r="S121" s="12"/>
+      <c r="T121" s="12"/>
+      <c r="U121" s="12"/>
+      <c r="V121" s="12"/>
+      <c r="W121" s="12"/>
+      <c r="X121" s="12"/>
+      <c r="Y121" s="7"/>
+    </row>
+    <row r="122" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B122" s="11" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C122" s="12"/>
       <c r="D122" s="12" t="s">
@@ -12169,45 +12585,45 @@
       <c r="X122" s="12"/>
       <c r="Y122" s="7"/>
     </row>
-    <row r="123" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="123" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="11" t="s">
         <v>209</v>
       </c>
-      <c r="B123" s="11" t="s">
-        <v>221</v>
-      </c>
-      <c r="C123" s="12"/>
-      <c r="D123" s="12" t="s">
+      <c r="B123" s="14" t="s">
+        <v>219</v>
+      </c>
+      <c r="C123" s="15"/>
+      <c r="D123" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="E123" s="12"/>
-      <c r="F123" s="12"/>
-      <c r="G123" s="12"/>
-      <c r="H123" s="12"/>
-      <c r="I123" s="12"/>
-      <c r="J123" s="12"/>
-      <c r="K123" s="12"/>
-      <c r="L123" s="12"/>
-      <c r="M123" s="12"/>
-      <c r="N123" s="12"/>
-      <c r="O123" s="12"/>
-      <c r="P123" s="12"/>
-      <c r="Q123" s="12"/>
-      <c r="R123" s="12"/>
-      <c r="S123" s="12"/>
-      <c r="T123" s="12"/>
-      <c r="U123" s="12"/>
-      <c r="V123" s="12"/>
-      <c r="W123" s="12"/>
-      <c r="X123" s="12"/>
-      <c r="Y123" s="7"/>
-    </row>
-    <row r="124" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E123" s="15"/>
+      <c r="F123" s="15"/>
+      <c r="G123" s="15"/>
+      <c r="H123" s="15"/>
+      <c r="I123" s="15"/>
+      <c r="J123" s="15"/>
+      <c r="K123" s="15"/>
+      <c r="L123" s="15"/>
+      <c r="M123" s="15"/>
+      <c r="N123" s="15"/>
+      <c r="O123" s="15"/>
+      <c r="P123" s="15"/>
+      <c r="Q123" s="15"/>
+      <c r="R123" s="15"/>
+      <c r="S123" s="15"/>
+      <c r="T123" s="15"/>
+      <c r="U123" s="15"/>
+      <c r="V123" s="15"/>
+      <c r="W123" s="15"/>
+      <c r="X123" s="15"/>
+      <c r="Y123" s="13"/>
+    </row>
+    <row r="124" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B124" s="11" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C124" s="12"/>
       <c r="D124" s="12" t="s">
@@ -12235,12 +12651,12 @@
       <c r="X124" s="12"/>
       <c r="Y124" s="7"/>
     </row>
-    <row r="125" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="125" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B125" s="11" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C125" s="12"/>
       <c r="D125" s="12" t="s">
@@ -12268,12 +12684,12 @@
       <c r="X125" s="12"/>
       <c r="Y125" s="7"/>
     </row>
-    <row r="126" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="126" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B126" s="11" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C126" s="12"/>
       <c r="D126" s="12" t="s">
@@ -12301,12 +12717,12 @@
       <c r="X126" s="12"/>
       <c r="Y126" s="7"/>
     </row>
-    <row r="127" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="127" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B127" s="11" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C127" s="12"/>
       <c r="D127" s="12" t="s">
@@ -12334,12 +12750,12 @@
       <c r="X127" s="12"/>
       <c r="Y127" s="7"/>
     </row>
-    <row r="128" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="128" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B128" s="11" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C128" s="12"/>
       <c r="D128" s="12" t="s">
@@ -12367,12 +12783,12 @@
       <c r="X128" s="12"/>
       <c r="Y128" s="7"/>
     </row>
-    <row r="129" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="129" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B129" s="11" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C129" s="12"/>
       <c r="D129" s="12" t="s">
@@ -12400,12 +12816,12 @@
       <c r="X129" s="12"/>
       <c r="Y129" s="7"/>
     </row>
-    <row r="130" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="130" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B130" s="11" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C130" s="12"/>
       <c r="D130" s="12" t="s">
@@ -12433,12 +12849,12 @@
       <c r="X130" s="12"/>
       <c r="Y130" s="7"/>
     </row>
-    <row r="131" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="131" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B131" s="11" t="s">
-        <v>264</v>
+        <v>227</v>
       </c>
       <c r="C131" s="12"/>
       <c r="D131" s="12" t="s">
@@ -12466,16 +12882,16 @@
       <c r="X131" s="12"/>
       <c r="Y131" s="7"/>
     </row>
-    <row r="132" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="132" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B132" s="11" t="s">
-        <v>270</v>
+        <v>228</v>
       </c>
       <c r="C132" s="12"/>
       <c r="D132" s="12" t="s">
-        <v>100</v>
+        <v>41</v>
       </c>
       <c r="E132" s="12"/>
       <c r="F132" s="12"/>
@@ -12499,12 +12915,12 @@
       <c r="X132" s="12"/>
       <c r="Y132" s="7"/>
     </row>
-    <row r="133" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="133" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B133" s="11" t="s">
-        <v>229</v>
+        <v>264</v>
       </c>
       <c r="C133" s="12"/>
       <c r="D133" s="12" t="s">
@@ -12532,138 +12948,210 @@
       <c r="X133" s="12"/>
       <c r="Y133" s="7"/>
     </row>
-    <row r="134" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="134" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="11" t="s">
+        <v>209</v>
+      </c>
+      <c r="B134" s="11" t="s">
+        <v>270</v>
+      </c>
+      <c r="C134" s="12"/>
+      <c r="D134" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="E134" s="12"/>
+      <c r="F134" s="12"/>
+      <c r="G134" s="12"/>
+      <c r="H134" s="12"/>
+      <c r="I134" s="12"/>
+      <c r="J134" s="12"/>
+      <c r="K134" s="12"/>
+      <c r="L134" s="12"/>
+      <c r="M134" s="12"/>
+      <c r="N134" s="12"/>
+      <c r="O134" s="12"/>
+      <c r="P134" s="12"/>
+      <c r="Q134" s="12"/>
+      <c r="R134" s="12"/>
+      <c r="S134" s="12"/>
+      <c r="T134" s="12"/>
+      <c r="U134" s="12"/>
+      <c r="V134" s="12"/>
+      <c r="W134" s="12"/>
+      <c r="X134" s="12"/>
+      <c r="Y134" s="7"/>
+    </row>
+    <row r="135" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A135" s="11" t="s">
+        <v>209</v>
+      </c>
+      <c r="B135" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="C135" s="12"/>
+      <c r="D135" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="E135" s="12"/>
+      <c r="F135" s="12"/>
+      <c r="G135" s="12"/>
+      <c r="H135" s="12"/>
+      <c r="I135" s="12"/>
+      <c r="J135" s="12"/>
+      <c r="K135" s="12"/>
+      <c r="L135" s="12"/>
+      <c r="M135" s="12"/>
+      <c r="N135" s="12"/>
+      <c r="O135" s="12"/>
+      <c r="P135" s="12"/>
+      <c r="Q135" s="12"/>
+      <c r="R135" s="12"/>
+      <c r="S135" s="12"/>
+      <c r="T135" s="12"/>
+      <c r="U135" s="12"/>
+      <c r="V135" s="12"/>
+      <c r="W135" s="12"/>
+      <c r="X135" s="12"/>
+      <c r="Y135" s="7"/>
+    </row>
+    <row r="136" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A136" s="11" t="s">
         <v>230</v>
       </c>
-      <c r="B134" s="11" t="s">
+      <c r="B136" s="11" t="s">
         <v>231</v>
-      </c>
-      <c r="C134" s="16"/>
-      <c r="D134" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="E134" s="16"/>
-      <c r="F134" s="16"/>
-      <c r="G134" s="16"/>
-      <c r="H134" s="16"/>
-      <c r="I134" s="16"/>
-      <c r="J134" s="16"/>
-      <c r="K134" s="16"/>
-      <c r="L134" s="16"/>
-      <c r="M134" s="16"/>
-      <c r="N134" s="16"/>
-      <c r="O134" s="16"/>
-      <c r="P134" s="16"/>
-      <c r="Q134" s="16"/>
-      <c r="R134" s="16"/>
-      <c r="S134" s="16"/>
-      <c r="T134" s="16"/>
-      <c r="U134" s="16"/>
-      <c r="V134" s="16"/>
-      <c r="W134" s="16"/>
-      <c r="X134" s="16"/>
-      <c r="Y134" s="7"/>
-    </row>
-    <row r="135" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A135" s="11" t="s">
-        <v>232</v>
-      </c>
-      <c r="B135" s="11" t="s">
-        <v>233</v>
-      </c>
-      <c r="C135" s="16"/>
-      <c r="D135" s="12" t="s">
-        <v>234</v>
-      </c>
-      <c r="E135" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="F135" s="31"/>
-      <c r="G135" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="H135" s="31"/>
-      <c r="I135" s="31"/>
-      <c r="J135" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="K135" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="L135" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="M135" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="N135" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="O135" s="31"/>
-      <c r="P135" s="31"/>
-      <c r="Q135" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="R135" s="31" t="s">
-        <v>236</v>
-      </c>
-      <c r="S135" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="T135" s="31"/>
-      <c r="U135" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="V135" s="31"/>
-      <c r="W135" s="31"/>
-      <c r="X135" s="31"/>
-      <c r="Y135" s="7"/>
-    </row>
-    <row r="136" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A136" s="11" t="s">
-        <v>265</v>
-      </c>
-      <c r="B136" s="11" t="s">
-        <v>265</v>
       </c>
       <c r="C136" s="16"/>
       <c r="D136" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="E136" s="31" t="s">
-        <v>38</v>
-      </c>
-      <c r="F136" s="31"/>
-      <c r="G136" s="31"/>
-      <c r="H136" s="31"/>
-      <c r="I136" s="31"/>
-      <c r="J136" s="31"/>
-      <c r="K136" s="31" t="s">
-        <v>38</v>
-      </c>
-      <c r="L136" s="31" t="s">
-        <v>38</v>
-      </c>
-      <c r="M136" s="31"/>
-      <c r="N136" s="31"/>
-      <c r="O136" s="31"/>
-      <c r="P136" s="31"/>
-      <c r="Q136" s="31"/>
-      <c r="R136" s="31"/>
-      <c r="S136" s="31"/>
-      <c r="T136" s="31"/>
-      <c r="U136" s="31"/>
-      <c r="V136" s="31"/>
-      <c r="W136" s="31"/>
-      <c r="X136" s="31"/>
+        <v>41</v>
+      </c>
+      <c r="E136" s="16"/>
+      <c r="F136" s="16"/>
+      <c r="G136" s="16"/>
+      <c r="H136" s="16"/>
+      <c r="I136" s="16"/>
+      <c r="J136" s="16"/>
+      <c r="K136" s="16"/>
+      <c r="L136" s="16"/>
+      <c r="M136" s="16"/>
+      <c r="N136" s="16"/>
+      <c r="O136" s="16"/>
+      <c r="P136" s="16"/>
+      <c r="Q136" s="16"/>
+      <c r="R136" s="16"/>
+      <c r="S136" s="16"/>
+      <c r="T136" s="16"/>
+      <c r="U136" s="16"/>
+      <c r="V136" s="16"/>
+      <c r="W136" s="16"/>
+      <c r="X136" s="16"/>
       <c r="Y136" s="7"/>
+    </row>
+    <row r="137" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A137" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="B137" s="11" t="s">
+        <v>233</v>
+      </c>
+      <c r="C137" s="16"/>
+      <c r="D137" s="12" t="s">
+        <v>234</v>
+      </c>
+      <c r="E137" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="F137" s="31"/>
+      <c r="G137" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="H137" s="31"/>
+      <c r="I137" s="31"/>
+      <c r="J137" s="31" t="s">
+        <v>235</v>
+      </c>
+      <c r="K137" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="L137" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="M137" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="N137" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="O137" s="31"/>
+      <c r="P137" s="31"/>
+      <c r="Q137" s="31" t="s">
+        <v>235</v>
+      </c>
+      <c r="R137" s="31" t="s">
+        <v>236</v>
+      </c>
+      <c r="S137" s="31" t="s">
+        <v>235</v>
+      </c>
+      <c r="T137" s="31"/>
+      <c r="U137" s="31" t="s">
+        <v>235</v>
+      </c>
+      <c r="V137" s="31"/>
+      <c r="W137" s="31"/>
+      <c r="X137" s="31"/>
+      <c r="Y137" s="7"/>
+    </row>
+    <row r="138" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A138" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="B138" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="C138" s="16"/>
+      <c r="D138" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="E138" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="F138" s="31"/>
+      <c r="G138" s="31"/>
+      <c r="H138" s="31"/>
+      <c r="I138" s="31"/>
+      <c r="J138" s="31"/>
+      <c r="K138" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="L138" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="M138" s="31"/>
+      <c r="N138" s="31"/>
+      <c r="O138" s="31"/>
+      <c r="P138" s="31"/>
+      <c r="Q138" s="31"/>
+      <c r="R138" s="31"/>
+      <c r="S138" s="31"/>
+      <c r="T138" s="31"/>
+      <c r="U138" s="31"/>
+      <c r="V138" s="31"/>
+      <c r="W138" s="31"/>
+      <c r="X138" s="31"/>
+      <c r="Y138" s="7"/>
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="115">
-      <pane xSplit="2" ySplit="6" topLeftCell="Q19" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="Y37" sqref="Y37"/>
+    <customSheetView guid="{810C905A-C0DA-4100-B6A9-F2260D80EA70}" scale="115">
+      <pane xSplit="2" ySplit="6" topLeftCell="Q101" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="B108" sqref="B108"/>
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+    </customSheetView>
+    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="130">
+      <pane xSplit="2" ySplit="6" topLeftCell="C53" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="B71" sqref="B71"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
@@ -12673,15 +13161,15 @@
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
-    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="130">
-      <pane xSplit="2" ySplit="6" topLeftCell="C53" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="B71" sqref="B71"/>
+    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="115">
+      <pane xSplit="2" ySplit="6" topLeftCell="Q19" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="Y37" sqref="Y37"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
   </customSheetViews>
   <mergeCells count="6">
-    <mergeCell ref="Y108:Y109"/>
+    <mergeCell ref="Y110:Y111"/>
     <mergeCell ref="C1:O1"/>
     <mergeCell ref="C2:O2"/>
     <mergeCell ref="C5:H5"/>
@@ -12697,7 +13185,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.6640625" customWidth="1"/>
     <col min="2" max="2" width="28.33203125" customWidth="1"/>
@@ -12705,7 +13193,7 @@
     <col min="5" max="5" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="32" t="s">
         <v>237</v>
       </c>
@@ -12722,7 +13210,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" s="33" t="s">
         <v>242</v>
       </c>
@@ -12735,7 +13223,7 @@
       <c r="D2" s="34"/>
       <c r="E2" s="34"/>
     </row>
-    <row r="3" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A3" s="33" t="s">
         <v>243</v>
       </c>
@@ -12748,7 +13236,7 @@
       <c r="D3" s="34"/>
       <c r="E3" s="34"/>
     </row>
-    <row r="4" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A4" s="33" t="s">
         <v>244</v>
       </c>
@@ -12761,7 +13249,7 @@
       <c r="D4" s="34"/>
       <c r="E4" s="34"/>
     </row>
-    <row r="5" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A5" s="33" t="s">
         <v>245</v>
       </c>
@@ -12776,7 +13264,7 @@
       </c>
       <c r="E5" s="34"/>
     </row>
-    <row r="6" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A6" s="33" t="s">
         <v>247</v>
       </c>
@@ -12791,7 +13279,7 @@
       </c>
       <c r="E6" s="34"/>
     </row>
-    <row r="7" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="33" t="s">
         <v>248</v>
       </c>
@@ -12806,7 +13294,7 @@
       </c>
       <c r="E7" s="34"/>
     </row>
-    <row r="8" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="33" t="s">
         <v>249</v>
       </c>
@@ -12821,7 +13309,7 @@
       </c>
       <c r="E8" s="34"/>
     </row>
-    <row r="9" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A9" s="33" t="s">
         <v>250</v>
       </c>
@@ -12836,7 +13324,7 @@
       </c>
       <c r="E9" s="34"/>
     </row>
-    <row r="10" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A10" s="33" t="s">
         <v>252</v>
       </c>
@@ -12849,7 +13337,7 @@
       <c r="D10" s="34"/>
       <c r="E10" s="34"/>
     </row>
-    <row r="11" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A11" s="33" t="s">
         <v>253</v>
       </c>
@@ -12862,7 +13350,7 @@
       <c r="D11" s="34"/>
       <c r="E11" s="34"/>
     </row>
-    <row r="12" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A12" s="33" t="s">
         <v>254</v>
       </c>
@@ -12875,7 +13363,7 @@
       <c r="D12" s="34"/>
       <c r="E12" s="34"/>
     </row>
-    <row r="13" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A13" s="33" t="s">
         <v>255</v>
       </c>
@@ -12890,7 +13378,7 @@
       </c>
       <c r="E13" s="34"/>
     </row>
-    <row r="14" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A14" s="33" t="s">
         <v>256</v>
       </c>
@@ -12905,7 +13393,7 @@
       </c>
       <c r="E14" s="34"/>
     </row>
-    <row r="15" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A15" s="33" t="s">
         <v>257</v>
       </c>
@@ -12920,7 +13408,7 @@
       </c>
       <c r="E15" s="34"/>
     </row>
-    <row r="16" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A16" s="33" t="s">
         <v>258</v>
       </c>
@@ -12935,7 +13423,7 @@
       </c>
       <c r="E16" s="34"/>
     </row>
-    <row r="17" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A17" s="33" t="s">
         <v>259</v>
       </c>
@@ -12950,7 +13438,7 @@
       </c>
       <c r="E17" s="34"/>
     </row>
-    <row r="18" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A18" s="33" t="s">
         <v>260</v>
       </c>
@@ -12965,7 +13453,7 @@
       </c>
       <c r="E18" s="34"/>
     </row>
-    <row r="19" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A19" s="33" t="s">
         <v>261</v>
       </c>
@@ -12980,7 +13468,7 @@
       </c>
       <c r="E19" s="34"/>
     </row>
-    <row r="20" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A20" s="33" t="s">
         <v>262</v>
       </c>
@@ -12995,7 +13483,7 @@
       </c>
       <c r="E20" s="34"/>
     </row>
-    <row r="21" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A21" s="33" t="s">
         <v>33</v>
       </c>
@@ -13010,7 +13498,7 @@
       </c>
       <c r="E21" s="34"/>
     </row>
-    <row r="22" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A22" s="33" t="s">
         <v>263</v>
       </c>
@@ -13027,7 +13515,12 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="150">
+    <customSheetView guid="{810C905A-C0DA-4100-B6A9-F2260D80EA70}" scale="150">
+      <selection activeCell="A22" sqref="A22"/>
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+    </customSheetView>
+    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="150">
       <selection activeCell="A22" sqref="A22"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -13037,7 +13530,7 @@
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
-    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="150">
+    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="150">
       <selection activeCell="A22" sqref="A22"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Revert "Muuta roolit.xlsx testiympäristöä varten"
This reverts commit f970ac4b1bd1c9197066ce64c0b63ef6beb63999.
</commit_message>
<xml_diff>
--- a/resources/roolit.xlsx
+++ b/resources/roolit.xlsx
@@ -1,48 +1,46 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\samuli\dev\harjaroot\harja\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lauri.nayha/Projects/harja/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:81_{C33009BB-AF4A-4311-9633-F3E6F0CC09C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:81_{A8790524-4076-984A-9AA0-56B44D9CB46B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23748" yWindow="156" windowWidth="25476" windowHeight="14232" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="98860" yWindow="2380" windowWidth="34560" windowHeight="14920" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Oikeudet" sheetId="1" r:id="rId1"/>
     <sheet name="Roolit" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_1CE83972_B6A5_C44D_86E5_E9D9B38739F4_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_1DD617EE_F308_3E45_A8EF_4713F47FA0DD_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_2064F962_35EF_41F3_8A86_D37B72D177C7_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_3EBD3306_FC69_2148_8542_F6313DC2056F_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_47348D7B_5AFC_4A25_B239_A26E1359728E_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_476C495F_6E55_F04C_8145_4E8EBD6B3DE3_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_5327B0A1_A5FC_7747_93A1_427B210F3DF4_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_56F6E422_2CD8_6B4D_9E39_69A269028D26_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_6AA8E519_028C_D745_9E2E_8FB60E5B789F_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_7A9649F2_657F_9445_B6E6_FE94C6A09957_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_810C905A_C0DA_4100_B6A9_F2260D80EA70_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_8411E1B5_4691_4435_A9A2_147FF80D0D98_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_843152D8_333A_1941_83E9_0CB5262068A2_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_87BEAE97_700C_BF40_B102_636C54D81F08_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_D01EF3E4_E485_4912_A9DA_396AAE5B8752_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_D57E2FB1_FF7F_8446_9C97_237A4D57F6BE_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_E3BBF62E_A283_4D48_98B7_21A2A94F634F_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_F86DF6F3_8AE5_3A44_B2D2_D623E01AE54F_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_1CE83972_B6A5_C44D_86E5_E9D9B38739F4_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_1DD617EE_F308_3E45_A8EF_4713F47FA0DD_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_2064F962_35EF_41F3_8A86_D37B72D177C7_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_3EBD3306_FC69_2148_8542_F6313DC2056F_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_47348D7B_5AFC_4A25_B239_A26E1359728E_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_476C495F_6E55_F04C_8145_4E8EBD6B3DE3_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_5327B0A1_A5FC_7747_93A1_427B210F3DF4_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_56F6E422_2CD8_6B4D_9E39_69A269028D26_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_6AA8E519_028C_D745_9E2E_8FB60E5B789F_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_7A9649F2_657F_9445_B6E6_FE94C6A09957_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_8411E1B5_4691_4435_A9A2_147FF80D0D98_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_843152D8_333A_1941_83E9_0CB5262068A2_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_87BEAE97_700C_BF40_B102_636C54D81F08_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_D01EF3E4_E485_4912_A9DA_396AAE5B8752_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_D57E2FB1_FF7F_8446_9C97_237A4D57F6BE_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_E3BBF62E_A283_4D48_98B7_21A2A94F634F_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="Z_F86DF6F3_8AE5_3A44_B2D2_D623E01AE54F_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
   </definedNames>
   <calcPr calcId="0"/>
   <customWorkbookViews>
-    <customWorkbookView name="Samuli Taskila - Personal View" guid="{810C905A-C0DA-4100-B6A9-F2260D80EA70}" mergeInterval="0" personalView="1" xWindow="1979" yWindow="13" windowWidth="2123" windowHeight="1186" tabRatio="500" activeSheetId="1"/>
+    <customWorkbookView name="Microsoft Office User - Personal View" guid="{843152D8-333A-1941-83E9-0CB5262068A2}" mergeInterval="0" personalView="1" xWindow="4943" yWindow="119" windowWidth="1728" windowHeight="746" tabRatio="500" activeSheetId="1"/>
+    <customWorkbookView name="Jarno Väyrynen - Personal View" guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" mergeInterval="0" personalView="1" xWindow="48" yWindow="25" windowWidth="2512" windowHeight="1336" tabRatio="500" activeSheetId="1"/>
     <customWorkbookView name="Microsoft Office User - Oma näkymä" guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" mergeInterval="0" personalView="1" xWindow="1440" yWindow="-515" windowWidth="2056" windowHeight="1366" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Jarno Väyrynen - Personal View" guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" mergeInterval="0" personalView="1" xWindow="48" yWindow="25" windowWidth="2512" windowHeight="1336" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Microsoft Office User - Personal View" guid="{843152D8-333A-1941-83E9-0CB5262068A2}" mergeInterval="0" personalView="1" xWindow="4943" yWindow="119" windowWidth="1728" windowHeight="746" tabRatio="500" activeSheetId="1"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -112,7 +110,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1989" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1947" uniqueCount="273">
   <si>
     <t xml:space="preserve">Roolimääritysten selitykset: </t>
   </si>
@@ -1003,12 +1001,6 @@
   </si>
   <si>
     <t>Koitetaan pärjätä yhdellä rivillä kaikkien välilehtien osalta</t>
-  </si>
-  <si>
-    <t>Tiemerkintä - Muut kustannukset</t>
-  </si>
-  <si>
-    <t>Tiemerkintä - Sakot ja bonukset</t>
   </si>
 </sst>
 </file>
@@ -1393,7 +1385,7 @@
 </file>
 
 <file path=xl/revisions/revisionHeaders.xml><?xml version="1.0" encoding="utf-8"?>
-<headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" guid="{4A6ED1B0-9135-4362-95CD-B6A2DDFC57B0}" diskRevisions="1" revisionId="269" version="14">
+<headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" guid="{16592C61-0221-A548-A820-56B21F0EE301}" diskRevisions="1" revisionId="224" version="13">
   <header guid="{8EBC2E30-8A6E-AD43-9F6F-B4500CF04203}" dateTime="2024-06-11T12:49:05" maxSheetId="3" userName="Jarno Väyrynen" r:id="rId9" minRId="87" maxRId="97">
     <sheetIdMap count="2">
       <sheetId val="1"/>
@@ -1448,12 +1440,6 @@
       <sheetId val="2"/>
     </sheetIdMap>
   </header>
-  <header guid="{4A6ED1B0-9135-4362-95CD-B6A2DDFC57B0}" dateTime="2025-04-02T11:13:06" maxSheetId="3" userName="Samuli Taskila" r:id="rId18" minRId="225" maxRId="268">
-    <sheetIdMap count="2">
-      <sheetId val="1"/>
-      <sheetId val="2"/>
-    </sheetIdMap>
-  </header>
 </headers>
 </file>
 
@@ -1485,335 +1471,6 @@
     <formula>Oikeudet!$A$5:$Y$128</formula>
   </rdn>
   <rcv guid="{843152D8-333A-1941-83E9-0CB5262068A2}" action="add"/>
-</revisions>
-</file>
-
-<file path=xl/revisions/revisionLog10.xml><?xml version="1.0" encoding="utf-8"?>
-<revisions xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <rrc rId="225" sId="1" ref="A107:XFD107" action="insertRow"/>
-  <rfmt sheetId="1" sqref="Y107" start="0" length="0">
-    <dxf>
-      <font>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-  </rfmt>
-  <rcc rId="226" sId="1">
-    <nc r="A107" t="inlineStr">
-      <is>
-        <t>Raportit</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="227" sId="1">
-    <nc r="D107" t="inlineStr">
-      <is>
-        <t>R*</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="228" sId="1">
-    <nc r="E107" t="inlineStr">
-      <is>
-        <t>R*</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="229" sId="1">
-    <nc r="F107" t="inlineStr">
-      <is>
-        <t>R*</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="230" sId="1">
-    <nc r="G107" t="inlineStr">
-      <is>
-        <t>R*</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="231" sId="1">
-    <nc r="H107" t="inlineStr">
-      <is>
-        <t>R*</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="232" sId="1">
-    <nc r="I107" t="inlineStr">
-      <is>
-        <t>R</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="233" sId="1">
-    <nc r="J107" t="inlineStr">
-      <is>
-        <t>R</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="234" sId="1">
-    <nc r="K107" t="inlineStr">
-      <is>
-        <t>R*</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="235" sId="1">
-    <nc r="L107" t="inlineStr">
-      <is>
-        <t>R*</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="236" sId="1">
-    <nc r="M107" t="inlineStr">
-      <is>
-        <t>R</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="237" sId="1">
-    <nc r="N107" t="inlineStr">
-      <is>
-        <t>R*</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="238" sId="1">
-    <nc r="P107" t="inlineStr">
-      <is>
-        <t>R</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="239" sId="1">
-    <nc r="Q107" t="inlineStr">
-      <is>
-        <t>R</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="240" sId="1">
-    <nc r="R107" t="inlineStr">
-      <is>
-        <t>R+</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="241" sId="1">
-    <nc r="S107" t="inlineStr">
-      <is>
-        <t>R</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="242" sId="1">
-    <nc r="T107" t="inlineStr">
-      <is>
-        <t>R+</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="243" sId="1">
-    <nc r="U107" t="inlineStr">
-      <is>
-        <t>R</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="244" sId="1">
-    <nc r="V107" t="inlineStr">
-      <is>
-        <t>R+</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="245" sId="1">
-    <nc r="X107" t="inlineStr">
-      <is>
-        <t>R</t>
-      </is>
-    </nc>
-  </rcc>
-  <rfmt sheetId="1" sqref="Y107" start="0" length="0">
-    <dxf>
-      <font>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-  </rfmt>
-  <rcc rId="246" sId="1">
-    <nc r="B107" t="inlineStr">
-      <is>
-        <t>Tiemerkintä - Muut kustannukset</t>
-      </is>
-    </nc>
-  </rcc>
-  <rrc rId="247" sId="1" ref="A107:XFD107" action="insertRow"/>
-  <rcc rId="248" sId="1">
-    <nc r="A107" t="inlineStr">
-      <is>
-        <t>Raportit</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="249" sId="1">
-    <nc r="D107" t="inlineStr">
-      <is>
-        <t>R*</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="250" sId="1">
-    <nc r="E107" t="inlineStr">
-      <is>
-        <t>R*</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="251" sId="1">
-    <nc r="F107" t="inlineStr">
-      <is>
-        <t>R*</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="252" sId="1">
-    <nc r="G107" t="inlineStr">
-      <is>
-        <t>R*</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="253" sId="1">
-    <nc r="H107" t="inlineStr">
-      <is>
-        <t>R*</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="254" sId="1">
-    <nc r="I107" t="inlineStr">
-      <is>
-        <t>R</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="255" sId="1">
-    <nc r="J107" t="inlineStr">
-      <is>
-        <t>R</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="256" sId="1">
-    <nc r="K107" t="inlineStr">
-      <is>
-        <t>R*</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="257" sId="1">
-    <nc r="L107" t="inlineStr">
-      <is>
-        <t>R*</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="258" sId="1">
-    <nc r="M107" t="inlineStr">
-      <is>
-        <t>R</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="259" sId="1">
-    <nc r="N107" t="inlineStr">
-      <is>
-        <t>R*</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="260" sId="1">
-    <nc r="P107" t="inlineStr">
-      <is>
-        <t>R</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="261" sId="1">
-    <nc r="Q107" t="inlineStr">
-      <is>
-        <t>R</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="262" sId="1">
-    <nc r="R107" t="inlineStr">
-      <is>
-        <t>R+</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="263" sId="1">
-    <nc r="S107" t="inlineStr">
-      <is>
-        <t>R</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="264" sId="1">
-    <nc r="T107" t="inlineStr">
-      <is>
-        <t>R+</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="265" sId="1">
-    <nc r="U107" t="inlineStr">
-      <is>
-        <t>R</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="266" sId="1">
-    <nc r="V107" t="inlineStr">
-      <is>
-        <t>R+</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="267" sId="1">
-    <nc r="X107" t="inlineStr">
-      <is>
-        <t>R</t>
-      </is>
-    </nc>
-  </rcc>
-  <rcc rId="268" sId="1">
-    <nc r="B107" t="inlineStr">
-      <is>
-        <t>Tiemerkintä - Sakot ja bonukset</t>
-      </is>
-    </nc>
-  </rcc>
-  <rdn rId="0" localSheetId="1" customView="1" name="Z_810C905A_C0DA_4100_B6A9_F2260D80EA70_.wvu.FilterData" hidden="1" oldHidden="1">
-    <formula>Oikeudet!$A$5:$Y$136</formula>
-  </rdn>
-  <rcv guid="{810C905A-C0DA-4100-B6A9-F2260D80EA70}" action="add"/>
 </revisions>
 </file>
 
@@ -5480,12 +5137,11 @@
 </file>
 
 <file path=xl/revisions/userNames.xml><?xml version="1.0" encoding="utf-8"?>
-<users xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" count="5">
+<users xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" count="4">
   <userInfo guid="{8EBC2E30-8A6E-AD43-9F6F-B4500CF04203}" name="Jarno Väyrynen" id="-589133089" dateTime="2024-06-10T14:55:26"/>
   <userInfo guid="{CFB45395-62D4-124C-9898-DEF874662F1B}" name="Microsoft Office User" id="-296973103" dateTime="2024-11-20T15:04:38"/>
   <userInfo guid="{CF3F0B66-D3D6-2C4C-93DF-DEE3169712D4}" name="Microsoft Office User" id="-296992802" dateTime="2024-12-13T10:34:14"/>
   <userInfo guid="{64AC07D8-8D49-4F46-96EF-A9E3AD0E8431}" name="Jarno Väyrynen" id="-589128654" dateTime="2025-02-12T12:58:37"/>
-  <userInfo guid="{4A6ED1B0-9135-4362-95CD-B6A2DDFC57B0}" name="Samuli Taskila" id="-1631752395" dateTime="2025-04-02T11:10:08"/>
 </users>
 </file>
 
@@ -5665,12 +5321,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y138"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:Y136"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="31.6640625" customWidth="1"/>
-    <col min="3" max="3" width="14.109375" customWidth="1"/>
+    <col min="3" max="3" width="14.1640625" customWidth="1"/>
     <col min="4" max="4" width="30.33203125" customWidth="1"/>
     <col min="5" max="5" width="26.33203125" customWidth="1"/>
     <col min="6" max="6" width="12.6640625" customWidth="1"/>
@@ -5679,22 +5335,22 @@
     <col min="9" max="9" width="18.33203125" customWidth="1"/>
     <col min="10" max="10" width="25.33203125" customWidth="1"/>
     <col min="11" max="11" width="40.6640625" customWidth="1"/>
-    <col min="12" max="12" width="38.109375" customWidth="1"/>
+    <col min="12" max="12" width="38.1640625" customWidth="1"/>
     <col min="13" max="13" width="12.33203125" customWidth="1"/>
     <col min="14" max="14" width="10.6640625" customWidth="1"/>
-    <col min="15" max="16" width="12.44140625" customWidth="1"/>
+    <col min="15" max="16" width="12.5" customWidth="1"/>
     <col min="17" max="17" width="21.6640625" customWidth="1"/>
     <col min="18" max="18" width="36" customWidth="1"/>
     <col min="19" max="19" width="29.6640625" customWidth="1"/>
     <col min="20" max="20" width="15" customWidth="1"/>
     <col min="21" max="21" width="17.6640625" customWidth="1"/>
-    <col min="22" max="22" width="11.44140625" customWidth="1"/>
+    <col min="22" max="22" width="11.5" customWidth="1"/>
     <col min="23" max="23" width="11.6640625" customWidth="1"/>
     <col min="24" max="24" width="11.33203125" customWidth="1"/>
     <col min="25" max="25" width="59" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" ht="24" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -5715,7 +5371,7 @@
       <c r="N1" s="36"/>
       <c r="O1" s="36"/>
     </row>
-    <row r="2" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="37" t="s">
@@ -5734,7 +5390,7 @@
       <c r="N2" s="37"/>
       <c r="O2" s="37"/>
     </row>
-    <row r="3" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="2"/>
       <c r="B3" s="2" t="s">
         <v>3</v>
@@ -5749,10 +5405,10 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="C4" s="6"/>
     </row>
-    <row r="5" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="7"/>
       <c r="B5" s="7"/>
       <c r="C5" s="38" t="s">
@@ -5787,7 +5443,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="1" t="s">
         <v>11</v>
       </c>
@@ -5860,7 +5516,7 @@
       </c>
       <c r="Y6" s="7"/>
     </row>
-    <row r="7" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="11" t="s">
         <v>34</v>
       </c>
@@ -5933,7 +5589,7 @@
       </c>
       <c r="Y7" s="13"/>
     </row>
-    <row r="8" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="11" t="s">
         <v>34</v>
       </c>
@@ -5992,7 +5648,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="11" t="s">
         <v>34</v>
       </c>
@@ -6045,7 +5701,7 @@
       <c r="X9" s="12"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="11" t="s">
         <v>34</v>
       </c>
@@ -6098,7 +5754,7 @@
       <c r="X10" s="12"/>
       <c r="Y10" s="13"/>
     </row>
-    <row r="11" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="11" t="s">
         <v>34</v>
       </c>
@@ -6157,7 +5813,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="11" t="s">
         <v>34</v>
       </c>
@@ -6210,7 +5866,7 @@
       <c r="X12" s="12"/>
       <c r="Y12" s="13"/>
     </row>
-    <row r="13" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="11" t="s">
         <v>34</v>
       </c>
@@ -6277,7 +5933,7 @@
       <c r="X13" s="12"/>
       <c r="Y13" s="13"/>
     </row>
-    <row r="14" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="11" t="s">
         <v>34</v>
       </c>
@@ -6344,7 +6000,7 @@
       <c r="X14" s="12"/>
       <c r="Y14" s="13"/>
     </row>
-    <row r="15" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="11" t="s">
         <v>34</v>
       </c>
@@ -6401,7 +6057,7 @@
       <c r="X15" s="12"/>
       <c r="Y15" s="13"/>
     </row>
-    <row r="16" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="11" t="s">
         <v>34</v>
       </c>
@@ -6458,7 +6114,7 @@
       <c r="X16" s="12"/>
       <c r="Y16" s="13"/>
     </row>
-    <row r="17" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="11" t="s">
         <v>34</v>
       </c>
@@ -6515,7 +6171,7 @@
       <c r="X17" s="12"/>
       <c r="Y17" s="13"/>
     </row>
-    <row r="18" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="11" t="s">
         <v>34</v>
       </c>
@@ -6582,7 +6238,7 @@
       <c r="X18" s="12"/>
       <c r="Y18" s="13"/>
     </row>
-    <row r="19" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="11" t="s">
         <v>34</v>
       </c>
@@ -6649,7 +6305,7 @@
       <c r="X19" s="12"/>
       <c r="Y19" s="13"/>
     </row>
-    <row r="20" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="11" t="s">
         <v>34</v>
       </c>
@@ -6704,7 +6360,7 @@
       <c r="X20" s="12"/>
       <c r="Y20" s="13"/>
     </row>
-    <row r="21" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="11" t="s">
         <v>34</v>
       </c>
@@ -6765,7 +6421,7 @@
       <c r="X21" s="12"/>
       <c r="Y21" s="13"/>
     </row>
-    <row r="22" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="11" t="s">
         <v>34</v>
       </c>
@@ -6832,7 +6488,7 @@
       <c r="X22" s="12"/>
       <c r="Y22" s="13"/>
     </row>
-    <row r="23" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="11" t="s">
         <v>34</v>
       </c>
@@ -6905,7 +6561,7 @@
       </c>
       <c r="Y23" s="13"/>
     </row>
-    <row r="24" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="11" t="s">
         <v>34</v>
       </c>
@@ -6978,7 +6634,7 @@
       </c>
       <c r="Y24" s="13"/>
     </row>
-    <row r="25" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="11" t="s">
         <v>34</v>
       </c>
@@ -7051,7 +6707,7 @@
       </c>
       <c r="Y25" s="13"/>
     </row>
-    <row r="26" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="11" t="s">
         <v>34</v>
       </c>
@@ -7122,7 +6778,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="27" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="11" t="s">
         <v>34</v>
       </c>
@@ -7191,7 +6847,7 @@
       <c r="X27" s="12"/>
       <c r="Y27" s="13"/>
     </row>
-    <row r="28" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="11" t="s">
         <v>34</v>
       </c>
@@ -7237,7 +6893,7 @@
       </c>
       <c r="Y28" s="13"/>
     </row>
-    <row r="29" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="11" t="s">
         <v>34</v>
       </c>
@@ -7306,7 +6962,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="30" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="11" t="s">
         <v>34</v>
       </c>
@@ -7367,7 +7023,7 @@
       <c r="X30" s="12"/>
       <c r="Y30" s="13"/>
     </row>
-    <row r="31" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="11" t="s">
         <v>34</v>
       </c>
@@ -7424,7 +7080,7 @@
       <c r="X31" s="12"/>
       <c r="Y31" s="13"/>
     </row>
-    <row r="32" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="11" t="s">
         <v>34</v>
       </c>
@@ -7477,7 +7133,7 @@
       <c r="X32" s="12"/>
       <c r="Y32" s="13"/>
     </row>
-    <row r="33" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="11" t="s">
         <v>34</v>
       </c>
@@ -7522,7 +7178,7 @@
       <c r="X33" s="12"/>
       <c r="Y33" s="13"/>
     </row>
-    <row r="34" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A34" s="17" t="s">
         <v>34</v>
       </c>
@@ -7551,7 +7207,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="35" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A35" s="11" t="s">
         <v>34</v>
       </c>
@@ -7598,7 +7254,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="36" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A36" s="11" t="s">
         <v>34</v>
       </c>
@@ -7655,7 +7311,7 @@
       </c>
       <c r="Y36" s="13"/>
     </row>
-    <row r="37" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A37" s="11" t="s">
         <v>34</v>
       </c>
@@ -7712,7 +7368,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="38" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A38" s="11" t="s">
         <v>34</v>
       </c>
@@ -7765,7 +7421,7 @@
       <c r="X38" s="12"/>
       <c r="Y38" s="13"/>
     </row>
-    <row r="39" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A39" s="11" t="s">
         <v>34</v>
       </c>
@@ -7834,7 +7490,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="40" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A40" s="11" t="s">
         <v>34</v>
       </c>
@@ -7897,7 +7553,7 @@
       <c r="X40" s="12"/>
       <c r="Y40" s="13"/>
     </row>
-    <row r="41" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A41" s="11" t="s">
         <v>34</v>
       </c>
@@ -7962,7 +7618,7 @@
       <c r="X41" s="12"/>
       <c r="Y41" s="13"/>
     </row>
-    <row r="42" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A42" s="11" t="s">
         <v>34</v>
       </c>
@@ -8025,7 +7681,7 @@
       <c r="X42" s="12"/>
       <c r="Y42" s="13"/>
     </row>
-    <row r="43" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A43" s="11" t="s">
         <v>34</v>
       </c>
@@ -8088,7 +7744,7 @@
       <c r="X43" s="12"/>
       <c r="Y43" s="13"/>
     </row>
-    <row r="44" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A44" s="11" t="s">
         <v>34</v>
       </c>
@@ -8151,7 +7807,7 @@
       <c r="X44" s="12"/>
       <c r="Y44" s="13"/>
     </row>
-    <row r="45" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A45" s="11" t="s">
         <v>34</v>
       </c>
@@ -8214,7 +7870,7 @@
       <c r="X45" s="12"/>
       <c r="Y45" s="7"/>
     </row>
-    <row r="46" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A46" s="11" t="s">
         <v>34</v>
       </c>
@@ -8277,7 +7933,7 @@
       <c r="X46" s="12"/>
       <c r="Y46" s="7"/>
     </row>
-    <row r="47" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A47" s="11" t="s">
         <v>34</v>
       </c>
@@ -8340,7 +7996,7 @@
       <c r="X47" s="12"/>
       <c r="Y47" s="7"/>
     </row>
-    <row r="48" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A48" s="11" t="s">
         <v>34</v>
       </c>
@@ -8413,7 +8069,7 @@
       </c>
       <c r="Y48" s="13"/>
     </row>
-    <row r="49" spans="1:25" ht="39.6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:25" ht="28" x14ac:dyDescent="0.15">
       <c r="A49" s="11" t="s">
         <v>34</v>
       </c>
@@ -8466,7 +8122,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="50" spans="1:25" ht="66" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:25" ht="70" x14ac:dyDescent="0.15">
       <c r="A50" s="11" t="s">
         <v>34</v>
       </c>
@@ -8519,7 +8175,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="51" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:25" x14ac:dyDescent="0.15">
       <c r="A51" s="11" t="s">
         <v>34</v>
       </c>
@@ -8570,7 +8226,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="52" spans="1:25" ht="26.4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:25" ht="14" x14ac:dyDescent="0.15">
       <c r="A52" s="11" t="s">
         <v>34</v>
       </c>
@@ -8619,7 +8275,7 @@
       <c r="X52" s="15"/>
       <c r="Y52" s="7"/>
     </row>
-    <row r="53" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A53" s="17" t="s">
         <v>34</v>
       </c>
@@ -8670,7 +8326,7 @@
       <c r="W53" s="22"/>
       <c r="X53" s="22"/>
     </row>
-    <row r="54" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A54" s="11" t="s">
         <v>34</v>
       </c>
@@ -8719,7 +8375,7 @@
       <c r="X54" s="15"/>
       <c r="Y54" s="13"/>
     </row>
-    <row r="55" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A55" s="11" t="s">
         <v>34</v>
       </c>
@@ -8752,7 +8408,7 @@
       <c r="X55" s="12"/>
       <c r="Y55" s="13"/>
     </row>
-    <row r="56" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A56" s="11" t="s">
         <v>34</v>
       </c>
@@ -8805,7 +8461,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="57" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A57" s="11" t="s">
         <v>34</v>
       </c>
@@ -8838,7 +8494,7 @@
       <c r="X57" s="12"/>
       <c r="Y57" s="13"/>
     </row>
-    <row r="58" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A58" s="11" t="s">
         <v>34</v>
       </c>
@@ -8889,7 +8545,7 @@
       <c r="X58" s="12"/>
       <c r="Y58" s="13"/>
     </row>
-    <row r="59" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A59" s="11" t="s">
         <v>34</v>
       </c>
@@ -8952,7 +8608,7 @@
       <c r="X59" s="12"/>
       <c r="Y59" s="13"/>
     </row>
-    <row r="60" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A60" s="23" t="s">
         <v>34</v>
       </c>
@@ -9011,7 +8667,7 @@
       <c r="X60" s="12"/>
       <c r="Y60" s="13"/>
     </row>
-    <row r="61" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A61" s="23" t="s">
         <v>34</v>
       </c>
@@ -9072,7 +8728,7 @@
       <c r="X61" s="12"/>
       <c r="Y61" s="13"/>
     </row>
-    <row r="62" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A62" s="23" t="s">
         <v>34</v>
       </c>
@@ -9127,7 +8783,7 @@
       <c r="X62" s="12"/>
       <c r="Y62" s="13"/>
     </row>
-    <row r="63" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A63" s="11" t="s">
         <v>34</v>
       </c>
@@ -9200,7 +8856,7 @@
       </c>
       <c r="Y63" s="13"/>
     </row>
-    <row r="64" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A64" s="11" t="s">
         <v>160</v>
       </c>
@@ -9253,7 +8909,7 @@
       <c r="X64" s="12"/>
       <c r="Y64" s="13"/>
     </row>
-    <row r="65" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A65" s="11" t="s">
         <v>160</v>
       </c>
@@ -9306,7 +8962,7 @@
       <c r="X65" s="12"/>
       <c r="Y65" s="13"/>
     </row>
-    <row r="66" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A66" s="11" t="s">
         <v>160</v>
       </c>
@@ -9359,7 +9015,7 @@
       <c r="X66" s="12"/>
       <c r="Y66" s="13"/>
     </row>
-    <row r="67" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A67" s="11" t="s">
         <v>160</v>
       </c>
@@ -9412,7 +9068,7 @@
       <c r="X67" s="12"/>
       <c r="Y67" s="13"/>
     </row>
-    <row r="68" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A68" s="11" t="s">
         <v>160</v>
       </c>
@@ -9459,7 +9115,7 @@
       <c r="X68" s="12"/>
       <c r="Y68" s="13"/>
     </row>
-    <row r="69" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A69" s="11" t="s">
         <v>160</v>
       </c>
@@ -9512,7 +9168,7 @@
       <c r="X69" s="12"/>
       <c r="Y69" s="13"/>
     </row>
-    <row r="70" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A70" s="11" t="s">
         <v>160</v>
       </c>
@@ -9565,7 +9221,7 @@
       <c r="X70" s="12"/>
       <c r="Y70" s="13"/>
     </row>
-    <row r="71" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A71" s="11" t="s">
         <v>160</v>
       </c>
@@ -9618,7 +9274,7 @@
       <c r="X71" s="12"/>
       <c r="Y71" s="13"/>
     </row>
-    <row r="72" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A72" s="11" t="s">
         <v>160</v>
       </c>
@@ -9671,7 +9327,7 @@
       <c r="X72" s="12"/>
       <c r="Y72" s="13"/>
     </row>
-    <row r="73" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A73" s="11" t="s">
         <v>160</v>
       </c>
@@ -9706,7 +9362,7 @@
       <c r="X73" s="12"/>
       <c r="Y73" s="13"/>
     </row>
-    <row r="74" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A74" s="11" t="s">
         <v>160</v>
       </c>
@@ -9777,7 +9433,7 @@
       </c>
       <c r="Y74" s="13"/>
     </row>
-    <row r="75" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A75" s="11" t="s">
         <v>160</v>
       </c>
@@ -9850,7 +9506,7 @@
       </c>
       <c r="Y75" s="13"/>
     </row>
-    <row r="76" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A76" s="11" t="s">
         <v>160</v>
       </c>
@@ -9921,7 +9577,7 @@
       </c>
       <c r="Y76" s="13"/>
     </row>
-    <row r="77" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A77" s="11" t="s">
         <v>160</v>
       </c>
@@ -9992,7 +9648,7 @@
       </c>
       <c r="Y77" s="13"/>
     </row>
-    <row r="78" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A78" s="11" t="s">
         <v>160</v>
       </c>
@@ -10027,7 +9683,7 @@
       <c r="X78" s="12"/>
       <c r="Y78" s="13"/>
     </row>
-    <row r="79" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A79" s="11" t="s">
         <v>160</v>
       </c>
@@ -10098,7 +9754,7 @@
       </c>
       <c r="Y79" s="13"/>
     </row>
-    <row r="80" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A80" s="11" t="s">
         <v>160</v>
       </c>
@@ -10169,7 +9825,7 @@
       </c>
       <c r="Y80" s="13"/>
     </row>
-    <row r="81" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A81" s="11" t="s">
         <v>160</v>
       </c>
@@ -10238,7 +9894,7 @@
       </c>
       <c r="Y81" s="13"/>
     </row>
-    <row r="82" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A82" s="11" t="s">
         <v>160</v>
       </c>
@@ -10309,7 +9965,7 @@
       </c>
       <c r="Y82" s="13"/>
     </row>
-    <row r="83" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A83" s="11" t="s">
         <v>160</v>
       </c>
@@ -10372,7 +10028,7 @@
       </c>
       <c r="Y83" s="13"/>
     </row>
-    <row r="84" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A84" s="11" t="s">
         <v>160</v>
       </c>
@@ -10429,7 +10085,7 @@
       <c r="X84" s="12"/>
       <c r="Y84" s="13"/>
     </row>
-    <row r="85" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A85" s="11" t="s">
         <v>160</v>
       </c>
@@ -10464,7 +10120,7 @@
       <c r="X85" s="12"/>
       <c r="Y85" s="13"/>
     </row>
-    <row r="86" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A86" s="11" t="s">
         <v>160</v>
       </c>
@@ -10499,7 +10155,7 @@
       <c r="X86" s="12"/>
       <c r="Y86" s="13"/>
     </row>
-    <row r="87" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A87" s="11" t="s">
         <v>160</v>
       </c>
@@ -10534,7 +10190,7 @@
       <c r="X87" s="12"/>
       <c r="Y87" s="13"/>
     </row>
-    <row r="88" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A88" s="11" t="s">
         <v>160</v>
       </c>
@@ -10603,7 +10259,7 @@
       </c>
       <c r="Y88" s="13"/>
     </row>
-    <row r="89" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A89" s="11" t="s">
         <v>160</v>
       </c>
@@ -10672,7 +10328,7 @@
       </c>
       <c r="Y89" s="13"/>
     </row>
-    <row r="90" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A90" s="11" t="s">
         <v>160</v>
       </c>
@@ -10743,7 +10399,7 @@
       </c>
       <c r="Y90" s="13"/>
     </row>
-    <row r="91" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A91" s="11" t="s">
         <v>160</v>
       </c>
@@ -10812,7 +10468,7 @@
       <c r="X91" s="12"/>
       <c r="Y91" s="13"/>
     </row>
-    <row r="92" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A92" s="11" t="s">
         <v>160</v>
       </c>
@@ -10881,7 +10537,7 @@
       <c r="X92" s="12"/>
       <c r="Y92" s="13"/>
     </row>
-    <row r="93" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A93" s="11" t="s">
         <v>160</v>
       </c>
@@ -10950,7 +10606,7 @@
       <c r="X93" s="12"/>
       <c r="Y93" s="13"/>
     </row>
-    <row r="94" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A94" s="11" t="s">
         <v>160</v>
       </c>
@@ -11019,7 +10675,7 @@
       <c r="X94" s="12"/>
       <c r="Y94" s="13"/>
     </row>
-    <row r="95" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A95" s="11" t="s">
         <v>160</v>
       </c>
@@ -11088,7 +10744,7 @@
       <c r="X95" s="12"/>
       <c r="Y95" s="13"/>
     </row>
-    <row r="96" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A96" s="11" t="s">
         <v>160</v>
       </c>
@@ -11123,7 +10779,7 @@
       <c r="X96" s="12"/>
       <c r="Y96" s="13"/>
     </row>
-    <row r="97" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A97" s="11" t="s">
         <v>160</v>
       </c>
@@ -11192,7 +10848,7 @@
       <c r="X97" s="12"/>
       <c r="Y97" s="13"/>
     </row>
-    <row r="98" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A98" s="11" t="s">
         <v>160</v>
       </c>
@@ -11245,7 +10901,7 @@
       <c r="X98" s="12"/>
       <c r="Y98" s="13"/>
     </row>
-    <row r="99" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A99" s="11" t="s">
         <v>160</v>
       </c>
@@ -11318,7 +10974,7 @@
       </c>
       <c r="Y99" s="13"/>
     </row>
-    <row r="100" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A100" s="11" t="s">
         <v>160</v>
       </c>
@@ -11391,7 +11047,7 @@
       </c>
       <c r="Y100" s="13"/>
     </row>
-    <row r="101" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A101" s="11" t="s">
         <v>160</v>
       </c>
@@ -11464,7 +11120,7 @@
       </c>
       <c r="Y101" s="13"/>
     </row>
-    <row r="102" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A102" s="11" t="s">
         <v>160</v>
       </c>
@@ -11535,7 +11191,7 @@
       </c>
       <c r="Y102" s="13"/>
     </row>
-    <row r="103" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A103" s="11" t="s">
         <v>160</v>
       </c>
@@ -11568,7 +11224,7 @@
       <c r="X103" s="12"/>
       <c r="Y103" s="13"/>
     </row>
-    <row r="104" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A104" s="11" t="s">
         <v>160</v>
       </c>
@@ -11639,7 +11295,7 @@
       </c>
       <c r="Y104" s="13"/>
     </row>
-    <row r="105" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A105" s="11" t="s">
         <v>160</v>
       </c>
@@ -11712,7 +11368,7 @@
       </c>
       <c r="Y105" s="13"/>
     </row>
-    <row r="106" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A106" s="11" t="s">
         <v>160</v>
       </c>
@@ -11785,40 +11441,34 @@
       </c>
       <c r="Y106" s="13"/>
     </row>
-    <row r="107" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A107" s="11" t="s">
         <v>160</v>
       </c>
       <c r="B107" s="11" t="s">
-        <v>274</v>
+        <v>200</v>
       </c>
       <c r="C107" s="12"/>
       <c r="D107" s="12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E107" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F107" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G107" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="H107" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="I107" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="G107" s="12"/>
+      <c r="H107" s="12"/>
+      <c r="I107" s="12"/>
       <c r="J107" s="12" t="s">
         <v>39</v>
       </c>
       <c r="K107" s="12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="L107" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="M107" s="12" t="s">
         <v>39</v>
@@ -11827,39 +11477,33 @@
         <v>38</v>
       </c>
       <c r="O107" s="12"/>
-      <c r="P107" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="P107" s="12"/>
       <c r="Q107" s="12" t="s">
         <v>39</v>
       </c>
       <c r="R107" s="12" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="S107" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="T107" s="12" t="s">
-        <v>44</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="T107" s="12"/>
       <c r="U107" s="12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="V107" s="12" t="s">
         <v>44</v>
       </c>
       <c r="W107" s="12"/>
-      <c r="X107" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="X107" s="12"/>
       <c r="Y107" s="13"/>
     </row>
-    <row r="108" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A108" s="11" t="s">
-        <v>160</v>
+        <v>201</v>
       </c>
       <c r="B108" s="11" t="s">
-        <v>273</v>
+        <v>202</v>
       </c>
       <c r="C108" s="12"/>
       <c r="D108" s="12" t="s">
@@ -11881,7 +11525,7 @@
         <v>39</v>
       </c>
       <c r="J108" s="12" t="s">
-        <v>39</v>
+        <v>203</v>
       </c>
       <c r="K108" s="12" t="s">
         <v>38</v>
@@ -11895,18 +11539,20 @@
       <c r="N108" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="O108" s="12"/>
+      <c r="O108" s="12" t="s">
+        <v>38</v>
+      </c>
       <c r="P108" s="12" t="s">
         <v>39</v>
       </c>
       <c r="Q108" s="12" t="s">
-        <v>39</v>
+        <v>203</v>
       </c>
       <c r="R108" s="12" t="s">
-        <v>44</v>
+        <v>204</v>
       </c>
       <c r="S108" s="12" t="s">
-        <v>39</v>
+        <v>203</v>
       </c>
       <c r="T108" s="12" t="s">
         <v>44</v>
@@ -11917,40 +11563,50 @@
       <c r="V108" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="W108" s="12"/>
+      <c r="W108" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="X108" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="Y108" s="13"/>
-    </row>
-    <row r="109" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Y108" s="35" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="109" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A109" s="11" t="s">
-        <v>160</v>
+        <v>201</v>
       </c>
       <c r="B109" s="11" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="C109" s="12"/>
       <c r="D109" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E109" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F109" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G109" s="12"/>
-      <c r="H109" s="12"/>
-      <c r="I109" s="12"/>
+      <c r="G109" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="H109" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I109" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="J109" s="12" t="s">
-        <v>39</v>
+        <v>203</v>
       </c>
       <c r="K109" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="L109" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="M109" s="12" t="s">
         <v>39</v>
@@ -11958,38 +11614,48 @@
       <c r="N109" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="O109" s="12"/>
-      <c r="P109" s="12"/>
+      <c r="O109" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="P109" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="Q109" s="12" t="s">
-        <v>39</v>
+        <v>203</v>
       </c>
       <c r="R109" s="12" t="s">
-        <v>42</v>
+        <v>204</v>
       </c>
       <c r="S109" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="T109" s="12"/>
+        <v>203</v>
+      </c>
+      <c r="T109" s="12" t="s">
+        <v>44</v>
+      </c>
       <c r="U109" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="V109" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="W109" s="12"/>
-      <c r="X109" s="12"/>
-      <c r="Y109" s="13"/>
-    </row>
-    <row r="110" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="W109" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="X109" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y109" s="35"/>
+    </row>
+    <row r="110" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A110" s="11" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="B110" s="11" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="C110" s="12"/>
       <c r="D110" s="12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E110" s="12" t="s">
         <v>38</v>
@@ -12007,10 +11673,10 @@
         <v>39</v>
       </c>
       <c r="J110" s="12" t="s">
-        <v>203</v>
+        <v>39</v>
       </c>
       <c r="K110" s="12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="L110" s="12" t="s">
         <v>38</v>
@@ -12028,43 +11694,41 @@
         <v>39</v>
       </c>
       <c r="Q110" s="12" t="s">
-        <v>203</v>
+        <v>39</v>
       </c>
       <c r="R110" s="12" t="s">
-        <v>204</v>
+        <v>42</v>
       </c>
       <c r="S110" s="12" t="s">
-        <v>203</v>
+        <v>40</v>
       </c>
       <c r="T110" s="12" t="s">
         <v>44</v>
       </c>
       <c r="U110" s="12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="V110" s="12" t="s">
         <v>44</v>
       </c>
       <c r="W110" s="12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="X110" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y110" s="35" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="111" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="Y110" s="7"/>
+    </row>
+    <row r="111" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A111" s="11" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B111" s="11" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="C111" s="12"/>
       <c r="D111" s="12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E111" s="12" t="s">
         <v>38</v>
@@ -12082,10 +11746,10 @@
         <v>39</v>
       </c>
       <c r="J111" s="12" t="s">
-        <v>203</v>
+        <v>39</v>
       </c>
       <c r="K111" s="12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="L111" s="12" t="s">
         <v>38</v>
@@ -12103,246 +11767,166 @@
         <v>39</v>
       </c>
       <c r="Q111" s="12" t="s">
-        <v>203</v>
+        <v>39</v>
       </c>
       <c r="R111" s="12" t="s">
-        <v>204</v>
+        <v>42</v>
       </c>
       <c r="S111" s="12" t="s">
-        <v>203</v>
+        <v>40</v>
       </c>
       <c r="T111" s="12" t="s">
         <v>44</v>
       </c>
       <c r="U111" s="12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="V111" s="12" t="s">
         <v>44</v>
       </c>
       <c r="W111" s="12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="X111" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y111" s="35"/>
-    </row>
-    <row r="112" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A112" s="11" t="s">
-        <v>207</v>
-      </c>
-      <c r="B112" s="11" t="s">
-        <v>208</v>
-      </c>
-      <c r="C112" s="12"/>
+        <v>40</v>
+      </c>
+      <c r="Y111" s="13"/>
+    </row>
+    <row r="112" spans="1:25" s="30" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A112" s="27" t="s">
+        <v>209</v>
+      </c>
+      <c r="B112" s="27" t="s">
+        <v>210</v>
+      </c>
+      <c r="C112" s="28"/>
       <c r="D112" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E112" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="F112" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="G112" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="H112" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="I112" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="J112" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="K112" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="L112" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="M112" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="N112" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="O112" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="P112" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q112" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="R112" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="S112" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="T112" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="U112" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="V112" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="W112" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="X112" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y112" s="7"/>
-    </row>
-    <row r="113" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E112" s="28"/>
+      <c r="F112" s="28"/>
+      <c r="G112" s="28"/>
+      <c r="H112" s="28"/>
+      <c r="I112" s="28"/>
+      <c r="J112" s="28"/>
+      <c r="K112" s="28"/>
+      <c r="L112" s="28"/>
+      <c r="M112" s="28"/>
+      <c r="N112" s="28"/>
+      <c r="O112" s="28"/>
+      <c r="P112" s="28"/>
+      <c r="Q112" s="28"/>
+      <c r="R112" s="28"/>
+      <c r="S112" s="28"/>
+      <c r="T112" s="28"/>
+      <c r="U112" s="28"/>
+      <c r="V112" s="28"/>
+      <c r="W112" s="28"/>
+      <c r="X112" s="28"/>
+      <c r="Y112" s="29" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="113" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A113" s="11" t="s">
-        <v>199</v>
+        <v>209</v>
       </c>
       <c r="B113" s="11" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
       <c r="C113" s="12"/>
       <c r="D113" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E113" s="12" t="s">
-        <v>38</v>
-      </c>
+      <c r="E113" s="12"/>
       <c r="F113" s="12" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="G113" s="12" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="H113" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="I113" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="J113" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="K113" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="L113" s="12" t="s">
-        <v>38</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="I113" s="12"/>
+      <c r="J113" s="12"/>
+      <c r="K113" s="12"/>
+      <c r="L113" s="12"/>
       <c r="M113" s="12" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="N113" s="12" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="O113" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="P113" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q113" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="R113" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="S113" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="T113" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="U113" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="V113" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="W113" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="X113" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y113" s="13"/>
-    </row>
-    <row r="114" spans="1:25" s="30" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A114" s="27" t="s">
+        <v>46</v>
+      </c>
+      <c r="P113" s="12"/>
+      <c r="Q113" s="12"/>
+      <c r="R113" s="12"/>
+      <c r="S113" s="12"/>
+      <c r="T113" s="12"/>
+      <c r="U113" s="12"/>
+      <c r="V113" s="12"/>
+      <c r="W113" s="12"/>
+      <c r="X113" s="12"/>
+      <c r="Y113" s="7"/>
+    </row>
+    <row r="114" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A114" s="11" t="s">
         <v>209</v>
       </c>
-      <c r="B114" s="27" t="s">
-        <v>210</v>
-      </c>
-      <c r="C114" s="28"/>
+      <c r="B114" s="11" t="s">
+        <v>213</v>
+      </c>
+      <c r="C114" s="12"/>
       <c r="D114" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E114" s="28"/>
-      <c r="F114" s="28"/>
-      <c r="G114" s="28"/>
-      <c r="H114" s="28"/>
-      <c r="I114" s="28"/>
-      <c r="J114" s="28"/>
-      <c r="K114" s="28"/>
-      <c r="L114" s="28"/>
-      <c r="M114" s="28"/>
-      <c r="N114" s="28"/>
-      <c r="O114" s="28"/>
-      <c r="P114" s="28"/>
-      <c r="Q114" s="28"/>
-      <c r="R114" s="28"/>
-      <c r="S114" s="28"/>
-      <c r="T114" s="28"/>
-      <c r="U114" s="28"/>
-      <c r="V114" s="28"/>
-      <c r="W114" s="28"/>
-      <c r="X114" s="28"/>
-      <c r="Y114" s="29" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="115" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E114" s="12"/>
+      <c r="F114" s="12"/>
+      <c r="G114" s="12"/>
+      <c r="H114" s="12"/>
+      <c r="I114" s="12"/>
+      <c r="J114" s="12"/>
+      <c r="K114" s="12"/>
+      <c r="L114" s="12"/>
+      <c r="M114" s="12"/>
+      <c r="N114" s="12"/>
+      <c r="O114" s="12"/>
+      <c r="P114" s="12"/>
+      <c r="Q114" s="12"/>
+      <c r="R114" s="12"/>
+      <c r="S114" s="12"/>
+      <c r="T114" s="12"/>
+      <c r="U114" s="12"/>
+      <c r="V114" s="12"/>
+      <c r="W114" s="12"/>
+      <c r="X114" s="12"/>
+      <c r="Y114" s="7"/>
+    </row>
+    <row r="115" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A115" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B115" s="11" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C115" s="12"/>
       <c r="D115" s="12" t="s">
         <v>41</v>
       </c>
       <c r="E115" s="12"/>
-      <c r="F115" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="G115" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="H115" s="12" t="s">
-        <v>46</v>
-      </c>
+      <c r="F115" s="12"/>
+      <c r="G115" s="12"/>
+      <c r="H115" s="12"/>
       <c r="I115" s="12"/>
       <c r="J115" s="12"/>
       <c r="K115" s="12"/>
       <c r="L115" s="12"/>
-      <c r="M115" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="N115" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="O115" s="12" t="s">
-        <v>46</v>
-      </c>
+      <c r="M115" s="12"/>
+      <c r="N115" s="12"/>
+      <c r="O115" s="12"/>
       <c r="P115" s="12"/>
       <c r="Q115" s="12"/>
       <c r="R115" s="12"/>
@@ -12354,12 +11938,12 @@
       <c r="X115" s="12"/>
       <c r="Y115" s="7"/>
     </row>
-    <row r="116" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A116" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B116" s="11" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C116" s="12"/>
       <c r="D116" s="12" t="s">
@@ -12387,12 +11971,12 @@
       <c r="X116" s="12"/>
       <c r="Y116" s="7"/>
     </row>
-    <row r="117" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A117" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B117" s="11" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C117" s="12"/>
       <c r="D117" s="12" t="s">
@@ -12420,12 +12004,12 @@
       <c r="X117" s="12"/>
       <c r="Y117" s="7"/>
     </row>
-    <row r="118" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A118" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B118" s="11" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C118" s="12"/>
       <c r="D118" s="12" t="s">
@@ -12453,12 +12037,12 @@
       <c r="X118" s="12"/>
       <c r="Y118" s="7"/>
     </row>
-    <row r="119" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A119" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B119" s="11" t="s">
-        <v>216</v>
+        <v>76</v>
       </c>
       <c r="C119" s="12"/>
       <c r="D119" s="12" t="s">
@@ -12486,12 +12070,12 @@
       <c r="X119" s="12"/>
       <c r="Y119" s="7"/>
     </row>
-    <row r="120" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A120" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B120" s="11" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C120" s="12"/>
       <c r="D120" s="12" t="s">
@@ -12519,45 +12103,45 @@
       <c r="X120" s="12"/>
       <c r="Y120" s="7"/>
     </row>
-    <row r="121" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A121" s="11" t="s">
         <v>209</v>
       </c>
-      <c r="B121" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="C121" s="12"/>
-      <c r="D121" s="12" t="s">
+      <c r="B121" s="14" t="s">
+        <v>219</v>
+      </c>
+      <c r="C121" s="15"/>
+      <c r="D121" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="E121" s="12"/>
-      <c r="F121" s="12"/>
-      <c r="G121" s="12"/>
-      <c r="H121" s="12"/>
-      <c r="I121" s="12"/>
-      <c r="J121" s="12"/>
-      <c r="K121" s="12"/>
-      <c r="L121" s="12"/>
-      <c r="M121" s="12"/>
-      <c r="N121" s="12"/>
-      <c r="O121" s="12"/>
-      <c r="P121" s="12"/>
-      <c r="Q121" s="12"/>
-      <c r="R121" s="12"/>
-      <c r="S121" s="12"/>
-      <c r="T121" s="12"/>
-      <c r="U121" s="12"/>
-      <c r="V121" s="12"/>
-      <c r="W121" s="12"/>
-      <c r="X121" s="12"/>
-      <c r="Y121" s="7"/>
-    </row>
-    <row r="122" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E121" s="15"/>
+      <c r="F121" s="15"/>
+      <c r="G121" s="15"/>
+      <c r="H121" s="15"/>
+      <c r="I121" s="15"/>
+      <c r="J121" s="15"/>
+      <c r="K121" s="15"/>
+      <c r="L121" s="15"/>
+      <c r="M121" s="15"/>
+      <c r="N121" s="15"/>
+      <c r="O121" s="15"/>
+      <c r="P121" s="15"/>
+      <c r="Q121" s="15"/>
+      <c r="R121" s="15"/>
+      <c r="S121" s="15"/>
+      <c r="T121" s="15"/>
+      <c r="U121" s="15"/>
+      <c r="V121" s="15"/>
+      <c r="W121" s="15"/>
+      <c r="X121" s="15"/>
+      <c r="Y121" s="13"/>
+    </row>
+    <row r="122" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A122" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B122" s="11" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C122" s="12"/>
       <c r="D122" s="12" t="s">
@@ -12585,45 +12169,45 @@
       <c r="X122" s="12"/>
       <c r="Y122" s="7"/>
     </row>
-    <row r="123" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A123" s="11" t="s">
         <v>209</v>
       </c>
-      <c r="B123" s="14" t="s">
-        <v>219</v>
-      </c>
-      <c r="C123" s="15"/>
-      <c r="D123" s="15" t="s">
+      <c r="B123" s="11" t="s">
+        <v>221</v>
+      </c>
+      <c r="C123" s="12"/>
+      <c r="D123" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E123" s="15"/>
-      <c r="F123" s="15"/>
-      <c r="G123" s="15"/>
-      <c r="H123" s="15"/>
-      <c r="I123" s="15"/>
-      <c r="J123" s="15"/>
-      <c r="K123" s="15"/>
-      <c r="L123" s="15"/>
-      <c r="M123" s="15"/>
-      <c r="N123" s="15"/>
-      <c r="O123" s="15"/>
-      <c r="P123" s="15"/>
-      <c r="Q123" s="15"/>
-      <c r="R123" s="15"/>
-      <c r="S123" s="15"/>
-      <c r="T123" s="15"/>
-      <c r="U123" s="15"/>
-      <c r="V123" s="15"/>
-      <c r="W123" s="15"/>
-      <c r="X123" s="15"/>
-      <c r="Y123" s="13"/>
-    </row>
-    <row r="124" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E123" s="12"/>
+      <c r="F123" s="12"/>
+      <c r="G123" s="12"/>
+      <c r="H123" s="12"/>
+      <c r="I123" s="12"/>
+      <c r="J123" s="12"/>
+      <c r="K123" s="12"/>
+      <c r="L123" s="12"/>
+      <c r="M123" s="12"/>
+      <c r="N123" s="12"/>
+      <c r="O123" s="12"/>
+      <c r="P123" s="12"/>
+      <c r="Q123" s="12"/>
+      <c r="R123" s="12"/>
+      <c r="S123" s="12"/>
+      <c r="T123" s="12"/>
+      <c r="U123" s="12"/>
+      <c r="V123" s="12"/>
+      <c r="W123" s="12"/>
+      <c r="X123" s="12"/>
+      <c r="Y123" s="7"/>
+    </row>
+    <row r="124" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A124" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B124" s="11" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C124" s="12"/>
       <c r="D124" s="12" t="s">
@@ -12651,12 +12235,12 @@
       <c r="X124" s="12"/>
       <c r="Y124" s="7"/>
     </row>
-    <row r="125" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A125" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B125" s="11" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C125" s="12"/>
       <c r="D125" s="12" t="s">
@@ -12684,12 +12268,12 @@
       <c r="X125" s="12"/>
       <c r="Y125" s="7"/>
     </row>
-    <row r="126" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A126" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B126" s="11" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C126" s="12"/>
       <c r="D126" s="12" t="s">
@@ -12717,12 +12301,12 @@
       <c r="X126" s="12"/>
       <c r="Y126" s="7"/>
     </row>
-    <row r="127" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A127" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B127" s="11" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C127" s="12"/>
       <c r="D127" s="12" t="s">
@@ -12750,12 +12334,12 @@
       <c r="X127" s="12"/>
       <c r="Y127" s="7"/>
     </row>
-    <row r="128" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A128" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B128" s="11" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C128" s="12"/>
       <c r="D128" s="12" t="s">
@@ -12783,12 +12367,12 @@
       <c r="X128" s="12"/>
       <c r="Y128" s="7"/>
     </row>
-    <row r="129" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A129" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B129" s="11" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C129" s="12"/>
       <c r="D129" s="12" t="s">
@@ -12816,12 +12400,12 @@
       <c r="X129" s="12"/>
       <c r="Y129" s="7"/>
     </row>
-    <row r="130" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A130" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B130" s="11" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C130" s="12"/>
       <c r="D130" s="12" t="s">
@@ -12849,12 +12433,12 @@
       <c r="X130" s="12"/>
       <c r="Y130" s="7"/>
     </row>
-    <row r="131" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A131" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B131" s="11" t="s">
-        <v>227</v>
+        <v>264</v>
       </c>
       <c r="C131" s="12"/>
       <c r="D131" s="12" t="s">
@@ -12882,16 +12466,16 @@
       <c r="X131" s="12"/>
       <c r="Y131" s="7"/>
     </row>
-    <row r="132" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A132" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B132" s="11" t="s">
-        <v>228</v>
+        <v>270</v>
       </c>
       <c r="C132" s="12"/>
       <c r="D132" s="12" t="s">
-        <v>41</v>
+        <v>100</v>
       </c>
       <c r="E132" s="12"/>
       <c r="F132" s="12"/>
@@ -12915,12 +12499,12 @@
       <c r="X132" s="12"/>
       <c r="Y132" s="7"/>
     </row>
-    <row r="133" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A133" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B133" s="11" t="s">
-        <v>264</v>
+        <v>229</v>
       </c>
       <c r="C133" s="12"/>
       <c r="D133" s="12" t="s">
@@ -12948,204 +12532,144 @@
       <c r="X133" s="12"/>
       <c r="Y133" s="7"/>
     </row>
-    <row r="134" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A134" s="11" t="s">
-        <v>209</v>
+        <v>230</v>
       </c>
       <c r="B134" s="11" t="s">
-        <v>270</v>
-      </c>
-      <c r="C134" s="12"/>
+        <v>231</v>
+      </c>
+      <c r="C134" s="16"/>
       <c r="D134" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="E134" s="12"/>
-      <c r="F134" s="12"/>
-      <c r="G134" s="12"/>
-      <c r="H134" s="12"/>
-      <c r="I134" s="12"/>
-      <c r="J134" s="12"/>
-      <c r="K134" s="12"/>
-      <c r="L134" s="12"/>
-      <c r="M134" s="12"/>
-      <c r="N134" s="12"/>
-      <c r="O134" s="12"/>
-      <c r="P134" s="12"/>
-      <c r="Q134" s="12"/>
-      <c r="R134" s="12"/>
-      <c r="S134" s="12"/>
-      <c r="T134" s="12"/>
-      <c r="U134" s="12"/>
-      <c r="V134" s="12"/>
-      <c r="W134" s="12"/>
-      <c r="X134" s="12"/>
+        <v>41</v>
+      </c>
+      <c r="E134" s="16"/>
+      <c r="F134" s="16"/>
+      <c r="G134" s="16"/>
+      <c r="H134" s="16"/>
+      <c r="I134" s="16"/>
+      <c r="J134" s="16"/>
+      <c r="K134" s="16"/>
+      <c r="L134" s="16"/>
+      <c r="M134" s="16"/>
+      <c r="N134" s="16"/>
+      <c r="O134" s="16"/>
+      <c r="P134" s="16"/>
+      <c r="Q134" s="16"/>
+      <c r="R134" s="16"/>
+      <c r="S134" s="16"/>
+      <c r="T134" s="16"/>
+      <c r="U134" s="16"/>
+      <c r="V134" s="16"/>
+      <c r="W134" s="16"/>
+      <c r="X134" s="16"/>
       <c r="Y134" s="7"/>
     </row>
-    <row r="135" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A135" s="11" t="s">
-        <v>209</v>
+        <v>232</v>
       </c>
       <c r="B135" s="11" t="s">
-        <v>229</v>
-      </c>
-      <c r="C135" s="12"/>
+        <v>233</v>
+      </c>
+      <c r="C135" s="16"/>
       <c r="D135" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="E135" s="12"/>
-      <c r="F135" s="12"/>
-      <c r="G135" s="12"/>
-      <c r="H135" s="12"/>
-      <c r="I135" s="12"/>
-      <c r="J135" s="12"/>
-      <c r="K135" s="12"/>
-      <c r="L135" s="12"/>
-      <c r="M135" s="12"/>
-      <c r="N135" s="12"/>
-      <c r="O135" s="12"/>
-      <c r="P135" s="12"/>
-      <c r="Q135" s="12"/>
-      <c r="R135" s="12"/>
-      <c r="S135" s="12"/>
-      <c r="T135" s="12"/>
-      <c r="U135" s="12"/>
-      <c r="V135" s="12"/>
-      <c r="W135" s="12"/>
-      <c r="X135" s="12"/>
+        <v>234</v>
+      </c>
+      <c r="E135" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="F135" s="31"/>
+      <c r="G135" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="H135" s="31"/>
+      <c r="I135" s="31"/>
+      <c r="J135" s="31" t="s">
+        <v>235</v>
+      </c>
+      <c r="K135" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="L135" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="M135" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="N135" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="O135" s="31"/>
+      <c r="P135" s="31"/>
+      <c r="Q135" s="31" t="s">
+        <v>235</v>
+      </c>
+      <c r="R135" s="31" t="s">
+        <v>236</v>
+      </c>
+      <c r="S135" s="31" t="s">
+        <v>235</v>
+      </c>
+      <c r="T135" s="31"/>
+      <c r="U135" s="31" t="s">
+        <v>235</v>
+      </c>
+      <c r="V135" s="31"/>
+      <c r="W135" s="31"/>
+      <c r="X135" s="31"/>
       <c r="Y135" s="7"/>
     </row>
-    <row r="136" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A136" s="11" t="s">
-        <v>230</v>
+        <v>265</v>
       </c>
       <c r="B136" s="11" t="s">
-        <v>231</v>
+        <v>265</v>
       </c>
       <c r="C136" s="16"/>
       <c r="D136" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="E136" s="16"/>
-      <c r="F136" s="16"/>
-      <c r="G136" s="16"/>
-      <c r="H136" s="16"/>
-      <c r="I136" s="16"/>
-      <c r="J136" s="16"/>
-      <c r="K136" s="16"/>
-      <c r="L136" s="16"/>
-      <c r="M136" s="16"/>
-      <c r="N136" s="16"/>
-      <c r="O136" s="16"/>
-      <c r="P136" s="16"/>
-      <c r="Q136" s="16"/>
-      <c r="R136" s="16"/>
-      <c r="S136" s="16"/>
-      <c r="T136" s="16"/>
-      <c r="U136" s="16"/>
-      <c r="V136" s="16"/>
-      <c r="W136" s="16"/>
-      <c r="X136" s="16"/>
+        <v>38</v>
+      </c>
+      <c r="E136" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="F136" s="31"/>
+      <c r="G136" s="31"/>
+      <c r="H136" s="31"/>
+      <c r="I136" s="31"/>
+      <c r="J136" s="31"/>
+      <c r="K136" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="L136" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="M136" s="31"/>
+      <c r="N136" s="31"/>
+      <c r="O136" s="31"/>
+      <c r="P136" s="31"/>
+      <c r="Q136" s="31"/>
+      <c r="R136" s="31"/>
+      <c r="S136" s="31"/>
+      <c r="T136" s="31"/>
+      <c r="U136" s="31"/>
+      <c r="V136" s="31"/>
+      <c r="W136" s="31"/>
+      <c r="X136" s="31"/>
       <c r="Y136" s="7"/>
-    </row>
-    <row r="137" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A137" s="11" t="s">
-        <v>232</v>
-      </c>
-      <c r="B137" s="11" t="s">
-        <v>233</v>
-      </c>
-      <c r="C137" s="16"/>
-      <c r="D137" s="12" t="s">
-        <v>234</v>
-      </c>
-      <c r="E137" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="F137" s="31"/>
-      <c r="G137" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="H137" s="31"/>
-      <c r="I137" s="31"/>
-      <c r="J137" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="K137" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="L137" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="M137" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="N137" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="O137" s="31"/>
-      <c r="P137" s="31"/>
-      <c r="Q137" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="R137" s="31" t="s">
-        <v>236</v>
-      </c>
-      <c r="S137" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="T137" s="31"/>
-      <c r="U137" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="V137" s="31"/>
-      <c r="W137" s="31"/>
-      <c r="X137" s="31"/>
-      <c r="Y137" s="7"/>
-    </row>
-    <row r="138" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A138" s="11" t="s">
-        <v>265</v>
-      </c>
-      <c r="B138" s="11" t="s">
-        <v>265</v>
-      </c>
-      <c r="C138" s="16"/>
-      <c r="D138" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="E138" s="31" t="s">
-        <v>38</v>
-      </c>
-      <c r="F138" s="31"/>
-      <c r="G138" s="31"/>
-      <c r="H138" s="31"/>
-      <c r="I138" s="31"/>
-      <c r="J138" s="31"/>
-      <c r="K138" s="31" t="s">
-        <v>38</v>
-      </c>
-      <c r="L138" s="31" t="s">
-        <v>38</v>
-      </c>
-      <c r="M138" s="31"/>
-      <c r="N138" s="31"/>
-      <c r="O138" s="31"/>
-      <c r="P138" s="31"/>
-      <c r="Q138" s="31"/>
-      <c r="R138" s="31"/>
-      <c r="S138" s="31"/>
-      <c r="T138" s="31"/>
-      <c r="U138" s="31"/>
-      <c r="V138" s="31"/>
-      <c r="W138" s="31"/>
-      <c r="X138" s="31"/>
-      <c r="Y138" s="7"/>
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{810C905A-C0DA-4100-B6A9-F2260D80EA70}" scale="115">
-      <pane xSplit="2" ySplit="6" topLeftCell="Q101" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="B108" sqref="B108"/>
+    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="115">
+      <pane xSplit="2" ySplit="6" topLeftCell="Q19" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="Y37" sqref="Y37"/>
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+    </customSheetView>
+    <customSheetView guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" scale="115">
+      <pane xSplit="2" ySplit="6" topLeftCell="C58" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="D81" sqref="D81:X81"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
@@ -13155,21 +12679,9 @@
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
-    <customSheetView guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" scale="115">
-      <pane xSplit="2" ySplit="6" topLeftCell="C58" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="D81" sqref="D81:X81"/>
-      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-    </customSheetView>
-    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="115">
-      <pane xSplit="2" ySplit="6" topLeftCell="Q19" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="Y37" sqref="Y37"/>
-      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-    </customSheetView>
   </customSheetViews>
   <mergeCells count="6">
-    <mergeCell ref="Y110:Y111"/>
+    <mergeCell ref="Y108:Y109"/>
     <mergeCell ref="C1:O1"/>
     <mergeCell ref="C2:O2"/>
     <mergeCell ref="C5:H5"/>
@@ -13185,7 +12697,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E22"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="29.6640625" customWidth="1"/>
     <col min="2" max="2" width="28.33203125" customWidth="1"/>
@@ -13193,7 +12705,7 @@
     <col min="5" max="5" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="32" t="s">
         <v>237</v>
       </c>
@@ -13210,7 +12722,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="33" t="s">
         <v>242</v>
       </c>
@@ -13223,7 +12735,7 @@
       <c r="D2" s="34"/>
       <c r="E2" s="34"/>
     </row>
-    <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A3" s="33" t="s">
         <v>243</v>
       </c>
@@ -13236,7 +12748,7 @@
       <c r="D3" s="34"/>
       <c r="E3" s="34"/>
     </row>
-    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" s="33" t="s">
         <v>244</v>
       </c>
@@ -13249,7 +12761,7 @@
       <c r="D4" s="34"/>
       <c r="E4" s="34"/>
     </row>
-    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" s="33" t="s">
         <v>245</v>
       </c>
@@ -13264,7 +12776,7 @@
       </c>
       <c r="E5" s="34"/>
     </row>
-    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" s="33" t="s">
         <v>247</v>
       </c>
@@ -13279,7 +12791,7 @@
       </c>
       <c r="E6" s="34"/>
     </row>
-    <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A7" s="33" t="s">
         <v>248</v>
       </c>
@@ -13294,7 +12806,7 @@
       </c>
       <c r="E7" s="34"/>
     </row>
-    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="33" t="s">
         <v>249</v>
       </c>
@@ -13309,7 +12821,7 @@
       </c>
       <c r="E8" s="34"/>
     </row>
-    <row r="9" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A9" s="33" t="s">
         <v>250</v>
       </c>
@@ -13324,7 +12836,7 @@
       </c>
       <c r="E9" s="34"/>
     </row>
-    <row r="10" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A10" s="33" t="s">
         <v>252</v>
       </c>
@@ -13337,7 +12849,7 @@
       <c r="D10" s="34"/>
       <c r="E10" s="34"/>
     </row>
-    <row r="11" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A11" s="33" t="s">
         <v>253</v>
       </c>
@@ -13350,7 +12862,7 @@
       <c r="D11" s="34"/>
       <c r="E11" s="34"/>
     </row>
-    <row r="12" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A12" s="33" t="s">
         <v>254</v>
       </c>
@@ -13363,7 +12875,7 @@
       <c r="D12" s="34"/>
       <c r="E12" s="34"/>
     </row>
-    <row r="13" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A13" s="33" t="s">
         <v>255</v>
       </c>
@@ -13378,7 +12890,7 @@
       </c>
       <c r="E13" s="34"/>
     </row>
-    <row r="14" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" s="33" t="s">
         <v>256</v>
       </c>
@@ -13393,7 +12905,7 @@
       </c>
       <c r="E14" s="34"/>
     </row>
-    <row r="15" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A15" s="33" t="s">
         <v>257</v>
       </c>
@@ -13408,7 +12920,7 @@
       </c>
       <c r="E15" s="34"/>
     </row>
-    <row r="16" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A16" s="33" t="s">
         <v>258</v>
       </c>
@@ -13423,7 +12935,7 @@
       </c>
       <c r="E16" s="34"/>
     </row>
-    <row r="17" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A17" s="33" t="s">
         <v>259</v>
       </c>
@@ -13438,7 +12950,7 @@
       </c>
       <c r="E17" s="34"/>
     </row>
-    <row r="18" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A18" s="33" t="s">
         <v>260</v>
       </c>
@@ -13453,7 +12965,7 @@
       </c>
       <c r="E18" s="34"/>
     </row>
-    <row r="19" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A19" s="33" t="s">
         <v>261</v>
       </c>
@@ -13468,7 +12980,7 @@
       </c>
       <c r="E19" s="34"/>
     </row>
-    <row r="20" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A20" s="33" t="s">
         <v>262</v>
       </c>
@@ -13483,7 +12995,7 @@
       </c>
       <c r="E20" s="34"/>
     </row>
-    <row r="21" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A21" s="33" t="s">
         <v>33</v>
       </c>
@@ -13498,7 +13010,7 @@
       </c>
       <c r="E21" s="34"/>
     </row>
-    <row r="22" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A22" s="33" t="s">
         <v>263</v>
       </c>
@@ -13515,7 +13027,12 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{810C905A-C0DA-4100-B6A9-F2260D80EA70}" scale="150">
+    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="150">
+      <selection activeCell="A22" sqref="A22"/>
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+    </customSheetView>
+    <customSheetView guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" scale="150">
       <selection activeCell="A22" sqref="A22"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -13525,16 +13042,6 @@
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
-    <customSheetView guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" scale="150">
-      <selection activeCell="A22" sqref="A22"/>
-      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-    </customSheetView>
-    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="150">
-      <selection activeCell="A22" sqref="A22"/>
-      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-    </customSheetView>
   </customSheetViews>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Reapply "Muuta roolit.xlsx testiympäristöä varten"
This reverts commit f9027f22c931c173fd061de9184b945cf9c5008d.
</commit_message>
<xml_diff>
--- a/resources/roolit.xlsx
+++ b/resources/roolit.xlsx
@@ -1,46 +1,48 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lauri.nayha/Projects/harja/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\samuli\dev\harjaroot\harja\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:81_{A8790524-4076-984A-9AA0-56B44D9CB46B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:81_{C33009BB-AF4A-4311-9633-F3E6F0CC09C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="98860" yWindow="2380" windowWidth="34560" windowHeight="14920" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="23748" yWindow="156" windowWidth="25476" windowHeight="14232" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Oikeudet" sheetId="1" r:id="rId1"/>
     <sheet name="Roolit" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_1CE83972_B6A5_C44D_86E5_E9D9B38739F4_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_1DD617EE_F308_3E45_A8EF_4713F47FA0DD_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_2064F962_35EF_41F3_8A86_D37B72D177C7_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_3EBD3306_FC69_2148_8542_F6313DC2056F_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_47348D7B_5AFC_4A25_B239_A26E1359728E_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_476C495F_6E55_F04C_8145_4E8EBD6B3DE3_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_5327B0A1_A5FC_7747_93A1_427B210F3DF4_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_56F6E422_2CD8_6B4D_9E39_69A269028D26_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_6AA8E519_028C_D745_9E2E_8FB60E5B789F_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_7A9649F2_657F_9445_B6E6_FE94C6A09957_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_8411E1B5_4691_4435_A9A2_147FF80D0D98_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_843152D8_333A_1941_83E9_0CB5262068A2_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_87BEAE97_700C_BF40_B102_636C54D81F08_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_D01EF3E4_E485_4912_A9DA_396AAE5B8752_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_D57E2FB1_FF7F_8446_9C97_237A4D57F6BE_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_E3BBF62E_A283_4D48_98B7_21A2A94F634F_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$134</definedName>
-    <definedName name="Z_F86DF6F3_8AE5_3A44_B2D2_D623E01AE54F_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$134</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_1CE83972_B6A5_C44D_86E5_E9D9B38739F4_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_1DD617EE_F308_3E45_A8EF_4713F47FA0DD_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_2064F962_35EF_41F3_8A86_D37B72D177C7_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_3EBD3306_FC69_2148_8542_F6313DC2056F_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_47348D7B_5AFC_4A25_B239_A26E1359728E_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_476C495F_6E55_F04C_8145_4E8EBD6B3DE3_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_5327B0A1_A5FC_7747_93A1_427B210F3DF4_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_56F6E422_2CD8_6B4D_9E39_69A269028D26_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_6AA8E519_028C_D745_9E2E_8FB60E5B789F_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_7A9649F2_657F_9445_B6E6_FE94C6A09957_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_810C905A_C0DA_4100_B6A9_F2260D80EA70_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_8411E1B5_4691_4435_A9A2_147FF80D0D98_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_843152D8_333A_1941_83E9_0CB5262068A2_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_87BEAE97_700C_BF40_B102_636C54D81F08_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_D01EF3E4_E485_4912_A9DA_396AAE5B8752_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_D57E2FB1_FF7F_8446_9C97_237A4D57F6BE_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_E3BBF62E_A283_4D48_98B7_21A2A94F634F_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="Z_F86DF6F3_8AE5_3A44_B2D2_D623E01AE54F_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
   </definedNames>
   <calcPr calcId="0"/>
   <customWorkbookViews>
+    <customWorkbookView name="Samuli Taskila - Personal View" guid="{810C905A-C0DA-4100-B6A9-F2260D80EA70}" mergeInterval="0" personalView="1" xWindow="1979" yWindow="13" windowWidth="2123" windowHeight="1186" tabRatio="500" activeSheetId="1"/>
+    <customWorkbookView name="Microsoft Office User - Oma näkymä" guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" mergeInterval="0" personalView="1" xWindow="1440" yWindow="-515" windowWidth="2056" windowHeight="1366" tabRatio="500" activeSheetId="1"/>
+    <customWorkbookView name="Jarno Väyrynen - Personal View" guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" mergeInterval="0" personalView="1" xWindow="48" yWindow="25" windowWidth="2512" windowHeight="1336" tabRatio="500" activeSheetId="1"/>
     <customWorkbookView name="Microsoft Office User - Personal View" guid="{843152D8-333A-1941-83E9-0CB5262068A2}" mergeInterval="0" personalView="1" xWindow="4943" yWindow="119" windowWidth="1728" windowHeight="746" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Jarno Väyrynen - Personal View" guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" mergeInterval="0" personalView="1" xWindow="48" yWindow="25" windowWidth="2512" windowHeight="1336" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Microsoft Office User - Oma näkymä" guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" mergeInterval="0" personalView="1" xWindow="1440" yWindow="-515" windowWidth="2056" windowHeight="1366" tabRatio="500" activeSheetId="1"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -110,7 +112,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1947" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1989" uniqueCount="275">
   <si>
     <t xml:space="preserve">Roolimääritysten selitykset: </t>
   </si>
@@ -1001,6 +1003,12 @@
   </si>
   <si>
     <t>Koitetaan pärjätä yhdellä rivillä kaikkien välilehtien osalta</t>
+  </si>
+  <si>
+    <t>Tiemerkintä - Muut kustannukset</t>
+  </si>
+  <si>
+    <t>Tiemerkintä - Sakot ja bonukset</t>
   </si>
 </sst>
 </file>
@@ -1385,7 +1393,7 @@
 </file>
 
 <file path=xl/revisions/revisionHeaders.xml><?xml version="1.0" encoding="utf-8"?>
-<headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" guid="{16592C61-0221-A548-A820-56B21F0EE301}" diskRevisions="1" revisionId="224" version="13">
+<headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" guid="{4A6ED1B0-9135-4362-95CD-B6A2DDFC57B0}" diskRevisions="1" revisionId="269" version="14">
   <header guid="{8EBC2E30-8A6E-AD43-9F6F-B4500CF04203}" dateTime="2024-06-11T12:49:05" maxSheetId="3" userName="Jarno Väyrynen" r:id="rId9" minRId="87" maxRId="97">
     <sheetIdMap count="2">
       <sheetId val="1"/>
@@ -1440,6 +1448,12 @@
       <sheetId val="2"/>
     </sheetIdMap>
   </header>
+  <header guid="{4A6ED1B0-9135-4362-95CD-B6A2DDFC57B0}" dateTime="2025-04-02T11:13:06" maxSheetId="3" userName="Samuli Taskila" r:id="rId18" minRId="225" maxRId="268">
+    <sheetIdMap count="2">
+      <sheetId val="1"/>
+      <sheetId val="2"/>
+    </sheetIdMap>
+  </header>
 </headers>
 </file>
 
@@ -1471,6 +1485,335 @@
     <formula>Oikeudet!$A$5:$Y$128</formula>
   </rdn>
   <rcv guid="{843152D8-333A-1941-83E9-0CB5262068A2}" action="add"/>
+</revisions>
+</file>
+
+<file path=xl/revisions/revisionLog10.xml><?xml version="1.0" encoding="utf-8"?>
+<revisions xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <rrc rId="225" sId="1" ref="A107:XFD107" action="insertRow"/>
+  <rfmt sheetId="1" sqref="Y107" start="0" length="0">
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+  </rfmt>
+  <rcc rId="226" sId="1">
+    <nc r="A107" t="inlineStr">
+      <is>
+        <t>Raportit</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="227" sId="1">
+    <nc r="D107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="228" sId="1">
+    <nc r="E107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="229" sId="1">
+    <nc r="F107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="230" sId="1">
+    <nc r="G107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="231" sId="1">
+    <nc r="H107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="232" sId="1">
+    <nc r="I107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="233" sId="1">
+    <nc r="J107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="234" sId="1">
+    <nc r="K107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="235" sId="1">
+    <nc r="L107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="236" sId="1">
+    <nc r="M107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="237" sId="1">
+    <nc r="N107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="238" sId="1">
+    <nc r="P107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="239" sId="1">
+    <nc r="Q107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="240" sId="1">
+    <nc r="R107" t="inlineStr">
+      <is>
+        <t>R+</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="241" sId="1">
+    <nc r="S107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="242" sId="1">
+    <nc r="T107" t="inlineStr">
+      <is>
+        <t>R+</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="243" sId="1">
+    <nc r="U107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="244" sId="1">
+    <nc r="V107" t="inlineStr">
+      <is>
+        <t>R+</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="245" sId="1">
+    <nc r="X107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rfmt sheetId="1" sqref="Y107" start="0" length="0">
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+  </rfmt>
+  <rcc rId="246" sId="1">
+    <nc r="B107" t="inlineStr">
+      <is>
+        <t>Tiemerkintä - Muut kustannukset</t>
+      </is>
+    </nc>
+  </rcc>
+  <rrc rId="247" sId="1" ref="A107:XFD107" action="insertRow"/>
+  <rcc rId="248" sId="1">
+    <nc r="A107" t="inlineStr">
+      <is>
+        <t>Raportit</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="249" sId="1">
+    <nc r="D107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="250" sId="1">
+    <nc r="E107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="251" sId="1">
+    <nc r="F107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="252" sId="1">
+    <nc r="G107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="253" sId="1">
+    <nc r="H107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="254" sId="1">
+    <nc r="I107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="255" sId="1">
+    <nc r="J107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="256" sId="1">
+    <nc r="K107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="257" sId="1">
+    <nc r="L107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="258" sId="1">
+    <nc r="M107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="259" sId="1">
+    <nc r="N107" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="260" sId="1">
+    <nc r="P107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="261" sId="1">
+    <nc r="Q107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="262" sId="1">
+    <nc r="R107" t="inlineStr">
+      <is>
+        <t>R+</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="263" sId="1">
+    <nc r="S107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="264" sId="1">
+    <nc r="T107" t="inlineStr">
+      <is>
+        <t>R+</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="265" sId="1">
+    <nc r="U107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="266" sId="1">
+    <nc r="V107" t="inlineStr">
+      <is>
+        <t>R+</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="267" sId="1">
+    <nc r="X107" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="268" sId="1">
+    <nc r="B107" t="inlineStr">
+      <is>
+        <t>Tiemerkintä - Sakot ja bonukset</t>
+      </is>
+    </nc>
+  </rcc>
+  <rdn rId="0" localSheetId="1" customView="1" name="Z_810C905A_C0DA_4100_B6A9_F2260D80EA70_.wvu.FilterData" hidden="1" oldHidden="1">
+    <formula>Oikeudet!$A$5:$Y$136</formula>
+  </rdn>
+  <rcv guid="{810C905A-C0DA-4100-B6A9-F2260D80EA70}" action="add"/>
 </revisions>
 </file>
 
@@ -5137,11 +5480,12 @@
 </file>
 
 <file path=xl/revisions/userNames.xml><?xml version="1.0" encoding="utf-8"?>
-<users xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" count="4">
+<users xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" count="5">
   <userInfo guid="{8EBC2E30-8A6E-AD43-9F6F-B4500CF04203}" name="Jarno Väyrynen" id="-589133089" dateTime="2024-06-10T14:55:26"/>
   <userInfo guid="{CFB45395-62D4-124C-9898-DEF874662F1B}" name="Microsoft Office User" id="-296973103" dateTime="2024-11-20T15:04:38"/>
   <userInfo guid="{CF3F0B66-D3D6-2C4C-93DF-DEE3169712D4}" name="Microsoft Office User" id="-296992802" dateTime="2024-12-13T10:34:14"/>
   <userInfo guid="{64AC07D8-8D49-4F46-96EF-A9E3AD0E8431}" name="Jarno Väyrynen" id="-589128654" dateTime="2025-02-12T12:58:37"/>
+  <userInfo guid="{4A6ED1B0-9135-4362-95CD-B6A2DDFC57B0}" name="Samuli Taskila" id="-1631752395" dateTime="2025-04-02T11:10:08"/>
 </users>
 </file>
 
@@ -5321,12 +5665,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y136"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <dimension ref="A1:Y138"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="31.6640625" customWidth="1"/>
-    <col min="3" max="3" width="14.1640625" customWidth="1"/>
+    <col min="3" max="3" width="14.109375" customWidth="1"/>
     <col min="4" max="4" width="30.33203125" customWidth="1"/>
     <col min="5" max="5" width="26.33203125" customWidth="1"/>
     <col min="6" max="6" width="12.6640625" customWidth="1"/>
@@ -5335,22 +5679,22 @@
     <col min="9" max="9" width="18.33203125" customWidth="1"/>
     <col min="10" max="10" width="25.33203125" customWidth="1"/>
     <col min="11" max="11" width="40.6640625" customWidth="1"/>
-    <col min="12" max="12" width="38.1640625" customWidth="1"/>
+    <col min="12" max="12" width="38.109375" customWidth="1"/>
     <col min="13" max="13" width="12.33203125" customWidth="1"/>
     <col min="14" max="14" width="10.6640625" customWidth="1"/>
-    <col min="15" max="16" width="12.5" customWidth="1"/>
+    <col min="15" max="16" width="12.44140625" customWidth="1"/>
     <col min="17" max="17" width="21.6640625" customWidth="1"/>
     <col min="18" max="18" width="36" customWidth="1"/>
     <col min="19" max="19" width="29.6640625" customWidth="1"/>
     <col min="20" max="20" width="15" customWidth="1"/>
     <col min="21" max="21" width="17.6640625" customWidth="1"/>
-    <col min="22" max="22" width="11.5" customWidth="1"/>
+    <col min="22" max="22" width="11.44140625" customWidth="1"/>
     <col min="23" max="23" width="11.6640625" customWidth="1"/>
     <col min="24" max="24" width="11.33203125" customWidth="1"/>
     <col min="25" max="25" width="59" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="24" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:25" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -5371,7 +5715,7 @@
       <c r="N1" s="36"/>
       <c r="O1" s="36"/>
     </row>
-    <row r="2" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="37" t="s">
@@ -5390,7 +5734,7 @@
       <c r="N2" s="37"/>
       <c r="O2" s="37"/>
     </row>
-    <row r="3" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3" s="2" t="s">
         <v>3</v>
@@ -5405,10 +5749,10 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C4" s="6"/>
     </row>
-    <row r="5" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7"/>
       <c r="B5" s="7"/>
       <c r="C5" s="38" t="s">
@@ -5443,7 +5787,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>11</v>
       </c>
@@ -5516,7 +5860,7 @@
       </c>
       <c r="Y6" s="7"/>
     </row>
-    <row r="7" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>34</v>
       </c>
@@ -5589,7 +5933,7 @@
       </c>
       <c r="Y7" s="13"/>
     </row>
-    <row r="8" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>34</v>
       </c>
@@ -5648,7 +5992,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>34</v>
       </c>
@@ -5701,7 +6045,7 @@
       <c r="X9" s="12"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>34</v>
       </c>
@@ -5754,7 +6098,7 @@
       <c r="X10" s="12"/>
       <c r="Y10" s="13"/>
     </row>
-    <row r="11" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
         <v>34</v>
       </c>
@@ -5813,7 +6157,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>34</v>
       </c>
@@ -5866,7 +6210,7 @@
       <c r="X12" s="12"/>
       <c r="Y12" s="13"/>
     </row>
-    <row r="13" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
         <v>34</v>
       </c>
@@ -5933,7 +6277,7 @@
       <c r="X13" s="12"/>
       <c r="Y13" s="13"/>
     </row>
-    <row r="14" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
         <v>34</v>
       </c>
@@ -6000,7 +6344,7 @@
       <c r="X14" s="12"/>
       <c r="Y14" s="13"/>
     </row>
-    <row r="15" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
         <v>34</v>
       </c>
@@ -6057,7 +6401,7 @@
       <c r="X15" s="12"/>
       <c r="Y15" s="13"/>
     </row>
-    <row r="16" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
         <v>34</v>
       </c>
@@ -6114,7 +6458,7 @@
       <c r="X16" s="12"/>
       <c r="Y16" s="13"/>
     </row>
-    <row r="17" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
         <v>34</v>
       </c>
@@ -6171,7 +6515,7 @@
       <c r="X17" s="12"/>
       <c r="Y17" s="13"/>
     </row>
-    <row r="18" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
         <v>34</v>
       </c>
@@ -6238,7 +6582,7 @@
       <c r="X18" s="12"/>
       <c r="Y18" s="13"/>
     </row>
-    <row r="19" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
         <v>34</v>
       </c>
@@ -6305,7 +6649,7 @@
       <c r="X19" s="12"/>
       <c r="Y19" s="13"/>
     </row>
-    <row r="20" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
         <v>34</v>
       </c>
@@ -6360,7 +6704,7 @@
       <c r="X20" s="12"/>
       <c r="Y20" s="13"/>
     </row>
-    <row r="21" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
         <v>34</v>
       </c>
@@ -6421,7 +6765,7 @@
       <c r="X21" s="12"/>
       <c r="Y21" s="13"/>
     </row>
-    <row r="22" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
         <v>34</v>
       </c>
@@ -6488,7 +6832,7 @@
       <c r="X22" s="12"/>
       <c r="Y22" s="13"/>
     </row>
-    <row r="23" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
         <v>34</v>
       </c>
@@ -6561,7 +6905,7 @@
       </c>
       <c r="Y23" s="13"/>
     </row>
-    <row r="24" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
         <v>34</v>
       </c>
@@ -6634,7 +6978,7 @@
       </c>
       <c r="Y24" s="13"/>
     </row>
-    <row r="25" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
         <v>34</v>
       </c>
@@ -6707,7 +7051,7 @@
       </c>
       <c r="Y25" s="13"/>
     </row>
-    <row r="26" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
         <v>34</v>
       </c>
@@ -6778,7 +7122,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="27" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
         <v>34</v>
       </c>
@@ -6847,7 +7191,7 @@
       <c r="X27" s="12"/>
       <c r="Y27" s="13"/>
     </row>
-    <row r="28" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
         <v>34</v>
       </c>
@@ -6893,7 +7237,7 @@
       </c>
       <c r="Y28" s="13"/>
     </row>
-    <row r="29" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
         <v>34</v>
       </c>
@@ -6962,7 +7306,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="30" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
         <v>34</v>
       </c>
@@ -7023,7 +7367,7 @@
       <c r="X30" s="12"/>
       <c r="Y30" s="13"/>
     </row>
-    <row r="31" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="11" t="s">
         <v>34</v>
       </c>
@@ -7080,7 +7424,7 @@
       <c r="X31" s="12"/>
       <c r="Y31" s="13"/>
     </row>
-    <row r="32" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
         <v>34</v>
       </c>
@@ -7133,7 +7477,7 @@
       <c r="X32" s="12"/>
       <c r="Y32" s="13"/>
     </row>
-    <row r="33" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="11" t="s">
         <v>34</v>
       </c>
@@ -7178,7 +7522,7 @@
       <c r="X33" s="12"/>
       <c r="Y33" s="13"/>
     </row>
-    <row r="34" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="34" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="17" t="s">
         <v>34</v>
       </c>
@@ -7207,7 +7551,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="35" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="11" t="s">
         <v>34</v>
       </c>
@@ -7254,7 +7598,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="36" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
         <v>34</v>
       </c>
@@ -7311,7 +7655,7 @@
       </c>
       <c r="Y36" s="13"/>
     </row>
-    <row r="37" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="11" t="s">
         <v>34</v>
       </c>
@@ -7368,7 +7712,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="38" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="38" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="11" t="s">
         <v>34</v>
       </c>
@@ -7421,7 +7765,7 @@
       <c r="X38" s="12"/>
       <c r="Y38" s="13"/>
     </row>
-    <row r="39" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="11" t="s">
         <v>34</v>
       </c>
@@ -7490,7 +7834,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="40" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="40" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
         <v>34</v>
       </c>
@@ -7553,7 +7897,7 @@
       <c r="X40" s="12"/>
       <c r="Y40" s="13"/>
     </row>
-    <row r="41" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="41" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="11" t="s">
         <v>34</v>
       </c>
@@ -7618,7 +7962,7 @@
       <c r="X41" s="12"/>
       <c r="Y41" s="13"/>
     </row>
-    <row r="42" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="42" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="11" t="s">
         <v>34</v>
       </c>
@@ -7681,7 +8025,7 @@
       <c r="X42" s="12"/>
       <c r="Y42" s="13"/>
     </row>
-    <row r="43" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="43" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="11" t="s">
         <v>34</v>
       </c>
@@ -7744,7 +8088,7 @@
       <c r="X43" s="12"/>
       <c r="Y43" s="13"/>
     </row>
-    <row r="44" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="44" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="11" t="s">
         <v>34</v>
       </c>
@@ -7807,7 +8151,7 @@
       <c r="X44" s="12"/>
       <c r="Y44" s="13"/>
     </row>
-    <row r="45" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="45" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="11" t="s">
         <v>34</v>
       </c>
@@ -7870,7 +8214,7 @@
       <c r="X45" s="12"/>
       <c r="Y45" s="7"/>
     </row>
-    <row r="46" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="46" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="11" t="s">
         <v>34</v>
       </c>
@@ -7933,7 +8277,7 @@
       <c r="X46" s="12"/>
       <c r="Y46" s="7"/>
     </row>
-    <row r="47" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="47" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="11" t="s">
         <v>34</v>
       </c>
@@ -7996,7 +8340,7 @@
       <c r="X47" s="12"/>
       <c r="Y47" s="7"/>
     </row>
-    <row r="48" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="48" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="11" t="s">
         <v>34</v>
       </c>
@@ -8069,7 +8413,7 @@
       </c>
       <c r="Y48" s="13"/>
     </row>
-    <row r="49" spans="1:25" ht="28" x14ac:dyDescent="0.15">
+    <row r="49" spans="1:25" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A49" s="11" t="s">
         <v>34</v>
       </c>
@@ -8122,7 +8466,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="50" spans="1:25" ht="70" x14ac:dyDescent="0.15">
+    <row r="50" spans="1:25" ht="66" x14ac:dyDescent="0.25">
       <c r="A50" s="11" t="s">
         <v>34</v>
       </c>
@@ -8175,7 +8519,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="51" spans="1:25" x14ac:dyDescent="0.15">
+    <row r="51" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A51" s="11" t="s">
         <v>34</v>
       </c>
@@ -8226,7 +8570,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="52" spans="1:25" ht="14" x14ac:dyDescent="0.15">
+    <row r="52" spans="1:25" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A52" s="11" t="s">
         <v>34</v>
       </c>
@@ -8275,7 +8619,7 @@
       <c r="X52" s="15"/>
       <c r="Y52" s="7"/>
     </row>
-    <row r="53" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="53" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="17" t="s">
         <v>34</v>
       </c>
@@ -8326,7 +8670,7 @@
       <c r="W53" s="22"/>
       <c r="X53" s="22"/>
     </row>
-    <row r="54" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="54" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11" t="s">
         <v>34</v>
       </c>
@@ -8375,7 +8719,7 @@
       <c r="X54" s="15"/>
       <c r="Y54" s="13"/>
     </row>
-    <row r="55" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="55" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="11" t="s">
         <v>34</v>
       </c>
@@ -8408,7 +8752,7 @@
       <c r="X55" s="12"/>
       <c r="Y55" s="13"/>
     </row>
-    <row r="56" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="56" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="11" t="s">
         <v>34</v>
       </c>
@@ -8461,7 +8805,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="57" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="57" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="11" t="s">
         <v>34</v>
       </c>
@@ -8494,7 +8838,7 @@
       <c r="X57" s="12"/>
       <c r="Y57" s="13"/>
     </row>
-    <row r="58" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="58" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="11" t="s">
         <v>34</v>
       </c>
@@ -8545,7 +8889,7 @@
       <c r="X58" s="12"/>
       <c r="Y58" s="13"/>
     </row>
-    <row r="59" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="59" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="11" t="s">
         <v>34</v>
       </c>
@@ -8608,7 +8952,7 @@
       <c r="X59" s="12"/>
       <c r="Y59" s="13"/>
     </row>
-    <row r="60" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="60" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="23" t="s">
         <v>34</v>
       </c>
@@ -8667,7 +9011,7 @@
       <c r="X60" s="12"/>
       <c r="Y60" s="13"/>
     </row>
-    <row r="61" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="61" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="23" t="s">
         <v>34</v>
       </c>
@@ -8728,7 +9072,7 @@
       <c r="X61" s="12"/>
       <c r="Y61" s="13"/>
     </row>
-    <row r="62" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="62" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="23" t="s">
         <v>34</v>
       </c>
@@ -8783,7 +9127,7 @@
       <c r="X62" s="12"/>
       <c r="Y62" s="13"/>
     </row>
-    <row r="63" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="63" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="11" t="s">
         <v>34</v>
       </c>
@@ -8856,7 +9200,7 @@
       </c>
       <c r="Y63" s="13"/>
     </row>
-    <row r="64" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="64" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="11" t="s">
         <v>160</v>
       </c>
@@ -8909,7 +9253,7 @@
       <c r="X64" s="12"/>
       <c r="Y64" s="13"/>
     </row>
-    <row r="65" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="65" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="11" t="s">
         <v>160</v>
       </c>
@@ -8962,7 +9306,7 @@
       <c r="X65" s="12"/>
       <c r="Y65" s="13"/>
     </row>
-    <row r="66" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="66" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="11" t="s">
         <v>160</v>
       </c>
@@ -9015,7 +9359,7 @@
       <c r="X66" s="12"/>
       <c r="Y66" s="13"/>
     </row>
-    <row r="67" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="67" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="11" t="s">
         <v>160</v>
       </c>
@@ -9068,7 +9412,7 @@
       <c r="X67" s="12"/>
       <c r="Y67" s="13"/>
     </row>
-    <row r="68" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="68" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="11" t="s">
         <v>160</v>
       </c>
@@ -9115,7 +9459,7 @@
       <c r="X68" s="12"/>
       <c r="Y68" s="13"/>
     </row>
-    <row r="69" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="69" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="11" t="s">
         <v>160</v>
       </c>
@@ -9168,7 +9512,7 @@
       <c r="X69" s="12"/>
       <c r="Y69" s="13"/>
     </row>
-    <row r="70" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="70" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="11" t="s">
         <v>160</v>
       </c>
@@ -9221,7 +9565,7 @@
       <c r="X70" s="12"/>
       <c r="Y70" s="13"/>
     </row>
-    <row r="71" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="71" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="11" t="s">
         <v>160</v>
       </c>
@@ -9274,7 +9618,7 @@
       <c r="X71" s="12"/>
       <c r="Y71" s="13"/>
     </row>
-    <row r="72" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="72" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="11" t="s">
         <v>160</v>
       </c>
@@ -9327,7 +9671,7 @@
       <c r="X72" s="12"/>
       <c r="Y72" s="13"/>
     </row>
-    <row r="73" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="73" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="11" t="s">
         <v>160</v>
       </c>
@@ -9362,7 +9706,7 @@
       <c r="X73" s="12"/>
       <c r="Y73" s="13"/>
     </row>
-    <row r="74" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="74" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="11" t="s">
         <v>160</v>
       </c>
@@ -9433,7 +9777,7 @@
       </c>
       <c r="Y74" s="13"/>
     </row>
-    <row r="75" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="75" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="11" t="s">
         <v>160</v>
       </c>
@@ -9506,7 +9850,7 @@
       </c>
       <c r="Y75" s="13"/>
     </row>
-    <row r="76" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="76" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="11" t="s">
         <v>160</v>
       </c>
@@ -9577,7 +9921,7 @@
       </c>
       <c r="Y76" s="13"/>
     </row>
-    <row r="77" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="77" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="11" t="s">
         <v>160</v>
       </c>
@@ -9648,7 +9992,7 @@
       </c>
       <c r="Y77" s="13"/>
     </row>
-    <row r="78" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="78" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="11" t="s">
         <v>160</v>
       </c>
@@ -9683,7 +10027,7 @@
       <c r="X78" s="12"/>
       <c r="Y78" s="13"/>
     </row>
-    <row r="79" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="79" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="11" t="s">
         <v>160</v>
       </c>
@@ -9754,7 +10098,7 @@
       </c>
       <c r="Y79" s="13"/>
     </row>
-    <row r="80" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="80" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="11" t="s">
         <v>160</v>
       </c>
@@ -9825,7 +10169,7 @@
       </c>
       <c r="Y80" s="13"/>
     </row>
-    <row r="81" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="81" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="11" t="s">
         <v>160</v>
       </c>
@@ -9894,7 +10238,7 @@
       </c>
       <c r="Y81" s="13"/>
     </row>
-    <row r="82" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="82" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="11" t="s">
         <v>160</v>
       </c>
@@ -9965,7 +10309,7 @@
       </c>
       <c r="Y82" s="13"/>
     </row>
-    <row r="83" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="83" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="11" t="s">
         <v>160</v>
       </c>
@@ -10028,7 +10372,7 @@
       </c>
       <c r="Y83" s="13"/>
     </row>
-    <row r="84" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="84" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="11" t="s">
         <v>160</v>
       </c>
@@ -10085,7 +10429,7 @@
       <c r="X84" s="12"/>
       <c r="Y84" s="13"/>
     </row>
-    <row r="85" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="85" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="11" t="s">
         <v>160</v>
       </c>
@@ -10120,7 +10464,7 @@
       <c r="X85" s="12"/>
       <c r="Y85" s="13"/>
     </row>
-    <row r="86" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="86" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="11" t="s">
         <v>160</v>
       </c>
@@ -10155,7 +10499,7 @@
       <c r="X86" s="12"/>
       <c r="Y86" s="13"/>
     </row>
-    <row r="87" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="87" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="11" t="s">
         <v>160</v>
       </c>
@@ -10190,7 +10534,7 @@
       <c r="X87" s="12"/>
       <c r="Y87" s="13"/>
     </row>
-    <row r="88" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="88" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="11" t="s">
         <v>160</v>
       </c>
@@ -10259,7 +10603,7 @@
       </c>
       <c r="Y88" s="13"/>
     </row>
-    <row r="89" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="89" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="11" t="s">
         <v>160</v>
       </c>
@@ -10328,7 +10672,7 @@
       </c>
       <c r="Y89" s="13"/>
     </row>
-    <row r="90" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="90" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="11" t="s">
         <v>160</v>
       </c>
@@ -10399,7 +10743,7 @@
       </c>
       <c r="Y90" s="13"/>
     </row>
-    <row r="91" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="91" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="11" t="s">
         <v>160</v>
       </c>
@@ -10468,7 +10812,7 @@
       <c r="X91" s="12"/>
       <c r="Y91" s="13"/>
     </row>
-    <row r="92" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="92" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="11" t="s">
         <v>160</v>
       </c>
@@ -10537,7 +10881,7 @@
       <c r="X92" s="12"/>
       <c r="Y92" s="13"/>
     </row>
-    <row r="93" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="93" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="11" t="s">
         <v>160</v>
       </c>
@@ -10606,7 +10950,7 @@
       <c r="X93" s="12"/>
       <c r="Y93" s="13"/>
     </row>
-    <row r="94" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="94" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="11" t="s">
         <v>160</v>
       </c>
@@ -10675,7 +11019,7 @@
       <c r="X94" s="12"/>
       <c r="Y94" s="13"/>
     </row>
-    <row r="95" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="95" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="11" t="s">
         <v>160</v>
       </c>
@@ -10744,7 +11088,7 @@
       <c r="X95" s="12"/>
       <c r="Y95" s="13"/>
     </row>
-    <row r="96" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="96" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="11" t="s">
         <v>160</v>
       </c>
@@ -10779,7 +11123,7 @@
       <c r="X96" s="12"/>
       <c r="Y96" s="13"/>
     </row>
-    <row r="97" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="97" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="11" t="s">
         <v>160</v>
       </c>
@@ -10848,7 +11192,7 @@
       <c r="X97" s="12"/>
       <c r="Y97" s="13"/>
     </row>
-    <row r="98" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="98" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="11" t="s">
         <v>160</v>
       </c>
@@ -10901,7 +11245,7 @@
       <c r="X98" s="12"/>
       <c r="Y98" s="13"/>
     </row>
-    <row r="99" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="99" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="11" t="s">
         <v>160</v>
       </c>
@@ -10974,7 +11318,7 @@
       </c>
       <c r="Y99" s="13"/>
     </row>
-    <row r="100" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="100" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="11" t="s">
         <v>160</v>
       </c>
@@ -11047,7 +11391,7 @@
       </c>
       <c r="Y100" s="13"/>
     </row>
-    <row r="101" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="101" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="11" t="s">
         <v>160</v>
       </c>
@@ -11120,7 +11464,7 @@
       </c>
       <c r="Y101" s="13"/>
     </row>
-    <row r="102" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="102" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="11" t="s">
         <v>160</v>
       </c>
@@ -11191,7 +11535,7 @@
       </c>
       <c r="Y102" s="13"/>
     </row>
-    <row r="103" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="103" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="11" t="s">
         <v>160</v>
       </c>
@@ -11224,7 +11568,7 @@
       <c r="X103" s="12"/>
       <c r="Y103" s="13"/>
     </row>
-    <row r="104" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="104" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="11" t="s">
         <v>160</v>
       </c>
@@ -11295,7 +11639,7 @@
       </c>
       <c r="Y104" s="13"/>
     </row>
-    <row r="105" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="105" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="11" t="s">
         <v>160</v>
       </c>
@@ -11368,7 +11712,7 @@
       </c>
       <c r="Y105" s="13"/>
     </row>
-    <row r="106" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="106" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="11" t="s">
         <v>160</v>
       </c>
@@ -11441,34 +11785,40 @@
       </c>
       <c r="Y106" s="13"/>
     </row>
-    <row r="107" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="107" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="11" t="s">
         <v>160</v>
       </c>
       <c r="B107" s="11" t="s">
-        <v>200</v>
+        <v>274</v>
       </c>
       <c r="C107" s="12"/>
       <c r="D107" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E107" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F107" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G107" s="12"/>
-      <c r="H107" s="12"/>
-      <c r="I107" s="12"/>
+      <c r="G107" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="H107" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I107" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="J107" s="12" t="s">
         <v>39</v>
       </c>
       <c r="K107" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="L107" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="M107" s="12" t="s">
         <v>39</v>
@@ -11477,33 +11827,39 @@
         <v>38</v>
       </c>
       <c r="O107" s="12"/>
-      <c r="P107" s="12"/>
+      <c r="P107" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="Q107" s="12" t="s">
         <v>39</v>
       </c>
       <c r="R107" s="12" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="S107" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="T107" s="12"/>
+        <v>39</v>
+      </c>
+      <c r="T107" s="12" t="s">
+        <v>44</v>
+      </c>
       <c r="U107" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="V107" s="12" t="s">
         <v>44</v>
       </c>
       <c r="W107" s="12"/>
-      <c r="X107" s="12"/>
+      <c r="X107" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="Y107" s="13"/>
     </row>
-    <row r="108" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="108" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="11" t="s">
-        <v>201</v>
+        <v>160</v>
       </c>
       <c r="B108" s="11" t="s">
-        <v>202</v>
+        <v>273</v>
       </c>
       <c r="C108" s="12"/>
       <c r="D108" s="12" t="s">
@@ -11525,7 +11881,7 @@
         <v>39</v>
       </c>
       <c r="J108" s="12" t="s">
-        <v>203</v>
+        <v>39</v>
       </c>
       <c r="K108" s="12" t="s">
         <v>38</v>
@@ -11539,20 +11895,18 @@
       <c r="N108" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="O108" s="12" t="s">
-        <v>38</v>
-      </c>
+      <c r="O108" s="12"/>
       <c r="P108" s="12" t="s">
         <v>39</v>
       </c>
       <c r="Q108" s="12" t="s">
-        <v>203</v>
+        <v>39</v>
       </c>
       <c r="R108" s="12" t="s">
-        <v>204</v>
+        <v>44</v>
       </c>
       <c r="S108" s="12" t="s">
-        <v>203</v>
+        <v>39</v>
       </c>
       <c r="T108" s="12" t="s">
         <v>44</v>
@@ -11563,50 +11917,40 @@
       <c r="V108" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="W108" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="W108" s="12"/>
       <c r="X108" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="Y108" s="35" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="109" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="Y108" s="13"/>
+    </row>
+    <row r="109" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="11" t="s">
-        <v>201</v>
+        <v>160</v>
       </c>
       <c r="B109" s="11" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="C109" s="12"/>
       <c r="D109" s="12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E109" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F109" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G109" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="H109" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="I109" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="G109" s="12"/>
+      <c r="H109" s="12"/>
+      <c r="I109" s="12"/>
       <c r="J109" s="12" t="s">
-        <v>203</v>
+        <v>39</v>
       </c>
       <c r="K109" s="12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="L109" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="M109" s="12" t="s">
         <v>39</v>
@@ -11614,48 +11958,38 @@
       <c r="N109" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="O109" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="P109" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="O109" s="12"/>
+      <c r="P109" s="12"/>
       <c r="Q109" s="12" t="s">
-        <v>203</v>
+        <v>39</v>
       </c>
       <c r="R109" s="12" t="s">
-        <v>204</v>
+        <v>42</v>
       </c>
       <c r="S109" s="12" t="s">
-        <v>203</v>
-      </c>
-      <c r="T109" s="12" t="s">
-        <v>44</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="T109" s="12"/>
       <c r="U109" s="12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="V109" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="W109" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="X109" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y109" s="35"/>
-    </row>
-    <row r="110" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="W109" s="12"/>
+      <c r="X109" s="12"/>
+      <c r="Y109" s="13"/>
+    </row>
+    <row r="110" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="11" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="B110" s="11" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="C110" s="12"/>
       <c r="D110" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E110" s="12" t="s">
         <v>38</v>
@@ -11673,10 +12007,10 @@
         <v>39</v>
       </c>
       <c r="J110" s="12" t="s">
-        <v>39</v>
+        <v>203</v>
       </c>
       <c r="K110" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="L110" s="12" t="s">
         <v>38</v>
@@ -11694,41 +12028,43 @@
         <v>39</v>
       </c>
       <c r="Q110" s="12" t="s">
-        <v>39</v>
+        <v>203</v>
       </c>
       <c r="R110" s="12" t="s">
-        <v>42</v>
+        <v>204</v>
       </c>
       <c r="S110" s="12" t="s">
-        <v>40</v>
+        <v>203</v>
       </c>
       <c r="T110" s="12" t="s">
         <v>44</v>
       </c>
       <c r="U110" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="V110" s="12" t="s">
         <v>44</v>
       </c>
       <c r="W110" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="X110" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y110" s="7"/>
-    </row>
-    <row r="111" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>39</v>
+      </c>
+      <c r="Y110" s="35" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="111" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="11" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B111" s="11" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="C111" s="12"/>
       <c r="D111" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E111" s="12" t="s">
         <v>38</v>
@@ -11746,10 +12082,10 @@
         <v>39</v>
       </c>
       <c r="J111" s="12" t="s">
-        <v>39</v>
+        <v>203</v>
       </c>
       <c r="K111" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="L111" s="12" t="s">
         <v>38</v>
@@ -11767,166 +12103,246 @@
         <v>39</v>
       </c>
       <c r="Q111" s="12" t="s">
-        <v>39</v>
+        <v>203</v>
       </c>
       <c r="R111" s="12" t="s">
-        <v>42</v>
+        <v>204</v>
       </c>
       <c r="S111" s="12" t="s">
-        <v>40</v>
+        <v>203</v>
       </c>
       <c r="T111" s="12" t="s">
         <v>44</v>
       </c>
       <c r="U111" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="V111" s="12" t="s">
         <v>44</v>
       </c>
       <c r="W111" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="X111" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y111" s="13"/>
-    </row>
-    <row r="112" spans="1:25" s="30" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A112" s="27" t="s">
-        <v>209</v>
-      </c>
-      <c r="B112" s="27" t="s">
-        <v>210</v>
-      </c>
-      <c r="C112" s="28"/>
+        <v>39</v>
+      </c>
+      <c r="Y111" s="35"/>
+    </row>
+    <row r="112" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A112" s="11" t="s">
+        <v>207</v>
+      </c>
+      <c r="B112" s="11" t="s">
+        <v>208</v>
+      </c>
+      <c r="C112" s="12"/>
       <c r="D112" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E112" s="28"/>
-      <c r="F112" s="28"/>
-      <c r="G112" s="28"/>
-      <c r="H112" s="28"/>
-      <c r="I112" s="28"/>
-      <c r="J112" s="28"/>
-      <c r="K112" s="28"/>
-      <c r="L112" s="28"/>
-      <c r="M112" s="28"/>
-      <c r="N112" s="28"/>
-      <c r="O112" s="28"/>
-      <c r="P112" s="28"/>
-      <c r="Q112" s="28"/>
-      <c r="R112" s="28"/>
-      <c r="S112" s="28"/>
-      <c r="T112" s="28"/>
-      <c r="U112" s="28"/>
-      <c r="V112" s="28"/>
-      <c r="W112" s="28"/>
-      <c r="X112" s="28"/>
-      <c r="Y112" s="29" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="113" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E112" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F112" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="G112" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="H112" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I112" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="J112" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="K112" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="L112" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="M112" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="N112" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="O112" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="P112" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q112" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="R112" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="S112" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="T112" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="U112" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="V112" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="W112" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="X112" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="Y112" s="7"/>
+    </row>
+    <row r="113" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="11" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="B113" s="11" t="s">
-        <v>212</v>
+        <v>199</v>
       </c>
       <c r="C113" s="12"/>
       <c r="D113" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E113" s="12"/>
+      <c r="E113" s="12" t="s">
+        <v>38</v>
+      </c>
       <c r="F113" s="12" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="G113" s="12" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="H113" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="I113" s="12"/>
-      <c r="J113" s="12"/>
-      <c r="K113" s="12"/>
-      <c r="L113" s="12"/>
+        <v>38</v>
+      </c>
+      <c r="I113" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="J113" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="K113" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="L113" s="12" t="s">
+        <v>38</v>
+      </c>
       <c r="M113" s="12" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="N113" s="12" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="O113" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="P113" s="12"/>
-      <c r="Q113" s="12"/>
-      <c r="R113" s="12"/>
-      <c r="S113" s="12"/>
-      <c r="T113" s="12"/>
-      <c r="U113" s="12"/>
-      <c r="V113" s="12"/>
-      <c r="W113" s="12"/>
-      <c r="X113" s="12"/>
-      <c r="Y113" s="7"/>
-    </row>
-    <row r="114" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A114" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="P113" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q113" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="R113" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="S113" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="T113" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="U113" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="V113" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="W113" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="X113" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="Y113" s="13"/>
+    </row>
+    <row r="114" spans="1:25" s="30" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A114" s="27" t="s">
         <v>209</v>
       </c>
-      <c r="B114" s="11" t="s">
-        <v>213</v>
-      </c>
-      <c r="C114" s="12"/>
+      <c r="B114" s="27" t="s">
+        <v>210</v>
+      </c>
+      <c r="C114" s="28"/>
       <c r="D114" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E114" s="12"/>
-      <c r="F114" s="12"/>
-      <c r="G114" s="12"/>
-      <c r="H114" s="12"/>
-      <c r="I114" s="12"/>
-      <c r="J114" s="12"/>
-      <c r="K114" s="12"/>
-      <c r="L114" s="12"/>
-      <c r="M114" s="12"/>
-      <c r="N114" s="12"/>
-      <c r="O114" s="12"/>
-      <c r="P114" s="12"/>
-      <c r="Q114" s="12"/>
-      <c r="R114" s="12"/>
-      <c r="S114" s="12"/>
-      <c r="T114" s="12"/>
-      <c r="U114" s="12"/>
-      <c r="V114" s="12"/>
-      <c r="W114" s="12"/>
-      <c r="X114" s="12"/>
-      <c r="Y114" s="7"/>
-    </row>
-    <row r="115" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E114" s="28"/>
+      <c r="F114" s="28"/>
+      <c r="G114" s="28"/>
+      <c r="H114" s="28"/>
+      <c r="I114" s="28"/>
+      <c r="J114" s="28"/>
+      <c r="K114" s="28"/>
+      <c r="L114" s="28"/>
+      <c r="M114" s="28"/>
+      <c r="N114" s="28"/>
+      <c r="O114" s="28"/>
+      <c r="P114" s="28"/>
+      <c r="Q114" s="28"/>
+      <c r="R114" s="28"/>
+      <c r="S114" s="28"/>
+      <c r="T114" s="28"/>
+      <c r="U114" s="28"/>
+      <c r="V114" s="28"/>
+      <c r="W114" s="28"/>
+      <c r="X114" s="28"/>
+      <c r="Y114" s="29" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="115" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B115" s="11" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C115" s="12"/>
       <c r="D115" s="12" t="s">
         <v>41</v>
       </c>
       <c r="E115" s="12"/>
-      <c r="F115" s="12"/>
-      <c r="G115" s="12"/>
-      <c r="H115" s="12"/>
+      <c r="F115" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="G115" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="H115" s="12" t="s">
+        <v>46</v>
+      </c>
       <c r="I115" s="12"/>
       <c r="J115" s="12"/>
       <c r="K115" s="12"/>
       <c r="L115" s="12"/>
-      <c r="M115" s="12"/>
-      <c r="N115" s="12"/>
-      <c r="O115" s="12"/>
+      <c r="M115" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="N115" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="O115" s="12" t="s">
+        <v>46</v>
+      </c>
       <c r="P115" s="12"/>
       <c r="Q115" s="12"/>
       <c r="R115" s="12"/>
@@ -11938,12 +12354,12 @@
       <c r="X115" s="12"/>
       <c r="Y115" s="7"/>
     </row>
-    <row r="116" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="116" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B116" s="11" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C116" s="12"/>
       <c r="D116" s="12" t="s">
@@ -11971,12 +12387,12 @@
       <c r="X116" s="12"/>
       <c r="Y116" s="7"/>
     </row>
-    <row r="117" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="117" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B117" s="11" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C117" s="12"/>
       <c r="D117" s="12" t="s">
@@ -12004,12 +12420,12 @@
       <c r="X117" s="12"/>
       <c r="Y117" s="7"/>
     </row>
-    <row r="118" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="118" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B118" s="11" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C118" s="12"/>
       <c r="D118" s="12" t="s">
@@ -12037,12 +12453,12 @@
       <c r="X118" s="12"/>
       <c r="Y118" s="7"/>
     </row>
-    <row r="119" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="119" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B119" s="11" t="s">
-        <v>76</v>
+        <v>216</v>
       </c>
       <c r="C119" s="12"/>
       <c r="D119" s="12" t="s">
@@ -12070,12 +12486,12 @@
       <c r="X119" s="12"/>
       <c r="Y119" s="7"/>
     </row>
-    <row r="120" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="120" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B120" s="11" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C120" s="12"/>
       <c r="D120" s="12" t="s">
@@ -12103,45 +12519,45 @@
       <c r="X120" s="12"/>
       <c r="Y120" s="7"/>
     </row>
-    <row r="121" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="121" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="11" t="s">
         <v>209</v>
       </c>
-      <c r="B121" s="14" t="s">
-        <v>219</v>
-      </c>
-      <c r="C121" s="15"/>
-      <c r="D121" s="15" t="s">
+      <c r="B121" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="C121" s="12"/>
+      <c r="D121" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E121" s="15"/>
-      <c r="F121" s="15"/>
-      <c r="G121" s="15"/>
-      <c r="H121" s="15"/>
-      <c r="I121" s="15"/>
-      <c r="J121" s="15"/>
-      <c r="K121" s="15"/>
-      <c r="L121" s="15"/>
-      <c r="M121" s="15"/>
-      <c r="N121" s="15"/>
-      <c r="O121" s="15"/>
-      <c r="P121" s="15"/>
-      <c r="Q121" s="15"/>
-      <c r="R121" s="15"/>
-      <c r="S121" s="15"/>
-      <c r="T121" s="15"/>
-      <c r="U121" s="15"/>
-      <c r="V121" s="15"/>
-      <c r="W121" s="15"/>
-      <c r="X121" s="15"/>
-      <c r="Y121" s="13"/>
-    </row>
-    <row r="122" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E121" s="12"/>
+      <c r="F121" s="12"/>
+      <c r="G121" s="12"/>
+      <c r="H121" s="12"/>
+      <c r="I121" s="12"/>
+      <c r="J121" s="12"/>
+      <c r="K121" s="12"/>
+      <c r="L121" s="12"/>
+      <c r="M121" s="12"/>
+      <c r="N121" s="12"/>
+      <c r="O121" s="12"/>
+      <c r="P121" s="12"/>
+      <c r="Q121" s="12"/>
+      <c r="R121" s="12"/>
+      <c r="S121" s="12"/>
+      <c r="T121" s="12"/>
+      <c r="U121" s="12"/>
+      <c r="V121" s="12"/>
+      <c r="W121" s="12"/>
+      <c r="X121" s="12"/>
+      <c r="Y121" s="7"/>
+    </row>
+    <row r="122" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B122" s="11" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C122" s="12"/>
       <c r="D122" s="12" t="s">
@@ -12169,45 +12585,45 @@
       <c r="X122" s="12"/>
       <c r="Y122" s="7"/>
     </row>
-    <row r="123" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="123" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="11" t="s">
         <v>209</v>
       </c>
-      <c r="B123" s="11" t="s">
-        <v>221</v>
-      </c>
-      <c r="C123" s="12"/>
-      <c r="D123" s="12" t="s">
+      <c r="B123" s="14" t="s">
+        <v>219</v>
+      </c>
+      <c r="C123" s="15"/>
+      <c r="D123" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="E123" s="12"/>
-      <c r="F123" s="12"/>
-      <c r="G123" s="12"/>
-      <c r="H123" s="12"/>
-      <c r="I123" s="12"/>
-      <c r="J123" s="12"/>
-      <c r="K123" s="12"/>
-      <c r="L123" s="12"/>
-      <c r="M123" s="12"/>
-      <c r="N123" s="12"/>
-      <c r="O123" s="12"/>
-      <c r="P123" s="12"/>
-      <c r="Q123" s="12"/>
-      <c r="R123" s="12"/>
-      <c r="S123" s="12"/>
-      <c r="T123" s="12"/>
-      <c r="U123" s="12"/>
-      <c r="V123" s="12"/>
-      <c r="W123" s="12"/>
-      <c r="X123" s="12"/>
-      <c r="Y123" s="7"/>
-    </row>
-    <row r="124" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E123" s="15"/>
+      <c r="F123" s="15"/>
+      <c r="G123" s="15"/>
+      <c r="H123" s="15"/>
+      <c r="I123" s="15"/>
+      <c r="J123" s="15"/>
+      <c r="K123" s="15"/>
+      <c r="L123" s="15"/>
+      <c r="M123" s="15"/>
+      <c r="N123" s="15"/>
+      <c r="O123" s="15"/>
+      <c r="P123" s="15"/>
+      <c r="Q123" s="15"/>
+      <c r="R123" s="15"/>
+      <c r="S123" s="15"/>
+      <c r="T123" s="15"/>
+      <c r="U123" s="15"/>
+      <c r="V123" s="15"/>
+      <c r="W123" s="15"/>
+      <c r="X123" s="15"/>
+      <c r="Y123" s="13"/>
+    </row>
+    <row r="124" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B124" s="11" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C124" s="12"/>
       <c r="D124" s="12" t="s">
@@ -12235,12 +12651,12 @@
       <c r="X124" s="12"/>
       <c r="Y124" s="7"/>
     </row>
-    <row r="125" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="125" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B125" s="11" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C125" s="12"/>
       <c r="D125" s="12" t="s">
@@ -12268,12 +12684,12 @@
       <c r="X125" s="12"/>
       <c r="Y125" s="7"/>
     </row>
-    <row r="126" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="126" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B126" s="11" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C126" s="12"/>
       <c r="D126" s="12" t="s">
@@ -12301,12 +12717,12 @@
       <c r="X126" s="12"/>
       <c r="Y126" s="7"/>
     </row>
-    <row r="127" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="127" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B127" s="11" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C127" s="12"/>
       <c r="D127" s="12" t="s">
@@ -12334,12 +12750,12 @@
       <c r="X127" s="12"/>
       <c r="Y127" s="7"/>
     </row>
-    <row r="128" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="128" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B128" s="11" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C128" s="12"/>
       <c r="D128" s="12" t="s">
@@ -12367,12 +12783,12 @@
       <c r="X128" s="12"/>
       <c r="Y128" s="7"/>
     </row>
-    <row r="129" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="129" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B129" s="11" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C129" s="12"/>
       <c r="D129" s="12" t="s">
@@ -12400,12 +12816,12 @@
       <c r="X129" s="12"/>
       <c r="Y129" s="7"/>
     </row>
-    <row r="130" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="130" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B130" s="11" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C130" s="12"/>
       <c r="D130" s="12" t="s">
@@ -12433,12 +12849,12 @@
       <c r="X130" s="12"/>
       <c r="Y130" s="7"/>
     </row>
-    <row r="131" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="131" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B131" s="11" t="s">
-        <v>264</v>
+        <v>227</v>
       </c>
       <c r="C131" s="12"/>
       <c r="D131" s="12" t="s">
@@ -12466,16 +12882,16 @@
       <c r="X131" s="12"/>
       <c r="Y131" s="7"/>
     </row>
-    <row r="132" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="132" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B132" s="11" t="s">
-        <v>270</v>
+        <v>228</v>
       </c>
       <c r="C132" s="12"/>
       <c r="D132" s="12" t="s">
-        <v>100</v>
+        <v>41</v>
       </c>
       <c r="E132" s="12"/>
       <c r="F132" s="12"/>
@@ -12499,12 +12915,12 @@
       <c r="X132" s="12"/>
       <c r="Y132" s="7"/>
     </row>
-    <row r="133" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="133" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B133" s="11" t="s">
-        <v>229</v>
+        <v>264</v>
       </c>
       <c r="C133" s="12"/>
       <c r="D133" s="12" t="s">
@@ -12532,138 +12948,210 @@
       <c r="X133" s="12"/>
       <c r="Y133" s="7"/>
     </row>
-    <row r="134" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="134" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="11" t="s">
+        <v>209</v>
+      </c>
+      <c r="B134" s="11" t="s">
+        <v>270</v>
+      </c>
+      <c r="C134" s="12"/>
+      <c r="D134" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="E134" s="12"/>
+      <c r="F134" s="12"/>
+      <c r="G134" s="12"/>
+      <c r="H134" s="12"/>
+      <c r="I134" s="12"/>
+      <c r="J134" s="12"/>
+      <c r="K134" s="12"/>
+      <c r="L134" s="12"/>
+      <c r="M134" s="12"/>
+      <c r="N134" s="12"/>
+      <c r="O134" s="12"/>
+      <c r="P134" s="12"/>
+      <c r="Q134" s="12"/>
+      <c r="R134" s="12"/>
+      <c r="S134" s="12"/>
+      <c r="T134" s="12"/>
+      <c r="U134" s="12"/>
+      <c r="V134" s="12"/>
+      <c r="W134" s="12"/>
+      <c r="X134" s="12"/>
+      <c r="Y134" s="7"/>
+    </row>
+    <row r="135" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A135" s="11" t="s">
+        <v>209</v>
+      </c>
+      <c r="B135" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="C135" s="12"/>
+      <c r="D135" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="E135" s="12"/>
+      <c r="F135" s="12"/>
+      <c r="G135" s="12"/>
+      <c r="H135" s="12"/>
+      <c r="I135" s="12"/>
+      <c r="J135" s="12"/>
+      <c r="K135" s="12"/>
+      <c r="L135" s="12"/>
+      <c r="M135" s="12"/>
+      <c r="N135" s="12"/>
+      <c r="O135" s="12"/>
+      <c r="P135" s="12"/>
+      <c r="Q135" s="12"/>
+      <c r="R135" s="12"/>
+      <c r="S135" s="12"/>
+      <c r="T135" s="12"/>
+      <c r="U135" s="12"/>
+      <c r="V135" s="12"/>
+      <c r="W135" s="12"/>
+      <c r="X135" s="12"/>
+      <c r="Y135" s="7"/>
+    </row>
+    <row r="136" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A136" s="11" t="s">
         <v>230</v>
       </c>
-      <c r="B134" s="11" t="s">
+      <c r="B136" s="11" t="s">
         <v>231</v>
-      </c>
-      <c r="C134" s="16"/>
-      <c r="D134" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="E134" s="16"/>
-      <c r="F134" s="16"/>
-      <c r="G134" s="16"/>
-      <c r="H134" s="16"/>
-      <c r="I134" s="16"/>
-      <c r="J134" s="16"/>
-      <c r="K134" s="16"/>
-      <c r="L134" s="16"/>
-      <c r="M134" s="16"/>
-      <c r="N134" s="16"/>
-      <c r="O134" s="16"/>
-      <c r="P134" s="16"/>
-      <c r="Q134" s="16"/>
-      <c r="R134" s="16"/>
-      <c r="S134" s="16"/>
-      <c r="T134" s="16"/>
-      <c r="U134" s="16"/>
-      <c r="V134" s="16"/>
-      <c r="W134" s="16"/>
-      <c r="X134" s="16"/>
-      <c r="Y134" s="7"/>
-    </row>
-    <row r="135" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A135" s="11" t="s">
-        <v>232</v>
-      </c>
-      <c r="B135" s="11" t="s">
-        <v>233</v>
-      </c>
-      <c r="C135" s="16"/>
-      <c r="D135" s="12" t="s">
-        <v>234</v>
-      </c>
-      <c r="E135" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="F135" s="31"/>
-      <c r="G135" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="H135" s="31"/>
-      <c r="I135" s="31"/>
-      <c r="J135" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="K135" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="L135" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="M135" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="N135" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="O135" s="31"/>
-      <c r="P135" s="31"/>
-      <c r="Q135" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="R135" s="31" t="s">
-        <v>236</v>
-      </c>
-      <c r="S135" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="T135" s="31"/>
-      <c r="U135" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="V135" s="31"/>
-      <c r="W135" s="31"/>
-      <c r="X135" s="31"/>
-      <c r="Y135" s="7"/>
-    </row>
-    <row r="136" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A136" s="11" t="s">
-        <v>265</v>
-      </c>
-      <c r="B136" s="11" t="s">
-        <v>265</v>
       </c>
       <c r="C136" s="16"/>
       <c r="D136" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="E136" s="31" t="s">
-        <v>38</v>
-      </c>
-      <c r="F136" s="31"/>
-      <c r="G136" s="31"/>
-      <c r="H136" s="31"/>
-      <c r="I136" s="31"/>
-      <c r="J136" s="31"/>
-      <c r="K136" s="31" t="s">
-        <v>38</v>
-      </c>
-      <c r="L136" s="31" t="s">
-        <v>38</v>
-      </c>
-      <c r="M136" s="31"/>
-      <c r="N136" s="31"/>
-      <c r="O136" s="31"/>
-      <c r="P136" s="31"/>
-      <c r="Q136" s="31"/>
-      <c r="R136" s="31"/>
-      <c r="S136" s="31"/>
-      <c r="T136" s="31"/>
-      <c r="U136" s="31"/>
-      <c r="V136" s="31"/>
-      <c r="W136" s="31"/>
-      <c r="X136" s="31"/>
+        <v>41</v>
+      </c>
+      <c r="E136" s="16"/>
+      <c r="F136" s="16"/>
+      <c r="G136" s="16"/>
+      <c r="H136" s="16"/>
+      <c r="I136" s="16"/>
+      <c r="J136" s="16"/>
+      <c r="K136" s="16"/>
+      <c r="L136" s="16"/>
+      <c r="M136" s="16"/>
+      <c r="N136" s="16"/>
+      <c r="O136" s="16"/>
+      <c r="P136" s="16"/>
+      <c r="Q136" s="16"/>
+      <c r="R136" s="16"/>
+      <c r="S136" s="16"/>
+      <c r="T136" s="16"/>
+      <c r="U136" s="16"/>
+      <c r="V136" s="16"/>
+      <c r="W136" s="16"/>
+      <c r="X136" s="16"/>
       <c r="Y136" s="7"/>
+    </row>
+    <row r="137" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A137" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="B137" s="11" t="s">
+        <v>233</v>
+      </c>
+      <c r="C137" s="16"/>
+      <c r="D137" s="12" t="s">
+        <v>234</v>
+      </c>
+      <c r="E137" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="F137" s="31"/>
+      <c r="G137" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="H137" s="31"/>
+      <c r="I137" s="31"/>
+      <c r="J137" s="31" t="s">
+        <v>235</v>
+      </c>
+      <c r="K137" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="L137" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="M137" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="N137" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="O137" s="31"/>
+      <c r="P137" s="31"/>
+      <c r="Q137" s="31" t="s">
+        <v>235</v>
+      </c>
+      <c r="R137" s="31" t="s">
+        <v>236</v>
+      </c>
+      <c r="S137" s="31" t="s">
+        <v>235</v>
+      </c>
+      <c r="T137" s="31"/>
+      <c r="U137" s="31" t="s">
+        <v>235</v>
+      </c>
+      <c r="V137" s="31"/>
+      <c r="W137" s="31"/>
+      <c r="X137" s="31"/>
+      <c r="Y137" s="7"/>
+    </row>
+    <row r="138" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A138" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="B138" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="C138" s="16"/>
+      <c r="D138" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="E138" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="F138" s="31"/>
+      <c r="G138" s="31"/>
+      <c r="H138" s="31"/>
+      <c r="I138" s="31"/>
+      <c r="J138" s="31"/>
+      <c r="K138" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="L138" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="M138" s="31"/>
+      <c r="N138" s="31"/>
+      <c r="O138" s="31"/>
+      <c r="P138" s="31"/>
+      <c r="Q138" s="31"/>
+      <c r="R138" s="31"/>
+      <c r="S138" s="31"/>
+      <c r="T138" s="31"/>
+      <c r="U138" s="31"/>
+      <c r="V138" s="31"/>
+      <c r="W138" s="31"/>
+      <c r="X138" s="31"/>
+      <c r="Y138" s="7"/>
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="115">
-      <pane xSplit="2" ySplit="6" topLeftCell="Q19" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="Y37" sqref="Y37"/>
+    <customSheetView guid="{810C905A-C0DA-4100-B6A9-F2260D80EA70}" scale="115">
+      <pane xSplit="2" ySplit="6" topLeftCell="Q101" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="B108" sqref="B108"/>
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+    </customSheetView>
+    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="130">
+      <pane xSplit="2" ySplit="6" topLeftCell="C53" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="B71" sqref="B71"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
@@ -12673,15 +13161,15 @@
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
-    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="130">
-      <pane xSplit="2" ySplit="6" topLeftCell="C53" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="B71" sqref="B71"/>
+    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="115">
+      <pane xSplit="2" ySplit="6" topLeftCell="Q19" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="Y37" sqref="Y37"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
   </customSheetViews>
   <mergeCells count="6">
-    <mergeCell ref="Y108:Y109"/>
+    <mergeCell ref="Y110:Y111"/>
     <mergeCell ref="C1:O1"/>
     <mergeCell ref="C2:O2"/>
     <mergeCell ref="C5:H5"/>
@@ -12697,7 +13185,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.6640625" customWidth="1"/>
     <col min="2" max="2" width="28.33203125" customWidth="1"/>
@@ -12705,7 +13193,7 @@
     <col min="5" max="5" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="32" t="s">
         <v>237</v>
       </c>
@@ -12722,7 +13210,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" s="33" t="s">
         <v>242</v>
       </c>
@@ -12735,7 +13223,7 @@
       <c r="D2" s="34"/>
       <c r="E2" s="34"/>
     </row>
-    <row r="3" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A3" s="33" t="s">
         <v>243</v>
       </c>
@@ -12748,7 +13236,7 @@
       <c r="D3" s="34"/>
       <c r="E3" s="34"/>
     </row>
-    <row r="4" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A4" s="33" t="s">
         <v>244</v>
       </c>
@@ -12761,7 +13249,7 @@
       <c r="D4" s="34"/>
       <c r="E4" s="34"/>
     </row>
-    <row r="5" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A5" s="33" t="s">
         <v>245</v>
       </c>
@@ -12776,7 +13264,7 @@
       </c>
       <c r="E5" s="34"/>
     </row>
-    <row r="6" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A6" s="33" t="s">
         <v>247</v>
       </c>
@@ -12791,7 +13279,7 @@
       </c>
       <c r="E6" s="34"/>
     </row>
-    <row r="7" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="33" t="s">
         <v>248</v>
       </c>
@@ -12806,7 +13294,7 @@
       </c>
       <c r="E7" s="34"/>
     </row>
-    <row r="8" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="33" t="s">
         <v>249</v>
       </c>
@@ -12821,7 +13309,7 @@
       </c>
       <c r="E8" s="34"/>
     </row>
-    <row r="9" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A9" s="33" t="s">
         <v>250</v>
       </c>
@@ -12836,7 +13324,7 @@
       </c>
       <c r="E9" s="34"/>
     </row>
-    <row r="10" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A10" s="33" t="s">
         <v>252</v>
       </c>
@@ -12849,7 +13337,7 @@
       <c r="D10" s="34"/>
       <c r="E10" s="34"/>
     </row>
-    <row r="11" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A11" s="33" t="s">
         <v>253</v>
       </c>
@@ -12862,7 +13350,7 @@
       <c r="D11" s="34"/>
       <c r="E11" s="34"/>
     </row>
-    <row r="12" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A12" s="33" t="s">
         <v>254</v>
       </c>
@@ -12875,7 +13363,7 @@
       <c r="D12" s="34"/>
       <c r="E12" s="34"/>
     </row>
-    <row r="13" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A13" s="33" t="s">
         <v>255</v>
       </c>
@@ -12890,7 +13378,7 @@
       </c>
       <c r="E13" s="34"/>
     </row>
-    <row r="14" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A14" s="33" t="s">
         <v>256</v>
       </c>
@@ -12905,7 +13393,7 @@
       </c>
       <c r="E14" s="34"/>
     </row>
-    <row r="15" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A15" s="33" t="s">
         <v>257</v>
       </c>
@@ -12920,7 +13408,7 @@
       </c>
       <c r="E15" s="34"/>
     </row>
-    <row r="16" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A16" s="33" t="s">
         <v>258</v>
       </c>
@@ -12935,7 +13423,7 @@
       </c>
       <c r="E16" s="34"/>
     </row>
-    <row r="17" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A17" s="33" t="s">
         <v>259</v>
       </c>
@@ -12950,7 +13438,7 @@
       </c>
       <c r="E17" s="34"/>
     </row>
-    <row r="18" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A18" s="33" t="s">
         <v>260</v>
       </c>
@@ -12965,7 +13453,7 @@
       </c>
       <c r="E18" s="34"/>
     </row>
-    <row r="19" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A19" s="33" t="s">
         <v>261</v>
       </c>
@@ -12980,7 +13468,7 @@
       </c>
       <c r="E19" s="34"/>
     </row>
-    <row r="20" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A20" s="33" t="s">
         <v>262</v>
       </c>
@@ -12995,7 +13483,7 @@
       </c>
       <c r="E20" s="34"/>
     </row>
-    <row r="21" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A21" s="33" t="s">
         <v>33</v>
       </c>
@@ -13010,7 +13498,7 @@
       </c>
       <c r="E21" s="34"/>
     </row>
-    <row r="22" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A22" s="33" t="s">
         <v>263</v>
       </c>
@@ -13027,7 +13515,12 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="150">
+    <customSheetView guid="{810C905A-C0DA-4100-B6A9-F2260D80EA70}" scale="150">
+      <selection activeCell="A22" sqref="A22"/>
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+    </customSheetView>
+    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="150">
       <selection activeCell="A22" sqref="A22"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -13037,7 +13530,7 @@
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
-    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="150">
+    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="150">
       <selection activeCell="A22" sqref="A22"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Lisää yhteenveto raportti rivi rooleihin
</commit_message>
<xml_diff>
--- a/resources/roolit.xlsx
+++ b/resources/roolit.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\samuli\dev\harjaroot\harja\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:81_{C33009BB-AF4A-4311-9633-F3E6F0CC09C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:81_{116B4C4A-38CD-40E6-B15E-39817FAEF29A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="23748" yWindow="156" windowWidth="25476" windowHeight="14232" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,32 +17,32 @@
     <sheet name="Roolit" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_1CE83972_B6A5_C44D_86E5_E9D9B38739F4_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_1DD617EE_F308_3E45_A8EF_4713F47FA0DD_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_2064F962_35EF_41F3_8A86_D37B72D177C7_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_3EBD3306_FC69_2148_8542_F6313DC2056F_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_47348D7B_5AFC_4A25_B239_A26E1359728E_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_476C495F_6E55_F04C_8145_4E8EBD6B3DE3_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_5327B0A1_A5FC_7747_93A1_427B210F3DF4_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_56F6E422_2CD8_6B4D_9E39_69A269028D26_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_6AA8E519_028C_D745_9E2E_8FB60E5B789F_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_7A9649F2_657F_9445_B6E6_FE94C6A09957_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_810C905A_C0DA_4100_B6A9_F2260D80EA70_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_8411E1B5_4691_4435_A9A2_147FF80D0D98_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_843152D8_333A_1941_83E9_0CB5262068A2_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_87BEAE97_700C_BF40_B102_636C54D81F08_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_D01EF3E4_E485_4912_A9DA_396AAE5B8752_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_D57E2FB1_FF7F_8446_9C97_237A4D57F6BE_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_E3BBF62E_A283_4D48_98B7_21A2A94F634F_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$136</definedName>
-    <definedName name="Z_F86DF6F3_8AE5_3A44_B2D2_D623E01AE54F_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$136</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Oikeudet!$A$5:$Y$137</definedName>
+    <definedName name="Z_1CE83972_B6A5_C44D_86E5_E9D9B38739F4_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$137</definedName>
+    <definedName name="Z_1DD617EE_F308_3E45_A8EF_4713F47FA0DD_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$137</definedName>
+    <definedName name="Z_2064F962_35EF_41F3_8A86_D37B72D177C7_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$137</definedName>
+    <definedName name="Z_3EBD3306_FC69_2148_8542_F6313DC2056F_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$137</definedName>
+    <definedName name="Z_47348D7B_5AFC_4A25_B239_A26E1359728E_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$137</definedName>
+    <definedName name="Z_476C495F_6E55_F04C_8145_4E8EBD6B3DE3_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$137</definedName>
+    <definedName name="Z_5327B0A1_A5FC_7747_93A1_427B210F3DF4_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$137</definedName>
+    <definedName name="Z_56F6E422_2CD8_6B4D_9E39_69A269028D26_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$137</definedName>
+    <definedName name="Z_6AA8E519_028C_D745_9E2E_8FB60E5B789F_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$137</definedName>
+    <definedName name="Z_7A9649F2_657F_9445_B6E6_FE94C6A09957_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$137</definedName>
+    <definedName name="Z_810C905A_C0DA_4100_B6A9_F2260D80EA70_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$137</definedName>
+    <definedName name="Z_8411E1B5_4691_4435_A9A2_147FF80D0D98_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$137</definedName>
+    <definedName name="Z_843152D8_333A_1941_83E9_0CB5262068A2_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$137</definedName>
+    <definedName name="Z_87BEAE97_700C_BF40_B102_636C54D81F08_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$137</definedName>
+    <definedName name="Z_D01EF3E4_E485_4912_A9DA_396AAE5B8752_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$137</definedName>
+    <definedName name="Z_D57E2FB1_FF7F_8446_9C97_237A4D57F6BE_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$137</definedName>
+    <definedName name="Z_E3BBF62E_A283_4D48_98B7_21A2A94F634F_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$137</definedName>
+    <definedName name="Z_F86DF6F3_8AE5_3A44_B2D2_D623E01AE54F_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$137</definedName>
   </definedNames>
   <calcPr calcId="0"/>
   <customWorkbookViews>
+    <customWorkbookView name="Microsoft Office User - Personal View" guid="{843152D8-333A-1941-83E9-0CB5262068A2}" mergeInterval="0" personalView="1" xWindow="4943" yWindow="119" windowWidth="1728" windowHeight="746" tabRatio="500" activeSheetId="1"/>
+    <customWorkbookView name="Jarno Väyrynen - Personal View" guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" mergeInterval="0" personalView="1" xWindow="48" yWindow="25" windowWidth="2512" windowHeight="1336" tabRatio="500" activeSheetId="1"/>
+    <customWorkbookView name="Microsoft Office User - Oma näkymä" guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" mergeInterval="0" personalView="1" xWindow="1440" yWindow="-515" windowWidth="2056" windowHeight="1366" tabRatio="500" activeSheetId="1"/>
     <customWorkbookView name="Samuli Taskila - Personal View" guid="{810C905A-C0DA-4100-B6A9-F2260D80EA70}" mergeInterval="0" personalView="1" xWindow="1979" yWindow="13" windowWidth="2123" windowHeight="1186" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Microsoft Office User - Oma näkymä" guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" mergeInterval="0" personalView="1" xWindow="1440" yWindow="-515" windowWidth="2056" windowHeight="1366" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Jarno Väyrynen - Personal View" guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" mergeInterval="0" personalView="1" xWindow="48" yWindow="25" windowWidth="2512" windowHeight="1336" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Microsoft Office User - Personal View" guid="{843152D8-333A-1941-83E9-0CB5262068A2}" mergeInterval="0" personalView="1" xWindow="4943" yWindow="119" windowWidth="1728" windowHeight="746" tabRatio="500" activeSheetId="1"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -112,7 +112,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1989" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2010" uniqueCount="276">
   <si>
     <t xml:space="preserve">Roolimääritysten selitykset: </t>
   </si>
@@ -1009,6 +1009,9 @@
   </si>
   <si>
     <t>Tiemerkintä - Sakot ja bonukset</t>
+  </si>
+  <si>
+    <t>Tiemerkintä - Yhteenveto</t>
   </si>
 </sst>
 </file>
@@ -1393,7 +1396,7 @@
 </file>
 
 <file path=xl/revisions/revisionHeaders.xml><?xml version="1.0" encoding="utf-8"?>
-<headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" guid="{4A6ED1B0-9135-4362-95CD-B6A2DDFC57B0}" diskRevisions="1" revisionId="269" version="14">
+<headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" guid="{53D7987A-7EDC-4AC3-9670-B01DA6273F6D}" diskRevisions="1" revisionId="292" version="15">
   <header guid="{8EBC2E30-8A6E-AD43-9F6F-B4500CF04203}" dateTime="2024-06-11T12:49:05" maxSheetId="3" userName="Jarno Väyrynen" r:id="rId9" minRId="87" maxRId="97">
     <sheetIdMap count="2">
       <sheetId val="1"/>
@@ -1454,6 +1457,12 @@
       <sheetId val="2"/>
     </sheetIdMap>
   </header>
+  <header guid="{53D7987A-7EDC-4AC3-9670-B01DA6273F6D}" dateTime="2025-04-03T12:26:20" maxSheetId="3" userName="Samuli Taskila" r:id="rId19" minRId="270" maxRId="292">
+    <sheetIdMap count="2">
+      <sheetId val="1"/>
+      <sheetId val="2"/>
+    </sheetIdMap>
+  </header>
 </headers>
 </file>
 
@@ -1814,6 +1823,171 @@
     <formula>Oikeudet!$A$5:$Y$136</formula>
   </rdn>
   <rcv guid="{810C905A-C0DA-4100-B6A9-F2260D80EA70}" action="add"/>
+</revisions>
+</file>
+
+<file path=xl/revisions/revisionLog11.xml><?xml version="1.0" encoding="utf-8"?>
+<revisions xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <rrc rId="270" sId="1" ref="A108:XFD108" action="insertRow"/>
+  <rcc rId="271" sId="1">
+    <nc r="A108" t="inlineStr">
+      <is>
+        <t>Raportit</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="272" sId="1">
+    <nc r="B108" t="inlineStr">
+      <is>
+        <t>Tiemerkintä - Muut kustannukset</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="273" sId="1">
+    <nc r="D108" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="274" sId="1">
+    <nc r="E108" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="275" sId="1">
+    <nc r="F108" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="276" sId="1">
+    <nc r="G108" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="277" sId="1">
+    <nc r="H108" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="278" sId="1">
+    <nc r="I108" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="279" sId="1">
+    <nc r="J108" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="280" sId="1">
+    <nc r="K108" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="281" sId="1">
+    <nc r="L108" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="282" sId="1">
+    <nc r="M108" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="283" sId="1">
+    <nc r="N108" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="284" sId="1">
+    <nc r="P108" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="285" sId="1">
+    <nc r="Q108" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="286" sId="1">
+    <nc r="R108" t="inlineStr">
+      <is>
+        <t>R+</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="287" sId="1">
+    <nc r="S108" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="288" sId="1">
+    <nc r="T108" t="inlineStr">
+      <is>
+        <t>R+</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="289" sId="1">
+    <nc r="U108" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="290" sId="1">
+    <nc r="V108" t="inlineStr">
+      <is>
+        <t>R+</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="291" sId="1">
+    <nc r="X108" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="292" sId="1">
+    <oc r="B109" t="inlineStr">
+      <is>
+        <t>Tiemerkintä - Muut kustannukset</t>
+      </is>
+    </oc>
+    <nc r="B109" t="inlineStr">
+      <is>
+        <t>Tiemerkintä - Yhteenveto</t>
+      </is>
+    </nc>
+  </rcc>
 </revisions>
 </file>
 
@@ -5665,7 +5839,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y138"/>
+  <dimension ref="A1:Y139"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -11928,29 +12102,35 @@
         <v>160</v>
       </c>
       <c r="B109" s="11" t="s">
-        <v>200</v>
+        <v>275</v>
       </c>
       <c r="C109" s="12"/>
       <c r="D109" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E109" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F109" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G109" s="12"/>
-      <c r="H109" s="12"/>
-      <c r="I109" s="12"/>
+      <c r="G109" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="H109" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I109" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="J109" s="12" t="s">
         <v>39</v>
       </c>
       <c r="K109" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="L109" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="M109" s="12" t="s">
         <v>39</v>
@@ -11959,61 +12139,61 @@
         <v>38</v>
       </c>
       <c r="O109" s="12"/>
-      <c r="P109" s="12"/>
+      <c r="P109" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="Q109" s="12" t="s">
         <v>39</v>
       </c>
       <c r="R109" s="12" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="S109" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="T109" s="12"/>
+        <v>39</v>
+      </c>
+      <c r="T109" s="12" t="s">
+        <v>44</v>
+      </c>
       <c r="U109" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="V109" s="12" t="s">
         <v>44</v>
       </c>
       <c r="W109" s="12"/>
-      <c r="X109" s="12"/>
+      <c r="X109" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="Y109" s="13"/>
     </row>
     <row r="110" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="11" t="s">
-        <v>201</v>
+        <v>160</v>
       </c>
       <c r="B110" s="11" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C110" s="12"/>
       <c r="D110" s="12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E110" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F110" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G110" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="H110" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="I110" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="G110" s="12"/>
+      <c r="H110" s="12"/>
+      <c r="I110" s="12"/>
       <c r="J110" s="12" t="s">
-        <v>203</v>
+        <v>39</v>
       </c>
       <c r="K110" s="12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="L110" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="M110" s="12" t="s">
         <v>39</v>
@@ -12021,46 +12201,34 @@
       <c r="N110" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="O110" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="P110" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="O110" s="12"/>
+      <c r="P110" s="12"/>
       <c r="Q110" s="12" t="s">
-        <v>203</v>
+        <v>39</v>
       </c>
       <c r="R110" s="12" t="s">
-        <v>204</v>
+        <v>42</v>
       </c>
       <c r="S110" s="12" t="s">
-        <v>203</v>
-      </c>
-      <c r="T110" s="12" t="s">
-        <v>44</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="T110" s="12"/>
       <c r="U110" s="12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="V110" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="W110" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="X110" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y110" s="35" t="s">
-        <v>205</v>
-      </c>
+      <c r="W110" s="12"/>
+      <c r="X110" s="12"/>
+      <c r="Y110" s="13"/>
     </row>
     <row r="111" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="11" t="s">
         <v>201</v>
       </c>
       <c r="B111" s="11" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="C111" s="12"/>
       <c r="D111" s="12" t="s">
@@ -12126,18 +12294,20 @@
       <c r="X111" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="Y111" s="35"/>
+      <c r="Y111" s="35" t="s">
+        <v>205</v>
+      </c>
     </row>
     <row r="112" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="11" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="B112" s="11" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C112" s="12"/>
       <c r="D112" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E112" s="12" t="s">
         <v>38</v>
@@ -12155,10 +12325,10 @@
         <v>39</v>
       </c>
       <c r="J112" s="12" t="s">
-        <v>39</v>
+        <v>203</v>
       </c>
       <c r="K112" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="L112" s="12" t="s">
         <v>38</v>
@@ -12176,37 +12346,37 @@
         <v>39</v>
       </c>
       <c r="Q112" s="12" t="s">
-        <v>39</v>
+        <v>203</v>
       </c>
       <c r="R112" s="12" t="s">
-        <v>42</v>
+        <v>204</v>
       </c>
       <c r="S112" s="12" t="s">
-        <v>40</v>
+        <v>203</v>
       </c>
       <c r="T112" s="12" t="s">
         <v>44</v>
       </c>
       <c r="U112" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="V112" s="12" t="s">
         <v>44</v>
       </c>
       <c r="W112" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="X112" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y112" s="7"/>
+        <v>39</v>
+      </c>
+      <c r="Y112" s="35"/>
     </row>
     <row r="113" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="11" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="B113" s="11" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="C113" s="12"/>
       <c r="D113" s="12" t="s">
@@ -12272,110 +12442,150 @@
       <c r="X113" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="Y113" s="13"/>
-    </row>
-    <row r="114" spans="1:25" s="30" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A114" s="27" t="s">
-        <v>209</v>
-      </c>
-      <c r="B114" s="27" t="s">
-        <v>210</v>
-      </c>
-      <c r="C114" s="28"/>
+      <c r="Y113" s="7"/>
+    </row>
+    <row r="114" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A114" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="B114" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="C114" s="12"/>
       <c r="D114" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E114" s="28"/>
-      <c r="F114" s="28"/>
-      <c r="G114" s="28"/>
-      <c r="H114" s="28"/>
-      <c r="I114" s="28"/>
-      <c r="J114" s="28"/>
-      <c r="K114" s="28"/>
-      <c r="L114" s="28"/>
-      <c r="M114" s="28"/>
-      <c r="N114" s="28"/>
-      <c r="O114" s="28"/>
-      <c r="P114" s="28"/>
-      <c r="Q114" s="28"/>
-      <c r="R114" s="28"/>
-      <c r="S114" s="28"/>
-      <c r="T114" s="28"/>
-      <c r="U114" s="28"/>
-      <c r="V114" s="28"/>
-      <c r="W114" s="28"/>
-      <c r="X114" s="28"/>
-      <c r="Y114" s="29" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="115" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A115" s="11" t="s">
+      <c r="E114" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F114" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="G114" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="H114" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I114" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="J114" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="K114" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="L114" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="M114" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="N114" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="O114" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="P114" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q114" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="R114" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="S114" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="T114" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="U114" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="V114" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="W114" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="X114" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="Y114" s="13"/>
+    </row>
+    <row r="115" spans="1:25" s="30" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A115" s="27" t="s">
         <v>209</v>
       </c>
-      <c r="B115" s="11" t="s">
-        <v>212</v>
-      </c>
-      <c r="C115" s="12"/>
+      <c r="B115" s="27" t="s">
+        <v>210</v>
+      </c>
+      <c r="C115" s="28"/>
       <c r="D115" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E115" s="12"/>
-      <c r="F115" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="G115" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="H115" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="I115" s="12"/>
-      <c r="J115" s="12"/>
-      <c r="K115" s="12"/>
-      <c r="L115" s="12"/>
-      <c r="M115" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="N115" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="O115" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="P115" s="12"/>
-      <c r="Q115" s="12"/>
-      <c r="R115" s="12"/>
-      <c r="S115" s="12"/>
-      <c r="T115" s="12"/>
-      <c r="U115" s="12"/>
-      <c r="V115" s="12"/>
-      <c r="W115" s="12"/>
-      <c r="X115" s="12"/>
-      <c r="Y115" s="7"/>
+      <c r="E115" s="28"/>
+      <c r="F115" s="28"/>
+      <c r="G115" s="28"/>
+      <c r="H115" s="28"/>
+      <c r="I115" s="28"/>
+      <c r="J115" s="28"/>
+      <c r="K115" s="28"/>
+      <c r="L115" s="28"/>
+      <c r="M115" s="28"/>
+      <c r="N115" s="28"/>
+      <c r="O115" s="28"/>
+      <c r="P115" s="28"/>
+      <c r="Q115" s="28"/>
+      <c r="R115" s="28"/>
+      <c r="S115" s="28"/>
+      <c r="T115" s="28"/>
+      <c r="U115" s="28"/>
+      <c r="V115" s="28"/>
+      <c r="W115" s="28"/>
+      <c r="X115" s="28"/>
+      <c r="Y115" s="29" t="s">
+        <v>211</v>
+      </c>
     </row>
     <row r="116" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B116" s="11" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C116" s="12"/>
       <c r="D116" s="12" t="s">
         <v>41</v>
       </c>
       <c r="E116" s="12"/>
-      <c r="F116" s="12"/>
-      <c r="G116" s="12"/>
-      <c r="H116" s="12"/>
+      <c r="F116" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="G116" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="H116" s="12" t="s">
+        <v>46</v>
+      </c>
       <c r="I116" s="12"/>
       <c r="J116" s="12"/>
       <c r="K116" s="12"/>
       <c r="L116" s="12"/>
-      <c r="M116" s="12"/>
-      <c r="N116" s="12"/>
-      <c r="O116" s="12"/>
+      <c r="M116" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="N116" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="O116" s="12" t="s">
+        <v>46</v>
+      </c>
       <c r="P116" s="12"/>
       <c r="Q116" s="12"/>
       <c r="R116" s="12"/>
@@ -12392,7 +12602,7 @@
         <v>209</v>
       </c>
       <c r="B117" s="11" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C117" s="12"/>
       <c r="D117" s="12" t="s">
@@ -12425,7 +12635,7 @@
         <v>209</v>
       </c>
       <c r="B118" s="11" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C118" s="12"/>
       <c r="D118" s="12" t="s">
@@ -12458,7 +12668,7 @@
         <v>209</v>
       </c>
       <c r="B119" s="11" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C119" s="12"/>
       <c r="D119" s="12" t="s">
@@ -12491,7 +12701,7 @@
         <v>209</v>
       </c>
       <c r="B120" s="11" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C120" s="12"/>
       <c r="D120" s="12" t="s">
@@ -12524,7 +12734,7 @@
         <v>209</v>
       </c>
       <c r="B121" s="11" t="s">
-        <v>76</v>
+        <v>217</v>
       </c>
       <c r="C121" s="12"/>
       <c r="D121" s="12" t="s">
@@ -12557,7 +12767,7 @@
         <v>209</v>
       </c>
       <c r="B122" s="11" t="s">
-        <v>218</v>
+        <v>76</v>
       </c>
       <c r="C122" s="12"/>
       <c r="D122" s="12" t="s">
@@ -12589,74 +12799,74 @@
       <c r="A123" s="11" t="s">
         <v>209</v>
       </c>
-      <c r="B123" s="14" t="s">
-        <v>219</v>
-      </c>
-      <c r="C123" s="15"/>
-      <c r="D123" s="15" t="s">
+      <c r="B123" s="11" t="s">
+        <v>218</v>
+      </c>
+      <c r="C123" s="12"/>
+      <c r="D123" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E123" s="15"/>
-      <c r="F123" s="15"/>
-      <c r="G123" s="15"/>
-      <c r="H123" s="15"/>
-      <c r="I123" s="15"/>
-      <c r="J123" s="15"/>
-      <c r="K123" s="15"/>
-      <c r="L123" s="15"/>
-      <c r="M123" s="15"/>
-      <c r="N123" s="15"/>
-      <c r="O123" s="15"/>
-      <c r="P123" s="15"/>
-      <c r="Q123" s="15"/>
-      <c r="R123" s="15"/>
-      <c r="S123" s="15"/>
-      <c r="T123" s="15"/>
-      <c r="U123" s="15"/>
-      <c r="V123" s="15"/>
-      <c r="W123" s="15"/>
-      <c r="X123" s="15"/>
-      <c r="Y123" s="13"/>
+      <c r="E123" s="12"/>
+      <c r="F123" s="12"/>
+      <c r="G123" s="12"/>
+      <c r="H123" s="12"/>
+      <c r="I123" s="12"/>
+      <c r="J123" s="12"/>
+      <c r="K123" s="12"/>
+      <c r="L123" s="12"/>
+      <c r="M123" s="12"/>
+      <c r="N123" s="12"/>
+      <c r="O123" s="12"/>
+      <c r="P123" s="12"/>
+      <c r="Q123" s="12"/>
+      <c r="R123" s="12"/>
+      <c r="S123" s="12"/>
+      <c r="T123" s="12"/>
+      <c r="U123" s="12"/>
+      <c r="V123" s="12"/>
+      <c r="W123" s="12"/>
+      <c r="X123" s="12"/>
+      <c r="Y123" s="7"/>
     </row>
     <row r="124" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="11" t="s">
         <v>209</v>
       </c>
-      <c r="B124" s="11" t="s">
-        <v>220</v>
-      </c>
-      <c r="C124" s="12"/>
-      <c r="D124" s="12" t="s">
+      <c r="B124" s="14" t="s">
+        <v>219</v>
+      </c>
+      <c r="C124" s="15"/>
+      <c r="D124" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="E124" s="12"/>
-      <c r="F124" s="12"/>
-      <c r="G124" s="12"/>
-      <c r="H124" s="12"/>
-      <c r="I124" s="12"/>
-      <c r="J124" s="12"/>
-      <c r="K124" s="12"/>
-      <c r="L124" s="12"/>
-      <c r="M124" s="12"/>
-      <c r="N124" s="12"/>
-      <c r="O124" s="12"/>
-      <c r="P124" s="12"/>
-      <c r="Q124" s="12"/>
-      <c r="R124" s="12"/>
-      <c r="S124" s="12"/>
-      <c r="T124" s="12"/>
-      <c r="U124" s="12"/>
-      <c r="V124" s="12"/>
-      <c r="W124" s="12"/>
-      <c r="X124" s="12"/>
-      <c r="Y124" s="7"/>
+      <c r="E124" s="15"/>
+      <c r="F124" s="15"/>
+      <c r="G124" s="15"/>
+      <c r="H124" s="15"/>
+      <c r="I124" s="15"/>
+      <c r="J124" s="15"/>
+      <c r="K124" s="15"/>
+      <c r="L124" s="15"/>
+      <c r="M124" s="15"/>
+      <c r="N124" s="15"/>
+      <c r="O124" s="15"/>
+      <c r="P124" s="15"/>
+      <c r="Q124" s="15"/>
+      <c r="R124" s="15"/>
+      <c r="S124" s="15"/>
+      <c r="T124" s="15"/>
+      <c r="U124" s="15"/>
+      <c r="V124" s="15"/>
+      <c r="W124" s="15"/>
+      <c r="X124" s="15"/>
+      <c r="Y124" s="13"/>
     </row>
     <row r="125" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B125" s="11" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C125" s="12"/>
       <c r="D125" s="12" t="s">
@@ -12689,7 +12899,7 @@
         <v>209</v>
       </c>
       <c r="B126" s="11" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C126" s="12"/>
       <c r="D126" s="12" t="s">
@@ -12722,7 +12932,7 @@
         <v>209</v>
       </c>
       <c r="B127" s="11" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C127" s="12"/>
       <c r="D127" s="12" t="s">
@@ -12750,12 +12960,12 @@
       <c r="X127" s="12"/>
       <c r="Y127" s="7"/>
     </row>
-    <row r="128" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="11" t="s">
         <v>209</v>
       </c>
       <c r="B128" s="11" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C128" s="12"/>
       <c r="D128" s="12" t="s">
@@ -12788,7 +12998,7 @@
         <v>209</v>
       </c>
       <c r="B129" s="11" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C129" s="12"/>
       <c r="D129" s="12" t="s">
@@ -12821,7 +13031,7 @@
         <v>209</v>
       </c>
       <c r="B130" s="11" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C130" s="12"/>
       <c r="D130" s="12" t="s">
@@ -12854,7 +13064,7 @@
         <v>209</v>
       </c>
       <c r="B131" s="11" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C131" s="12"/>
       <c r="D131" s="12" t="s">
@@ -12887,7 +13097,7 @@
         <v>209</v>
       </c>
       <c r="B132" s="11" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C132" s="12"/>
       <c r="D132" s="12" t="s">
@@ -12920,7 +13130,7 @@
         <v>209</v>
       </c>
       <c r="B133" s="11" t="s">
-        <v>264</v>
+        <v>228</v>
       </c>
       <c r="C133" s="12"/>
       <c r="D133" s="12" t="s">
@@ -12953,11 +13163,11 @@
         <v>209</v>
       </c>
       <c r="B134" s="11" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="C134" s="12"/>
       <c r="D134" s="12" t="s">
-        <v>100</v>
+        <v>41</v>
       </c>
       <c r="E134" s="12"/>
       <c r="F134" s="12"/>
@@ -12986,11 +13196,11 @@
         <v>209</v>
       </c>
       <c r="B135" s="11" t="s">
-        <v>229</v>
+        <v>270</v>
       </c>
       <c r="C135" s="12"/>
       <c r="D135" s="12" t="s">
-        <v>41</v>
+        <v>100</v>
       </c>
       <c r="E135" s="12"/>
       <c r="F135" s="12"/>
@@ -13016,136 +13226,175 @@
     </row>
     <row r="136" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="11" t="s">
-        <v>230</v>
+        <v>209</v>
       </c>
       <c r="B136" s="11" t="s">
-        <v>231</v>
-      </c>
-      <c r="C136" s="16"/>
+        <v>229</v>
+      </c>
+      <c r="C136" s="12"/>
       <c r="D136" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E136" s="16"/>
-      <c r="F136" s="16"/>
-      <c r="G136" s="16"/>
-      <c r="H136" s="16"/>
-      <c r="I136" s="16"/>
-      <c r="J136" s="16"/>
-      <c r="K136" s="16"/>
-      <c r="L136" s="16"/>
-      <c r="M136" s="16"/>
-      <c r="N136" s="16"/>
-      <c r="O136" s="16"/>
-      <c r="P136" s="16"/>
-      <c r="Q136" s="16"/>
-      <c r="R136" s="16"/>
-      <c r="S136" s="16"/>
-      <c r="T136" s="16"/>
-      <c r="U136" s="16"/>
-      <c r="V136" s="16"/>
-      <c r="W136" s="16"/>
-      <c r="X136" s="16"/>
+      <c r="E136" s="12"/>
+      <c r="F136" s="12"/>
+      <c r="G136" s="12"/>
+      <c r="H136" s="12"/>
+      <c r="I136" s="12"/>
+      <c r="J136" s="12"/>
+      <c r="K136" s="12"/>
+      <c r="L136" s="12"/>
+      <c r="M136" s="12"/>
+      <c r="N136" s="12"/>
+      <c r="O136" s="12"/>
+      <c r="P136" s="12"/>
+      <c r="Q136" s="12"/>
+      <c r="R136" s="12"/>
+      <c r="S136" s="12"/>
+      <c r="T136" s="12"/>
+      <c r="U136" s="12"/>
+      <c r="V136" s="12"/>
+      <c r="W136" s="12"/>
+      <c r="X136" s="12"/>
       <c r="Y136" s="7"/>
     </row>
     <row r="137" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="11" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B137" s="11" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C137" s="16"/>
       <c r="D137" s="12" t="s">
-        <v>234</v>
-      </c>
-      <c r="E137" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="F137" s="31"/>
-      <c r="G137" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="H137" s="31"/>
-      <c r="I137" s="31"/>
-      <c r="J137" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="K137" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="L137" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="M137" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="N137" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="O137" s="31"/>
-      <c r="P137" s="31"/>
-      <c r="Q137" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="R137" s="31" t="s">
-        <v>236</v>
-      </c>
-      <c r="S137" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="T137" s="31"/>
-      <c r="U137" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="V137" s="31"/>
-      <c r="W137" s="31"/>
-      <c r="X137" s="31"/>
+        <v>41</v>
+      </c>
+      <c r="E137" s="16"/>
+      <c r="F137" s="16"/>
+      <c r="G137" s="16"/>
+      <c r="H137" s="16"/>
+      <c r="I137" s="16"/>
+      <c r="J137" s="16"/>
+      <c r="K137" s="16"/>
+      <c r="L137" s="16"/>
+      <c r="M137" s="16"/>
+      <c r="N137" s="16"/>
+      <c r="O137" s="16"/>
+      <c r="P137" s="16"/>
+      <c r="Q137" s="16"/>
+      <c r="R137" s="16"/>
+      <c r="S137" s="16"/>
+      <c r="T137" s="16"/>
+      <c r="U137" s="16"/>
+      <c r="V137" s="16"/>
+      <c r="W137" s="16"/>
+      <c r="X137" s="16"/>
       <c r="Y137" s="7"/>
     </row>
     <row r="138" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="11" t="s">
-        <v>265</v>
+        <v>232</v>
       </c>
       <c r="B138" s="11" t="s">
-        <v>265</v>
+        <v>233</v>
       </c>
       <c r="C138" s="16"/>
       <c r="D138" s="12" t="s">
-        <v>38</v>
+        <v>234</v>
       </c>
       <c r="E138" s="31" t="s">
-        <v>38</v>
+        <v>234</v>
       </c>
       <c r="F138" s="31"/>
-      <c r="G138" s="31"/>
+      <c r="G138" s="31" t="s">
+        <v>234</v>
+      </c>
       <c r="H138" s="31"/>
       <c r="I138" s="31"/>
-      <c r="J138" s="31"/>
+      <c r="J138" s="31" t="s">
+        <v>235</v>
+      </c>
       <c r="K138" s="31" t="s">
-        <v>38</v>
+        <v>234</v>
       </c>
       <c r="L138" s="31" t="s">
-        <v>38</v>
-      </c>
-      <c r="M138" s="31"/>
-      <c r="N138" s="31"/>
+        <v>234</v>
+      </c>
+      <c r="M138" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="N138" s="31" t="s">
+        <v>234</v>
+      </c>
       <c r="O138" s="31"/>
       <c r="P138" s="31"/>
-      <c r="Q138" s="31"/>
-      <c r="R138" s="31"/>
-      <c r="S138" s="31"/>
+      <c r="Q138" s="31" t="s">
+        <v>235</v>
+      </c>
+      <c r="R138" s="31" t="s">
+        <v>236</v>
+      </c>
+      <c r="S138" s="31" t="s">
+        <v>235</v>
+      </c>
       <c r="T138" s="31"/>
-      <c r="U138" s="31"/>
+      <c r="U138" s="31" t="s">
+        <v>235</v>
+      </c>
       <c r="V138" s="31"/>
       <c r="W138" s="31"/>
       <c r="X138" s="31"/>
       <c r="Y138" s="7"/>
     </row>
+    <row r="139" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A139" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="B139" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="C139" s="16"/>
+      <c r="D139" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="E139" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="F139" s="31"/>
+      <c r="G139" s="31"/>
+      <c r="H139" s="31"/>
+      <c r="I139" s="31"/>
+      <c r="J139" s="31"/>
+      <c r="K139" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="L139" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="M139" s="31"/>
+      <c r="N139" s="31"/>
+      <c r="O139" s="31"/>
+      <c r="P139" s="31"/>
+      <c r="Q139" s="31"/>
+      <c r="R139" s="31"/>
+      <c r="S139" s="31"/>
+      <c r="T139" s="31"/>
+      <c r="U139" s="31"/>
+      <c r="V139" s="31"/>
+      <c r="W139" s="31"/>
+      <c r="X139" s="31"/>
+      <c r="Y139" s="7"/>
+    </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{810C905A-C0DA-4100-B6A9-F2260D80EA70}" scale="115">
-      <pane xSplit="2" ySplit="6" topLeftCell="Q101" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="B108" sqref="B108"/>
+    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="115">
+      <pane xSplit="2" ySplit="6" topLeftCell="Q19" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="Y37" sqref="Y37"/>
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+    </customSheetView>
+    <customSheetView guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" scale="115">
+      <pane xSplit="2" ySplit="6" topLeftCell="C58" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="D81" sqref="D81:X81"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
@@ -13155,21 +13404,15 @@
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
-    <customSheetView guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" scale="115">
-      <pane xSplit="2" ySplit="6" topLeftCell="C58" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="D81" sqref="D81:X81"/>
-      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-    </customSheetView>
-    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="115">
-      <pane xSplit="2" ySplit="6" topLeftCell="Q19" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="Y37" sqref="Y37"/>
+    <customSheetView guid="{810C905A-C0DA-4100-B6A9-F2260D80EA70}" scale="115">
+      <pane xSplit="2" ySplit="6" topLeftCell="Q101" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="B108" sqref="B108"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
   </customSheetViews>
   <mergeCells count="6">
-    <mergeCell ref="Y110:Y111"/>
+    <mergeCell ref="Y111:Y112"/>
     <mergeCell ref="C1:O1"/>
     <mergeCell ref="C2:O2"/>
     <mergeCell ref="C5:H5"/>
@@ -13515,7 +13758,12 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{810C905A-C0DA-4100-B6A9-F2260D80EA70}" scale="150">
+    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="150">
+      <selection activeCell="A22" sqref="A22"/>
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+    </customSheetView>
+    <customSheetView guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" scale="150">
       <selection activeCell="A22" sqref="A22"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -13525,12 +13773,7 @@
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
-    <customSheetView guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" scale="150">
-      <selection activeCell="A22" sqref="A22"/>
-      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-    </customSheetView>
-    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="150">
+    <customSheetView guid="{810C905A-C0DA-4100-B6A9-F2260D80EA70}" scale="150">
       <selection activeCell="A22" sqref="A22"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Korjaa tiemerkinnän kustannuksien roolit
</commit_message>
<xml_diff>
--- a/resources/roolit.xlsx
+++ b/resources/roolit.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\samuli\dev\harjaroot\harja\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:81_{1F4D09BB-474B-4F77-BA0E-639DC5265069}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:81_{AE896ADE-AD64-49AF-8AB6-77EEA9B91A85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27912" yWindow="504" windowWidth="25476" windowHeight="14232" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-40935" yWindow="-1620" windowWidth="33120" windowHeight="16470" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Oikeudet" sheetId="1" r:id="rId1"/>
@@ -39,10 +39,10 @@
   </definedNames>
   <calcPr calcId="0"/>
   <customWorkbookViews>
+    <customWorkbookView name="Microsoft Office User - Personal View" guid="{843152D8-333A-1941-83E9-0CB5262068A2}" mergeInterval="0" personalView="1" xWindow="4943" yWindow="119" windowWidth="1728" windowHeight="746" tabRatio="500" activeSheetId="1"/>
+    <customWorkbookView name="Jarno Väyrynen - Personal View" guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" mergeInterval="0" personalView="1" xWindow="48" yWindow="25" windowWidth="2512" windowHeight="1336" tabRatio="500" activeSheetId="1"/>
+    <customWorkbookView name="Microsoft Office User - Oma näkymä" guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" mergeInterval="0" personalView="1" xWindow="1440" yWindow="-515" windowWidth="2056" windowHeight="1366" tabRatio="500" activeSheetId="1"/>
     <customWorkbookView name="Samuli Taskila - Personal View" guid="{B8461C08-78CA-4BAA-BBDB-16DCE44957A3}" mergeInterval="0" personalView="1" xWindow="2326" yWindow="42" windowWidth="2123" windowHeight="1186" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Microsoft Office User - Oma näkymä" guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" mergeInterval="0" personalView="1" xWindow="1440" yWindow="-515" windowWidth="2056" windowHeight="1366" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Jarno Väyrynen - Personal View" guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" mergeInterval="0" personalView="1" xWindow="48" yWindow="25" windowWidth="2512" windowHeight="1336" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Microsoft Office User - Personal View" guid="{843152D8-333A-1941-83E9-0CB5262068A2}" mergeInterval="0" personalView="1" xWindow="4943" yWindow="119" windowWidth="1728" windowHeight="746" tabRatio="500" activeSheetId="1"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -112,7 +112,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2010" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2013" uniqueCount="275">
   <si>
     <t xml:space="preserve">Roolimääritysten selitykset: </t>
   </si>
@@ -1000,9 +1000,6 @@
   </si>
   <si>
     <t>Tiemerkinnän kustannukset</t>
-  </si>
-  <si>
-    <t>Koitetaan pärjätä yhdellä rivillä kaikkien välilehtien osalta</t>
   </si>
   <si>
     <t>Tiemerkintä - Yhteenveto</t>
@@ -1396,7 +1393,7 @@
 </file>
 
 <file path=xl/revisions/revisionHeaders.xml><?xml version="1.0" encoding="utf-8"?>
-<headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" guid="{831A92D1-02E0-4095-80A8-F54C5209A530}" diskRevisions="1" revisionId="291" version="14">
+<headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" guid="{40CEC047-1DCE-421E-B201-659B500E1570}" diskRevisions="1" revisionId="301" version="15">
   <header guid="{8EBC2E30-8A6E-AD43-9F6F-B4500CF04203}" dateTime="2024-06-11T12:49:05" maxSheetId="3" userName="Jarno Väyrynen" r:id="rId9" minRId="87" maxRId="97">
     <sheetIdMap count="2">
       <sheetId val="1"/>
@@ -1457,6 +1454,12 @@
       <sheetId val="2"/>
     </sheetIdMap>
   </header>
+  <header guid="{40CEC047-1DCE-421E-B201-659B500E1570}" dateTime="2025-04-30T12:34:14" maxSheetId="3" userName="Samuli Taskila" r:id="rId19" minRId="292" maxRId="301">
+    <sheetIdMap count="2">
+      <sheetId val="1"/>
+      <sheetId val="2"/>
+    </sheetIdMap>
+  </header>
 </headers>
 </file>
 
@@ -1941,6 +1944,122 @@
     <formula>Oikeudet!$A$5:$Y$137</formula>
   </rdn>
   <rcv guid="{B8461C08-78CA-4BAA-BBDB-16DCE44957A3}" action="add"/>
+</revisions>
+</file>
+
+<file path=xl/revisions/revisionLog11.xml><?xml version="1.0" encoding="utf-8"?>
+<revisions xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <rfmt sheetId="1" sqref="B37" start="0" length="0">
+    <dxf>
+      <font>
+        <color auto="1"/>
+        <family val="2"/>
+      </font>
+    </dxf>
+  </rfmt>
+  <rcc rId="292" sId="1">
+    <oc r="E37" t="inlineStr">
+      <is>
+        <t>R*,W*</t>
+      </is>
+    </oc>
+    <nc r="E37" t="inlineStr">
+      <is>
+        <t>R*,W</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="293" sId="1">
+    <nc r="H37" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="294" sId="1">
+    <nc r="I37" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="295" sId="1">
+    <oc r="J37" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </oc>
+    <nc r="J37" t="inlineStr">
+      <is>
+        <t>R,W</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="296" sId="1">
+    <oc r="M37" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </oc>
+    <nc r="M37"/>
+  </rcc>
+  <rcc rId="297" sId="1">
+    <nc r="O37" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="298" sId="1">
+    <nc r="Q37" t="inlineStr">
+      <is>
+        <t>R,W</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="299" sId="1">
+    <nc r="T37" t="inlineStr">
+      <is>
+        <t>R+</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="300" sId="1">
+    <oc r="U37" t="inlineStr">
+      <is>
+        <t>R,W</t>
+      </is>
+    </oc>
+    <nc r="U37" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="301" sId="1" odxf="1" dxf="1">
+    <oc r="Y37" t="inlineStr">
+      <is>
+        <t>Koitetaan pärjätä yhdellä rivillä kaikkien välilehtien osalta</t>
+      </is>
+    </oc>
+    <nc r="Y37"/>
+    <odxf>
+      <font>
+        <color auto="1"/>
+        <family val="2"/>
+      </font>
+    </odxf>
+    <ndxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+    </ndxf>
+  </rcc>
 </revisions>
 </file>
 
@@ -7785,7 +7904,7 @@
       <c r="A37" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B37" s="16" t="s">
+      <c r="B37" s="11" t="s">
         <v>271</v>
       </c>
       <c r="C37" s="12"/>
@@ -7793,16 +7912,20 @@
         <v>41</v>
       </c>
       <c r="E37" s="12" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F37" s="12" t="s">
         <v>38</v>
       </c>
       <c r="G37" s="12"/>
-      <c r="H37" s="12"/>
-      <c r="I37" s="12"/>
+      <c r="H37" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I37" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="J37" s="12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K37" s="12" t="s">
         <v>41</v>
@@ -7810,33 +7933,35 @@
       <c r="L37" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="M37" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="M37" s="12"/>
       <c r="N37" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="O37" s="12"/>
+      <c r="O37" s="12" t="s">
+        <v>38</v>
+      </c>
       <c r="P37" s="12"/>
-      <c r="Q37" s="12"/>
+      <c r="Q37" s="12" t="s">
+        <v>40</v>
+      </c>
       <c r="R37" s="12" t="s">
         <v>42</v>
       </c>
       <c r="S37" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="T37" s="12"/>
+      <c r="T37" s="12" t="s">
+        <v>44</v>
+      </c>
       <c r="U37" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="V37" s="12" t="s">
         <v>44</v>
       </c>
       <c r="W37" s="12"/>
       <c r="X37" s="12"/>
-      <c r="Y37" s="13" t="s">
-        <v>272</v>
-      </c>
+      <c r="Y37" s="7"/>
     </row>
     <row r="38" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="11" t="s">
@@ -10665,7 +10790,7 @@
         <v>160</v>
       </c>
       <c r="B88" s="11" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C88" s="12"/>
       <c r="D88" s="12" t="s">
@@ -10734,7 +10859,7 @@
         <v>160</v>
       </c>
       <c r="B89" s="11" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C89" s="12"/>
       <c r="D89" s="12" t="s">
@@ -10803,7 +10928,7 @@
         <v>160</v>
       </c>
       <c r="B90" s="11" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C90" s="12"/>
       <c r="D90" s="12" t="s">
@@ -13338,9 +13463,15 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{B8461C08-78CA-4BAA-BBDB-16DCE44957A3}" scale="115">
-      <pane xSplit="2" ySplit="6" topLeftCell="C74" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="B89" sqref="B89"/>
+    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="115">
+      <pane xSplit="2" ySplit="6" topLeftCell="Q19" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="Y37" sqref="Y37"/>
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+    </customSheetView>
+    <customSheetView guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" scale="115">
+      <pane xSplit="2" ySplit="6" topLeftCell="C58" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="D81" sqref="D81:X81"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
@@ -13350,15 +13481,9 @@
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
-    <customSheetView guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" scale="115">
-      <pane xSplit="2" ySplit="6" topLeftCell="C58" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="D81" sqref="D81:X81"/>
-      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-    </customSheetView>
-    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="115">
-      <pane xSplit="2" ySplit="6" topLeftCell="Q19" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="Y37" sqref="Y37"/>
+    <customSheetView guid="{B8461C08-78CA-4BAA-BBDB-16DCE44957A3}" scale="115">
+      <pane xSplit="2" ySplit="6" topLeftCell="C74" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="B89" sqref="B89"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
@@ -13710,7 +13835,12 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{B8461C08-78CA-4BAA-BBDB-16DCE44957A3}" scale="150">
+    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="150">
+      <selection activeCell="A22" sqref="A22"/>
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+    </customSheetView>
+    <customSheetView guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" scale="150">
       <selection activeCell="A22" sqref="A22"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -13720,12 +13850,7 @@
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
-    <customSheetView guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" scale="150">
-      <selection activeCell="A22" sqref="A22"/>
-      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-    </customSheetView>
-    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="150">
+    <customSheetView guid="{B8461C08-78CA-4BAA-BBDB-16DCE44957A3}" scale="150">
       <selection activeCell="A22" sqref="A22"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Näytä talvihoitoreitit urakan myös vastuuhenkilölle
</commit_message>
<xml_diff>
--- a/resources/roolit.xlsx
+++ b/resources/roolit.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\samuli\dev\harjaroot\harja\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:81_{9C135951-6B6F-4789-A226-B4FFA1E58967}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:81_{06D8ADD0-19FE-4026-B692-06A3BCF92CB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-168" yWindow="108" windowWidth="22116" windowHeight="11352" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Oikeudet" sheetId="1" r:id="rId1"/>
@@ -39,10 +39,10 @@
   </definedNames>
   <calcPr calcId="0"/>
   <customWorkbookViews>
+    <customWorkbookView name="Microsoft Office User - Personal View" guid="{843152D8-333A-1941-83E9-0CB5262068A2}" mergeInterval="0" personalView="1" xWindow="4943" yWindow="119" windowWidth="1728" windowHeight="746" tabRatio="500" activeSheetId="1"/>
+    <customWorkbookView name="Jarno Väyrynen - Personal View" guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" mergeInterval="0" personalView="1" xWindow="48" yWindow="25" windowWidth="2512" windowHeight="1336" tabRatio="500" activeSheetId="1"/>
+    <customWorkbookView name="Microsoft Office User - Oma näkymä" guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" mergeInterval="0" personalView="1" xWindow="1440" yWindow="-515" windowWidth="2056" windowHeight="1366" tabRatio="500" activeSheetId="1"/>
     <customWorkbookView name="Samuli Taskila - Personal View" guid="{B8461C08-78CA-4BAA-BBDB-16DCE44957A3}" mergeInterval="0" personalView="1" xWindow="2326" yWindow="42" windowWidth="2123" windowHeight="1186" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Microsoft Office User - Oma näkymä" guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" mergeInterval="0" personalView="1" xWindow="1440" yWindow="-515" windowWidth="2056" windowHeight="1366" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Jarno Väyrynen - Personal View" guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" mergeInterval="0" personalView="1" xWindow="48" yWindow="25" windowWidth="2512" windowHeight="1336" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Microsoft Office User - Personal View" guid="{843152D8-333A-1941-83E9-0CB5262068A2}" mergeInterval="0" personalView="1" xWindow="4943" yWindow="119" windowWidth="1728" windowHeight="746" tabRatio="500" activeSheetId="1"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -112,7 +112,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2013" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1995" uniqueCount="275">
   <si>
     <t xml:space="preserve">Roolimääritysten selitykset: </t>
   </si>
@@ -1393,7 +1393,7 @@
 </file>
 
 <file path=xl/revisions/revisionHeaders.xml><?xml version="1.0" encoding="utf-8"?>
-<headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" guid="{AFB060D9-1129-4A2B-9A21-20692074B2F4}" diskRevisions="1" revisionId="302" version="16">
+<headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" guid="{65DB2B6E-EAE6-4BCB-9E6B-6C0CCEFA17C2}" diskRevisions="1" revisionId="320" version="17">
   <header guid="{8EBC2E30-8A6E-AD43-9F6F-B4500CF04203}" dateTime="2024-06-11T12:49:05" maxSheetId="3" userName="Jarno Väyrynen" r:id="rId9" minRId="87" maxRId="97">
     <sheetIdMap count="2">
       <sheetId val="1"/>
@@ -1466,6 +1466,12 @@
       <sheetId val="2"/>
     </sheetIdMap>
   </header>
+  <header guid="{65DB2B6E-EAE6-4BCB-9E6B-6C0CCEFA17C2}" dateTime="2025-05-27T14:04:27" maxSheetId="3" userName="Samuli Taskila" r:id="rId21" minRId="303" maxRId="320">
+    <sheetIdMap count="2">
+      <sheetId val="1"/>
+      <sheetId val="2"/>
+    </sheetIdMap>
+  </header>
 </headers>
 </file>
 
@@ -2082,6 +2088,155 @@
         <t>Tiemerkintä / Kustannukset</t>
       </is>
     </nc>
+  </rcc>
+</revisions>
+</file>
+
+<file path=xl/revisions/revisionLog13.xml><?xml version="1.0" encoding="utf-8"?>
+<revisions xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <rcc rId="303" sId="1">
+    <oc r="E24" t="inlineStr">
+      <is>
+        <t>R*,W</t>
+      </is>
+    </oc>
+    <nc r="E24"/>
+  </rcc>
+  <rcc rId="304" sId="1">
+    <oc r="F24" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </oc>
+    <nc r="F24"/>
+  </rcc>
+  <rcc rId="305" sId="1">
+    <oc r="G24" t="inlineStr">
+      <is>
+        <t>R*,W+</t>
+      </is>
+    </oc>
+    <nc r="G24"/>
+  </rcc>
+  <rcc rId="306" sId="1">
+    <oc r="H24" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </oc>
+    <nc r="H24"/>
+  </rcc>
+  <rcc rId="307" sId="1">
+    <oc r="I24" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </oc>
+    <nc r="I24"/>
+  </rcc>
+  <rcc rId="308" sId="1">
+    <oc r="J24" t="inlineStr">
+      <is>
+        <t>R,W</t>
+      </is>
+    </oc>
+    <nc r="J24"/>
+  </rcc>
+  <rcc rId="309" sId="1">
+    <oc r="K24" t="inlineStr">
+      <is>
+        <t>R*,W*</t>
+      </is>
+    </oc>
+    <nc r="K24"/>
+  </rcc>
+  <rcc rId="310" sId="1">
+    <oc r="M24" t="inlineStr">
+      <is>
+        <t>R,W</t>
+      </is>
+    </oc>
+    <nc r="M24"/>
+  </rcc>
+  <rcc rId="311" sId="1">
+    <oc r="N24" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </oc>
+    <nc r="N24"/>
+  </rcc>
+  <rcc rId="312" sId="1">
+    <oc r="O24" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </oc>
+    <nc r="O24"/>
+  </rcc>
+  <rcc rId="313" sId="1">
+    <oc r="P24" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </oc>
+    <nc r="P24"/>
+  </rcc>
+  <rcc rId="314" sId="1">
+    <oc r="Q24" t="inlineStr">
+      <is>
+        <t>R,W</t>
+      </is>
+    </oc>
+    <nc r="Q24"/>
+  </rcc>
+  <rcc rId="315" sId="1">
+    <oc r="R24" t="inlineStr">
+      <is>
+        <t>R+,W+</t>
+      </is>
+    </oc>
+    <nc r="R24"/>
+  </rcc>
+  <rcc rId="316" sId="1">
+    <oc r="T24" t="inlineStr">
+      <is>
+        <t>R+</t>
+      </is>
+    </oc>
+    <nc r="T24"/>
+  </rcc>
+  <rcc rId="317" sId="1">
+    <oc r="U24" t="inlineStr">
+      <is>
+        <t>R,W</t>
+      </is>
+    </oc>
+    <nc r="U24"/>
+  </rcc>
+  <rcc rId="318" sId="1">
+    <oc r="V24" t="inlineStr">
+      <is>
+        <t>R+</t>
+      </is>
+    </oc>
+    <nc r="V24"/>
+  </rcc>
+  <rcc rId="319" sId="1">
+    <oc r="W24" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </oc>
+    <nc r="W24"/>
+  </rcc>
+  <rcc rId="320" sId="1">
+    <oc r="X24" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </oc>
+    <nc r="X24"/>
   </rcc>
 </revisions>
 </file>
@@ -5934,35 +6089,35 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Y139"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="31.6640625" customWidth="1"/>
-    <col min="3" max="3" width="14.109375" customWidth="1"/>
-    <col min="4" max="4" width="30.33203125" customWidth="1"/>
-    <col min="5" max="5" width="26.33203125" customWidth="1"/>
-    <col min="6" max="6" width="12.6640625" customWidth="1"/>
-    <col min="7" max="7" width="14.33203125" customWidth="1"/>
-    <col min="8" max="8" width="10.6640625" customWidth="1"/>
-    <col min="9" max="9" width="18.33203125" customWidth="1"/>
-    <col min="10" max="10" width="25.33203125" customWidth="1"/>
-    <col min="11" max="11" width="40.6640625" customWidth="1"/>
-    <col min="12" max="12" width="38.109375" customWidth="1"/>
-    <col min="13" max="13" width="12.33203125" customWidth="1"/>
-    <col min="14" max="14" width="10.6640625" customWidth="1"/>
-    <col min="15" max="16" width="12.44140625" customWidth="1"/>
-    <col min="17" max="17" width="21.6640625" customWidth="1"/>
+    <col min="2" max="2" width="31.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.140625" customWidth="1"/>
+    <col min="4" max="4" width="30.28515625" customWidth="1"/>
+    <col min="5" max="5" width="26.28515625" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" customWidth="1"/>
+    <col min="7" max="7" width="14.28515625" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" customWidth="1"/>
+    <col min="9" max="9" width="18.28515625" customWidth="1"/>
+    <col min="10" max="10" width="25.28515625" customWidth="1"/>
+    <col min="11" max="11" width="40.7109375" customWidth="1"/>
+    <col min="12" max="12" width="38.140625" customWidth="1"/>
+    <col min="13" max="13" width="12.28515625" customWidth="1"/>
+    <col min="14" max="14" width="10.7109375" customWidth="1"/>
+    <col min="15" max="16" width="12.42578125" customWidth="1"/>
+    <col min="17" max="17" width="21.7109375" customWidth="1"/>
     <col min="18" max="18" width="36" customWidth="1"/>
-    <col min="19" max="19" width="29.6640625" customWidth="1"/>
+    <col min="19" max="19" width="29.7109375" customWidth="1"/>
     <col min="20" max="20" width="15" customWidth="1"/>
-    <col min="21" max="21" width="17.6640625" customWidth="1"/>
-    <col min="22" max="22" width="11.44140625" customWidth="1"/>
-    <col min="23" max="23" width="11.6640625" customWidth="1"/>
-    <col min="24" max="24" width="11.33203125" customWidth="1"/>
+    <col min="21" max="21" width="17.7109375" customWidth="1"/>
+    <col min="22" max="22" width="11.42578125" customWidth="1"/>
+    <col min="23" max="23" width="11.7109375" customWidth="1"/>
+    <col min="24" max="24" width="11.28515625" customWidth="1"/>
     <col min="25" max="25" width="59" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -5983,7 +6138,7 @@
       <c r="N1" s="36"/>
       <c r="O1" s="36"/>
     </row>
-    <row r="2" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="37" t="s">
@@ -6002,7 +6157,7 @@
       <c r="N2" s="37"/>
       <c r="O2" s="37"/>
     </row>
-    <row r="3" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2"/>
       <c r="B3" s="2" t="s">
         <v>3</v>
@@ -6017,10 +6172,10 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C4" s="6"/>
     </row>
-    <row r="5" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="7"/>
       <c r="B5" s="7"/>
       <c r="C5" s="38" t="s">
@@ -6055,7 +6210,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>11</v>
       </c>
@@ -6128,7 +6283,7 @@
       </c>
       <c r="Y6" s="7"/>
     </row>
-    <row r="7" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
         <v>34</v>
       </c>
@@ -6201,7 +6356,7 @@
       </c>
       <c r="Y7" s="13"/>
     </row>
-    <row r="8" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
         <v>34</v>
       </c>
@@ -6260,7 +6415,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
         <v>34</v>
       </c>
@@ -6313,7 +6468,7 @@
       <c r="X9" s="12"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="11" t="s">
         <v>34</v>
       </c>
@@ -6366,7 +6521,7 @@
       <c r="X10" s="12"/>
       <c r="Y10" s="13"/>
     </row>
-    <row r="11" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="11" t="s">
         <v>34</v>
       </c>
@@ -6425,7 +6580,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="11" t="s">
         <v>34</v>
       </c>
@@ -6478,7 +6633,7 @@
       <c r="X12" s="12"/>
       <c r="Y12" s="13"/>
     </row>
-    <row r="13" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="11" t="s">
         <v>34</v>
       </c>
@@ -6545,7 +6700,7 @@
       <c r="X13" s="12"/>
       <c r="Y13" s="13"/>
     </row>
-    <row r="14" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="11" t="s">
         <v>34</v>
       </c>
@@ -6612,7 +6767,7 @@
       <c r="X14" s="12"/>
       <c r="Y14" s="13"/>
     </row>
-    <row r="15" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
         <v>34</v>
       </c>
@@ -6669,7 +6824,7 @@
       <c r="X15" s="12"/>
       <c r="Y15" s="13"/>
     </row>
-    <row r="16" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="11" t="s">
         <v>34</v>
       </c>
@@ -6726,7 +6881,7 @@
       <c r="X16" s="12"/>
       <c r="Y16" s="13"/>
     </row>
-    <row r="17" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="11" t="s">
         <v>34</v>
       </c>
@@ -6783,7 +6938,7 @@
       <c r="X17" s="12"/>
       <c r="Y17" s="13"/>
     </row>
-    <row r="18" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="11" t="s">
         <v>34</v>
       </c>
@@ -6850,7 +7005,7 @@
       <c r="X18" s="12"/>
       <c r="Y18" s="13"/>
     </row>
-    <row r="19" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="11" t="s">
         <v>34</v>
       </c>
@@ -6917,7 +7072,7 @@
       <c r="X19" s="12"/>
       <c r="Y19" s="13"/>
     </row>
-    <row r="20" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="11" t="s">
         <v>34</v>
       </c>
@@ -6972,7 +7127,7 @@
       <c r="X20" s="12"/>
       <c r="Y20" s="13"/>
     </row>
-    <row r="21" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="11" t="s">
         <v>34</v>
       </c>
@@ -7033,7 +7188,7 @@
       <c r="X21" s="12"/>
       <c r="Y21" s="13"/>
     </row>
-    <row r="22" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="11" t="s">
         <v>34</v>
       </c>
@@ -7100,7 +7255,7 @@
       <c r="X22" s="12"/>
       <c r="Y22" s="13"/>
     </row>
-    <row r="23" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="11" t="s">
         <v>34</v>
       </c>
@@ -7173,7 +7328,7 @@
       </c>
       <c r="Y23" s="13"/>
     </row>
-    <row r="24" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="11" t="s">
         <v>34</v>
       </c>
@@ -7184,69 +7339,33 @@
       <c r="D24" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E24" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="F24" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="G24" s="12" t="s">
-        <v>68</v>
-      </c>
-      <c r="H24" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="I24" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="J24" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="K24" s="12" t="s">
-        <v>41</v>
-      </c>
+      <c r="E24" s="12"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="12"/>
+      <c r="H24" s="12"/>
+      <c r="I24" s="12"/>
+      <c r="J24" s="12"/>
+      <c r="K24" s="12"/>
       <c r="L24" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="M24" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="N24" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="O24" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="P24" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q24" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="R24" s="12" t="s">
-        <v>42</v>
-      </c>
+      <c r="M24" s="12"/>
+      <c r="N24" s="12"/>
+      <c r="O24" s="12"/>
+      <c r="P24" s="12"/>
+      <c r="Q24" s="12"/>
+      <c r="R24" s="12"/>
       <c r="S24" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="T24" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="U24" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="V24" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="W24" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="X24" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="T24" s="12"/>
+      <c r="U24" s="12"/>
+      <c r="V24" s="12"/>
+      <c r="W24" s="12"/>
+      <c r="X24" s="12"/>
       <c r="Y24" s="13"/>
     </row>
-    <row r="25" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="11" t="s">
         <v>34</v>
       </c>
@@ -7319,7 +7438,7 @@
       </c>
       <c r="Y25" s="13"/>
     </row>
-    <row r="26" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="11" t="s">
         <v>34</v>
       </c>
@@ -7390,7 +7509,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="27" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="11" t="s">
         <v>34</v>
       </c>
@@ -7459,7 +7578,7 @@
       <c r="X27" s="12"/>
       <c r="Y27" s="13"/>
     </row>
-    <row r="28" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="11" t="s">
         <v>34</v>
       </c>
@@ -7505,7 +7624,7 @@
       </c>
       <c r="Y28" s="13"/>
     </row>
-    <row r="29" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="11" t="s">
         <v>34</v>
       </c>
@@ -7574,7 +7693,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="30" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="11" t="s">
         <v>34</v>
       </c>
@@ -7635,7 +7754,7 @@
       <c r="X30" s="12"/>
       <c r="Y30" s="13"/>
     </row>
-    <row r="31" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="11" t="s">
         <v>34</v>
       </c>
@@ -7692,7 +7811,7 @@
       <c r="X31" s="12"/>
       <c r="Y31" s="13"/>
     </row>
-    <row r="32" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="11" t="s">
         <v>34</v>
       </c>
@@ -7745,7 +7864,7 @@
       <c r="X32" s="12"/>
       <c r="Y32" s="13"/>
     </row>
-    <row r="33" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="11" t="s">
         <v>34</v>
       </c>
@@ -7790,7 +7909,7 @@
       <c r="X33" s="12"/>
       <c r="Y33" s="13"/>
     </row>
-    <row r="34" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="17" t="s">
         <v>34</v>
       </c>
@@ -7819,7 +7938,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="35" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="11" t="s">
         <v>34</v>
       </c>
@@ -7866,7 +7985,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="36" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="11" t="s">
         <v>34</v>
       </c>
@@ -7923,7 +8042,7 @@
       </c>
       <c r="Y36" s="13"/>
     </row>
-    <row r="37" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="11" t="s">
         <v>34</v>
       </c>
@@ -7986,7 +8105,7 @@
       <c r="X37" s="12"/>
       <c r="Y37" s="7"/>
     </row>
-    <row r="38" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="11" t="s">
         <v>34</v>
       </c>
@@ -8039,7 +8158,7 @@
       <c r="X38" s="12"/>
       <c r="Y38" s="13"/>
     </row>
-    <row r="39" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="11" t="s">
         <v>34</v>
       </c>
@@ -8108,7 +8227,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="40" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="11" t="s">
         <v>34</v>
       </c>
@@ -8171,7 +8290,7 @@
       <c r="X40" s="12"/>
       <c r="Y40" s="13"/>
     </row>
-    <row r="41" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="11" t="s">
         <v>34</v>
       </c>
@@ -8236,7 +8355,7 @@
       <c r="X41" s="12"/>
       <c r="Y41" s="13"/>
     </row>
-    <row r="42" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="11" t="s">
         <v>34</v>
       </c>
@@ -8299,7 +8418,7 @@
       <c r="X42" s="12"/>
       <c r="Y42" s="13"/>
     </row>
-    <row r="43" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="11" t="s">
         <v>34</v>
       </c>
@@ -8362,7 +8481,7 @@
       <c r="X43" s="12"/>
       <c r="Y43" s="13"/>
     </row>
-    <row r="44" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="11" t="s">
         <v>34</v>
       </c>
@@ -8425,7 +8544,7 @@
       <c r="X44" s="12"/>
       <c r="Y44" s="13"/>
     </row>
-    <row r="45" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="11" t="s">
         <v>34</v>
       </c>
@@ -8488,7 +8607,7 @@
       <c r="X45" s="12"/>
       <c r="Y45" s="7"/>
     </row>
-    <row r="46" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="11" t="s">
         <v>34</v>
       </c>
@@ -8551,7 +8670,7 @@
       <c r="X46" s="12"/>
       <c r="Y46" s="7"/>
     </row>
-    <row r="47" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="11" t="s">
         <v>34</v>
       </c>
@@ -8614,7 +8733,7 @@
       <c r="X47" s="12"/>
       <c r="Y47" s="7"/>
     </row>
-    <row r="48" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="11" t="s">
         <v>34</v>
       </c>
@@ -8687,7 +8806,7 @@
       </c>
       <c r="Y48" s="13"/>
     </row>
-    <row r="49" spans="1:25" ht="39.6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:25" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A49" s="11" t="s">
         <v>34</v>
       </c>
@@ -8740,7 +8859,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="50" spans="1:25" ht="66" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:25" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A50" s="11" t="s">
         <v>34</v>
       </c>
@@ -8793,7 +8912,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="51" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A51" s="11" t="s">
         <v>34</v>
       </c>
@@ -8844,7 +8963,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="52" spans="1:25" ht="26.4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:25" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A52" s="11" t="s">
         <v>34</v>
       </c>
@@ -8893,7 +9012,7 @@
       <c r="X52" s="15"/>
       <c r="Y52" s="7"/>
     </row>
-    <row r="53" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="17" t="s">
         <v>34</v>
       </c>
@@ -8944,7 +9063,7 @@
       <c r="W53" s="22"/>
       <c r="X53" s="22"/>
     </row>
-    <row r="54" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="11" t="s">
         <v>34</v>
       </c>
@@ -8993,7 +9112,7 @@
       <c r="X54" s="15"/>
       <c r="Y54" s="13"/>
     </row>
-    <row r="55" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="11" t="s">
         <v>34</v>
       </c>
@@ -9026,7 +9145,7 @@
       <c r="X55" s="12"/>
       <c r="Y55" s="13"/>
     </row>
-    <row r="56" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="11" t="s">
         <v>34</v>
       </c>
@@ -9079,7 +9198,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="57" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="11" t="s">
         <v>34</v>
       </c>
@@ -9112,7 +9231,7 @@
       <c r="X57" s="12"/>
       <c r="Y57" s="13"/>
     </row>
-    <row r="58" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="11" t="s">
         <v>34</v>
       </c>
@@ -9163,7 +9282,7 @@
       <c r="X58" s="12"/>
       <c r="Y58" s="13"/>
     </row>
-    <row r="59" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="11" t="s">
         <v>34</v>
       </c>
@@ -9226,7 +9345,7 @@
       <c r="X59" s="12"/>
       <c r="Y59" s="13"/>
     </row>
-    <row r="60" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="23" t="s">
         <v>34</v>
       </c>
@@ -9285,7 +9404,7 @@
       <c r="X60" s="12"/>
       <c r="Y60" s="13"/>
     </row>
-    <row r="61" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="23" t="s">
         <v>34</v>
       </c>
@@ -9346,7 +9465,7 @@
       <c r="X61" s="12"/>
       <c r="Y61" s="13"/>
     </row>
-    <row r="62" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="23" t="s">
         <v>34</v>
       </c>
@@ -9401,7 +9520,7 @@
       <c r="X62" s="12"/>
       <c r="Y62" s="13"/>
     </row>
-    <row r="63" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="11" t="s">
         <v>34</v>
       </c>
@@ -9474,7 +9593,7 @@
       </c>
       <c r="Y63" s="13"/>
     </row>
-    <row r="64" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="11" t="s">
         <v>160</v>
       </c>
@@ -9527,7 +9646,7 @@
       <c r="X64" s="12"/>
       <c r="Y64" s="13"/>
     </row>
-    <row r="65" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="11" t="s">
         <v>160</v>
       </c>
@@ -9580,7 +9699,7 @@
       <c r="X65" s="12"/>
       <c r="Y65" s="13"/>
     </row>
-    <row r="66" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="11" t="s">
         <v>160</v>
       </c>
@@ -9633,7 +9752,7 @@
       <c r="X66" s="12"/>
       <c r="Y66" s="13"/>
     </row>
-    <row r="67" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="11" t="s">
         <v>160</v>
       </c>
@@ -9686,7 +9805,7 @@
       <c r="X67" s="12"/>
       <c r="Y67" s="13"/>
     </row>
-    <row r="68" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="11" t="s">
         <v>160</v>
       </c>
@@ -9733,7 +9852,7 @@
       <c r="X68" s="12"/>
       <c r="Y68" s="13"/>
     </row>
-    <row r="69" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="11" t="s">
         <v>160</v>
       </c>
@@ -9786,7 +9905,7 @@
       <c r="X69" s="12"/>
       <c r="Y69" s="13"/>
     </row>
-    <row r="70" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="11" t="s">
         <v>160</v>
       </c>
@@ -9839,7 +9958,7 @@
       <c r="X70" s="12"/>
       <c r="Y70" s="13"/>
     </row>
-    <row r="71" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="11" t="s">
         <v>160</v>
       </c>
@@ -9892,7 +10011,7 @@
       <c r="X71" s="12"/>
       <c r="Y71" s="13"/>
     </row>
-    <row r="72" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="11" t="s">
         <v>160</v>
       </c>
@@ -9945,7 +10064,7 @@
       <c r="X72" s="12"/>
       <c r="Y72" s="13"/>
     </row>
-    <row r="73" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="11" t="s">
         <v>160</v>
       </c>
@@ -9980,7 +10099,7 @@
       <c r="X73" s="12"/>
       <c r="Y73" s="13"/>
     </row>
-    <row r="74" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="11" t="s">
         <v>160</v>
       </c>
@@ -10051,7 +10170,7 @@
       </c>
       <c r="Y74" s="13"/>
     </row>
-    <row r="75" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="11" t="s">
         <v>160</v>
       </c>
@@ -10124,7 +10243,7 @@
       </c>
       <c r="Y75" s="13"/>
     </row>
-    <row r="76" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="11" t="s">
         <v>160</v>
       </c>
@@ -10195,7 +10314,7 @@
       </c>
       <c r="Y76" s="13"/>
     </row>
-    <row r="77" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="11" t="s">
         <v>160</v>
       </c>
@@ -10266,7 +10385,7 @@
       </c>
       <c r="Y77" s="13"/>
     </row>
-    <row r="78" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="11" t="s">
         <v>160</v>
       </c>
@@ -10301,7 +10420,7 @@
       <c r="X78" s="12"/>
       <c r="Y78" s="13"/>
     </row>
-    <row r="79" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="11" t="s">
         <v>160</v>
       </c>
@@ -10372,7 +10491,7 @@
       </c>
       <c r="Y79" s="13"/>
     </row>
-    <row r="80" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="11" t="s">
         <v>160</v>
       </c>
@@ -10443,7 +10562,7 @@
       </c>
       <c r="Y80" s="13"/>
     </row>
-    <row r="81" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="11" t="s">
         <v>160</v>
       </c>
@@ -10512,7 +10631,7 @@
       </c>
       <c r="Y81" s="13"/>
     </row>
-    <row r="82" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="11" t="s">
         <v>160</v>
       </c>
@@ -10583,7 +10702,7 @@
       </c>
       <c r="Y82" s="13"/>
     </row>
-    <row r="83" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="11" t="s">
         <v>160</v>
       </c>
@@ -10646,7 +10765,7 @@
       </c>
       <c r="Y83" s="13"/>
     </row>
-    <row r="84" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="11" t="s">
         <v>160</v>
       </c>
@@ -10703,7 +10822,7 @@
       <c r="X84" s="12"/>
       <c r="Y84" s="13"/>
     </row>
-    <row r="85" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="11" t="s">
         <v>160</v>
       </c>
@@ -10738,7 +10857,7 @@
       <c r="X85" s="12"/>
       <c r="Y85" s="13"/>
     </row>
-    <row r="86" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="11" t="s">
         <v>160</v>
       </c>
@@ -10773,7 +10892,7 @@
       <c r="X86" s="12"/>
       <c r="Y86" s="13"/>
     </row>
-    <row r="87" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="11" t="s">
         <v>160</v>
       </c>
@@ -10808,7 +10927,7 @@
       <c r="X87" s="12"/>
       <c r="Y87" s="13"/>
     </row>
-    <row r="88" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="11" t="s">
         <v>160</v>
       </c>
@@ -10877,7 +10996,7 @@
       </c>
       <c r="Y88" s="13"/>
     </row>
-    <row r="89" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="11" t="s">
         <v>160</v>
       </c>
@@ -10946,7 +11065,7 @@
       </c>
       <c r="Y89" s="13"/>
     </row>
-    <row r="90" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="11" t="s">
         <v>160</v>
       </c>
@@ -11015,7 +11134,7 @@
       </c>
       <c r="Y90" s="13"/>
     </row>
-    <row r="91" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="11" t="s">
         <v>160</v>
       </c>
@@ -11084,7 +11203,7 @@
       </c>
       <c r="Y91" s="13"/>
     </row>
-    <row r="92" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="11" t="s">
         <v>160</v>
       </c>
@@ -11153,7 +11272,7 @@
       </c>
       <c r="Y92" s="13"/>
     </row>
-    <row r="93" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="11" t="s">
         <v>160</v>
       </c>
@@ -11224,7 +11343,7 @@
       </c>
       <c r="Y93" s="13"/>
     </row>
-    <row r="94" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="11" t="s">
         <v>160</v>
       </c>
@@ -11293,7 +11412,7 @@
       <c r="X94" s="12"/>
       <c r="Y94" s="13"/>
     </row>
-    <row r="95" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="11" t="s">
         <v>160</v>
       </c>
@@ -11362,7 +11481,7 @@
       <c r="X95" s="12"/>
       <c r="Y95" s="13"/>
     </row>
-    <row r="96" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="11" t="s">
         <v>160</v>
       </c>
@@ -11431,7 +11550,7 @@
       <c r="X96" s="12"/>
       <c r="Y96" s="13"/>
     </row>
-    <row r="97" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="11" t="s">
         <v>160</v>
       </c>
@@ -11500,7 +11619,7 @@
       <c r="X97" s="12"/>
       <c r="Y97" s="13"/>
     </row>
-    <row r="98" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="11" t="s">
         <v>160</v>
       </c>
@@ -11569,7 +11688,7 @@
       <c r="X98" s="12"/>
       <c r="Y98" s="13"/>
     </row>
-    <row r="99" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="11" t="s">
         <v>160</v>
       </c>
@@ -11604,7 +11723,7 @@
       <c r="X99" s="12"/>
       <c r="Y99" s="13"/>
     </row>
-    <row r="100" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="11" t="s">
         <v>160</v>
       </c>
@@ -11673,7 +11792,7 @@
       <c r="X100" s="12"/>
       <c r="Y100" s="13"/>
     </row>
-    <row r="101" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="11" t="s">
         <v>160</v>
       </c>
@@ -11726,7 +11845,7 @@
       <c r="X101" s="12"/>
       <c r="Y101" s="13"/>
     </row>
-    <row r="102" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="11" t="s">
         <v>160</v>
       </c>
@@ -11799,7 +11918,7 @@
       </c>
       <c r="Y102" s="13"/>
     </row>
-    <row r="103" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="11" t="s">
         <v>160</v>
       </c>
@@ -11872,7 +11991,7 @@
       </c>
       <c r="Y103" s="13"/>
     </row>
-    <row r="104" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="11" t="s">
         <v>160</v>
       </c>
@@ -11945,7 +12064,7 @@
       </c>
       <c r="Y104" s="13"/>
     </row>
-    <row r="105" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="11" t="s">
         <v>160</v>
       </c>
@@ -12016,7 +12135,7 @@
       </c>
       <c r="Y105" s="13"/>
     </row>
-    <row r="106" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="11" t="s">
         <v>160</v>
       </c>
@@ -12049,7 +12168,7 @@
       <c r="X106" s="12"/>
       <c r="Y106" s="13"/>
     </row>
-    <row r="107" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="11" t="s">
         <v>160</v>
       </c>
@@ -12120,7 +12239,7 @@
       </c>
       <c r="Y107" s="13"/>
     </row>
-    <row r="108" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="11" t="s">
         <v>160</v>
       </c>
@@ -12193,7 +12312,7 @@
       </c>
       <c r="Y108" s="13"/>
     </row>
-    <row r="109" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="11" t="s">
         <v>160</v>
       </c>
@@ -12266,7 +12385,7 @@
       </c>
       <c r="Y109" s="13"/>
     </row>
-    <row r="110" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="11" t="s">
         <v>160</v>
       </c>
@@ -12323,7 +12442,7 @@
       <c r="X110" s="12"/>
       <c r="Y110" s="13"/>
     </row>
-    <row r="111" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="11" t="s">
         <v>201</v>
       </c>
@@ -12398,7 +12517,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="112" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="11" t="s">
         <v>201</v>
       </c>
@@ -12471,7 +12590,7 @@
       </c>
       <c r="Y112" s="35"/>
     </row>
-    <row r="113" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="11" t="s">
         <v>207</v>
       </c>
@@ -12544,7 +12663,7 @@
       </c>
       <c r="Y113" s="7"/>
     </row>
-    <row r="114" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="11" t="s">
         <v>199</v>
       </c>
@@ -12617,7 +12736,7 @@
       </c>
       <c r="Y114" s="13"/>
     </row>
-    <row r="115" spans="1:25" s="30" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:25" s="30" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="27" t="s">
         <v>209</v>
       </c>
@@ -12652,7 +12771,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="116" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="11" t="s">
         <v>209</v>
       </c>
@@ -12697,7 +12816,7 @@
       <c r="X116" s="12"/>
       <c r="Y116" s="7"/>
     </row>
-    <row r="117" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="11" t="s">
         <v>209</v>
       </c>
@@ -12730,7 +12849,7 @@
       <c r="X117" s="12"/>
       <c r="Y117" s="7"/>
     </row>
-    <row r="118" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="11" t="s">
         <v>209</v>
       </c>
@@ -12763,7 +12882,7 @@
       <c r="X118" s="12"/>
       <c r="Y118" s="7"/>
     </row>
-    <row r="119" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="11" t="s">
         <v>209</v>
       </c>
@@ -12796,7 +12915,7 @@
       <c r="X119" s="12"/>
       <c r="Y119" s="7"/>
     </row>
-    <row r="120" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="11" t="s">
         <v>209</v>
       </c>
@@ -12829,7 +12948,7 @@
       <c r="X120" s="12"/>
       <c r="Y120" s="7"/>
     </row>
-    <row r="121" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="11" t="s">
         <v>209</v>
       </c>
@@ -12862,7 +12981,7 @@
       <c r="X121" s="12"/>
       <c r="Y121" s="7"/>
     </row>
-    <row r="122" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" s="11" t="s">
         <v>209</v>
       </c>
@@ -12895,7 +13014,7 @@
       <c r="X122" s="12"/>
       <c r="Y122" s="7"/>
     </row>
-    <row r="123" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="11" t="s">
         <v>209</v>
       </c>
@@ -12928,7 +13047,7 @@
       <c r="X123" s="12"/>
       <c r="Y123" s="7"/>
     </row>
-    <row r="124" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="11" t="s">
         <v>209</v>
       </c>
@@ -12961,7 +13080,7 @@
       <c r="X124" s="15"/>
       <c r="Y124" s="13"/>
     </row>
-    <row r="125" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="11" t="s">
         <v>209</v>
       </c>
@@ -12994,7 +13113,7 @@
       <c r="X125" s="12"/>
       <c r="Y125" s="7"/>
     </row>
-    <row r="126" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="11" t="s">
         <v>209</v>
       </c>
@@ -13027,7 +13146,7 @@
       <c r="X126" s="12"/>
       <c r="Y126" s="7"/>
     </row>
-    <row r="127" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="11" t="s">
         <v>209</v>
       </c>
@@ -13060,7 +13179,7 @@
       <c r="X127" s="12"/>
       <c r="Y127" s="7"/>
     </row>
-    <row r="128" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="11" t="s">
         <v>209</v>
       </c>
@@ -13093,7 +13212,7 @@
       <c r="X128" s="12"/>
       <c r="Y128" s="7"/>
     </row>
-    <row r="129" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129" s="11" t="s">
         <v>209</v>
       </c>
@@ -13126,7 +13245,7 @@
       <c r="X129" s="12"/>
       <c r="Y129" s="7"/>
     </row>
-    <row r="130" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" s="11" t="s">
         <v>209</v>
       </c>
@@ -13159,7 +13278,7 @@
       <c r="X130" s="12"/>
       <c r="Y130" s="7"/>
     </row>
-    <row r="131" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" s="11" t="s">
         <v>209</v>
       </c>
@@ -13192,7 +13311,7 @@
       <c r="X131" s="12"/>
       <c r="Y131" s="7"/>
     </row>
-    <row r="132" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A132" s="11" t="s">
         <v>209</v>
       </c>
@@ -13225,7 +13344,7 @@
       <c r="X132" s="12"/>
       <c r="Y132" s="7"/>
     </row>
-    <row r="133" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A133" s="11" t="s">
         <v>209</v>
       </c>
@@ -13258,7 +13377,7 @@
       <c r="X133" s="12"/>
       <c r="Y133" s="7"/>
     </row>
-    <row r="134" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A134" s="11" t="s">
         <v>209</v>
       </c>
@@ -13291,7 +13410,7 @@
       <c r="X134" s="12"/>
       <c r="Y134" s="7"/>
     </row>
-    <row r="135" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A135" s="11" t="s">
         <v>209</v>
       </c>
@@ -13324,7 +13443,7 @@
       <c r="X135" s="12"/>
       <c r="Y135" s="7"/>
     </row>
-    <row r="136" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" s="11" t="s">
         <v>209</v>
       </c>
@@ -13357,7 +13476,7 @@
       <c r="X136" s="12"/>
       <c r="Y136" s="7"/>
     </row>
-    <row r="137" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" s="11" t="s">
         <v>230</v>
       </c>
@@ -13390,7 +13509,7 @@
       <c r="X137" s="16"/>
       <c r="Y137" s="7"/>
     </row>
-    <row r="138" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" s="11" t="s">
         <v>232</v>
       </c>
@@ -13445,7 +13564,7 @@
       <c r="X138" s="31"/>
       <c r="Y138" s="7"/>
     </row>
-    <row r="139" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A139" s="11" t="s">
         <v>265</v>
       </c>
@@ -13486,9 +13605,15 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{B8461C08-78CA-4BAA-BBDB-16DCE44957A3}" scale="115">
-      <pane xSplit="2" ySplit="6" topLeftCell="C74" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="B89" sqref="B89"/>
+    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="115">
+      <pane xSplit="2" ySplit="6" topLeftCell="Q19" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="Y37" sqref="Y37"/>
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+    </customSheetView>
+    <customSheetView guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" scale="115">
+      <pane xSplit="2" ySplit="6" topLeftCell="C58" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="D81" sqref="D81:X81"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
@@ -13498,15 +13623,9 @@
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
-    <customSheetView guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" scale="115">
-      <pane xSplit="2" ySplit="6" topLeftCell="C58" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="D81" sqref="D81:X81"/>
-      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-    </customSheetView>
-    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="115">
-      <pane xSplit="2" ySplit="6" topLeftCell="Q19" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="Y37" sqref="Y37"/>
+    <customSheetView guid="{B8461C08-78CA-4BAA-BBDB-16DCE44957A3}" scale="115">
+      <pane xSplit="2" ySplit="6" topLeftCell="C74" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="B89" sqref="B89"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
@@ -13528,15 +13647,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E22"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="29.6640625" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="42.33203125" customWidth="1"/>
+    <col min="1" max="1" width="29.7109375" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="42.28515625" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="32" t="s">
         <v>237</v>
       </c>
@@ -13553,7 +13672,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A2" s="33" t="s">
         <v>242</v>
       </c>
@@ -13566,7 +13685,7 @@
       <c r="D2" s="34"/>
       <c r="E2" s="34"/>
     </row>
-    <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A3" s="33" t="s">
         <v>243</v>
       </c>
@@ -13579,7 +13698,7 @@
       <c r="D3" s="34"/>
       <c r="E3" s="34"/>
     </row>
-    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A4" s="33" t="s">
         <v>244</v>
       </c>
@@ -13592,7 +13711,7 @@
       <c r="D4" s="34"/>
       <c r="E4" s="34"/>
     </row>
-    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A5" s="33" t="s">
         <v>245</v>
       </c>
@@ -13607,7 +13726,7 @@
       </c>
       <c r="E5" s="34"/>
     </row>
-    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A6" s="33" t="s">
         <v>247</v>
       </c>
@@ -13622,7 +13741,7 @@
       </c>
       <c r="E6" s="34"/>
     </row>
-    <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.2">
       <c r="A7" s="33" t="s">
         <v>248</v>
       </c>
@@ -13637,7 +13756,7 @@
       </c>
       <c r="E7" s="34"/>
     </row>
-    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.2">
       <c r="A8" s="33" t="s">
         <v>249</v>
       </c>
@@ -13652,7 +13771,7 @@
       </c>
       <c r="E8" s="34"/>
     </row>
-    <row r="9" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A9" s="33" t="s">
         <v>250</v>
       </c>
@@ -13667,7 +13786,7 @@
       </c>
       <c r="E9" s="34"/>
     </row>
-    <row r="10" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A10" s="33" t="s">
         <v>252</v>
       </c>
@@ -13680,7 +13799,7 @@
       <c r="D10" s="34"/>
       <c r="E10" s="34"/>
     </row>
-    <row r="11" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A11" s="33" t="s">
         <v>253</v>
       </c>
@@ -13693,7 +13812,7 @@
       <c r="D11" s="34"/>
       <c r="E11" s="34"/>
     </row>
-    <row r="12" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A12" s="33" t="s">
         <v>254</v>
       </c>
@@ -13706,7 +13825,7 @@
       <c r="D12" s="34"/>
       <c r="E12" s="34"/>
     </row>
-    <row r="13" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A13" s="33" t="s">
         <v>255</v>
       </c>
@@ -13721,7 +13840,7 @@
       </c>
       <c r="E13" s="34"/>
     </row>
-    <row r="14" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A14" s="33" t="s">
         <v>256</v>
       </c>
@@ -13736,7 +13855,7 @@
       </c>
       <c r="E14" s="34"/>
     </row>
-    <row r="15" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A15" s="33" t="s">
         <v>257</v>
       </c>
@@ -13751,7 +13870,7 @@
       </c>
       <c r="E15" s="34"/>
     </row>
-    <row r="16" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A16" s="33" t="s">
         <v>258</v>
       </c>
@@ -13766,7 +13885,7 @@
       </c>
       <c r="E16" s="34"/>
     </row>
-    <row r="17" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A17" s="33" t="s">
         <v>259</v>
       </c>
@@ -13781,7 +13900,7 @@
       </c>
       <c r="E17" s="34"/>
     </row>
-    <row r="18" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A18" s="33" t="s">
         <v>260</v>
       </c>
@@ -13796,7 +13915,7 @@
       </c>
       <c r="E18" s="34"/>
     </row>
-    <row r="19" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A19" s="33" t="s">
         <v>261</v>
       </c>
@@ -13811,7 +13930,7 @@
       </c>
       <c r="E19" s="34"/>
     </row>
-    <row r="20" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A20" s="33" t="s">
         <v>262</v>
       </c>
@@ -13826,7 +13945,7 @@
       </c>
       <c r="E20" s="34"/>
     </row>
-    <row r="21" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A21" s="33" t="s">
         <v>33</v>
       </c>
@@ -13841,7 +13960,7 @@
       </c>
       <c r="E21" s="34"/>
     </row>
-    <row r="22" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A22" s="33" t="s">
         <v>263</v>
       </c>
@@ -13858,7 +13977,12 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{B8461C08-78CA-4BAA-BBDB-16DCE44957A3}" scale="150">
+    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="150">
+      <selection activeCell="A22" sqref="A22"/>
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+    </customSheetView>
+    <customSheetView guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" scale="150">
       <selection activeCell="A22" sqref="A22"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -13868,12 +13992,7 @@
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
-    <customSheetView guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" scale="150">
-      <selection activeCell="A22" sqref="A22"/>
-      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-    </customSheetView>
-    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="150">
+    <customSheetView guid="{B8461C08-78CA-4BAA-BBDB-16DCE44957A3}" scale="150">
       <selection activeCell="A22" sqref="A22"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Anna ELYn pääkäyttäjälle oikeus vahvistaa kustannussuunnitelma
</commit_message>
<xml_diff>
--- a/resources/roolit.xlsx
+++ b/resources/roolit.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\samuli\dev\harjaroot\harja\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maarit.laine/Sources/harja/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:81_{06D8ADD0-19FE-4026-B692-06A3BCF92CB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:81_{6324C653-F24D-0849-8A6C-C70CF39492F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Oikeudet" sheetId="1" r:id="rId1"/>
@@ -26,6 +26,7 @@
     <definedName name="Z_476C495F_6E55_F04C_8145_4E8EBD6B3DE3_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$137</definedName>
     <definedName name="Z_5327B0A1_A5FC_7747_93A1_427B210F3DF4_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$137</definedName>
     <definedName name="Z_56F6E422_2CD8_6B4D_9E39_69A269028D26_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$137</definedName>
+    <definedName name="Z_58389A3C_0D32_7C4E_B363_794E8E4E7869_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$137</definedName>
     <definedName name="Z_6AA8E519_028C_D745_9E2E_8FB60E5B789F_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$137</definedName>
     <definedName name="Z_7A9649F2_657F_9445_B6E6_FE94C6A09957_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$137</definedName>
     <definedName name="Z_8411E1B5_4691_4435_A9A2_147FF80D0D98_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$137</definedName>
@@ -39,10 +40,11 @@
   </definedNames>
   <calcPr calcId="0"/>
   <customWorkbookViews>
+    <customWorkbookView name="Maarit Laine - Personal View" guid="{58389A3C-0D32-7C4E-B363-794E8E4E7869}" mergeInterval="0" personalView="1" maximized="1" yWindow="25" windowWidth="2560" windowHeight="1415" tabRatio="500" activeSheetId="1"/>
+    <customWorkbookView name="Samuli Taskila - Personal View" guid="{B8461C08-78CA-4BAA-BBDB-16DCE44957A3}" mergeInterval="0" personalView="1" xWindow="2326" yWindow="42" windowWidth="2123" windowHeight="1186" tabRatio="500" activeSheetId="1"/>
+    <customWorkbookView name="Microsoft Office User - Oma näkymä" guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" mergeInterval="0" personalView="1" xWindow="1440" yWindow="-515" windowWidth="2056" windowHeight="1366" tabRatio="500" activeSheetId="1"/>
+    <customWorkbookView name="Jarno Väyrynen - Personal View" guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" mergeInterval="0" personalView="1" xWindow="48" yWindow="25" windowWidth="2512" windowHeight="1336" tabRatio="500" activeSheetId="1"/>
     <customWorkbookView name="Microsoft Office User - Personal View" guid="{843152D8-333A-1941-83E9-0CB5262068A2}" mergeInterval="0" personalView="1" xWindow="4943" yWindow="119" windowWidth="1728" windowHeight="746" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Jarno Väyrynen - Personal View" guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" mergeInterval="0" personalView="1" xWindow="48" yWindow="25" windowWidth="2512" windowHeight="1336" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Microsoft Office User - Oma näkymä" guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" mergeInterval="0" personalView="1" xWindow="1440" yWindow="-515" windowWidth="2056" windowHeight="1366" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Samuli Taskila - Personal View" guid="{B8461C08-78CA-4BAA-BBDB-16DCE44957A3}" mergeInterval="0" personalView="1" xWindow="2326" yWindow="42" windowWidth="2123" windowHeight="1186" tabRatio="500" activeSheetId="1"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -112,7 +114,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1995" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1995" uniqueCount="278">
   <si>
     <t xml:space="preserve">Roolimääritysten selitykset: </t>
   </si>
@@ -1009,6 +1011,15 @@
   </si>
   <si>
     <t>Tiemerkintä / Kustannukset</t>
+  </si>
+  <si>
+    <t>R*,W*,vahvistus*</t>
+  </si>
+  <si>
+    <t>R*,W,vahvistus</t>
+  </si>
+  <si>
+    <t>Erikoisoikeudet: vahvistus (kustannussuunnitelman vahvistaminen ja vahvistetun kustannussuunnitelman muokkaus)</t>
   </si>
 </sst>
 </file>
@@ -1393,7 +1404,7 @@
 </file>
 
 <file path=xl/revisions/revisionHeaders.xml><?xml version="1.0" encoding="utf-8"?>
-<headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" guid="{65DB2B6E-EAE6-4BCB-9E6B-6C0CCEFA17C2}" diskRevisions="1" revisionId="320" version="17">
+<headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" guid="{90D29C1C-C846-9949-A28E-46AD1C87D24B}" diskRevisions="1" revisionId="325" version="18">
   <header guid="{8EBC2E30-8A6E-AD43-9F6F-B4500CF04203}" dateTime="2024-06-11T12:49:05" maxSheetId="3" userName="Jarno Väyrynen" r:id="rId9" minRId="87" maxRId="97">
     <sheetIdMap count="2">
       <sheetId val="1"/>
@@ -1472,6 +1483,12 @@
       <sheetId val="2"/>
     </sheetIdMap>
   </header>
+  <header guid="{90D29C1C-C846-9949-A28E-46AD1C87D24B}" dateTime="2025-07-08T13:32:47" maxSheetId="3" userName="Maarit Laine" r:id="rId22" minRId="321" maxRId="324">
+    <sheetIdMap count="2">
+      <sheetId val="1"/>
+      <sheetId val="2"/>
+    </sheetIdMap>
+  </header>
 </headers>
 </file>
 
@@ -2238,6 +2255,63 @@
     </oc>
     <nc r="X24"/>
   </rcc>
+</revisions>
+</file>
+
+<file path=xl/revisions/revisionLog14.xml><?xml version="1.0" encoding="utf-8"?>
+<revisions xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <rcc rId="321" sId="1">
+    <oc r="D11" t="inlineStr">
+      <is>
+        <t>R*,W*</t>
+      </is>
+    </oc>
+    <nc r="D11" t="inlineStr">
+      <is>
+        <t>R*,W*,vahvistus*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="322" sId="1">
+    <oc r="K11" t="inlineStr">
+      <is>
+        <t>R*,W*</t>
+      </is>
+    </oc>
+    <nc r="K11" t="inlineStr">
+      <is>
+        <t>R*,W*,vahvistus*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="323" sId="1">
+    <oc r="L11" t="inlineStr">
+      <is>
+        <t>R*,W</t>
+      </is>
+    </oc>
+    <nc r="L11" t="inlineStr">
+      <is>
+        <t>R*,W,vahvistus</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="324" sId="1">
+    <oc r="Y11" t="inlineStr">
+      <is>
+        <t>Sallitaanko urakoitsijalle hintojen syöttö?</t>
+      </is>
+    </oc>
+    <nc r="Y11" t="inlineStr">
+      <is>
+        <t>Erikoisoikeudet: vahvistus (kustannussuunnitelman vahvistaminen ja vahvistetun kustannussuunnitelman muokkaus)</t>
+      </is>
+    </nc>
+  </rcc>
+  <rdn rId="0" localSheetId="1" customView="1" name="Z_58389A3C_0D32_7C4E_B363_794E8E4E7869_.wvu.FilterData" hidden="1" oldHidden="1">
+    <formula>Oikeudet!$A$5:$Y$137</formula>
+  </rdn>
+  <rcv guid="{58389A3C-0D32-7C4E-B363-794E8E4E7869}" action="add"/>
 </revisions>
 </file>
 
@@ -5904,11 +5978,12 @@
 </file>
 
 <file path=xl/revisions/userNames.xml><?xml version="1.0" encoding="utf-8"?>
-<users xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" count="4">
+<users xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" count="5">
   <userInfo guid="{8EBC2E30-8A6E-AD43-9F6F-B4500CF04203}" name="Jarno Väyrynen" id="-589133089" dateTime="2024-06-10T14:55:26"/>
   <userInfo guid="{CFB45395-62D4-124C-9898-DEF874662F1B}" name="Microsoft Office User" id="-296973103" dateTime="2024-11-20T15:04:38"/>
   <userInfo guid="{CF3F0B66-D3D6-2C4C-93DF-DEE3169712D4}" name="Microsoft Office User" id="-296992802" dateTime="2024-12-13T10:34:14"/>
   <userInfo guid="{64AC07D8-8D49-4F46-96EF-A9E3AD0E8431}" name="Jarno Väyrynen" id="-589128654" dateTime="2025-02-12T12:58:37"/>
+  <userInfo guid="{90D29C1C-C846-9949-A28E-46AD1C87D24B}" name="Maarit Laine" id="-1051111788" dateTime="2025-07-08T12:28:46"/>
 </users>
 </file>
 
@@ -6089,35 +6164,35 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Y139"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="31.7109375" customWidth="1"/>
-    <col min="3" max="3" width="14.140625" customWidth="1"/>
-    <col min="4" max="4" width="30.28515625" customWidth="1"/>
-    <col min="5" max="5" width="26.28515625" customWidth="1"/>
-    <col min="6" max="6" width="12.7109375" customWidth="1"/>
-    <col min="7" max="7" width="14.28515625" customWidth="1"/>
-    <col min="8" max="8" width="10.7109375" customWidth="1"/>
-    <col min="9" max="9" width="18.28515625" customWidth="1"/>
-    <col min="10" max="10" width="25.28515625" customWidth="1"/>
-    <col min="11" max="11" width="40.7109375" customWidth="1"/>
-    <col min="12" max="12" width="38.140625" customWidth="1"/>
-    <col min="13" max="13" width="12.28515625" customWidth="1"/>
-    <col min="14" max="14" width="10.7109375" customWidth="1"/>
-    <col min="15" max="16" width="12.42578125" customWidth="1"/>
-    <col min="17" max="17" width="21.7109375" customWidth="1"/>
+    <col min="2" max="2" width="31.6640625" customWidth="1"/>
+    <col min="3" max="3" width="14.1640625" customWidth="1"/>
+    <col min="4" max="4" width="30.33203125" customWidth="1"/>
+    <col min="5" max="5" width="26.33203125" customWidth="1"/>
+    <col min="6" max="6" width="12.6640625" customWidth="1"/>
+    <col min="7" max="7" width="14.33203125" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" customWidth="1"/>
+    <col min="9" max="9" width="18.33203125" customWidth="1"/>
+    <col min="10" max="10" width="25.33203125" customWidth="1"/>
+    <col min="11" max="11" width="40.6640625" customWidth="1"/>
+    <col min="12" max="12" width="38.1640625" customWidth="1"/>
+    <col min="13" max="13" width="12.33203125" customWidth="1"/>
+    <col min="14" max="14" width="10.6640625" customWidth="1"/>
+    <col min="15" max="16" width="12.5" customWidth="1"/>
+    <col min="17" max="17" width="21.6640625" customWidth="1"/>
     <col min="18" max="18" width="36" customWidth="1"/>
-    <col min="19" max="19" width="29.7109375" customWidth="1"/>
+    <col min="19" max="19" width="29.6640625" customWidth="1"/>
     <col min="20" max="20" width="15" customWidth="1"/>
-    <col min="21" max="21" width="17.7109375" customWidth="1"/>
-    <col min="22" max="22" width="11.42578125" customWidth="1"/>
-    <col min="23" max="23" width="11.7109375" customWidth="1"/>
-    <col min="24" max="24" width="11.28515625" customWidth="1"/>
+    <col min="21" max="21" width="17.6640625" customWidth="1"/>
+    <col min="22" max="22" width="11.5" customWidth="1"/>
+    <col min="23" max="23" width="11.6640625" customWidth="1"/>
+    <col min="24" max="24" width="11.33203125" customWidth="1"/>
     <col min="25" max="25" width="59" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:25" ht="24" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -6138,7 +6213,7 @@
       <c r="N1" s="36"/>
       <c r="O1" s="36"/>
     </row>
-    <row r="2" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="37" t="s">
@@ -6157,7 +6232,7 @@
       <c r="N2" s="37"/>
       <c r="O2" s="37"/>
     </row>
-    <row r="3" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="2"/>
       <c r="B3" s="2" t="s">
         <v>3</v>
@@ -6172,10 +6247,10 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="C4" s="6"/>
     </row>
-    <row r="5" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="7"/>
       <c r="B5" s="7"/>
       <c r="C5" s="38" t="s">
@@ -6210,7 +6285,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="1" t="s">
         <v>11</v>
       </c>
@@ -6283,7 +6358,7 @@
       </c>
       <c r="Y6" s="7"/>
     </row>
-    <row r="7" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="11" t="s">
         <v>34</v>
       </c>
@@ -6356,7 +6431,7 @@
       </c>
       <c r="Y7" s="13"/>
     </row>
-    <row r="8" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="11" t="s">
         <v>34</v>
       </c>
@@ -6415,7 +6490,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="11" t="s">
         <v>34</v>
       </c>
@@ -6468,7 +6543,7 @@
       <c r="X9" s="12"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="11" t="s">
         <v>34</v>
       </c>
@@ -6521,7 +6596,7 @@
       <c r="X10" s="12"/>
       <c r="Y10" s="13"/>
     </row>
-    <row r="11" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="11" t="s">
         <v>34</v>
       </c>
@@ -6530,7 +6605,7 @@
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12" t="s">
-        <v>41</v>
+        <v>275</v>
       </c>
       <c r="E11" s="12" t="s">
         <v>37</v>
@@ -6545,10 +6620,10 @@
         <v>40</v>
       </c>
       <c r="K11" s="12" t="s">
-        <v>41</v>
+        <v>275</v>
       </c>
       <c r="L11" s="12" t="s">
-        <v>37</v>
+        <v>276</v>
       </c>
       <c r="M11" s="12"/>
       <c r="N11" s="12" t="s">
@@ -6577,10 +6652,10 @@
         <v>46</v>
       </c>
       <c r="Y11" s="13" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="12" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="12" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="11" t="s">
         <v>34</v>
       </c>
@@ -6633,7 +6708,7 @@
       <c r="X12" s="12"/>
       <c r="Y12" s="13"/>
     </row>
-    <row r="13" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="11" t="s">
         <v>34</v>
       </c>
@@ -6700,7 +6775,7 @@
       <c r="X13" s="12"/>
       <c r="Y13" s="13"/>
     </row>
-    <row r="14" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="11" t="s">
         <v>34</v>
       </c>
@@ -6767,7 +6842,7 @@
       <c r="X14" s="12"/>
       <c r="Y14" s="13"/>
     </row>
-    <row r="15" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="11" t="s">
         <v>34</v>
       </c>
@@ -6824,7 +6899,7 @@
       <c r="X15" s="12"/>
       <c r="Y15" s="13"/>
     </row>
-    <row r="16" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="11" t="s">
         <v>34</v>
       </c>
@@ -6881,7 +6956,7 @@
       <c r="X16" s="12"/>
       <c r="Y16" s="13"/>
     </row>
-    <row r="17" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="11" t="s">
         <v>34</v>
       </c>
@@ -6938,7 +7013,7 @@
       <c r="X17" s="12"/>
       <c r="Y17" s="13"/>
     </row>
-    <row r="18" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="11" t="s">
         <v>34</v>
       </c>
@@ -7005,7 +7080,7 @@
       <c r="X18" s="12"/>
       <c r="Y18" s="13"/>
     </row>
-    <row r="19" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="11" t="s">
         <v>34</v>
       </c>
@@ -7072,7 +7147,7 @@
       <c r="X19" s="12"/>
       <c r="Y19" s="13"/>
     </row>
-    <row r="20" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="11" t="s">
         <v>34</v>
       </c>
@@ -7127,7 +7202,7 @@
       <c r="X20" s="12"/>
       <c r="Y20" s="13"/>
     </row>
-    <row r="21" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="11" t="s">
         <v>34</v>
       </c>
@@ -7188,7 +7263,7 @@
       <c r="X21" s="12"/>
       <c r="Y21" s="13"/>
     </row>
-    <row r="22" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="11" t="s">
         <v>34</v>
       </c>
@@ -7255,7 +7330,7 @@
       <c r="X22" s="12"/>
       <c r="Y22" s="13"/>
     </row>
-    <row r="23" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="11" t="s">
         <v>34</v>
       </c>
@@ -7328,7 +7403,7 @@
       </c>
       <c r="Y23" s="13"/>
     </row>
-    <row r="24" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="11" t="s">
         <v>34</v>
       </c>
@@ -7365,7 +7440,7 @@
       <c r="X24" s="12"/>
       <c r="Y24" s="13"/>
     </row>
-    <row r="25" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="11" t="s">
         <v>34</v>
       </c>
@@ -7438,7 +7513,7 @@
       </c>
       <c r="Y25" s="13"/>
     </row>
-    <row r="26" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="11" t="s">
         <v>34</v>
       </c>
@@ -7509,7 +7584,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="27" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="11" t="s">
         <v>34</v>
       </c>
@@ -7578,7 +7653,7 @@
       <c r="X27" s="12"/>
       <c r="Y27" s="13"/>
     </row>
-    <row r="28" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="11" t="s">
         <v>34</v>
       </c>
@@ -7624,7 +7699,7 @@
       </c>
       <c r="Y28" s="13"/>
     </row>
-    <row r="29" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="11" t="s">
         <v>34</v>
       </c>
@@ -7693,7 +7768,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="30" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="11" t="s">
         <v>34</v>
       </c>
@@ -7754,7 +7829,7 @@
       <c r="X30" s="12"/>
       <c r="Y30" s="13"/>
     </row>
-    <row r="31" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="11" t="s">
         <v>34</v>
       </c>
@@ -7811,7 +7886,7 @@
       <c r="X31" s="12"/>
       <c r="Y31" s="13"/>
     </row>
-    <row r="32" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="11" t="s">
         <v>34</v>
       </c>
@@ -7864,7 +7939,7 @@
       <c r="X32" s="12"/>
       <c r="Y32" s="13"/>
     </row>
-    <row r="33" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="11" t="s">
         <v>34</v>
       </c>
@@ -7909,7 +7984,7 @@
       <c r="X33" s="12"/>
       <c r="Y33" s="13"/>
     </row>
-    <row r="34" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A34" s="17" t="s">
         <v>34</v>
       </c>
@@ -7938,7 +8013,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="35" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A35" s="11" t="s">
         <v>34</v>
       </c>
@@ -7985,7 +8060,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="36" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A36" s="11" t="s">
         <v>34</v>
       </c>
@@ -8042,7 +8117,7 @@
       </c>
       <c r="Y36" s="13"/>
     </row>
-    <row r="37" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A37" s="11" t="s">
         <v>34</v>
       </c>
@@ -8105,7 +8180,7 @@
       <c r="X37" s="12"/>
       <c r="Y37" s="7"/>
     </row>
-    <row r="38" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A38" s="11" t="s">
         <v>34</v>
       </c>
@@ -8158,7 +8233,7 @@
       <c r="X38" s="12"/>
       <c r="Y38" s="13"/>
     </row>
-    <row r="39" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A39" s="11" t="s">
         <v>34</v>
       </c>
@@ -8227,7 +8302,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="40" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A40" s="11" t="s">
         <v>34</v>
       </c>
@@ -8290,7 +8365,7 @@
       <c r="X40" s="12"/>
       <c r="Y40" s="13"/>
     </row>
-    <row r="41" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A41" s="11" t="s">
         <v>34</v>
       </c>
@@ -8355,7 +8430,7 @@
       <c r="X41" s="12"/>
       <c r="Y41" s="13"/>
     </row>
-    <row r="42" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A42" s="11" t="s">
         <v>34</v>
       </c>
@@ -8418,7 +8493,7 @@
       <c r="X42" s="12"/>
       <c r="Y42" s="13"/>
     </row>
-    <row r="43" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A43" s="11" t="s">
         <v>34</v>
       </c>
@@ -8481,7 +8556,7 @@
       <c r="X43" s="12"/>
       <c r="Y43" s="13"/>
     </row>
-    <row r="44" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A44" s="11" t="s">
         <v>34</v>
       </c>
@@ -8544,7 +8619,7 @@
       <c r="X44" s="12"/>
       <c r="Y44" s="13"/>
     </row>
-    <row r="45" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A45" s="11" t="s">
         <v>34</v>
       </c>
@@ -8607,7 +8682,7 @@
       <c r="X45" s="12"/>
       <c r="Y45" s="7"/>
     </row>
-    <row r="46" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A46" s="11" t="s">
         <v>34</v>
       </c>
@@ -8670,7 +8745,7 @@
       <c r="X46" s="12"/>
       <c r="Y46" s="7"/>
     </row>
-    <row r="47" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A47" s="11" t="s">
         <v>34</v>
       </c>
@@ -8733,7 +8808,7 @@
       <c r="X47" s="12"/>
       <c r="Y47" s="7"/>
     </row>
-    <row r="48" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A48" s="11" t="s">
         <v>34</v>
       </c>
@@ -8806,7 +8881,7 @@
       </c>
       <c r="Y48" s="13"/>
     </row>
-    <row r="49" spans="1:25" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:25" ht="28" x14ac:dyDescent="0.15">
       <c r="A49" s="11" t="s">
         <v>34</v>
       </c>
@@ -8859,7 +8934,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="50" spans="1:25" ht="76.5" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:25" ht="70" x14ac:dyDescent="0.15">
       <c r="A50" s="11" t="s">
         <v>34</v>
       </c>
@@ -8912,7 +8987,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="51" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:25" x14ac:dyDescent="0.15">
       <c r="A51" s="11" t="s">
         <v>34</v>
       </c>
@@ -8963,7 +9038,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="52" spans="1:25" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:25" ht="14" x14ac:dyDescent="0.15">
       <c r="A52" s="11" t="s">
         <v>34</v>
       </c>
@@ -9012,7 +9087,7 @@
       <c r="X52" s="15"/>
       <c r="Y52" s="7"/>
     </row>
-    <row r="53" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A53" s="17" t="s">
         <v>34</v>
       </c>
@@ -9063,7 +9138,7 @@
       <c r="W53" s="22"/>
       <c r="X53" s="22"/>
     </row>
-    <row r="54" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A54" s="11" t="s">
         <v>34</v>
       </c>
@@ -9112,7 +9187,7 @@
       <c r="X54" s="15"/>
       <c r="Y54" s="13"/>
     </row>
-    <row r="55" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A55" s="11" t="s">
         <v>34</v>
       </c>
@@ -9145,7 +9220,7 @@
       <c r="X55" s="12"/>
       <c r="Y55" s="13"/>
     </row>
-    <row r="56" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A56" s="11" t="s">
         <v>34</v>
       </c>
@@ -9198,7 +9273,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="57" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A57" s="11" t="s">
         <v>34</v>
       </c>
@@ -9231,7 +9306,7 @@
       <c r="X57" s="12"/>
       <c r="Y57" s="13"/>
     </row>
-    <row r="58" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A58" s="11" t="s">
         <v>34</v>
       </c>
@@ -9282,7 +9357,7 @@
       <c r="X58" s="12"/>
       <c r="Y58" s="13"/>
     </row>
-    <row r="59" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A59" s="11" t="s">
         <v>34</v>
       </c>
@@ -9345,7 +9420,7 @@
       <c r="X59" s="12"/>
       <c r="Y59" s="13"/>
     </row>
-    <row r="60" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A60" s="23" t="s">
         <v>34</v>
       </c>
@@ -9404,7 +9479,7 @@
       <c r="X60" s="12"/>
       <c r="Y60" s="13"/>
     </row>
-    <row r="61" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A61" s="23" t="s">
         <v>34</v>
       </c>
@@ -9465,7 +9540,7 @@
       <c r="X61" s="12"/>
       <c r="Y61" s="13"/>
     </row>
-    <row r="62" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A62" s="23" t="s">
         <v>34</v>
       </c>
@@ -9520,7 +9595,7 @@
       <c r="X62" s="12"/>
       <c r="Y62" s="13"/>
     </row>
-    <row r="63" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A63" s="11" t="s">
         <v>34</v>
       </c>
@@ -9593,7 +9668,7 @@
       </c>
       <c r="Y63" s="13"/>
     </row>
-    <row r="64" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A64" s="11" t="s">
         <v>160</v>
       </c>
@@ -9646,7 +9721,7 @@
       <c r="X64" s="12"/>
       <c r="Y64" s="13"/>
     </row>
-    <row r="65" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A65" s="11" t="s">
         <v>160</v>
       </c>
@@ -9699,7 +9774,7 @@
       <c r="X65" s="12"/>
       <c r="Y65" s="13"/>
     </row>
-    <row r="66" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A66" s="11" t="s">
         <v>160</v>
       </c>
@@ -9752,7 +9827,7 @@
       <c r="X66" s="12"/>
       <c r="Y66" s="13"/>
     </row>
-    <row r="67" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A67" s="11" t="s">
         <v>160</v>
       </c>
@@ -9805,7 +9880,7 @@
       <c r="X67" s="12"/>
       <c r="Y67" s="13"/>
     </row>
-    <row r="68" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A68" s="11" t="s">
         <v>160</v>
       </c>
@@ -9852,7 +9927,7 @@
       <c r="X68" s="12"/>
       <c r="Y68" s="13"/>
     </row>
-    <row r="69" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A69" s="11" t="s">
         <v>160</v>
       </c>
@@ -9905,7 +9980,7 @@
       <c r="X69" s="12"/>
       <c r="Y69" s="13"/>
     </row>
-    <row r="70" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A70" s="11" t="s">
         <v>160</v>
       </c>
@@ -9958,7 +10033,7 @@
       <c r="X70" s="12"/>
       <c r="Y70" s="13"/>
     </row>
-    <row r="71" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A71" s="11" t="s">
         <v>160</v>
       </c>
@@ -10011,7 +10086,7 @@
       <c r="X71" s="12"/>
       <c r="Y71" s="13"/>
     </row>
-    <row r="72" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A72" s="11" t="s">
         <v>160</v>
       </c>
@@ -10064,7 +10139,7 @@
       <c r="X72" s="12"/>
       <c r="Y72" s="13"/>
     </row>
-    <row r="73" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A73" s="11" t="s">
         <v>160</v>
       </c>
@@ -10099,7 +10174,7 @@
       <c r="X73" s="12"/>
       <c r="Y73" s="13"/>
     </row>
-    <row r="74" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A74" s="11" t="s">
         <v>160</v>
       </c>
@@ -10170,7 +10245,7 @@
       </c>
       <c r="Y74" s="13"/>
     </row>
-    <row r="75" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A75" s="11" t="s">
         <v>160</v>
       </c>
@@ -10243,7 +10318,7 @@
       </c>
       <c r="Y75" s="13"/>
     </row>
-    <row r="76" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A76" s="11" t="s">
         <v>160</v>
       </c>
@@ -10314,7 +10389,7 @@
       </c>
       <c r="Y76" s="13"/>
     </row>
-    <row r="77" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A77" s="11" t="s">
         <v>160</v>
       </c>
@@ -10385,7 +10460,7 @@
       </c>
       <c r="Y77" s="13"/>
     </row>
-    <row r="78" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A78" s="11" t="s">
         <v>160</v>
       </c>
@@ -10420,7 +10495,7 @@
       <c r="X78" s="12"/>
       <c r="Y78" s="13"/>
     </row>
-    <row r="79" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A79" s="11" t="s">
         <v>160</v>
       </c>
@@ -10491,7 +10566,7 @@
       </c>
       <c r="Y79" s="13"/>
     </row>
-    <row r="80" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A80" s="11" t="s">
         <v>160</v>
       </c>
@@ -10562,7 +10637,7 @@
       </c>
       <c r="Y80" s="13"/>
     </row>
-    <row r="81" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A81" s="11" t="s">
         <v>160</v>
       </c>
@@ -10631,7 +10706,7 @@
       </c>
       <c r="Y81" s="13"/>
     </row>
-    <row r="82" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A82" s="11" t="s">
         <v>160</v>
       </c>
@@ -10702,7 +10777,7 @@
       </c>
       <c r="Y82" s="13"/>
     </row>
-    <row r="83" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A83" s="11" t="s">
         <v>160</v>
       </c>
@@ -10765,7 +10840,7 @@
       </c>
       <c r="Y83" s="13"/>
     </row>
-    <row r="84" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A84" s="11" t="s">
         <v>160</v>
       </c>
@@ -10822,7 +10897,7 @@
       <c r="X84" s="12"/>
       <c r="Y84" s="13"/>
     </row>
-    <row r="85" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A85" s="11" t="s">
         <v>160</v>
       </c>
@@ -10857,7 +10932,7 @@
       <c r="X85" s="12"/>
       <c r="Y85" s="13"/>
     </row>
-    <row r="86" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A86" s="11" t="s">
         <v>160</v>
       </c>
@@ -10892,7 +10967,7 @@
       <c r="X86" s="12"/>
       <c r="Y86" s="13"/>
     </row>
-    <row r="87" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A87" s="11" t="s">
         <v>160</v>
       </c>
@@ -10927,7 +11002,7 @@
       <c r="X87" s="12"/>
       <c r="Y87" s="13"/>
     </row>
-    <row r="88" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A88" s="11" t="s">
         <v>160</v>
       </c>
@@ -10996,7 +11071,7 @@
       </c>
       <c r="Y88" s="13"/>
     </row>
-    <row r="89" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A89" s="11" t="s">
         <v>160</v>
       </c>
@@ -11065,7 +11140,7 @@
       </c>
       <c r="Y89" s="13"/>
     </row>
-    <row r="90" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A90" s="11" t="s">
         <v>160</v>
       </c>
@@ -11134,7 +11209,7 @@
       </c>
       <c r="Y90" s="13"/>
     </row>
-    <row r="91" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A91" s="11" t="s">
         <v>160</v>
       </c>
@@ -11203,7 +11278,7 @@
       </c>
       <c r="Y91" s="13"/>
     </row>
-    <row r="92" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A92" s="11" t="s">
         <v>160</v>
       </c>
@@ -11272,7 +11347,7 @@
       </c>
       <c r="Y92" s="13"/>
     </row>
-    <row r="93" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A93" s="11" t="s">
         <v>160</v>
       </c>
@@ -11343,7 +11418,7 @@
       </c>
       <c r="Y93" s="13"/>
     </row>
-    <row r="94" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A94" s="11" t="s">
         <v>160</v>
       </c>
@@ -11412,7 +11487,7 @@
       <c r="X94" s="12"/>
       <c r="Y94" s="13"/>
     </row>
-    <row r="95" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A95" s="11" t="s">
         <v>160</v>
       </c>
@@ -11481,7 +11556,7 @@
       <c r="X95" s="12"/>
       <c r="Y95" s="13"/>
     </row>
-    <row r="96" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A96" s="11" t="s">
         <v>160</v>
       </c>
@@ -11550,7 +11625,7 @@
       <c r="X96" s="12"/>
       <c r="Y96" s="13"/>
     </row>
-    <row r="97" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A97" s="11" t="s">
         <v>160</v>
       </c>
@@ -11619,7 +11694,7 @@
       <c r="X97" s="12"/>
       <c r="Y97" s="13"/>
     </row>
-    <row r="98" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A98" s="11" t="s">
         <v>160</v>
       </c>
@@ -11688,7 +11763,7 @@
       <c r="X98" s="12"/>
       <c r="Y98" s="13"/>
     </row>
-    <row r="99" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A99" s="11" t="s">
         <v>160</v>
       </c>
@@ -11723,7 +11798,7 @@
       <c r="X99" s="12"/>
       <c r="Y99" s="13"/>
     </row>
-    <row r="100" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A100" s="11" t="s">
         <v>160</v>
       </c>
@@ -11792,7 +11867,7 @@
       <c r="X100" s="12"/>
       <c r="Y100" s="13"/>
     </row>
-    <row r="101" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A101" s="11" t="s">
         <v>160</v>
       </c>
@@ -11845,7 +11920,7 @@
       <c r="X101" s="12"/>
       <c r="Y101" s="13"/>
     </row>
-    <row r="102" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A102" s="11" t="s">
         <v>160</v>
       </c>
@@ -11918,7 +11993,7 @@
       </c>
       <c r="Y102" s="13"/>
     </row>
-    <row r="103" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A103" s="11" t="s">
         <v>160</v>
       </c>
@@ -11991,7 +12066,7 @@
       </c>
       <c r="Y103" s="13"/>
     </row>
-    <row r="104" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A104" s="11" t="s">
         <v>160</v>
       </c>
@@ -12064,7 +12139,7 @@
       </c>
       <c r="Y104" s="13"/>
     </row>
-    <row r="105" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A105" s="11" t="s">
         <v>160</v>
       </c>
@@ -12135,7 +12210,7 @@
       </c>
       <c r="Y105" s="13"/>
     </row>
-    <row r="106" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A106" s="11" t="s">
         <v>160</v>
       </c>
@@ -12168,7 +12243,7 @@
       <c r="X106" s="12"/>
       <c r="Y106" s="13"/>
     </row>
-    <row r="107" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A107" s="11" t="s">
         <v>160</v>
       </c>
@@ -12239,7 +12314,7 @@
       </c>
       <c r="Y107" s="13"/>
     </row>
-    <row r="108" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A108" s="11" t="s">
         <v>160</v>
       </c>
@@ -12312,7 +12387,7 @@
       </c>
       <c r="Y108" s="13"/>
     </row>
-    <row r="109" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A109" s="11" t="s">
         <v>160</v>
       </c>
@@ -12385,7 +12460,7 @@
       </c>
       <c r="Y109" s="13"/>
     </row>
-    <row r="110" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A110" s="11" t="s">
         <v>160</v>
       </c>
@@ -12442,7 +12517,7 @@
       <c r="X110" s="12"/>
       <c r="Y110" s="13"/>
     </row>
-    <row r="111" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A111" s="11" t="s">
         <v>201</v>
       </c>
@@ -12517,7 +12592,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="112" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A112" s="11" t="s">
         <v>201</v>
       </c>
@@ -12590,7 +12665,7 @@
       </c>
       <c r="Y112" s="35"/>
     </row>
-    <row r="113" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A113" s="11" t="s">
         <v>207</v>
       </c>
@@ -12663,7 +12738,7 @@
       </c>
       <c r="Y113" s="7"/>
     </row>
-    <row r="114" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A114" s="11" t="s">
         <v>199</v>
       </c>
@@ -12736,7 +12811,7 @@
       </c>
       <c r="Y114" s="13"/>
     </row>
-    <row r="115" spans="1:25" s="30" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:25" s="30" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A115" s="27" t="s">
         <v>209</v>
       </c>
@@ -12771,7 +12846,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="116" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A116" s="11" t="s">
         <v>209</v>
       </c>
@@ -12816,7 +12891,7 @@
       <c r="X116" s="12"/>
       <c r="Y116" s="7"/>
     </row>
-    <row r="117" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A117" s="11" t="s">
         <v>209</v>
       </c>
@@ -12849,7 +12924,7 @@
       <c r="X117" s="12"/>
       <c r="Y117" s="7"/>
     </row>
-    <row r="118" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A118" s="11" t="s">
         <v>209</v>
       </c>
@@ -12882,7 +12957,7 @@
       <c r="X118" s="12"/>
       <c r="Y118" s="7"/>
     </row>
-    <row r="119" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A119" s="11" t="s">
         <v>209</v>
       </c>
@@ -12915,7 +12990,7 @@
       <c r="X119" s="12"/>
       <c r="Y119" s="7"/>
     </row>
-    <row r="120" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A120" s="11" t="s">
         <v>209</v>
       </c>
@@ -12948,7 +13023,7 @@
       <c r="X120" s="12"/>
       <c r="Y120" s="7"/>
     </row>
-    <row r="121" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A121" s="11" t="s">
         <v>209</v>
       </c>
@@ -12981,7 +13056,7 @@
       <c r="X121" s="12"/>
       <c r="Y121" s="7"/>
     </row>
-    <row r="122" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A122" s="11" t="s">
         <v>209</v>
       </c>
@@ -13014,7 +13089,7 @@
       <c r="X122" s="12"/>
       <c r="Y122" s="7"/>
     </row>
-    <row r="123" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A123" s="11" t="s">
         <v>209</v>
       </c>
@@ -13047,7 +13122,7 @@
       <c r="X123" s="12"/>
       <c r="Y123" s="7"/>
     </row>
-    <row r="124" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A124" s="11" t="s">
         <v>209</v>
       </c>
@@ -13080,7 +13155,7 @@
       <c r="X124" s="15"/>
       <c r="Y124" s="13"/>
     </row>
-    <row r="125" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A125" s="11" t="s">
         <v>209</v>
       </c>
@@ -13113,7 +13188,7 @@
       <c r="X125" s="12"/>
       <c r="Y125" s="7"/>
     </row>
-    <row r="126" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A126" s="11" t="s">
         <v>209</v>
       </c>
@@ -13146,7 +13221,7 @@
       <c r="X126" s="12"/>
       <c r="Y126" s="7"/>
     </row>
-    <row r="127" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A127" s="11" t="s">
         <v>209</v>
       </c>
@@ -13179,7 +13254,7 @@
       <c r="X127" s="12"/>
       <c r="Y127" s="7"/>
     </row>
-    <row r="128" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A128" s="11" t="s">
         <v>209</v>
       </c>
@@ -13212,7 +13287,7 @@
       <c r="X128" s="12"/>
       <c r="Y128" s="7"/>
     </row>
-    <row r="129" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A129" s="11" t="s">
         <v>209</v>
       </c>
@@ -13245,7 +13320,7 @@
       <c r="X129" s="12"/>
       <c r="Y129" s="7"/>
     </row>
-    <row r="130" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A130" s="11" t="s">
         <v>209</v>
       </c>
@@ -13278,7 +13353,7 @@
       <c r="X130" s="12"/>
       <c r="Y130" s="7"/>
     </row>
-    <row r="131" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A131" s="11" t="s">
         <v>209</v>
       </c>
@@ -13311,7 +13386,7 @@
       <c r="X131" s="12"/>
       <c r="Y131" s="7"/>
     </row>
-    <row r="132" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A132" s="11" t="s">
         <v>209</v>
       </c>
@@ -13344,7 +13419,7 @@
       <c r="X132" s="12"/>
       <c r="Y132" s="7"/>
     </row>
-    <row r="133" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A133" s="11" t="s">
         <v>209</v>
       </c>
@@ -13377,7 +13452,7 @@
       <c r="X133" s="12"/>
       <c r="Y133" s="7"/>
     </row>
-    <row r="134" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A134" s="11" t="s">
         <v>209</v>
       </c>
@@ -13410,7 +13485,7 @@
       <c r="X134" s="12"/>
       <c r="Y134" s="7"/>
     </row>
-    <row r="135" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A135" s="11" t="s">
         <v>209</v>
       </c>
@@ -13443,7 +13518,7 @@
       <c r="X135" s="12"/>
       <c r="Y135" s="7"/>
     </row>
-    <row r="136" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A136" s="11" t="s">
         <v>209</v>
       </c>
@@ -13476,7 +13551,7 @@
       <c r="X136" s="12"/>
       <c r="Y136" s="7"/>
     </row>
-    <row r="137" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A137" s="11" t="s">
         <v>230</v>
       </c>
@@ -13509,7 +13584,7 @@
       <c r="X137" s="16"/>
       <c r="Y137" s="7"/>
     </row>
-    <row r="138" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A138" s="11" t="s">
         <v>232</v>
       </c>
@@ -13564,7 +13639,7 @@
       <c r="X138" s="31"/>
       <c r="Y138" s="7"/>
     </row>
-    <row r="139" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A139" s="11" t="s">
         <v>265</v>
       </c>
@@ -13605,9 +13680,21 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="115">
-      <pane xSplit="2" ySplit="6" topLeftCell="Q19" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="Y37" sqref="Y37"/>
+    <customSheetView guid="{58389A3C-0D32-7C4E-B363-794E8E4E7869}" scale="162">
+      <pane xSplit="2" ySplit="6" topLeftCell="K7" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="K17" sqref="K17"/>
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+    </customSheetView>
+    <customSheetView guid="{B8461C08-78CA-4BAA-BBDB-16DCE44957A3}" scale="115">
+      <pane xSplit="2" ySplit="6" topLeftCell="C74" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="B89" sqref="B89"/>
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+    </customSheetView>
+    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="130">
+      <pane xSplit="2" ySplit="6" topLeftCell="C53" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="B71" sqref="B71"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
@@ -13617,15 +13704,9 @@
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
-    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="130">
-      <pane xSplit="2" ySplit="6" topLeftCell="C53" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="B71" sqref="B71"/>
-      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-    </customSheetView>
-    <customSheetView guid="{B8461C08-78CA-4BAA-BBDB-16DCE44957A3}" scale="115">
-      <pane xSplit="2" ySplit="6" topLeftCell="C74" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="B89" sqref="B89"/>
+    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="115">
+      <pane xSplit="2" ySplit="6" topLeftCell="Q19" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="Y37" sqref="Y37"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
@@ -13647,15 +13728,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E22"/>
-  <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="29.7109375" customWidth="1"/>
-    <col min="2" max="2" width="28.28515625" customWidth="1"/>
-    <col min="3" max="3" width="42.28515625" customWidth="1"/>
+    <col min="1" max="1" width="29.6640625" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="3" max="3" width="42.33203125" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="32" t="s">
         <v>237</v>
       </c>
@@ -13672,7 +13753,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="33" t="s">
         <v>242</v>
       </c>
@@ -13685,7 +13766,7 @@
       <c r="D2" s="34"/>
       <c r="E2" s="34"/>
     </row>
-    <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A3" s="33" t="s">
         <v>243</v>
       </c>
@@ -13698,7 +13779,7 @@
       <c r="D3" s="34"/>
       <c r="E3" s="34"/>
     </row>
-    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" s="33" t="s">
         <v>244</v>
       </c>
@@ -13711,7 +13792,7 @@
       <c r="D4" s="34"/>
       <c r="E4" s="34"/>
     </row>
-    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" s="33" t="s">
         <v>245</v>
       </c>
@@ -13726,7 +13807,7 @@
       </c>
       <c r="E5" s="34"/>
     </row>
-    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" s="33" t="s">
         <v>247</v>
       </c>
@@ -13741,7 +13822,7 @@
       </c>
       <c r="E6" s="34"/>
     </row>
-    <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A7" s="33" t="s">
         <v>248</v>
       </c>
@@ -13756,7 +13837,7 @@
       </c>
       <c r="E7" s="34"/>
     </row>
-    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="33" t="s">
         <v>249</v>
       </c>
@@ -13771,7 +13852,7 @@
       </c>
       <c r="E8" s="34"/>
     </row>
-    <row r="9" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A9" s="33" t="s">
         <v>250</v>
       </c>
@@ -13786,7 +13867,7 @@
       </c>
       <c r="E9" s="34"/>
     </row>
-    <row r="10" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A10" s="33" t="s">
         <v>252</v>
       </c>
@@ -13799,7 +13880,7 @@
       <c r="D10" s="34"/>
       <c r="E10" s="34"/>
     </row>
-    <row r="11" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A11" s="33" t="s">
         <v>253</v>
       </c>
@@ -13812,7 +13893,7 @@
       <c r="D11" s="34"/>
       <c r="E11" s="34"/>
     </row>
-    <row r="12" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A12" s="33" t="s">
         <v>254</v>
       </c>
@@ -13825,7 +13906,7 @@
       <c r="D12" s="34"/>
       <c r="E12" s="34"/>
     </row>
-    <row r="13" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A13" s="33" t="s">
         <v>255</v>
       </c>
@@ -13840,7 +13921,7 @@
       </c>
       <c r="E13" s="34"/>
     </row>
-    <row r="14" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" s="33" t="s">
         <v>256</v>
       </c>
@@ -13855,7 +13936,7 @@
       </c>
       <c r="E14" s="34"/>
     </row>
-    <row r="15" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A15" s="33" t="s">
         <v>257</v>
       </c>
@@ -13870,7 +13951,7 @@
       </c>
       <c r="E15" s="34"/>
     </row>
-    <row r="16" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A16" s="33" t="s">
         <v>258</v>
       </c>
@@ -13885,7 +13966,7 @@
       </c>
       <c r="E16" s="34"/>
     </row>
-    <row r="17" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A17" s="33" t="s">
         <v>259</v>
       </c>
@@ -13900,7 +13981,7 @@
       </c>
       <c r="E17" s="34"/>
     </row>
-    <row r="18" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A18" s="33" t="s">
         <v>260</v>
       </c>
@@ -13915,7 +13996,7 @@
       </c>
       <c r="E18" s="34"/>
     </row>
-    <row r="19" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A19" s="33" t="s">
         <v>261</v>
       </c>
@@ -13930,7 +14011,7 @@
       </c>
       <c r="E19" s="34"/>
     </row>
-    <row r="20" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A20" s="33" t="s">
         <v>262</v>
       </c>
@@ -13945,7 +14026,7 @@
       </c>
       <c r="E20" s="34"/>
     </row>
-    <row r="21" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A21" s="33" t="s">
         <v>33</v>
       </c>
@@ -13960,7 +14041,7 @@
       </c>
       <c r="E21" s="34"/>
     </row>
-    <row r="22" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A22" s="33" t="s">
         <v>263</v>
       </c>
@@ -13977,7 +14058,17 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="150">
+    <customSheetView guid="{58389A3C-0D32-7C4E-B363-794E8E4E7869}" scale="150">
+      <selection activeCell="A22" sqref="A22"/>
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+    </customSheetView>
+    <customSheetView guid="{B8461C08-78CA-4BAA-BBDB-16DCE44957A3}" scale="150">
+      <selection activeCell="A22" sqref="A22"/>
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+    </customSheetView>
+    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="150">
       <selection activeCell="A22" sqref="A22"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -13987,12 +14078,7 @@
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
-    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="150">
-      <selection activeCell="A22" sqref="A22"/>
-      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-    </customSheetView>
-    <customSheetView guid="{B8461C08-78CA-4BAA-BBDB-16DCE44957A3}" scale="150">
+    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="150">
       <selection activeCell="A22" sqref="A22"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Lisää talvihoitoreittien näkymään oikeuksia
</commit_message>
<xml_diff>
--- a/resources/roolit.xlsx
+++ b/resources/roolit.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maarit.laine/Sources/harja/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\marik\repos\harja\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:81_{6324C653-F24D-0849-8A6C-C70CF39492F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:81_{DF371EFD-4617-424F-A2CA-E75900D9B68E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Oikeudet" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">Oikeudet!$A$5:$Y$137</definedName>
+    <definedName name="Z_13156CEF_1324_493B_BC78_7F90522FC5C9_.wvu.FilterData" localSheetId="0" hidden="1">Oikeudet!$A$5:$Y$137</definedName>
     <definedName name="Z_1CE83972_B6A5_C44D_86E5_E9D9B38739F4_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$137</definedName>
     <definedName name="Z_1DD617EE_F308_3E45_A8EF_4713F47FA0DD_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$137</definedName>
     <definedName name="Z_2064F962_35EF_41F3_8A86_D37B72D177C7_.wvu.FilterData" localSheetId="0">Oikeudet!$A$5:$Y$137</definedName>
@@ -40,11 +41,12 @@
   </definedNames>
   <calcPr calcId="0"/>
   <customWorkbookViews>
+    <customWorkbookView name="Mari Korkka - Oma näkymä" guid="{13156CEF-1324-493B-BC78-7F90522FC5C9}" mergeInterval="0" personalView="1" maximized="1" xWindow="-8" yWindow="-8" windowWidth="1936" windowHeight="1048" tabRatio="500" activeSheetId="1"/>
+    <customWorkbookView name="Microsoft Office User - Personal View" guid="{843152D8-333A-1941-83E9-0CB5262068A2}" mergeInterval="0" personalView="1" xWindow="4943" yWindow="119" windowWidth="1728" windowHeight="746" tabRatio="500" activeSheetId="1"/>
+    <customWorkbookView name="Jarno Väyrynen - Personal View" guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" mergeInterval="0" personalView="1" xWindow="48" yWindow="25" windowWidth="2512" windowHeight="1336" tabRatio="500" activeSheetId="1"/>
+    <customWorkbookView name="Microsoft Office User - Oma näkymä" guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" mergeInterval="0" personalView="1" xWindow="1440" yWindow="-515" windowWidth="2056" windowHeight="1366" tabRatio="500" activeSheetId="1"/>
+    <customWorkbookView name="Samuli Taskila - Personal View" guid="{B8461C08-78CA-4BAA-BBDB-16DCE44957A3}" mergeInterval="0" personalView="1" xWindow="2326" yWindow="42" windowWidth="2123" windowHeight="1186" tabRatio="500" activeSheetId="1"/>
     <customWorkbookView name="Maarit Laine - Personal View" guid="{58389A3C-0D32-7C4E-B363-794E8E4E7869}" mergeInterval="0" personalView="1" maximized="1" yWindow="25" windowWidth="2560" windowHeight="1415" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Samuli Taskila - Personal View" guid="{B8461C08-78CA-4BAA-BBDB-16DCE44957A3}" mergeInterval="0" personalView="1" xWindow="2326" yWindow="42" windowWidth="2123" windowHeight="1186" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Microsoft Office User - Oma näkymä" guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" mergeInterval="0" personalView="1" xWindow="1440" yWindow="-515" windowWidth="2056" windowHeight="1366" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Jarno Väyrynen - Personal View" guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" mergeInterval="0" personalView="1" xWindow="48" yWindow="25" windowWidth="2512" windowHeight="1336" tabRatio="500" activeSheetId="1"/>
-    <customWorkbookView name="Microsoft Office User - Personal View" guid="{843152D8-333A-1941-83E9-0CB5262068A2}" mergeInterval="0" personalView="1" xWindow="4943" yWindow="119" windowWidth="1728" windowHeight="746" tabRatio="500" activeSheetId="1"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -114,7 +116,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1995" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2008" uniqueCount="278">
   <si>
     <t xml:space="preserve">Roolimääritysten selitykset: </t>
   </si>
@@ -1320,7 +1322,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normaali" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1404,7 +1406,7 @@
 </file>
 
 <file path=xl/revisions/revisionHeaders.xml><?xml version="1.0" encoding="utf-8"?>
-<headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" guid="{90D29C1C-C846-9949-A28E-46AD1C87D24B}" diskRevisions="1" revisionId="325" version="18">
+<headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" guid="{EA1ED50D-6247-4B9D-8B0E-0353F2BB6D7D}" diskRevisions="1" revisionId="339" version="19">
   <header guid="{8EBC2E30-8A6E-AD43-9F6F-B4500CF04203}" dateTime="2024-06-11T12:49:05" maxSheetId="3" userName="Jarno Väyrynen" r:id="rId9" minRId="87" maxRId="97">
     <sheetIdMap count="2">
       <sheetId val="1"/>
@@ -1489,6 +1491,12 @@
       <sheetId val="2"/>
     </sheetIdMap>
   </header>
+  <header guid="{EA1ED50D-6247-4B9D-8B0E-0353F2BB6D7D}" dateTime="2025-10-31T15:38:57" maxSheetId="3" userName="Mari Korkka" r:id="rId23" minRId="326" maxRId="338">
+    <sheetIdMap count="2">
+      <sheetId val="1"/>
+      <sheetId val="2"/>
+    </sheetIdMap>
+  </header>
 </headers>
 </file>
 
@@ -2312,6 +2320,309 @@
     <formula>Oikeudet!$A$5:$Y$137</formula>
   </rdn>
   <rcv guid="{58389A3C-0D32-7C4E-B363-794E8E4E7869}" action="add"/>
+</revisions>
+</file>
+
+<file path=xl/revisions/revisionLog15.xml><?xml version="1.0" encoding="utf-8"?>
+<revisions xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <rcc rId="326" sId="1">
+    <nc r="K24" t="inlineStr">
+      <is>
+        <t>R*,W*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="327" sId="1">
+    <nc r="R24" t="inlineStr">
+      <is>
+        <t>R+,W+</t>
+      </is>
+    </nc>
+  </rcc>
+  <rfmt sheetId="1" xfDxf="1" sqref="Q24" start="0" length="0">
+    <dxf>
+      <font>
+        <color auto="1"/>
+        <family val="2"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rcc rId="328" sId="1" xfDxf="1" dxf="1">
+    <nc r="E24" t="inlineStr">
+      <is>
+        <t>R*,W</t>
+      </is>
+    </nc>
+    <ndxf>
+      <font>
+        <color auto="1"/>
+        <family val="2"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </ndxf>
+  </rcc>
+  <rcc rId="329" sId="1" xfDxf="1" dxf="1">
+    <nc r="J24" t="inlineStr">
+      <is>
+        <t>R*,W</t>
+      </is>
+    </nc>
+    <ndxf>
+      <font>
+        <color auto="1"/>
+        <family val="2"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </ndxf>
+  </rcc>
+  <rfmt sheetId="1" xfDxf="1" sqref="F24" start="0" length="0">
+    <dxf>
+      <font>
+        <color auto="1"/>
+        <family val="2"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rcc rId="330" sId="1">
+    <nc r="F24" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rfmt sheetId="1" xfDxf="1" sqref="G24" start="0" length="0">
+    <dxf>
+      <font>
+        <color auto="1"/>
+        <family val="2"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rcc rId="331" sId="1">
+    <nc r="G24" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rfmt sheetId="1" xfDxf="1" sqref="H24" start="0" length="0">
+    <dxf>
+      <font>
+        <color auto="1"/>
+        <family val="2"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rcc rId="332" sId="1">
+    <nc r="H24" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rfmt sheetId="1" xfDxf="1" sqref="I24" start="0" length="0">
+    <dxf>
+      <font>
+        <color auto="1"/>
+        <family val="2"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rcc rId="333" sId="1">
+    <nc r="I24" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rfmt sheetId="1" xfDxf="1" sqref="M24" start="0" length="0">
+    <dxf>
+      <font>
+        <color auto="1"/>
+        <family val="2"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rcc rId="334" sId="1">
+    <nc r="M24" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rfmt sheetId="1" xfDxf="1" sqref="N24" start="0" length="0">
+    <dxf>
+      <font>
+        <color auto="1"/>
+        <family val="2"/>
+      </font>
+      <alignment horizontal="center" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </rfmt>
+  <rcc rId="335" sId="1">
+    <nc r="N24" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="336" sId="1">
+    <nc r="O24" t="inlineStr">
+      <is>
+        <t>R*</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="337" sId="1">
+    <nc r="P24" t="inlineStr">
+      <is>
+        <t>R</t>
+      </is>
+    </nc>
+  </rcc>
+  <rcc rId="338" sId="1">
+    <nc r="Q24" t="inlineStr">
+      <is>
+        <t>R,W</t>
+      </is>
+    </nc>
+  </rcc>
+  <rdn rId="0" localSheetId="1" customView="1" name="Z_13156CEF_1324_493B_BC78_7F90522FC5C9_.wvu.FilterData" hidden="1" oldHidden="1">
+    <formula>Oikeudet!$A$5:$Y$137</formula>
+  </rdn>
+  <rcv guid="{13156CEF-1324-493B-BC78-7F90522FC5C9}" action="add"/>
 </revisions>
 </file>
 
@@ -6164,35 +6475,35 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Y139"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="31.6640625" customWidth="1"/>
-    <col min="3" max="3" width="14.1640625" customWidth="1"/>
-    <col min="4" max="4" width="30.33203125" customWidth="1"/>
-    <col min="5" max="5" width="26.33203125" customWidth="1"/>
-    <col min="6" max="6" width="12.6640625" customWidth="1"/>
-    <col min="7" max="7" width="14.33203125" customWidth="1"/>
-    <col min="8" max="8" width="10.6640625" customWidth="1"/>
-    <col min="9" max="9" width="18.33203125" customWidth="1"/>
-    <col min="10" max="10" width="25.33203125" customWidth="1"/>
-    <col min="11" max="11" width="40.6640625" customWidth="1"/>
-    <col min="12" max="12" width="38.1640625" customWidth="1"/>
-    <col min="13" max="13" width="12.33203125" customWidth="1"/>
-    <col min="14" max="14" width="10.6640625" customWidth="1"/>
-    <col min="15" max="16" width="12.5" customWidth="1"/>
-    <col min="17" max="17" width="21.6640625" customWidth="1"/>
+    <col min="2" max="2" width="31.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.140625" customWidth="1"/>
+    <col min="4" max="4" width="30.28515625" customWidth="1"/>
+    <col min="5" max="5" width="26.28515625" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" customWidth="1"/>
+    <col min="7" max="7" width="14.28515625" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" customWidth="1"/>
+    <col min="9" max="9" width="18.28515625" customWidth="1"/>
+    <col min="10" max="10" width="25.28515625" customWidth="1"/>
+    <col min="11" max="11" width="40.7109375" customWidth="1"/>
+    <col min="12" max="12" width="38.140625" customWidth="1"/>
+    <col min="13" max="13" width="12.28515625" customWidth="1"/>
+    <col min="14" max="14" width="10.7109375" customWidth="1"/>
+    <col min="15" max="16" width="12.42578125" customWidth="1"/>
+    <col min="17" max="17" width="21.7109375" customWidth="1"/>
     <col min="18" max="18" width="36" customWidth="1"/>
-    <col min="19" max="19" width="29.6640625" customWidth="1"/>
+    <col min="19" max="19" width="29.7109375" customWidth="1"/>
     <col min="20" max="20" width="15" customWidth="1"/>
-    <col min="21" max="21" width="17.6640625" customWidth="1"/>
-    <col min="22" max="22" width="11.5" customWidth="1"/>
-    <col min="23" max="23" width="11.6640625" customWidth="1"/>
-    <col min="24" max="24" width="11.33203125" customWidth="1"/>
+    <col min="21" max="21" width="17.7109375" customWidth="1"/>
+    <col min="22" max="22" width="11.42578125" customWidth="1"/>
+    <col min="23" max="23" width="11.7109375" customWidth="1"/>
+    <col min="24" max="24" width="11.28515625" customWidth="1"/>
     <col min="25" max="25" width="59" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="24" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:25" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -6213,7 +6524,7 @@
       <c r="N1" s="36"/>
       <c r="O1" s="36"/>
     </row>
-    <row r="2" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="37" t="s">
@@ -6232,7 +6543,7 @@
       <c r="N2" s="37"/>
       <c r="O2" s="37"/>
     </row>
-    <row r="3" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2"/>
       <c r="B3" s="2" t="s">
         <v>3</v>
@@ -6247,10 +6558,10 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C4" s="6"/>
     </row>
-    <row r="5" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="7"/>
       <c r="B5" s="7"/>
       <c r="C5" s="38" t="s">
@@ -6285,7 +6596,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>11</v>
       </c>
@@ -6358,7 +6669,7 @@
       </c>
       <c r="Y6" s="7"/>
     </row>
-    <row r="7" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
         <v>34</v>
       </c>
@@ -6431,7 +6742,7 @@
       </c>
       <c r="Y7" s="13"/>
     </row>
-    <row r="8" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
         <v>34</v>
       </c>
@@ -6490,7 +6801,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
         <v>34</v>
       </c>
@@ -6543,7 +6854,7 @@
       <c r="X9" s="12"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="11" t="s">
         <v>34</v>
       </c>
@@ -6596,7 +6907,7 @@
       <c r="X10" s="12"/>
       <c r="Y10" s="13"/>
     </row>
-    <row r="11" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="11" t="s">
         <v>34</v>
       </c>
@@ -6655,7 +6966,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="12" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="11" t="s">
         <v>34</v>
       </c>
@@ -6708,7 +7019,7 @@
       <c r="X12" s="12"/>
       <c r="Y12" s="13"/>
     </row>
-    <row r="13" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="11" t="s">
         <v>34</v>
       </c>
@@ -6775,7 +7086,7 @@
       <c r="X13" s="12"/>
       <c r="Y13" s="13"/>
     </row>
-    <row r="14" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="11" t="s">
         <v>34</v>
       </c>
@@ -6842,7 +7153,7 @@
       <c r="X14" s="12"/>
       <c r="Y14" s="13"/>
     </row>
-    <row r="15" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
         <v>34</v>
       </c>
@@ -6899,7 +7210,7 @@
       <c r="X15" s="12"/>
       <c r="Y15" s="13"/>
     </row>
-    <row r="16" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="11" t="s">
         <v>34</v>
       </c>
@@ -6956,7 +7267,7 @@
       <c r="X16" s="12"/>
       <c r="Y16" s="13"/>
     </row>
-    <row r="17" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="11" t="s">
         <v>34</v>
       </c>
@@ -7013,7 +7324,7 @@
       <c r="X17" s="12"/>
       <c r="Y17" s="13"/>
     </row>
-    <row r="18" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="11" t="s">
         <v>34</v>
       </c>
@@ -7080,7 +7391,7 @@
       <c r="X18" s="12"/>
       <c r="Y18" s="13"/>
     </row>
-    <row r="19" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="11" t="s">
         <v>34</v>
       </c>
@@ -7147,7 +7458,7 @@
       <c r="X19" s="12"/>
       <c r="Y19" s="13"/>
     </row>
-    <row r="20" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="11" t="s">
         <v>34</v>
       </c>
@@ -7202,7 +7513,7 @@
       <c r="X20" s="12"/>
       <c r="Y20" s="13"/>
     </row>
-    <row r="21" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="11" t="s">
         <v>34</v>
       </c>
@@ -7263,7 +7574,7 @@
       <c r="X21" s="12"/>
       <c r="Y21" s="13"/>
     </row>
-    <row r="22" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="11" t="s">
         <v>34</v>
       </c>
@@ -7330,7 +7641,7 @@
       <c r="X22" s="12"/>
       <c r="Y22" s="13"/>
     </row>
-    <row r="23" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="11" t="s">
         <v>34</v>
       </c>
@@ -7403,7 +7714,7 @@
       </c>
       <c r="Y23" s="13"/>
     </row>
-    <row r="24" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="11" t="s">
         <v>34</v>
       </c>
@@ -7414,22 +7725,48 @@
       <c r="D24" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E24" s="12"/>
-      <c r="F24" s="12"/>
-      <c r="G24" s="12"/>
-      <c r="H24" s="12"/>
-      <c r="I24" s="12"/>
-      <c r="J24" s="12"/>
-      <c r="K24" s="12"/>
+      <c r="E24" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="F24" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="G24" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="H24" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I24" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="J24" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="K24" s="12" t="s">
+        <v>41</v>
+      </c>
       <c r="L24" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="M24" s="12"/>
-      <c r="N24" s="12"/>
-      <c r="O24" s="12"/>
-      <c r="P24" s="12"/>
-      <c r="Q24" s="12"/>
-      <c r="R24" s="12"/>
+      <c r="M24" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="N24" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="O24" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="P24" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q24" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="R24" s="12" t="s">
+        <v>42</v>
+      </c>
       <c r="S24" s="12" t="s">
         <v>40</v>
       </c>
@@ -7440,7 +7777,7 @@
       <c r="X24" s="12"/>
       <c r="Y24" s="13"/>
     </row>
-    <row r="25" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="11" t="s">
         <v>34</v>
       </c>
@@ -7513,7 +7850,7 @@
       </c>
       <c r="Y25" s="13"/>
     </row>
-    <row r="26" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="11" t="s">
         <v>34</v>
       </c>
@@ -7584,7 +7921,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="27" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="11" t="s">
         <v>34</v>
       </c>
@@ -7653,7 +7990,7 @@
       <c r="X27" s="12"/>
       <c r="Y27" s="13"/>
     </row>
-    <row r="28" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="11" t="s">
         <v>34</v>
       </c>
@@ -7699,7 +8036,7 @@
       </c>
       <c r="Y28" s="13"/>
     </row>
-    <row r="29" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="11" t="s">
         <v>34</v>
       </c>
@@ -7768,7 +8105,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="30" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="11" t="s">
         <v>34</v>
       </c>
@@ -7829,7 +8166,7 @@
       <c r="X30" s="12"/>
       <c r="Y30" s="13"/>
     </row>
-    <row r="31" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="11" t="s">
         <v>34</v>
       </c>
@@ -7886,7 +8223,7 @@
       <c r="X31" s="12"/>
       <c r="Y31" s="13"/>
     </row>
-    <row r="32" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="11" t="s">
         <v>34</v>
       </c>
@@ -7939,7 +8276,7 @@
       <c r="X32" s="12"/>
       <c r="Y32" s="13"/>
     </row>
-    <row r="33" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="11" t="s">
         <v>34</v>
       </c>
@@ -7984,7 +8321,7 @@
       <c r="X33" s="12"/>
       <c r="Y33" s="13"/>
     </row>
-    <row r="34" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="34" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="17" t="s">
         <v>34</v>
       </c>
@@ -8013,7 +8350,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="35" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="11" t="s">
         <v>34</v>
       </c>
@@ -8060,7 +8397,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="36" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="11" t="s">
         <v>34</v>
       </c>
@@ -8117,7 +8454,7 @@
       </c>
       <c r="Y36" s="13"/>
     </row>
-    <row r="37" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="11" t="s">
         <v>34</v>
       </c>
@@ -8180,7 +8517,7 @@
       <c r="X37" s="12"/>
       <c r="Y37" s="7"/>
     </row>
-    <row r="38" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="38" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="11" t="s">
         <v>34</v>
       </c>
@@ -8233,7 +8570,7 @@
       <c r="X38" s="12"/>
       <c r="Y38" s="13"/>
     </row>
-    <row r="39" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="11" t="s">
         <v>34</v>
       </c>
@@ -8302,7 +8639,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="40" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="40" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="11" t="s">
         <v>34</v>
       </c>
@@ -8365,7 +8702,7 @@
       <c r="X40" s="12"/>
       <c r="Y40" s="13"/>
     </row>
-    <row r="41" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="41" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="11" t="s">
         <v>34</v>
       </c>
@@ -8430,7 +8767,7 @@
       <c r="X41" s="12"/>
       <c r="Y41" s="13"/>
     </row>
-    <row r="42" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="42" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="11" t="s">
         <v>34</v>
       </c>
@@ -8493,7 +8830,7 @@
       <c r="X42" s="12"/>
       <c r="Y42" s="13"/>
     </row>
-    <row r="43" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="43" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="11" t="s">
         <v>34</v>
       </c>
@@ -8556,7 +8893,7 @@
       <c r="X43" s="12"/>
       <c r="Y43" s="13"/>
     </row>
-    <row r="44" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="44" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="11" t="s">
         <v>34</v>
       </c>
@@ -8619,7 +8956,7 @@
       <c r="X44" s="12"/>
       <c r="Y44" s="13"/>
     </row>
-    <row r="45" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="45" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="11" t="s">
         <v>34</v>
       </c>
@@ -8682,7 +9019,7 @@
       <c r="X45" s="12"/>
       <c r="Y45" s="7"/>
     </row>
-    <row r="46" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="46" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="11" t="s">
         <v>34</v>
       </c>
@@ -8745,7 +9082,7 @@
       <c r="X46" s="12"/>
       <c r="Y46" s="7"/>
     </row>
-    <row r="47" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="47" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="11" t="s">
         <v>34</v>
       </c>
@@ -8808,7 +9145,7 @@
       <c r="X47" s="12"/>
       <c r="Y47" s="7"/>
     </row>
-    <row r="48" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="48" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="11" t="s">
         <v>34</v>
       </c>
@@ -8881,7 +9218,7 @@
       </c>
       <c r="Y48" s="13"/>
     </row>
-    <row r="49" spans="1:25" ht="28" x14ac:dyDescent="0.15">
+    <row r="49" spans="1:25" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A49" s="11" t="s">
         <v>34</v>
       </c>
@@ -8934,7 +9271,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="50" spans="1:25" ht="70" x14ac:dyDescent="0.15">
+    <row r="50" spans="1:25" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A50" s="11" t="s">
         <v>34</v>
       </c>
@@ -8987,7 +9324,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="51" spans="1:25" x14ac:dyDescent="0.15">
+    <row r="51" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A51" s="11" t="s">
         <v>34</v>
       </c>
@@ -9038,7 +9375,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="52" spans="1:25" ht="14" x14ac:dyDescent="0.15">
+    <row r="52" spans="1:25" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A52" s="11" t="s">
         <v>34</v>
       </c>
@@ -9087,7 +9424,7 @@
       <c r="X52" s="15"/>
       <c r="Y52" s="7"/>
     </row>
-    <row r="53" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="53" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="17" t="s">
         <v>34</v>
       </c>
@@ -9138,7 +9475,7 @@
       <c r="W53" s="22"/>
       <c r="X53" s="22"/>
     </row>
-    <row r="54" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="54" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="11" t="s">
         <v>34</v>
       </c>
@@ -9187,7 +9524,7 @@
       <c r="X54" s="15"/>
       <c r="Y54" s="13"/>
     </row>
-    <row r="55" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="55" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="11" t="s">
         <v>34</v>
       </c>
@@ -9220,7 +9557,7 @@
       <c r="X55" s="12"/>
       <c r="Y55" s="13"/>
     </row>
-    <row r="56" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="56" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="11" t="s">
         <v>34</v>
       </c>
@@ -9273,7 +9610,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="57" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="57" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="11" t="s">
         <v>34</v>
       </c>
@@ -9306,7 +9643,7 @@
       <c r="X57" s="12"/>
       <c r="Y57" s="13"/>
     </row>
-    <row r="58" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="58" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="11" t="s">
         <v>34</v>
       </c>
@@ -9357,7 +9694,7 @@
       <c r="X58" s="12"/>
       <c r="Y58" s="13"/>
     </row>
-    <row r="59" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="59" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="11" t="s">
         <v>34</v>
       </c>
@@ -9420,7 +9757,7 @@
       <c r="X59" s="12"/>
       <c r="Y59" s="13"/>
     </row>
-    <row r="60" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="60" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="23" t="s">
         <v>34</v>
       </c>
@@ -9479,7 +9816,7 @@
       <c r="X60" s="12"/>
       <c r="Y60" s="13"/>
     </row>
-    <row r="61" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="61" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="23" t="s">
         <v>34</v>
       </c>
@@ -9540,7 +9877,7 @@
       <c r="X61" s="12"/>
       <c r="Y61" s="13"/>
     </row>
-    <row r="62" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="62" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="23" t="s">
         <v>34</v>
       </c>
@@ -9595,7 +9932,7 @@
       <c r="X62" s="12"/>
       <c r="Y62" s="13"/>
     </row>
-    <row r="63" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="63" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="11" t="s">
         <v>34</v>
       </c>
@@ -9668,7 +10005,7 @@
       </c>
       <c r="Y63" s="13"/>
     </row>
-    <row r="64" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="64" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="11" t="s">
         <v>160</v>
       </c>
@@ -9721,7 +10058,7 @@
       <c r="X64" s="12"/>
       <c r="Y64" s="13"/>
     </row>
-    <row r="65" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="65" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="11" t="s">
         <v>160</v>
       </c>
@@ -9774,7 +10111,7 @@
       <c r="X65" s="12"/>
       <c r="Y65" s="13"/>
     </row>
-    <row r="66" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="66" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="11" t="s">
         <v>160</v>
       </c>
@@ -9827,7 +10164,7 @@
       <c r="X66" s="12"/>
       <c r="Y66" s="13"/>
     </row>
-    <row r="67" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="67" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="11" t="s">
         <v>160</v>
       </c>
@@ -9880,7 +10217,7 @@
       <c r="X67" s="12"/>
       <c r="Y67" s="13"/>
     </row>
-    <row r="68" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="68" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="11" t="s">
         <v>160</v>
       </c>
@@ -9927,7 +10264,7 @@
       <c r="X68" s="12"/>
       <c r="Y68" s="13"/>
     </row>
-    <row r="69" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="69" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="11" t="s">
         <v>160</v>
       </c>
@@ -9980,7 +10317,7 @@
       <c r="X69" s="12"/>
       <c r="Y69" s="13"/>
     </row>
-    <row r="70" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="70" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="11" t="s">
         <v>160</v>
       </c>
@@ -10033,7 +10370,7 @@
       <c r="X70" s="12"/>
       <c r="Y70" s="13"/>
     </row>
-    <row r="71" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="71" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="11" t="s">
         <v>160</v>
       </c>
@@ -10086,7 +10423,7 @@
       <c r="X71" s="12"/>
       <c r="Y71" s="13"/>
     </row>
-    <row r="72" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="72" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="11" t="s">
         <v>160</v>
       </c>
@@ -10139,7 +10476,7 @@
       <c r="X72" s="12"/>
       <c r="Y72" s="13"/>
     </row>
-    <row r="73" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="73" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="11" t="s">
         <v>160</v>
       </c>
@@ -10174,7 +10511,7 @@
       <c r="X73" s="12"/>
       <c r="Y73" s="13"/>
     </row>
-    <row r="74" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="74" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="11" t="s">
         <v>160</v>
       </c>
@@ -10245,7 +10582,7 @@
       </c>
       <c r="Y74" s="13"/>
     </row>
-    <row r="75" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="75" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="11" t="s">
         <v>160</v>
       </c>
@@ -10318,7 +10655,7 @@
       </c>
       <c r="Y75" s="13"/>
     </row>
-    <row r="76" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="76" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="11" t="s">
         <v>160</v>
       </c>
@@ -10389,7 +10726,7 @@
       </c>
       <c r="Y76" s="13"/>
     </row>
-    <row r="77" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="77" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="11" t="s">
         <v>160</v>
       </c>
@@ -10460,7 +10797,7 @@
       </c>
       <c r="Y77" s="13"/>
     </row>
-    <row r="78" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="78" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="11" t="s">
         <v>160</v>
       </c>
@@ -10495,7 +10832,7 @@
       <c r="X78" s="12"/>
       <c r="Y78" s="13"/>
     </row>
-    <row r="79" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="79" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="11" t="s">
         <v>160</v>
       </c>
@@ -10566,7 +10903,7 @@
       </c>
       <c r="Y79" s="13"/>
     </row>
-    <row r="80" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="80" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="11" t="s">
         <v>160</v>
       </c>
@@ -10637,7 +10974,7 @@
       </c>
       <c r="Y80" s="13"/>
     </row>
-    <row r="81" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="81" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="11" t="s">
         <v>160</v>
       </c>
@@ -10706,7 +11043,7 @@
       </c>
       <c r="Y81" s="13"/>
     </row>
-    <row r="82" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="82" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="11" t="s">
         <v>160</v>
       </c>
@@ -10777,7 +11114,7 @@
       </c>
       <c r="Y82" s="13"/>
     </row>
-    <row r="83" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="83" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="11" t="s">
         <v>160</v>
       </c>
@@ -10840,7 +11177,7 @@
       </c>
       <c r="Y83" s="13"/>
     </row>
-    <row r="84" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="84" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="11" t="s">
         <v>160</v>
       </c>
@@ -10897,7 +11234,7 @@
       <c r="X84" s="12"/>
       <c r="Y84" s="13"/>
     </row>
-    <row r="85" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="85" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="11" t="s">
         <v>160</v>
       </c>
@@ -10932,7 +11269,7 @@
       <c r="X85" s="12"/>
       <c r="Y85" s="13"/>
     </row>
-    <row r="86" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="86" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="11" t="s">
         <v>160</v>
       </c>
@@ -10967,7 +11304,7 @@
       <c r="X86" s="12"/>
       <c r="Y86" s="13"/>
     </row>
-    <row r="87" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="87" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="11" t="s">
         <v>160</v>
       </c>
@@ -11002,7 +11339,7 @@
       <c r="X87" s="12"/>
       <c r="Y87" s="13"/>
     </row>
-    <row r="88" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="88" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="11" t="s">
         <v>160</v>
       </c>
@@ -11071,7 +11408,7 @@
       </c>
       <c r="Y88" s="13"/>
     </row>
-    <row r="89" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="89" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="11" t="s">
         <v>160</v>
       </c>
@@ -11140,7 +11477,7 @@
       </c>
       <c r="Y89" s="13"/>
     </row>
-    <row r="90" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="90" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="11" t="s">
         <v>160</v>
       </c>
@@ -11209,7 +11546,7 @@
       </c>
       <c r="Y90" s="13"/>
     </row>
-    <row r="91" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="91" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="11" t="s">
         <v>160</v>
       </c>
@@ -11278,7 +11615,7 @@
       </c>
       <c r="Y91" s="13"/>
     </row>
-    <row r="92" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="92" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="11" t="s">
         <v>160</v>
       </c>
@@ -11347,7 +11684,7 @@
       </c>
       <c r="Y92" s="13"/>
     </row>
-    <row r="93" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="93" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="11" t="s">
         <v>160</v>
       </c>
@@ -11418,7 +11755,7 @@
       </c>
       <c r="Y93" s="13"/>
     </row>
-    <row r="94" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="94" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="11" t="s">
         <v>160</v>
       </c>
@@ -11487,7 +11824,7 @@
       <c r="X94" s="12"/>
       <c r="Y94" s="13"/>
     </row>
-    <row r="95" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="95" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="11" t="s">
         <v>160</v>
       </c>
@@ -11556,7 +11893,7 @@
       <c r="X95" s="12"/>
       <c r="Y95" s="13"/>
     </row>
-    <row r="96" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="96" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="11" t="s">
         <v>160</v>
       </c>
@@ -11625,7 +11962,7 @@
       <c r="X96" s="12"/>
       <c r="Y96" s="13"/>
     </row>
-    <row r="97" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="97" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="11" t="s">
         <v>160</v>
       </c>
@@ -11694,7 +12031,7 @@
       <c r="X97" s="12"/>
       <c r="Y97" s="13"/>
     </row>
-    <row r="98" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="98" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="11" t="s">
         <v>160</v>
       </c>
@@ -11763,7 +12100,7 @@
       <c r="X98" s="12"/>
       <c r="Y98" s="13"/>
     </row>
-    <row r="99" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="99" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="11" t="s">
         <v>160</v>
       </c>
@@ -11798,7 +12135,7 @@
       <c r="X99" s="12"/>
       <c r="Y99" s="13"/>
     </row>
-    <row r="100" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="100" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="11" t="s">
         <v>160</v>
       </c>
@@ -11867,7 +12204,7 @@
       <c r="X100" s="12"/>
       <c r="Y100" s="13"/>
     </row>
-    <row r="101" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="101" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="11" t="s">
         <v>160</v>
       </c>
@@ -11920,7 +12257,7 @@
       <c r="X101" s="12"/>
       <c r="Y101" s="13"/>
     </row>
-    <row r="102" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="102" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="11" t="s">
         <v>160</v>
       </c>
@@ -11993,7 +12330,7 @@
       </c>
       <c r="Y102" s="13"/>
     </row>
-    <row r="103" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="103" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="11" t="s">
         <v>160</v>
       </c>
@@ -12066,7 +12403,7 @@
       </c>
       <c r="Y103" s="13"/>
     </row>
-    <row r="104" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="104" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="11" t="s">
         <v>160</v>
       </c>
@@ -12139,7 +12476,7 @@
       </c>
       <c r="Y104" s="13"/>
     </row>
-    <row r="105" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="105" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="11" t="s">
         <v>160</v>
       </c>
@@ -12210,7 +12547,7 @@
       </c>
       <c r="Y105" s="13"/>
     </row>
-    <row r="106" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="106" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="11" t="s">
         <v>160</v>
       </c>
@@ -12243,7 +12580,7 @@
       <c r="X106" s="12"/>
       <c r="Y106" s="13"/>
     </row>
-    <row r="107" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="107" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="11" t="s">
         <v>160</v>
       </c>
@@ -12314,7 +12651,7 @@
       </c>
       <c r="Y107" s="13"/>
     </row>
-    <row r="108" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="108" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="11" t="s">
         <v>160</v>
       </c>
@@ -12387,7 +12724,7 @@
       </c>
       <c r="Y108" s="13"/>
     </row>
-    <row r="109" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="109" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="11" t="s">
         <v>160</v>
       </c>
@@ -12460,7 +12797,7 @@
       </c>
       <c r="Y109" s="13"/>
     </row>
-    <row r="110" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="110" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="11" t="s">
         <v>160</v>
       </c>
@@ -12517,7 +12854,7 @@
       <c r="X110" s="12"/>
       <c r="Y110" s="13"/>
     </row>
-    <row r="111" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="111" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="11" t="s">
         <v>201</v>
       </c>
@@ -12592,7 +12929,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="112" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="112" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="11" t="s">
         <v>201</v>
       </c>
@@ -12665,7 +13002,7 @@
       </c>
       <c r="Y112" s="35"/>
     </row>
-    <row r="113" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="113" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="11" t="s">
         <v>207</v>
       </c>
@@ -12738,7 +13075,7 @@
       </c>
       <c r="Y113" s="7"/>
     </row>
-    <row r="114" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="114" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="11" t="s">
         <v>199</v>
       </c>
@@ -12811,7 +13148,7 @@
       </c>
       <c r="Y114" s="13"/>
     </row>
-    <row r="115" spans="1:25" s="30" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="115" spans="1:25" s="30" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="27" t="s">
         <v>209</v>
       </c>
@@ -12846,7 +13183,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="116" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="116" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="11" t="s">
         <v>209</v>
       </c>
@@ -12891,7 +13228,7 @@
       <c r="X116" s="12"/>
       <c r="Y116" s="7"/>
     </row>
-    <row r="117" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="117" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="11" t="s">
         <v>209</v>
       </c>
@@ -12924,7 +13261,7 @@
       <c r="X117" s="12"/>
       <c r="Y117" s="7"/>
     </row>
-    <row r="118" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="118" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="11" t="s">
         <v>209</v>
       </c>
@@ -12957,7 +13294,7 @@
       <c r="X118" s="12"/>
       <c r="Y118" s="7"/>
     </row>
-    <row r="119" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="119" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="11" t="s">
         <v>209</v>
       </c>
@@ -12990,7 +13327,7 @@
       <c r="X119" s="12"/>
       <c r="Y119" s="7"/>
     </row>
-    <row r="120" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="120" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="11" t="s">
         <v>209</v>
       </c>
@@ -13023,7 +13360,7 @@
       <c r="X120" s="12"/>
       <c r="Y120" s="7"/>
     </row>
-    <row r="121" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="121" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="11" t="s">
         <v>209</v>
       </c>
@@ -13056,7 +13393,7 @@
       <c r="X121" s="12"/>
       <c r="Y121" s="7"/>
     </row>
-    <row r="122" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="122" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" s="11" t="s">
         <v>209</v>
       </c>
@@ -13089,7 +13426,7 @@
       <c r="X122" s="12"/>
       <c r="Y122" s="7"/>
     </row>
-    <row r="123" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="123" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="11" t="s">
         <v>209</v>
       </c>
@@ -13122,7 +13459,7 @@
       <c r="X123" s="12"/>
       <c r="Y123" s="7"/>
     </row>
-    <row r="124" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="124" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="11" t="s">
         <v>209</v>
       </c>
@@ -13155,7 +13492,7 @@
       <c r="X124" s="15"/>
       <c r="Y124" s="13"/>
     </row>
-    <row r="125" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="125" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="11" t="s">
         <v>209</v>
       </c>
@@ -13188,7 +13525,7 @@
       <c r="X125" s="12"/>
       <c r="Y125" s="7"/>
     </row>
-    <row r="126" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="126" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="11" t="s">
         <v>209</v>
       </c>
@@ -13221,7 +13558,7 @@
       <c r="X126" s="12"/>
       <c r="Y126" s="7"/>
     </row>
-    <row r="127" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="127" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="11" t="s">
         <v>209</v>
       </c>
@@ -13254,7 +13591,7 @@
       <c r="X127" s="12"/>
       <c r="Y127" s="7"/>
     </row>
-    <row r="128" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="128" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="11" t="s">
         <v>209</v>
       </c>
@@ -13287,7 +13624,7 @@
       <c r="X128" s="12"/>
       <c r="Y128" s="7"/>
     </row>
-    <row r="129" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="129" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129" s="11" t="s">
         <v>209</v>
       </c>
@@ -13320,7 +13657,7 @@
       <c r="X129" s="12"/>
       <c r="Y129" s="7"/>
     </row>
-    <row r="130" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="130" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" s="11" t="s">
         <v>209</v>
       </c>
@@ -13353,7 +13690,7 @@
       <c r="X130" s="12"/>
       <c r="Y130" s="7"/>
     </row>
-    <row r="131" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="131" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" s="11" t="s">
         <v>209</v>
       </c>
@@ -13386,7 +13723,7 @@
       <c r="X131" s="12"/>
       <c r="Y131" s="7"/>
     </row>
-    <row r="132" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="132" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A132" s="11" t="s">
         <v>209</v>
       </c>
@@ -13419,7 +13756,7 @@
       <c r="X132" s="12"/>
       <c r="Y132" s="7"/>
     </row>
-    <row r="133" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="133" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A133" s="11" t="s">
         <v>209</v>
       </c>
@@ -13452,7 +13789,7 @@
       <c r="X133" s="12"/>
       <c r="Y133" s="7"/>
     </row>
-    <row r="134" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="134" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A134" s="11" t="s">
         <v>209</v>
       </c>
@@ -13485,7 +13822,7 @@
       <c r="X134" s="12"/>
       <c r="Y134" s="7"/>
     </row>
-    <row r="135" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="135" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A135" s="11" t="s">
         <v>209</v>
       </c>
@@ -13518,7 +13855,7 @@
       <c r="X135" s="12"/>
       <c r="Y135" s="7"/>
     </row>
-    <row r="136" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="136" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" s="11" t="s">
         <v>209</v>
       </c>
@@ -13551,7 +13888,7 @@
       <c r="X136" s="12"/>
       <c r="Y136" s="7"/>
     </row>
-    <row r="137" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="137" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" s="11" t="s">
         <v>230</v>
       </c>
@@ -13584,7 +13921,7 @@
       <c r="X137" s="16"/>
       <c r="Y137" s="7"/>
     </row>
-    <row r="138" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="138" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" s="11" t="s">
         <v>232</v>
       </c>
@@ -13639,7 +13976,7 @@
       <c r="X138" s="31"/>
       <c r="Y138" s="7"/>
     </row>
-    <row r="139" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="139" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A139" s="11" t="s">
         <v>265</v>
       </c>
@@ -13680,9 +14017,27 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{58389A3C-0D32-7C4E-B363-794E8E4E7869}" scale="162">
-      <pane xSplit="2" ySplit="6" topLeftCell="K7" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="K17" sqref="K17"/>
+    <customSheetView guid="{13156CEF-1324-493B-BC78-7F90522FC5C9}">
+      <pane xSplit="2" ySplit="6" topLeftCell="C14" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="A24" sqref="A24:XFD24"/>
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+    </customSheetView>
+    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="115">
+      <pane xSplit="2" ySplit="6" topLeftCell="Q19" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="Y37" sqref="Y37"/>
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+    </customSheetView>
+    <customSheetView guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" scale="115">
+      <pane xSplit="2" ySplit="6" topLeftCell="C58" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="D81" sqref="D81:X81"/>
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+    </customSheetView>
+    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="130">
+      <pane xSplit="2" ySplit="6" topLeftCell="C53" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="B71" sqref="B71"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
@@ -13692,21 +14047,9 @@
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
-    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="130">
-      <pane xSplit="2" ySplit="6" topLeftCell="C53" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="B71" sqref="B71"/>
-      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-    </customSheetView>
-    <customSheetView guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" scale="115">
-      <pane xSplit="2" ySplit="6" topLeftCell="C58" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="D81" sqref="D81:X81"/>
-      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-    </customSheetView>
-    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="115">
-      <pane xSplit="2" ySplit="6" topLeftCell="Q19" activePane="bottomRight" state="frozen"/>
-      <selection pane="bottomRight" activeCell="Y37" sqref="Y37"/>
+    <customSheetView guid="{58389A3C-0D32-7C4E-B363-794E8E4E7869}" scale="162">
+      <pane xSplit="2" ySplit="6" topLeftCell="K7" activePane="bottomRight" state="frozen"/>
+      <selection pane="bottomRight" activeCell="K17" sqref="K17"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
@@ -13728,15 +14071,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="29.6640625" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="42.33203125" customWidth="1"/>
+    <col min="1" max="1" width="29.7109375" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="42.28515625" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="32" t="s">
         <v>237</v>
       </c>
@@ -13753,7 +14096,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A2" s="33" t="s">
         <v>242</v>
       </c>
@@ -13766,7 +14109,7 @@
       <c r="D2" s="34"/>
       <c r="E2" s="34"/>
     </row>
-    <row r="3" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A3" s="33" t="s">
         <v>243</v>
       </c>
@@ -13779,7 +14122,7 @@
       <c r="D3" s="34"/>
       <c r="E3" s="34"/>
     </row>
-    <row r="4" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A4" s="33" t="s">
         <v>244</v>
       </c>
@@ -13792,7 +14135,7 @@
       <c r="D4" s="34"/>
       <c r="E4" s="34"/>
     </row>
-    <row r="5" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A5" s="33" t="s">
         <v>245</v>
       </c>
@@ -13807,7 +14150,7 @@
       </c>
       <c r="E5" s="34"/>
     </row>
-    <row r="6" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A6" s="33" t="s">
         <v>247</v>
       </c>
@@ -13822,7 +14165,7 @@
       </c>
       <c r="E6" s="34"/>
     </row>
-    <row r="7" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.2">
       <c r="A7" s="33" t="s">
         <v>248</v>
       </c>
@@ -13837,7 +14180,7 @@
       </c>
       <c r="E7" s="34"/>
     </row>
-    <row r="8" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.2">
       <c r="A8" s="33" t="s">
         <v>249</v>
       </c>
@@ -13852,7 +14195,7 @@
       </c>
       <c r="E8" s="34"/>
     </row>
-    <row r="9" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A9" s="33" t="s">
         <v>250</v>
       </c>
@@ -13867,7 +14210,7 @@
       </c>
       <c r="E9" s="34"/>
     </row>
-    <row r="10" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A10" s="33" t="s">
         <v>252</v>
       </c>
@@ -13880,7 +14223,7 @@
       <c r="D10" s="34"/>
       <c r="E10" s="34"/>
     </row>
-    <row r="11" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A11" s="33" t="s">
         <v>253</v>
       </c>
@@ -13893,7 +14236,7 @@
       <c r="D11" s="34"/>
       <c r="E11" s="34"/>
     </row>
-    <row r="12" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A12" s="33" t="s">
         <v>254</v>
       </c>
@@ -13906,7 +14249,7 @@
       <c r="D12" s="34"/>
       <c r="E12" s="34"/>
     </row>
-    <row r="13" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A13" s="33" t="s">
         <v>255</v>
       </c>
@@ -13921,7 +14264,7 @@
       </c>
       <c r="E13" s="34"/>
     </row>
-    <row r="14" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A14" s="33" t="s">
         <v>256</v>
       </c>
@@ -13936,7 +14279,7 @@
       </c>
       <c r="E14" s="34"/>
     </row>
-    <row r="15" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A15" s="33" t="s">
         <v>257</v>
       </c>
@@ -13951,7 +14294,7 @@
       </c>
       <c r="E15" s="34"/>
     </row>
-    <row r="16" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A16" s="33" t="s">
         <v>258</v>
       </c>
@@ -13966,7 +14309,7 @@
       </c>
       <c r="E16" s="34"/>
     </row>
-    <row r="17" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A17" s="33" t="s">
         <v>259</v>
       </c>
@@ -13981,7 +14324,7 @@
       </c>
       <c r="E17" s="34"/>
     </row>
-    <row r="18" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A18" s="33" t="s">
         <v>260</v>
       </c>
@@ -13996,7 +14339,7 @@
       </c>
       <c r="E18" s="34"/>
     </row>
-    <row r="19" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A19" s="33" t="s">
         <v>261</v>
       </c>
@@ -14011,7 +14354,7 @@
       </c>
       <c r="E19" s="34"/>
     </row>
-    <row r="20" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A20" s="33" t="s">
         <v>262</v>
       </c>
@@ -14026,7 +14369,7 @@
       </c>
       <c r="E20" s="34"/>
     </row>
-    <row r="21" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A21" s="33" t="s">
         <v>33</v>
       </c>
@@ -14041,7 +14384,7 @@
       </c>
       <c r="E21" s="34"/>
     </row>
-    <row r="22" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A22" s="33" t="s">
         <v>263</v>
       </c>
@@ -14058,7 +14401,22 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{58389A3C-0D32-7C4E-B363-794E8E4E7869}" scale="150">
+    <customSheetView guid="{13156CEF-1324-493B-BC78-7F90522FC5C9}" scale="150">
+      <selection activeCell="A16" sqref="A16"/>
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+    </customSheetView>
+    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="150">
+      <selection activeCell="A22" sqref="A22"/>
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+    </customSheetView>
+    <customSheetView guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" scale="150">
+      <selection activeCell="A22" sqref="A22"/>
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+    </customSheetView>
+    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="150">
       <selection activeCell="A22" sqref="A22"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -14068,17 +14426,7 @@
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
     </customSheetView>
-    <customSheetView guid="{476C495F-6E55-F04C-8145-4E8EBD6B3DE3}" scale="150">
-      <selection activeCell="A22" sqref="A22"/>
-      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-    </customSheetView>
-    <customSheetView guid="{E3BBF62E-A283-4D48-98B7-21A2A94F634F}" scale="150">
-      <selection activeCell="A22" sqref="A22"/>
-      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-      <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-    </customSheetView>
-    <customSheetView guid="{843152D8-333A-1941-83E9-0CB5262068A2}" scale="150">
+    <customSheetView guid="{58389A3C-0D32-7C4E-B363-794E8E4E7869}" scale="150">
       <selection activeCell="A22" sqref="A22"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
       <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Salli Tilaajan_Urakanvalvoja roolilla kulun kohdistaminen
</commit_message>
<xml_diff>
--- a/resources/roolit.xlsx
+++ b/resources/roolit.xlsx
@@ -1289,14 +1289,14 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="30.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="26.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10.65"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="18.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="25.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="40.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="2" width="38.17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="12.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="10.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="10.65"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="1" width="12.5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="21.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="36"/>
@@ -1304,7 +1304,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="17.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="11.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="11.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="11.65"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="1" width="11.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="1" width="59"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="26" style="1" width="14.5"/>
@@ -3127,7 +3127,7 @@
         <v>41</v>
       </c>
       <c r="E32" s="27" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F32" s="26" t="s">
         <v>38</v>
@@ -9061,14 +9061,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E22"/>
-  <sheetFormatPr defaultColWidth="10.6796875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.66796875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="28.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="42.33"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.66"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.65"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14.01"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="6" style="1" width="10.66"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="6" style="1" width="10.65"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
HARJA-2248: Lisää ELY_Urakanvalvoja rooliin liittyvät oikeudet takaisin ja päivitä roolitiedoston kuvaus
</commit_message>
<xml_diff>
--- a/resources/roolit.xlsx
+++ b/resources/roolit.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elias.tahto/projects/harjaroot/harja/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46DB1EAF-5D42-7946-83DF-C21F03E53A0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC3C01F3-98F2-2C4D-B411-54C29932077C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Oikeudet" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Unknown Author:
 Tatu Tarvainen:
@@ -52,7 +52,7 @@
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Unknown Author:
 Tatu Tarvainen:
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2049" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2049" uniqueCount="287">
   <si>
     <t xml:space="preserve">Roolimääritysten selitykset: </t>
   </si>
@@ -927,9 +927,6 @@
   </si>
   <si>
     <t>Suunnittelu / Kalustoresurssit</t>
-  </si>
-  <si>
-    <t>ELY urakanvalvoja, Hoidon projektipäälikkö</t>
   </si>
 </sst>
 </file>
@@ -1190,6 +1187,9 @@
     <xf numFmtId="49" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1199,9 +1199,6 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1571,21 +1568,21 @@
       <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="41" t="s">
+      <c r="C1" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
-      <c r="H1" s="41"/>
-      <c r="I1" s="41"/>
-      <c r="J1" s="41"/>
-      <c r="K1" s="41"/>
-      <c r="L1" s="41"/>
-      <c r="M1" s="41"/>
-      <c r="N1" s="41"/>
-      <c r="O1" s="41"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="42"/>
+      <c r="I1" s="42"/>
+      <c r="J1" s="42"/>
+      <c r="K1" s="42"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
       <c r="R1" s="2"/>
@@ -1600,21 +1597,21 @@
     <row r="2" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
-      <c r="C2" s="42" t="s">
+      <c r="C2" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42"/>
-      <c r="I2" s="42"/>
-      <c r="J2" s="42"/>
-      <c r="K2" s="42"/>
-      <c r="L2" s="42"/>
-      <c r="M2" s="42"/>
-      <c r="N2" s="42"/>
-      <c r="O2" s="42"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
+      <c r="I2" s="43"/>
+      <c r="J2" s="43"/>
+      <c r="K2" s="43"/>
+      <c r="L2" s="43"/>
+      <c r="M2" s="43"/>
+      <c r="N2" s="43"/>
+      <c r="O2" s="43"/>
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
       <c r="R2" s="2"/>
@@ -1691,34 +1688,34 @@
     <row r="5" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="12"/>
       <c r="B5" s="12"/>
-      <c r="C5" s="43" t="s">
+      <c r="C5" s="44" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="43"/>
-      <c r="E5" s="43"/>
-      <c r="F5" s="43"/>
-      <c r="G5" s="43"/>
-      <c r="H5" s="43"/>
+      <c r="D5" s="44"/>
+      <c r="E5" s="44"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
+      <c r="H5" s="44"/>
       <c r="I5" s="13"/>
       <c r="J5" s="13"/>
-      <c r="K5" s="43" t="s">
+      <c r="K5" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="43"/>
-      <c r="M5" s="43"/>
-      <c r="N5" s="43"/>
-      <c r="O5" s="43"/>
+      <c r="L5" s="44"/>
+      <c r="M5" s="44"/>
+      <c r="N5" s="44"/>
+      <c r="O5" s="44"/>
       <c r="P5" s="13"/>
       <c r="Q5" s="13"/>
-      <c r="R5" s="43" t="s">
+      <c r="R5" s="44" t="s">
         <v>9</v>
       </c>
-      <c r="S5" s="43"/>
-      <c r="T5" s="43"/>
-      <c r="U5" s="43"/>
-      <c r="V5" s="43"/>
-      <c r="W5" s="43"/>
-      <c r="X5" s="43"/>
+      <c r="S5" s="44"/>
+      <c r="T5" s="44"/>
+      <c r="U5" s="44"/>
+      <c r="V5" s="44"/>
+      <c r="W5" s="44"/>
+      <c r="X5" s="44"/>
       <c r="Y5" s="14" t="s">
         <v>10</v>
       </c>
@@ -2289,7 +2286,7 @@
       </c>
       <c r="C15" s="21"/>
       <c r="D15" s="22"/>
-      <c r="E15" s="44" t="s">
+      <c r="E15" s="40" t="s">
         <v>37</v>
       </c>
       <c r="F15" s="22"/>
@@ -2298,7 +2295,7 @@
       <c r="I15" s="22"/>
       <c r="J15" s="22"/>
       <c r="K15" s="22"/>
-      <c r="L15" s="44" t="s">
+      <c r="L15" s="40" t="s">
         <v>37</v>
       </c>
       <c r="M15" s="22"/>
@@ -8236,7 +8233,7 @@
       <c r="X114" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="Y114" s="40" t="s">
+      <c r="Y114" s="41" t="s">
         <v>224</v>
       </c>
     </row>
@@ -8311,7 +8308,7 @@
       <c r="X115" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="Y115" s="40"/>
+      <c r="Y115" s="41"/>
     </row>
     <row r="116" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A116" s="20" t="s">
@@ -9563,7 +9560,7 @@
         <v>276</v>
       </c>
       <c r="B13" s="36" t="s">
-        <v>287</v>
+        <v>21</v>
       </c>
       <c r="C13" s="36" t="s">
         <v>6</v>

</xml_diff>

<commit_message>
HARJA-2248: Päivitä roolit excel ja testidata
</commit_message>
<xml_diff>
--- a/resources/roolit.xlsx
+++ b/resources/roolit.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elias.tahto/projects/harjaroot/harja/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC3C01F3-98F2-2C4D-B411-54C29932077C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37528237-4E58-E341-9BC0-07455B9533C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Oikeudet" sheetId="1" r:id="rId1"/>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2049" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2050" uniqueCount="287">
   <si>
     <t xml:space="preserve">Roolimääritysten selitykset: </t>
   </si>
@@ -1096,7 +1096,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1199,6 +1199,9 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2285,7 +2288,9 @@
         <v>286</v>
       </c>
       <c r="C15" s="21"/>
-      <c r="D15" s="22"/>
+      <c r="D15" s="45" t="s">
+        <v>41</v>
+      </c>
       <c r="E15" s="40" t="s">
         <v>37</v>
       </c>

</xml_diff>

<commit_message>
HARJA-2107: Lisää oikeudet laatupoikkeaman sanktioiden muokkaamiseen ja poistamiseen ja luo uusi poista-laatupoikkeaman-sanktio toiminallisuus. Palauta poista suorasanktio ennalleen
</commit_message>
<xml_diff>
--- a/resources/roolit.xlsx
+++ b/resources/roolit.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elias.tahto/projects/harjaroot/harja/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37528237-4E58-E341-9BC0-07455B9533C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD43CD03-7BE3-FF4A-9950-7BDB342ECF89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2050" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2050" uniqueCount="290">
   <si>
     <t xml:space="preserve">Roolimääritysten selitykset: </t>
   </si>
@@ -927,6 +927,15 @@
   </si>
   <si>
     <t>Suunnittelu / Kalustoresurssit</t>
+  </si>
+  <si>
+    <t>R*,W,päätös,poisto</t>
+  </si>
+  <si>
+    <t>R*,W*,päätös*,poisto*</t>
+  </si>
+  <si>
+    <t>R*,W*,poisto*</t>
   </si>
 </sst>
 </file>
@@ -1190,6 +1199,9 @@
     <xf numFmtId="49" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="49" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1199,9 +1211,6 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1571,21 +1580,21 @@
       <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="42" t="s">
+      <c r="C1" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
-      <c r="I1" s="42"/>
-      <c r="J1" s="42"/>
-      <c r="K1" s="42"/>
-      <c r="L1" s="42"/>
-      <c r="M1" s="42"/>
-      <c r="N1" s="42"/>
-      <c r="O1" s="42"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="O1" s="43"/>
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
       <c r="R1" s="2"/>
@@ -1600,21 +1609,21 @@
     <row r="2" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
-      <c r="C2" s="43" t="s">
+      <c r="C2" s="44" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
-      <c r="I2" s="43"/>
-      <c r="J2" s="43"/>
-      <c r="K2" s="43"/>
-      <c r="L2" s="43"/>
-      <c r="M2" s="43"/>
-      <c r="N2" s="43"/>
-      <c r="O2" s="43"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
+      <c r="N2" s="44"/>
+      <c r="O2" s="44"/>
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
       <c r="R2" s="2"/>
@@ -1691,34 +1700,34 @@
     <row r="5" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="12"/>
       <c r="B5" s="12"/>
-      <c r="C5" s="44" t="s">
+      <c r="C5" s="45" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
-      <c r="G5" s="44"/>
-      <c r="H5" s="44"/>
+      <c r="D5" s="45"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="45"/>
+      <c r="G5" s="45"/>
+      <c r="H5" s="45"/>
       <c r="I5" s="13"/>
       <c r="J5" s="13"/>
-      <c r="K5" s="44" t="s">
+      <c r="K5" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="44"/>
-      <c r="M5" s="44"/>
-      <c r="N5" s="44"/>
-      <c r="O5" s="44"/>
+      <c r="L5" s="45"/>
+      <c r="M5" s="45"/>
+      <c r="N5" s="45"/>
+      <c r="O5" s="45"/>
       <c r="P5" s="13"/>
       <c r="Q5" s="13"/>
-      <c r="R5" s="44" t="s">
+      <c r="R5" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="S5" s="44"/>
-      <c r="T5" s="44"/>
-      <c r="U5" s="44"/>
-      <c r="V5" s="44"/>
-      <c r="W5" s="44"/>
-      <c r="X5" s="44"/>
+      <c r="S5" s="45"/>
+      <c r="T5" s="45"/>
+      <c r="U5" s="45"/>
+      <c r="V5" s="45"/>
+      <c r="W5" s="45"/>
+      <c r="X5" s="45"/>
       <c r="Y5" s="14" t="s">
         <v>10</v>
       </c>
@@ -2288,7 +2297,7 @@
         <v>286</v>
       </c>
       <c r="C15" s="21"/>
-      <c r="D15" s="45" t="s">
+      <c r="D15" s="41" t="s">
         <v>41</v>
       </c>
       <c r="E15" s="40" t="s">
@@ -3022,11 +3031,11 @@
         <v>73</v>
       </c>
       <c r="C27" s="21"/>
-      <c r="D27" s="22" t="s">
-        <v>74</v>
-      </c>
-      <c r="E27" s="23" t="s">
-        <v>75</v>
+      <c r="D27" s="41" t="s">
+        <v>288</v>
+      </c>
+      <c r="E27" s="40" t="s">
+        <v>287</v>
       </c>
       <c r="F27" s="22" t="s">
         <v>38</v>
@@ -3043,11 +3052,11 @@
       <c r="J27" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="K27" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="L27" s="23" t="s">
-        <v>75</v>
+      <c r="K27" s="41" t="s">
+        <v>289</v>
+      </c>
+      <c r="L27" s="40" t="s">
+        <v>287</v>
       </c>
       <c r="M27" s="22" t="s">
         <v>39</v>
@@ -8238,7 +8247,7 @@
       <c r="X114" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="Y114" s="41" t="s">
+      <c r="Y114" s="42" t="s">
         <v>224</v>
       </c>
     </row>
@@ -8313,7 +8322,7 @@
       <c r="X115" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="Y115" s="41"/>
+      <c r="Y115" s="42"/>
     </row>
     <row r="116" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A116" s="20" t="s">

</xml_diff>

<commit_message>
HARJA-2107: Päivitä roolitiedosto sanktioiden muokkausprosessin tueksi
</commit_message>
<xml_diff>
--- a/resources/roolit.xlsx
+++ b/resources/roolit.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elias.tahto/projects/harjaroot/harja/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD43CD03-7BE3-FF4A-9950-7BDB342ECF89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECA5E79A-88D3-AA48-A821-26849CF199B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -935,7 +935,7 @@
     <t>R*,W*,päätös*,poisto*</t>
   </si>
   <si>
-    <t>R*,W*,poisto*</t>
+    <t>R*,W*,poisto*,päätös*</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Muuta raportin nimi ja päivitä testit
</commit_message>
<xml_diff>
--- a/resources/roolit.xlsx
+++ b/resources/roolit.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elias.tahto/projects/harjaroot/harja/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marikorkkasolita/Projektit/repos/harja/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37528237-4E58-E341-9BC0-07455B9533C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D774BE6A-3A09-3448-8C23-503D4F7F1F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26400" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Oikeudet" sheetId="1" r:id="rId1"/>
     <sheet name="Roolit" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -719,9 +719,6 @@
     <t>Suolatoteumat - Kaikki pohjavesialueet</t>
   </si>
   <si>
-    <t>Talvisuolanlämpötilaraportti</t>
-  </si>
-  <si>
     <t>Ilmoitukset</t>
   </si>
   <si>
@@ -927,6 +924,9 @@
   </si>
   <si>
     <t>Suunnittelu / Kalustoresurssit</t>
+  </si>
+  <si>
+    <t>Talvisuolan kokonaiskäyttö</t>
   </si>
 </sst>
 </file>
@@ -1190,6 +1190,9 @@
     <xf numFmtId="49" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="49" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1200,12 +1203,9 @@
     <xf numFmtId="49" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normaali" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1571,21 +1571,21 @@
       <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="42" t="s">
+      <c r="C1" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
-      <c r="I1" s="42"/>
-      <c r="J1" s="42"/>
-      <c r="K1" s="42"/>
-      <c r="L1" s="42"/>
-      <c r="M1" s="42"/>
-      <c r="N1" s="42"/>
-      <c r="O1" s="42"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="O1" s="43"/>
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
       <c r="R1" s="2"/>
@@ -1600,21 +1600,21 @@
     <row r="2" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
-      <c r="C2" s="43" t="s">
+      <c r="C2" s="44" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
-      <c r="I2" s="43"/>
-      <c r="J2" s="43"/>
-      <c r="K2" s="43"/>
-      <c r="L2" s="43"/>
-      <c r="M2" s="43"/>
-      <c r="N2" s="43"/>
-      <c r="O2" s="43"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
+      <c r="N2" s="44"/>
+      <c r="O2" s="44"/>
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
       <c r="R2" s="2"/>
@@ -1691,34 +1691,34 @@
     <row r="5" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="12"/>
       <c r="B5" s="12"/>
-      <c r="C5" s="44" t="s">
+      <c r="C5" s="45" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
-      <c r="G5" s="44"/>
-      <c r="H5" s="44"/>
+      <c r="D5" s="45"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="45"/>
+      <c r="G5" s="45"/>
+      <c r="H5" s="45"/>
       <c r="I5" s="13"/>
       <c r="J5" s="13"/>
-      <c r="K5" s="44" t="s">
+      <c r="K5" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="44"/>
-      <c r="M5" s="44"/>
-      <c r="N5" s="44"/>
-      <c r="O5" s="44"/>
+      <c r="L5" s="45"/>
+      <c r="M5" s="45"/>
+      <c r="N5" s="45"/>
+      <c r="O5" s="45"/>
       <c r="P5" s="13"/>
       <c r="Q5" s="13"/>
-      <c r="R5" s="44" t="s">
+      <c r="R5" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="S5" s="44"/>
-      <c r="T5" s="44"/>
-      <c r="U5" s="44"/>
-      <c r="V5" s="44"/>
-      <c r="W5" s="44"/>
-      <c r="X5" s="44"/>
+      <c r="S5" s="45"/>
+      <c r="T5" s="45"/>
+      <c r="U5" s="45"/>
+      <c r="V5" s="45"/>
+      <c r="W5" s="45"/>
+      <c r="X5" s="45"/>
       <c r="Y5" s="14" t="s">
         <v>10</v>
       </c>
@@ -2285,10 +2285,10 @@
         <v>34</v>
       </c>
       <c r="B15" s="39" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C15" s="21"/>
-      <c r="D15" s="45" t="s">
+      <c r="D15" s="41" t="s">
         <v>41</v>
       </c>
       <c r="E15" s="40" t="s">
@@ -7897,8 +7897,8 @@
       <c r="A110" s="20" t="s">
         <v>172</v>
       </c>
-      <c r="B110" s="20" t="s">
-        <v>217</v>
+      <c r="B110" s="39" t="s">
+        <v>286</v>
       </c>
       <c r="C110" s="21"/>
       <c r="D110" s="22" t="s">
@@ -7969,7 +7969,7 @@
         <v>172</v>
       </c>
       <c r="B111" s="20" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C111" s="21"/>
       <c r="D111" s="22" t="s">
@@ -8115,7 +8115,7 @@
         <v>172</v>
       </c>
       <c r="B113" s="20" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C113" s="21"/>
       <c r="D113" s="22" t="s">
@@ -8169,10 +8169,10 @@
     </row>
     <row r="114" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A114" s="20" t="s">
+        <v>219</v>
+      </c>
+      <c r="B114" s="20" t="s">
         <v>220</v>
-      </c>
-      <c r="B114" s="20" t="s">
-        <v>221</v>
       </c>
       <c r="C114" s="21"/>
       <c r="D114" s="22" t="s">
@@ -8194,60 +8194,60 @@
         <v>39</v>
       </c>
       <c r="J114" s="22" t="s">
+        <v>221</v>
+      </c>
+      <c r="K114" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="L114" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="M114" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N114" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="O114" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="P114" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q114" s="22" t="s">
+        <v>221</v>
+      </c>
+      <c r="R114" s="22" t="s">
         <v>222</v>
       </c>
-      <c r="K114" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="L114" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="M114" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="N114" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="O114" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="P114" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q114" s="22" t="s">
-        <v>222</v>
-      </c>
-      <c r="R114" s="22" t="s">
+      <c r="S114" s="22" t="s">
+        <v>221</v>
+      </c>
+      <c r="T114" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="U114" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="V114" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="W114" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="X114" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y114" s="42" t="s">
         <v>223</v>
-      </c>
-      <c r="S114" s="22" t="s">
-        <v>222</v>
-      </c>
-      <c r="T114" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="U114" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="V114" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="W114" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="X114" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y114" s="41" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="115" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A115" s="20" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B115" s="20" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C115" s="21"/>
       <c r="D115" s="22" t="s">
@@ -8269,34 +8269,34 @@
         <v>39</v>
       </c>
       <c r="J115" s="22" t="s">
+        <v>221</v>
+      </c>
+      <c r="K115" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="L115" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="M115" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N115" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="O115" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="P115" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q115" s="22" t="s">
+        <v>221</v>
+      </c>
+      <c r="R115" s="22" t="s">
         <v>222</v>
       </c>
-      <c r="K115" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="L115" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="M115" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="N115" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="O115" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="P115" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q115" s="22" t="s">
-        <v>222</v>
-      </c>
-      <c r="R115" s="22" t="s">
-        <v>223</v>
-      </c>
       <c r="S115" s="22" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="T115" s="22" t="s">
         <v>44</v>
@@ -8313,14 +8313,14 @@
       <c r="X115" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="Y115" s="41"/>
+      <c r="Y115" s="42"/>
     </row>
     <row r="116" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A116" s="20" t="s">
+        <v>225</v>
+      </c>
+      <c r="B116" s="20" t="s">
         <v>226</v>
-      </c>
-      <c r="B116" s="20" t="s">
-        <v>227</v>
       </c>
       <c r="C116" s="21"/>
       <c r="D116" s="22" t="s">
@@ -8390,10 +8390,10 @@
     </row>
     <row r="117" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A117" s="20" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B117" s="20" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C117" s="21"/>
       <c r="D117" s="22" t="s">
@@ -8463,10 +8463,10 @@
     </row>
     <row r="118" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A118" s="20" t="s">
+        <v>227</v>
+      </c>
+      <c r="B118" s="20" t="s">
         <v>228</v>
-      </c>
-      <c r="B118" s="20" t="s">
-        <v>229</v>
       </c>
       <c r="C118" s="21"/>
       <c r="D118" s="22" t="s">
@@ -8493,15 +8493,15 @@
       <c r="W118" s="21"/>
       <c r="X118" s="21"/>
       <c r="Y118" s="32" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="119" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A119" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B119" s="20" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C119" s="21"/>
       <c r="D119" s="22" t="s">
@@ -8543,10 +8543,10 @@
     </row>
     <row r="120" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A120" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B120" s="20" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C120" s="21"/>
       <c r="D120" s="22" t="s">
@@ -8576,10 +8576,10 @@
     </row>
     <row r="121" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A121" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B121" s="20" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C121" s="21"/>
       <c r="D121" s="22" t="s">
@@ -8609,10 +8609,10 @@
     </row>
     <row r="122" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A122" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B122" s="39" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C122" s="21"/>
       <c r="D122" s="22" t="s">
@@ -8642,10 +8642,10 @@
     </row>
     <row r="123" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A123" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B123" s="20" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C123" s="21"/>
       <c r="D123" s="22" t="s">
@@ -8675,10 +8675,10 @@
     </row>
     <row r="124" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A124" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B124" s="20" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C124" s="21"/>
       <c r="D124" s="22" t="s">
@@ -8708,7 +8708,7 @@
     </row>
     <row r="125" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A125" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B125" s="20" t="s">
         <v>87</v>
@@ -8741,10 +8741,10 @@
     </row>
     <row r="126" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A126" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B126" s="20" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C126" s="21"/>
       <c r="D126" s="22" t="s">
@@ -8774,10 +8774,10 @@
     </row>
     <row r="127" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A127" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B127" s="20" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C127" s="21"/>
       <c r="D127" s="22" t="s">
@@ -8807,10 +8807,10 @@
     </row>
     <row r="128" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A128" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B128" s="20" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C128" s="21"/>
       <c r="D128" s="22" t="s">
@@ -8840,10 +8840,10 @@
     </row>
     <row r="129" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A129" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B129" s="20" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C129" s="21"/>
       <c r="D129" s="22" t="s">
@@ -8873,10 +8873,10 @@
     </row>
     <row r="130" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A130" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B130" s="20" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C130" s="21"/>
       <c r="D130" s="22" t="s">
@@ -8906,10 +8906,10 @@
     </row>
     <row r="131" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A131" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B131" s="20" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C131" s="21"/>
       <c r="D131" s="22" t="s">
@@ -8939,10 +8939,10 @@
     </row>
     <row r="132" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A132" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B132" s="20" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C132" s="21"/>
       <c r="D132" s="22" t="s">
@@ -8972,10 +8972,10 @@
     </row>
     <row r="133" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A133" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B133" s="20" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C133" s="21"/>
       <c r="D133" s="22" t="s">
@@ -9005,10 +9005,10 @@
     </row>
     <row r="134" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A134" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B134" s="20" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C134" s="21"/>
       <c r="D134" s="22" t="s">
@@ -9038,10 +9038,10 @@
     </row>
     <row r="135" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A135" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B135" s="20" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C135" s="21"/>
       <c r="D135" s="22" t="s">
@@ -9071,10 +9071,10 @@
     </row>
     <row r="136" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A136" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B136" s="20" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C136" s="21"/>
       <c r="D136" s="22" t="s">
@@ -9104,7 +9104,7 @@
     </row>
     <row r="137" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A137" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B137" s="20" t="s">
         <v>80</v>
@@ -9137,10 +9137,10 @@
     </row>
     <row r="138" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A138" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B138" s="20" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C138" s="21"/>
       <c r="D138" s="22" t="s">
@@ -9170,10 +9170,10 @@
     </row>
     <row r="139" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A139" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B139" s="20" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C139" s="21"/>
       <c r="D139" s="22" t="s">
@@ -9203,10 +9203,10 @@
     </row>
     <row r="140" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A140" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B140" s="39" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C140" s="21"/>
       <c r="D140" s="22" t="s">
@@ -9236,10 +9236,10 @@
     </row>
     <row r="141" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A141" s="20" t="s">
+        <v>249</v>
+      </c>
+      <c r="B141" s="20" t="s">
         <v>250</v>
-      </c>
-      <c r="B141" s="20" t="s">
-        <v>251</v>
       </c>
       <c r="C141" s="12"/>
       <c r="D141" s="22" t="s">
@@ -9269,53 +9269,53 @@
     </row>
     <row r="142" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A142" s="20" t="s">
+        <v>251</v>
+      </c>
+      <c r="B142" s="20" t="s">
         <v>252</v>
-      </c>
-      <c r="B142" s="20" t="s">
-        <v>253</v>
       </c>
       <c r="C142" s="12"/>
       <c r="D142" s="22" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E142" s="23" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F142" s="21"/>
       <c r="G142" s="22" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="H142" s="21"/>
       <c r="I142" s="21"/>
       <c r="J142" s="22" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="K142" s="22" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="L142" s="23" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="M142" s="22" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="N142" s="22" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="O142" s="21"/>
       <c r="P142" s="21"/>
       <c r="Q142" s="22" t="s">
+        <v>254</v>
+      </c>
+      <c r="R142" s="22" t="s">
         <v>255</v>
       </c>
-      <c r="R142" s="22" t="s">
-        <v>256</v>
-      </c>
       <c r="S142" s="22" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="T142" s="21"/>
       <c r="U142" s="22" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="V142" s="21"/>
       <c r="W142" s="21"/>
@@ -9324,10 +9324,10 @@
     </row>
     <row r="143" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A143" s="20" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B143" s="20" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C143" s="12"/>
       <c r="D143" s="22" t="s">
@@ -9392,24 +9392,24 @@
   <sheetData>
     <row r="1" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="35" t="s">
+        <v>257</v>
+      </c>
+      <c r="B1" s="35" t="s">
         <v>258</v>
       </c>
-      <c r="B1" s="35" t="s">
+      <c r="C1" s="35" t="s">
         <v>259</v>
       </c>
-      <c r="C1" s="35" t="s">
+      <c r="D1" s="35" t="s">
         <v>260</v>
       </c>
-      <c r="D1" s="35" t="s">
+      <c r="E1" s="35" t="s">
         <v>261</v>
-      </c>
-      <c r="E1" s="35" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="36" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B2" s="36" t="s">
         <v>13</v>
@@ -9422,7 +9422,7 @@
     </row>
     <row r="3" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="36" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B3" s="36" t="s">
         <v>15</v>
@@ -9435,7 +9435,7 @@
     </row>
     <row r="4" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="36" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B4" s="36" t="s">
         <v>17</v>
@@ -9448,7 +9448,7 @@
     </row>
     <row r="5" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="36" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B5" s="36" t="s">
         <v>14</v>
@@ -9457,13 +9457,13 @@
         <v>4</v>
       </c>
       <c r="D5" s="38" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E5" s="37"/>
     </row>
     <row r="6" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B6" s="36" t="s">
         <v>16</v>
@@ -9472,13 +9472,13 @@
         <v>4</v>
       </c>
       <c r="D6" s="38" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E6" s="37"/>
     </row>
     <row r="7" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B7" s="36" t="s">
         <v>18</v>
@@ -9487,13 +9487,13 @@
         <v>4</v>
       </c>
       <c r="D7" s="38" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E7" s="37"/>
     </row>
     <row r="8" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="36" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B8" s="36" t="s">
         <v>19</v>
@@ -9502,13 +9502,13 @@
         <v>4</v>
       </c>
       <c r="D8" s="38" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E8" s="37"/>
     </row>
     <row r="9" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="36" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B9" s="36" t="s">
         <v>27</v>
@@ -9517,13 +9517,13 @@
         <v>5</v>
       </c>
       <c r="D9" s="38" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="E9" s="37"/>
     </row>
     <row r="10" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="36" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B10" s="36" t="s">
         <v>20</v>
@@ -9536,7 +9536,7 @@
     </row>
     <row r="11" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="36" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B11" s="36" t="s">
         <v>23</v>
@@ -9549,7 +9549,7 @@
     </row>
     <row r="12" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="36" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B12" s="36" t="s">
         <v>24</v>
@@ -9562,7 +9562,7 @@
     </row>
     <row r="13" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="36" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B13" s="36" t="s">
         <v>21</v>
@@ -9571,13 +9571,13 @@
         <v>6</v>
       </c>
       <c r="D13" s="38" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E13" s="37"/>
     </row>
     <row r="14" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="36" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B14" s="36" t="s">
         <v>22</v>
@@ -9586,13 +9586,13 @@
         <v>6</v>
       </c>
       <c r="D14" s="38" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E14" s="37"/>
     </row>
     <row r="15" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="36" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B15" s="36" t="s">
         <v>25</v>
@@ -9601,13 +9601,13 @@
         <v>6</v>
       </c>
       <c r="D15" s="38" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E15" s="37"/>
     </row>
     <row r="16" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="36" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B16" s="36" t="s">
         <v>26</v>
@@ -9616,13 +9616,13 @@
         <v>6</v>
       </c>
       <c r="D16" s="38" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E16" s="37"/>
     </row>
     <row r="17" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="36" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B17" s="36" t="s">
         <v>29</v>
@@ -9631,13 +9631,13 @@
         <v>5</v>
       </c>
       <c r="D17" s="38" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="E17" s="37"/>
     </row>
     <row r="18" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="36" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B18" s="36" t="s">
         <v>31</v>
@@ -9646,13 +9646,13 @@
         <v>5</v>
       </c>
       <c r="D18" s="38" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="E18" s="37"/>
     </row>
     <row r="19" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="36" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B19" s="36" t="s">
         <v>28</v>
@@ -9661,13 +9661,13 @@
         <v>5</v>
       </c>
       <c r="D19" s="38" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E19" s="37"/>
     </row>
     <row r="20" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="36" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B20" s="36" t="s">
         <v>30</v>
@@ -9676,7 +9676,7 @@
         <v>5</v>
       </c>
       <c r="D20" s="38" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E20" s="37"/>
     </row>
@@ -9691,13 +9691,13 @@
         <v>5</v>
       </c>
       <c r="D21" s="38" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E21" s="37"/>
     </row>
     <row r="22" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="36" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B22" s="36" t="s">
         <v>32</v>
@@ -9706,7 +9706,7 @@
         <v>5</v>
       </c>
       <c r="D22" s="38" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E22" s="37"/>
     </row>

</xml_diff>

<commit_message>
Poista roolimuutokset konfliktien takia
</commit_message>
<xml_diff>
--- a/resources/roolit.xlsx
+++ b/resources/roolit.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marikorkkasolita/Projektit/repos/harja/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D774BE6A-3A09-3448-8C23-503D4F7F1F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BEE0F83-F1E8-454C-BE8F-9F160AE2CB2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26400" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -926,7 +926,7 @@
     <t>Suunnittelu / Kalustoresurssit</t>
   </si>
   <si>
-    <t>Talvisuolan kokonaiskäyttö</t>
+    <t>Talvisuolanlämpötilaraportti</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
HARJA-2710 Muuta tilaajan tarkastusten näkyminen erityisoikeudeksi
</commit_message>
<xml_diff>
--- a/resources/roolit.xlsx
+++ b/resources/roolit.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marikorkkasolita/Projektit/repos/harja/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\henrikkorpi\harjaroot\harja\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD60B6C3-AEE9-6340-BA02-63ABAAD81610}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFA29749-5C72-4187-A467-817E96F07074}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26400" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-57720" yWindow="-9060" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Oikeudet" sheetId="1" r:id="rId1"/>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2050" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2050" uniqueCount="292">
   <si>
     <t xml:space="preserve">Roolimääritysten selitykset: </t>
   </si>
@@ -266,18 +266,6 @@
     <t>Laadunseuranta / Tarkastukset</t>
   </si>
   <si>
-    <t>R*,W*,aseta-näkyviin-urakoitsijalle*</t>
-  </si>
-  <si>
-    <t>R*,W,aseta-näkyviin-urakoitsijalle</t>
-  </si>
-  <si>
-    <t>R*,W+,aseta-näkyviin-urakoitsijalle+</t>
-  </si>
-  <si>
-    <t>R,W,aseta-näkyviin-urakoitsijalle</t>
-  </si>
-  <si>
     <t>Laadunseuranta / Talvihoitoreititys</t>
   </si>
   <si>
@@ -936,6 +924,24 @@
   </si>
   <si>
     <t>Talvisuolan kokonaiskäyttö</t>
+  </si>
+  <si>
+    <t>R*,W*,aseta-näkyviin-urakoitsijalle*,nakee-tilaajan-tarkastukset</t>
+  </si>
+  <si>
+    <t>R*,W,aseta-näkyviin-urakoitsijalle,nakee-tilaajan-tarkastukset</t>
+  </si>
+  <si>
+    <t>R*,nakee-tilaajan-tarkastukset</t>
+  </si>
+  <si>
+    <t>R*,W+,aseta-näkyviin-urakoitsijalle+,nakee-tilaajan-tarkastukset</t>
+  </si>
+  <si>
+    <t>R,nakee-tilaajan-tarkastukset</t>
+  </si>
+  <si>
+    <t>R,W,aseta-näkyviin-urakoitsijalle,nakee-tilaajan-tarkastukset</t>
   </si>
 </sst>
 </file>
@@ -1214,7 +1220,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normaali" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1230,7 +1236,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office-teema">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1547,11 +1553,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Y143"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="31.6640625" customWidth="1"/>
-    <col min="3" max="3" width="14.1640625" customWidth="1"/>
+    <col min="3" max="3" width="14.109375" customWidth="1"/>
     <col min="4" max="4" width="30.33203125" customWidth="1"/>
     <col min="5" max="5" width="26.33203125" style="1" customWidth="1"/>
     <col min="6" max="6" width="12.6640625" customWidth="1"/>
@@ -1560,22 +1566,22 @@
     <col min="9" max="9" width="18.33203125" customWidth="1"/>
     <col min="10" max="10" width="25.33203125" customWidth="1"/>
     <col min="11" max="11" width="40.6640625" customWidth="1"/>
-    <col min="12" max="12" width="38.1640625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="38.109375" style="1" customWidth="1"/>
     <col min="13" max="13" width="12.33203125" customWidth="1"/>
     <col min="14" max="14" width="10.6640625" customWidth="1"/>
-    <col min="15" max="16" width="12.5" customWidth="1"/>
+    <col min="15" max="16" width="12.44140625" customWidth="1"/>
     <col min="17" max="17" width="21.6640625" customWidth="1"/>
     <col min="18" max="18" width="36" customWidth="1"/>
     <col min="19" max="19" width="29.6640625" customWidth="1"/>
     <col min="20" max="20" width="15" customWidth="1"/>
     <col min="21" max="21" width="17.6640625" customWidth="1"/>
-    <col min="22" max="22" width="11.5" customWidth="1"/>
+    <col min="22" max="22" width="11.44140625" customWidth="1"/>
     <col min="23" max="23" width="11.6640625" customWidth="1"/>
     <col min="24" max="24" width="11.33203125" customWidth="1"/>
     <col min="25" max="25" width="59" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="24" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:25" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
       <c r="B1" s="3" t="s">
         <v>0</v>
@@ -1606,7 +1612,7 @@
       <c r="X1" s="2"/>
       <c r="Y1" s="2"/>
     </row>
-    <row r="2" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="44" t="s">
@@ -1635,7 +1641,7 @@
       <c r="X2" s="2"/>
       <c r="Y2" s="2"/>
     </row>
-    <row r="3" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3" s="4" t="s">
         <v>3</v>
@@ -1670,7 +1676,7 @@
       <c r="X3" s="2"/>
       <c r="Y3" s="2"/>
     </row>
-    <row r="4" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="9"/>
@@ -1697,7 +1703,7 @@
       <c r="X4" s="2"/>
       <c r="Y4" s="2"/>
     </row>
-    <row r="5" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="12"/>
       <c r="B5" s="12"/>
       <c r="C5" s="45" t="s">
@@ -1732,7 +1738,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>11</v>
       </c>
@@ -1805,7 +1811,7 @@
       </c>
       <c r="Y6" s="19"/>
     </row>
-    <row r="7" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="20" t="s">
         <v>34</v>
       </c>
@@ -1878,7 +1884,7 @@
       </c>
       <c r="Y7" s="12"/>
     </row>
-    <row r="8" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="20" t="s">
         <v>34</v>
       </c>
@@ -1937,7 +1943,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="20" t="s">
         <v>34</v>
       </c>
@@ -1990,7 +1996,7 @@
       <c r="X9" s="21"/>
       <c r="Y9" s="12"/>
     </row>
-    <row r="10" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="20" t="s">
         <v>34</v>
       </c>
@@ -2043,7 +2049,7 @@
       <c r="X10" s="21"/>
       <c r="Y10" s="12"/>
     </row>
-    <row r="11" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="20" t="s">
         <v>34</v>
       </c>
@@ -2102,7 +2108,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="12" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="20" t="s">
         <v>34</v>
       </c>
@@ -2155,7 +2161,7 @@
       <c r="X12" s="21"/>
       <c r="Y12" s="12"/>
     </row>
-    <row r="13" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="20" t="s">
         <v>34</v>
       </c>
@@ -2222,7 +2228,7 @@
       <c r="X13" s="21"/>
       <c r="Y13" s="12"/>
     </row>
-    <row r="14" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="20" t="s">
         <v>34</v>
       </c>
@@ -2289,12 +2295,12 @@
       <c r="X14" s="21"/>
       <c r="Y14" s="12"/>
     </row>
-    <row r="15" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
         <v>34</v>
       </c>
       <c r="B15" s="39" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="C15" s="21"/>
       <c r="D15" s="41" t="s">
@@ -2326,7 +2332,7 @@
       <c r="X15" s="21"/>
       <c r="Y15" s="12"/>
     </row>
-    <row r="16" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="20" t="s">
         <v>34</v>
       </c>
@@ -2383,7 +2389,7 @@
       <c r="X16" s="21"/>
       <c r="Y16" s="12"/>
     </row>
-    <row r="17" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="20" t="s">
         <v>34</v>
       </c>
@@ -2440,7 +2446,7 @@
       <c r="X17" s="21"/>
       <c r="Y17" s="12"/>
     </row>
-    <row r="18" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="20" t="s">
         <v>34</v>
       </c>
@@ -2497,7 +2503,7 @@
       <c r="X18" s="21"/>
       <c r="Y18" s="12"/>
     </row>
-    <row r="19" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="20" t="s">
         <v>34</v>
       </c>
@@ -2564,7 +2570,7 @@
       <c r="X19" s="21"/>
       <c r="Y19" s="12"/>
     </row>
-    <row r="20" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="20" t="s">
         <v>34</v>
       </c>
@@ -2631,7 +2637,7 @@
       <c r="X20" s="21"/>
       <c r="Y20" s="12"/>
     </row>
-    <row r="21" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="20" t="s">
         <v>34</v>
       </c>
@@ -2686,7 +2692,7 @@
       <c r="X21" s="21"/>
       <c r="Y21" s="12"/>
     </row>
-    <row r="22" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="20" t="s">
         <v>34</v>
       </c>
@@ -2747,7 +2753,7 @@
       <c r="X22" s="21"/>
       <c r="Y22" s="12"/>
     </row>
-    <row r="23" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="20" t="s">
         <v>34</v>
       </c>
@@ -2814,7 +2820,7 @@
       <c r="X23" s="21"/>
       <c r="Y23" s="12"/>
     </row>
-    <row r="24" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="20" t="s">
         <v>34</v>
       </c>
@@ -2823,46 +2829,46 @@
       </c>
       <c r="C24" s="21"/>
       <c r="D24" s="22" t="s">
-        <v>66</v>
+        <v>286</v>
       </c>
       <c r="E24" s="23" t="s">
-        <v>67</v>
+        <v>287</v>
       </c>
       <c r="F24" s="22" t="s">
-        <v>38</v>
+        <v>288</v>
       </c>
       <c r="G24" s="22" t="s">
-        <v>68</v>
+        <v>289</v>
       </c>
       <c r="H24" s="22" t="s">
-        <v>38</v>
+        <v>288</v>
       </c>
       <c r="I24" s="22" t="s">
-        <v>39</v>
+        <v>290</v>
       </c>
       <c r="J24" s="22" t="s">
-        <v>69</v>
+        <v>291</v>
       </c>
       <c r="K24" s="22" t="s">
-        <v>66</v>
+        <v>286</v>
       </c>
       <c r="L24" s="23" t="s">
-        <v>67</v>
+        <v>287</v>
       </c>
       <c r="M24" s="22" t="s">
-        <v>69</v>
+        <v>291</v>
       </c>
       <c r="N24" s="22" t="s">
-        <v>38</v>
+        <v>288</v>
       </c>
       <c r="O24" s="22" t="s">
-        <v>38</v>
+        <v>288</v>
       </c>
       <c r="P24" s="22" t="s">
-        <v>39</v>
+        <v>290</v>
       </c>
       <c r="Q24" s="22" t="s">
-        <v>69</v>
+        <v>291</v>
       </c>
       <c r="R24" s="22" t="s">
         <v>42</v>
@@ -2887,12 +2893,12 @@
       </c>
       <c r="Y24" s="12"/>
     </row>
-    <row r="25" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B25" s="20" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C25" s="21"/>
       <c r="D25" s="22" t="s">
@@ -2950,12 +2956,12 @@
       <c r="X25" s="21"/>
       <c r="Y25" s="12"/>
     </row>
-    <row r="26" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C26" s="21"/>
       <c r="D26" s="22" t="s">
@@ -2968,7 +2974,7 @@
         <v>38</v>
       </c>
       <c r="G26" s="22" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="H26" s="22" t="s">
         <v>38</v>
@@ -3023,19 +3029,19 @@
       </c>
       <c r="Y26" s="12"/>
     </row>
-    <row r="27" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B27" s="20" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C27" s="21"/>
       <c r="D27" s="41" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="E27" s="40" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="F27" s="22" t="s">
         <v>38</v>
@@ -3050,13 +3056,13 @@
         <v>39</v>
       </c>
       <c r="J27" s="22" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="K27" s="41" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="L27" s="40" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="M27" s="22" t="s">
         <v>39</v>
@@ -3071,7 +3077,7 @@
         <v>39</v>
       </c>
       <c r="Q27" s="22" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="R27" s="22" t="s">
         <v>44</v>
@@ -3091,15 +3097,15 @@
       <c r="W27" s="21"/>
       <c r="X27" s="21"/>
       <c r="Y27" s="20" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="28" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="28" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C28" s="21"/>
       <c r="D28" s="22" t="s">
@@ -3163,12 +3169,12 @@
       <c r="X28" s="21"/>
       <c r="Y28" s="12"/>
     </row>
-    <row r="29" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C29" s="21"/>
       <c r="D29" s="22" t="s">
@@ -3218,19 +3224,19 @@
       <c r="X29" s="2"/>
       <c r="Y29" s="12"/>
     </row>
-    <row r="30" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C30" s="21"/>
       <c r="D30" s="22" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E30" s="23" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="F30" s="22" t="s">
         <v>38</v>
@@ -3248,10 +3254,10 @@
         <v>40</v>
       </c>
       <c r="K30" s="22" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="L30" s="23" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="M30" s="22" t="s">
         <v>39</v>
@@ -3267,10 +3273,10 @@
         <v>40</v>
       </c>
       <c r="R30" s="22" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="S30" s="22" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="T30" s="22" t="s">
         <v>44</v>
@@ -3284,22 +3290,22 @@
       <c r="W30" s="21"/>
       <c r="X30" s="21"/>
       <c r="Y30" s="20" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="31" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="31" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B31" s="20" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C31" s="21"/>
       <c r="D31" s="22" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="E31" s="23" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="F31" s="22" t="s">
         <v>38</v>
@@ -3314,13 +3320,13 @@
         <v>39</v>
       </c>
       <c r="J31" s="22" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="K31" s="22" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="L31" s="23" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="M31" s="22" t="s">
         <v>39</v>
@@ -3333,19 +3339,19 @@
       </c>
       <c r="P31" s="21"/>
       <c r="Q31" s="22" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="R31" s="22" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="S31" s="22" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="T31" s="22" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="U31" s="22" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="V31" s="22" t="s">
         <v>44</v>
@@ -3353,15 +3359,15 @@
       <c r="W31" s="21"/>
       <c r="X31" s="21"/>
       <c r="Y31" s="20" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="32" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="32" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B32" s="20" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C32" s="21"/>
       <c r="D32" s="22" t="s">
@@ -3417,12 +3423,12 @@
       <c r="X32" s="21"/>
       <c r="Y32" s="12"/>
     </row>
-    <row r="33" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B33" s="20" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C33" s="21"/>
       <c r="D33" s="22" t="s">
@@ -3474,12 +3480,12 @@
       <c r="X33" s="21"/>
       <c r="Y33" s="12"/>
     </row>
-    <row r="34" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="34" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B34" s="24" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C34" s="21"/>
       <c r="D34" s="22" t="s">
@@ -3527,12 +3533,12 @@
       <c r="X34" s="21"/>
       <c r="Y34" s="12"/>
     </row>
-    <row r="35" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B35" s="20" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="C35" s="21"/>
       <c r="D35" s="22" t="s">
@@ -3572,12 +3578,12 @@
       <c r="X35" s="21"/>
       <c r="Y35" s="12"/>
     </row>
-    <row r="36" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B36" s="24" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="22" t="s">
@@ -3617,12 +3623,12 @@
       <c r="X36" s="2"/>
       <c r="Y36" s="2"/>
     </row>
-    <row r="37" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C37" s="21"/>
       <c r="D37" s="22" t="s">
@@ -3661,15 +3667,15 @@
       <c r="W37" s="21"/>
       <c r="X37" s="21"/>
       <c r="Y37" s="20" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="38" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="38" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B38" s="24" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C38" s="21"/>
       <c r="D38" s="22" t="s">
@@ -3721,12 +3727,12 @@
       </c>
       <c r="Y38" s="12"/>
     </row>
-    <row r="39" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C39" s="21"/>
       <c r="D39" s="22" t="s">
@@ -3784,12 +3790,12 @@
       <c r="X39" s="21"/>
       <c r="Y39" s="12"/>
     </row>
-    <row r="40" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="40" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="C40" s="21"/>
       <c r="D40" s="22" t="s">
@@ -3837,19 +3843,19 @@
       <c r="X40" s="21"/>
       <c r="Y40" s="12"/>
     </row>
-    <row r="41" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="41" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B41" s="20" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C41" s="21"/>
       <c r="D41" s="22" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="E41" s="23" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="F41" s="22" t="s">
         <v>38</v>
@@ -3864,13 +3870,13 @@
         <v>39</v>
       </c>
       <c r="J41" s="26" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="K41" s="22" t="s">
         <v>41</v>
       </c>
       <c r="L41" s="23" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="M41" s="22" t="s">
         <v>40</v>
@@ -3883,13 +3889,13 @@
       </c>
       <c r="P41" s="21"/>
       <c r="Q41" s="26" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="R41" s="22" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="S41" s="22" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="T41" s="22" t="s">
         <v>44</v>
@@ -3903,22 +3909,22 @@
       <c r="W41" s="21"/>
       <c r="X41" s="21"/>
       <c r="Y41" s="20" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="42" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="42" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B42" s="20" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="C42" s="21"/>
       <c r="D42" s="22" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E42" s="23" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F42" s="22" t="s">
         <v>38</v>
@@ -3934,10 +3940,10 @@
         <v>40</v>
       </c>
       <c r="K42" s="22" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="L42" s="23" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="M42" s="21"/>
       <c r="N42" s="22" t="s">
@@ -3948,7 +3954,7 @@
       </c>
       <c r="P42" s="21"/>
       <c r="Q42" s="22" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="R42" s="22" t="s">
         <v>42</v>
@@ -3969,25 +3975,25 @@
       <c r="X42" s="21"/>
       <c r="Y42" s="12"/>
     </row>
-    <row r="43" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="43" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C43" s="21"/>
       <c r="D43" s="22" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="E43" s="23" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="F43" s="22" t="s">
         <v>38</v>
       </c>
       <c r="G43" s="22" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="H43" s="22" t="s">
         <v>38</v>
@@ -3996,13 +4002,13 @@
         <v>39</v>
       </c>
       <c r="J43" s="22" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="K43" s="22" t="s">
         <v>41</v>
       </c>
       <c r="L43" s="23" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="M43" s="21"/>
       <c r="N43" s="22" t="s">
@@ -4013,7 +4019,7 @@
       </c>
       <c r="P43" s="21"/>
       <c r="Q43" s="22" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="R43" s="22" t="s">
         <v>42</v>
@@ -4034,19 +4040,19 @@
       <c r="X43" s="21"/>
       <c r="Y43" s="12"/>
     </row>
-    <row r="44" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="44" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B44" s="20" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C44" s="21"/>
       <c r="D44" s="22" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E44" s="23" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F44" s="22" t="s">
         <v>38</v>
@@ -4062,10 +4068,10 @@
         <v>40</v>
       </c>
       <c r="K44" s="22" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="L44" s="23" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="M44" s="21"/>
       <c r="N44" s="22" t="s">
@@ -4076,7 +4082,7 @@
       </c>
       <c r="P44" s="21"/>
       <c r="Q44" s="22" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="R44" s="22" t="s">
         <v>42</v>
@@ -4097,16 +4103,16 @@
       <c r="X44" s="21"/>
       <c r="Y44" s="12"/>
     </row>
-    <row r="45" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="45" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B45" s="20" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C45" s="21"/>
       <c r="D45" s="22" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E45" s="23" t="s">
         <v>37</v>
@@ -4160,19 +4166,19 @@
       <c r="X45" s="21"/>
       <c r="Y45" s="12"/>
     </row>
-    <row r="46" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="46" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B46" s="20" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="C46" s="21"/>
       <c r="D46" s="22" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E46" s="23" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="F46" s="22" t="s">
         <v>38</v>
@@ -4188,10 +4194,10 @@
         <v>40</v>
       </c>
       <c r="K46" s="22" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="L46" s="23" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="M46" s="21"/>
       <c r="N46" s="22" t="s">
@@ -4205,10 +4211,10 @@
         <v>40</v>
       </c>
       <c r="R46" s="22" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="S46" s="22" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="T46" s="22" t="s">
         <v>44</v>
@@ -4223,12 +4229,12 @@
       <c r="X46" s="21"/>
       <c r="Y46" s="12"/>
     </row>
-    <row r="47" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="47" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C47" s="21"/>
       <c r="D47" s="22" t="s">
@@ -4286,12 +4292,12 @@
       <c r="X47" s="21"/>
       <c r="Y47" s="12"/>
     </row>
-    <row r="48" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="48" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B48" s="20" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C48" s="21"/>
       <c r="D48" s="22" t="s">
@@ -4349,12 +4355,12 @@
       <c r="X48" s="21"/>
       <c r="Y48" s="12"/>
     </row>
-    <row r="49" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="49" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C49" s="21"/>
       <c r="D49" s="22" t="s">
@@ -4412,25 +4418,25 @@
       <c r="X49" s="21"/>
       <c r="Y49" s="12"/>
     </row>
-    <row r="50" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="50" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B50" s="20" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C50" s="21"/>
       <c r="D50" s="22" t="s">
         <v>41</v>
       </c>
       <c r="E50" s="23" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="F50" s="22" t="s">
         <v>38</v>
       </c>
       <c r="G50" s="22" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="H50" s="22" t="s">
         <v>38</v>
@@ -4445,7 +4451,7 @@
         <v>41</v>
       </c>
       <c r="L50" s="23" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="M50" s="22" t="s">
         <v>40</v>
@@ -4485,19 +4491,19 @@
       </c>
       <c r="Y50" s="12"/>
     </row>
-    <row r="51" spans="1:25" ht="27.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="51" spans="1:25" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B51" s="20" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C51" s="21"/>
       <c r="D51" s="27" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="E51" s="28" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="F51" s="22" t="s">
         <v>38</v>
@@ -4508,7 +4514,7 @@
       </c>
       <c r="I51" s="21"/>
       <c r="J51" s="27" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="K51" s="21"/>
       <c r="L51" s="25"/>
@@ -4518,10 +4524,10 @@
       <c r="P51" s="21"/>
       <c r="Q51" s="21"/>
       <c r="R51" s="27" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="S51" s="27" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="T51" s="22" t="s">
         <v>44</v>
@@ -4535,22 +4541,22 @@
       <c r="W51" s="21"/>
       <c r="X51" s="21"/>
       <c r="Y51" s="20" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="52" spans="1:25" ht="69.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="52" spans="1:25" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B52" s="20" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="C52" s="21"/>
       <c r="D52" s="27" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="E52" s="28" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="F52" s="22" t="s">
         <v>38</v>
@@ -4561,7 +4567,7 @@
       </c>
       <c r="I52" s="21"/>
       <c r="J52" s="27" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="K52" s="29"/>
       <c r="L52" s="30"/>
@@ -4571,10 +4577,10 @@
       <c r="P52" s="21"/>
       <c r="Q52" s="21"/>
       <c r="R52" s="27" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="S52" s="27" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="T52" s="22" t="s">
         <v>44</v>
@@ -4588,15 +4594,15 @@
       <c r="W52" s="21"/>
       <c r="X52" s="21"/>
       <c r="Y52" s="20" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="53" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="53" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B53" s="20" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C53" s="21"/>
       <c r="D53" s="22" t="s">
@@ -4639,22 +4645,22 @@
       <c r="W53" s="21"/>
       <c r="X53" s="21"/>
       <c r="Y53" s="20" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="54" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="54" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B54" s="20" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="C54" s="21"/>
       <c r="D54" s="27" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E54" s="28" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="F54" s="27" t="s">
         <v>38</v>
@@ -4663,7 +4669,7 @@
       <c r="H54" s="29"/>
       <c r="I54" s="29"/>
       <c r="J54" s="27" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="K54" s="21"/>
       <c r="L54" s="25"/>
@@ -4673,10 +4679,10 @@
       <c r="P54" s="21"/>
       <c r="Q54" s="21"/>
       <c r="R54" s="27" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="S54" s="27" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="T54" s="22" t="s">
         <v>44</v>
@@ -4691,12 +4697,12 @@
       <c r="X54" s="21"/>
       <c r="Y54" s="12"/>
     </row>
-    <row r="55" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="55" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B55" s="20" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" s="22" t="s">
@@ -4744,19 +4750,19 @@
       <c r="X55" s="2"/>
       <c r="Y55" s="2"/>
     </row>
-    <row r="56" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="56" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B56" s="20" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="C56" s="21"/>
       <c r="D56" s="22" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="E56" s="23" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="F56" s="22" t="s">
         <v>38</v>
@@ -4765,7 +4771,7 @@
       <c r="H56" s="21"/>
       <c r="I56" s="21"/>
       <c r="J56" s="22" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="K56" s="21"/>
       <c r="L56" s="25"/>
@@ -4775,10 +4781,10 @@
       <c r="P56" s="21"/>
       <c r="Q56" s="21"/>
       <c r="R56" s="22" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="S56" s="22" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="T56" s="22" t="s">
         <v>44</v>
@@ -4793,12 +4799,12 @@
       <c r="X56" s="21"/>
       <c r="Y56" s="12"/>
     </row>
-    <row r="57" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="57" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B57" s="20" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="C57" s="21"/>
       <c r="D57" s="22" t="s">
@@ -4826,19 +4832,19 @@
       <c r="X57" s="21"/>
       <c r="Y57" s="12"/>
     </row>
-    <row r="58" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="58" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B58" s="20" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="C58" s="21"/>
       <c r="D58" s="22" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="E58" s="31" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="F58" s="22" t="s">
         <v>38</v>
@@ -4849,7 +4855,7 @@
       </c>
       <c r="I58" s="21"/>
       <c r="J58" s="22" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="K58" s="21"/>
       <c r="L58" s="25"/>
@@ -4859,32 +4865,32 @@
       <c r="P58" s="21"/>
       <c r="Q58" s="21"/>
       <c r="R58" s="22" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="S58" s="22" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="T58" s="22" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="U58" s="22" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="V58" s="22" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="W58" s="21"/>
       <c r="X58" s="21"/>
       <c r="Y58" s="20" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="59" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="59" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B59" s="20" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C59" s="21"/>
       <c r="D59" s="22" t="s">
@@ -4912,12 +4918,12 @@
       <c r="X59" s="21"/>
       <c r="Y59" s="12"/>
     </row>
-    <row r="60" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="60" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B60" s="20" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C60" s="21"/>
       <c r="D60" s="22" t="s">
@@ -4963,12 +4969,12 @@
       <c r="X60" s="21"/>
       <c r="Y60" s="12"/>
     </row>
-    <row r="61" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="61" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B61" s="20" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C61" s="21"/>
       <c r="D61" s="22" t="s">
@@ -5026,12 +5032,12 @@
       <c r="X61" s="21"/>
       <c r="Y61" s="12"/>
     </row>
-    <row r="62" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="62" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B62" s="20" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C62" s="21"/>
       <c r="D62" s="22" t="s">
@@ -5085,12 +5091,12 @@
       <c r="X62" s="21"/>
       <c r="Y62" s="12"/>
     </row>
-    <row r="63" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="63" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B63" s="20" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C63" s="21"/>
       <c r="D63" s="22" t="s">
@@ -5146,12 +5152,12 @@
       <c r="X63" s="21"/>
       <c r="Y63" s="12"/>
     </row>
-    <row r="64" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="64" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B64" s="20" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C64" s="21"/>
       <c r="D64" s="22" t="s">
@@ -5201,12 +5207,12 @@
       <c r="X64" s="21"/>
       <c r="Y64" s="12"/>
     </row>
-    <row r="65" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="65" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B65" s="20" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C65" s="21"/>
       <c r="D65" s="22" t="s">
@@ -5274,12 +5280,12 @@
       </c>
       <c r="Y65" s="12"/>
     </row>
-    <row r="66" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="66" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B66" s="20" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C66" s="21"/>
       <c r="D66" s="22" t="s">
@@ -5327,12 +5333,12 @@
       <c r="X66" s="21"/>
       <c r="Y66" s="12"/>
     </row>
-    <row r="67" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="67" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B67" s="20" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C67" s="21"/>
       <c r="D67" s="22" t="s">
@@ -5380,12 +5386,12 @@
       <c r="X67" s="21"/>
       <c r="Y67" s="12"/>
     </row>
-    <row r="68" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="68" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B68" s="20" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="C68" s="21"/>
       <c r="D68" s="22" t="s">
@@ -5433,12 +5439,12 @@
       <c r="X68" s="21"/>
       <c r="Y68" s="12"/>
     </row>
-    <row r="69" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="69" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="20" t="s">
+        <v>168</v>
+      </c>
+      <c r="B69" s="20" t="s">
         <v>172</v>
-      </c>
-      <c r="B69" s="20" t="s">
-        <v>176</v>
       </c>
       <c r="C69" s="21"/>
       <c r="D69" s="22" t="s">
@@ -5486,12 +5492,12 @@
       <c r="X69" s="21"/>
       <c r="Y69" s="12"/>
     </row>
-    <row r="70" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="70" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B70" s="20" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="C70" s="21"/>
       <c r="D70" s="22" t="s">
@@ -5533,12 +5539,12 @@
       <c r="X70" s="21"/>
       <c r="Y70" s="12"/>
     </row>
-    <row r="71" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="71" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B71" s="20" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="C71" s="21"/>
       <c r="D71" s="22" t="s">
@@ -5586,12 +5592,12 @@
       <c r="X71" s="21"/>
       <c r="Y71" s="12"/>
     </row>
-    <row r="72" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="72" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B72" s="20" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="C72" s="21"/>
       <c r="D72" s="22" t="s">
@@ -5639,12 +5645,12 @@
       <c r="X72" s="21"/>
       <c r="Y72" s="12"/>
     </row>
-    <row r="73" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="73" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B73" s="20" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="C73" s="21"/>
       <c r="D73" s="22" t="s">
@@ -5692,12 +5698,12 @@
       <c r="X73" s="21"/>
       <c r="Y73" s="12"/>
     </row>
-    <row r="74" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="74" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B74" s="20" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="C74" s="21"/>
       <c r="D74" s="22" t="s">
@@ -5745,12 +5751,12 @@
       <c r="X74" s="21"/>
       <c r="Y74" s="12"/>
     </row>
-    <row r="75" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="75" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B75" s="20" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="C75" s="21"/>
       <c r="D75" s="22" t="s">
@@ -5780,12 +5786,12 @@
       <c r="X75" s="21"/>
       <c r="Y75" s="12"/>
     </row>
-    <row r="76" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="76" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B76" s="20" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="C76" s="21"/>
       <c r="D76" s="22" t="s">
@@ -5851,12 +5857,12 @@
       </c>
       <c r="Y76" s="12"/>
     </row>
-    <row r="77" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="77" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B77" s="20" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="C77" s="21"/>
       <c r="D77" s="22" t="s">
@@ -5924,12 +5930,12 @@
       </c>
       <c r="Y77" s="12"/>
     </row>
-    <row r="78" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="78" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B78" s="20" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="C78" s="21"/>
       <c r="D78" s="22" t="s">
@@ -5995,12 +6001,12 @@
       </c>
       <c r="Y78" s="12"/>
     </row>
-    <row r="79" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="79" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B79" s="20" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="C79" s="21"/>
       <c r="D79" s="22" t="s">
@@ -6066,12 +6072,12 @@
       </c>
       <c r="Y79" s="12"/>
     </row>
-    <row r="80" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="80" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B80" s="20" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="C80" s="21"/>
       <c r="D80" s="22" t="s">
@@ -6119,12 +6125,12 @@
       <c r="X80" s="21"/>
       <c r="Y80" s="12"/>
     </row>
-    <row r="81" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="81" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B81" s="20" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="C81" s="21"/>
       <c r="D81" s="22" t="s">
@@ -6154,12 +6160,12 @@
       <c r="X81" s="21"/>
       <c r="Y81" s="12"/>
     </row>
-    <row r="82" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="82" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B82" s="20" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="C82" s="21"/>
       <c r="D82" s="22" t="s">
@@ -6225,12 +6231,12 @@
       </c>
       <c r="Y82" s="12"/>
     </row>
-    <row r="83" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="83" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B83" s="20" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="C83" s="21"/>
       <c r="D83" s="22" t="s">
@@ -6296,12 +6302,12 @@
       </c>
       <c r="Y83" s="12"/>
     </row>
-    <row r="84" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="84" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B84" s="20" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="C84" s="21"/>
       <c r="D84" s="22" t="s">
@@ -6365,12 +6371,12 @@
       </c>
       <c r="Y84" s="12"/>
     </row>
-    <row r="85" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="85" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B85" s="20" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="C85" s="21"/>
       <c r="D85" s="22" t="s">
@@ -6436,12 +6442,12 @@
       </c>
       <c r="Y85" s="12"/>
     </row>
-    <row r="86" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="86" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B86" s="20" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="C86" s="21"/>
       <c r="D86" s="22" t="s">
@@ -6499,12 +6505,12 @@
       </c>
       <c r="Y86" s="12"/>
     </row>
-    <row r="87" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="87" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B87" s="20" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="C87" s="21"/>
       <c r="D87" s="22" t="s">
@@ -6556,12 +6562,12 @@
       <c r="X87" s="21"/>
       <c r="Y87" s="12"/>
     </row>
-    <row r="88" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="88" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B88" s="20" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="C88" s="21"/>
       <c r="D88" s="22" t="s">
@@ -6591,12 +6597,12 @@
       <c r="X88" s="21"/>
       <c r="Y88" s="12"/>
     </row>
-    <row r="89" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="89" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B89" s="20" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="C89" s="21"/>
       <c r="D89" s="22" t="s">
@@ -6626,12 +6632,12 @@
       <c r="X89" s="21"/>
       <c r="Y89" s="12"/>
     </row>
-    <row r="90" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="90" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B90" s="20" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="C90" s="21"/>
       <c r="D90" s="22" t="s">
@@ -6661,12 +6667,12 @@
       <c r="X90" s="21"/>
       <c r="Y90" s="12"/>
     </row>
-    <row r="91" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="91" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B91" s="20" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="C91" s="21"/>
       <c r="D91" s="22" t="s">
@@ -6730,12 +6736,12 @@
       </c>
       <c r="Y91" s="12"/>
     </row>
-    <row r="92" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="92" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B92" s="20" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C92" s="21"/>
       <c r="D92" s="22" t="s">
@@ -6799,12 +6805,12 @@
       </c>
       <c r="Y92" s="12"/>
     </row>
-    <row r="93" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="93" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B93" s="20" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="C93" s="21"/>
       <c r="D93" s="22" t="s">
@@ -6868,12 +6874,12 @@
       </c>
       <c r="Y93" s="12"/>
     </row>
-    <row r="94" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="94" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B94" s="20" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="C94" s="21"/>
       <c r="D94" s="22" t="s">
@@ -6937,12 +6943,12 @@
       </c>
       <c r="Y94" s="12"/>
     </row>
-    <row r="95" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="95" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B95" s="20" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="C95" s="21"/>
       <c r="D95" s="22" t="s">
@@ -7006,12 +7012,12 @@
       </c>
       <c r="Y95" s="12"/>
     </row>
-    <row r="96" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="96" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B96" s="20" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C96" s="21"/>
       <c r="D96" s="22" t="s">
@@ -7077,12 +7083,12 @@
       </c>
       <c r="Y96" s="12"/>
     </row>
-    <row r="97" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="97" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B97" s="20" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="C97" s="21"/>
       <c r="D97" s="22" t="s">
@@ -7146,12 +7152,12 @@
       <c r="X97" s="21"/>
       <c r="Y97" s="12"/>
     </row>
-    <row r="98" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="98" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B98" s="20" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="C98" s="21"/>
       <c r="D98" s="22" t="s">
@@ -7215,12 +7221,12 @@
       <c r="X98" s="21"/>
       <c r="Y98" s="12"/>
     </row>
-    <row r="99" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="99" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B99" s="20" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="C99" s="21"/>
       <c r="D99" s="22" t="s">
@@ -7284,12 +7290,12 @@
       <c r="X99" s="21"/>
       <c r="Y99" s="12"/>
     </row>
-    <row r="100" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="100" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B100" s="20" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="C100" s="21"/>
       <c r="D100" s="22" t="s">
@@ -7353,12 +7359,12 @@
       <c r="X100" s="21"/>
       <c r="Y100" s="12"/>
     </row>
-    <row r="101" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="101" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B101" s="20" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="C101" s="21"/>
       <c r="D101" s="22" t="s">
@@ -7422,12 +7428,12 @@
       <c r="X101" s="21"/>
       <c r="Y101" s="12"/>
     </row>
-    <row r="102" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="102" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B102" s="20" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="C102" s="21"/>
       <c r="D102" s="22" t="s">
@@ -7457,12 +7463,12 @@
       <c r="X102" s="21"/>
       <c r="Y102" s="12"/>
     </row>
-    <row r="103" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="103" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B103" s="20" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="C103" s="21"/>
       <c r="D103" s="22" t="s">
@@ -7526,12 +7532,12 @@
       <c r="X103" s="21"/>
       <c r="Y103" s="12"/>
     </row>
-    <row r="104" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="104" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B104" s="20" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="C104" s="21"/>
       <c r="D104" s="22" t="s">
@@ -7579,12 +7585,12 @@
       <c r="X104" s="21"/>
       <c r="Y104" s="12"/>
     </row>
-    <row r="105" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="105" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B105" s="20" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="C105" s="21"/>
       <c r="D105" s="22" t="s">
@@ -7652,12 +7658,12 @@
       </c>
       <c r="Y105" s="12"/>
     </row>
-    <row r="106" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="106" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B106" s="20" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="C106" s="21"/>
       <c r="D106" s="22" t="s">
@@ -7725,12 +7731,12 @@
       </c>
       <c r="Y106" s="12"/>
     </row>
-    <row r="107" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="107" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B107" s="20" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="C107" s="21"/>
       <c r="D107" s="22" t="s">
@@ -7798,12 +7804,12 @@
       </c>
       <c r="Y107" s="12"/>
     </row>
-    <row r="108" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="108" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B108" s="20" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="C108" s="21"/>
       <c r="D108" s="22" t="s">
@@ -7869,12 +7875,12 @@
       </c>
       <c r="Y108" s="12"/>
     </row>
-    <row r="109" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="109" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B109" s="20" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="C109" s="21"/>
       <c r="D109" s="22" t="s">
@@ -7902,12 +7908,12 @@
       <c r="X109" s="21"/>
       <c r="Y109" s="12"/>
     </row>
-    <row r="110" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="110" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B110" s="39" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="C110" s="21"/>
       <c r="D110" s="22" t="s">
@@ -7973,12 +7979,12 @@
       </c>
       <c r="Y110" s="12"/>
     </row>
-    <row r="111" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="111" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B111" s="20" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="C111" s="21"/>
       <c r="D111" s="22" t="s">
@@ -8046,12 +8052,12 @@
       </c>
       <c r="Y111" s="12"/>
     </row>
-    <row r="112" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="112" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B112" s="20" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C112" s="21"/>
       <c r="D112" s="22" t="s">
@@ -8119,12 +8125,12 @@
       </c>
       <c r="Y112" s="12"/>
     </row>
-    <row r="113" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="113" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B113" s="20" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="C113" s="21"/>
       <c r="D113" s="22" t="s">
@@ -8176,12 +8182,12 @@
       <c r="X113" s="21"/>
       <c r="Y113" s="12"/>
     </row>
-    <row r="114" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="114" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="20" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="B114" s="20" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="C114" s="21"/>
       <c r="D114" s="22" t="s">
@@ -8203,7 +8209,7 @@
         <v>39</v>
       </c>
       <c r="J114" s="22" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="K114" s="22" t="s">
         <v>38</v>
@@ -8224,13 +8230,13 @@
         <v>39</v>
       </c>
       <c r="Q114" s="22" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="R114" s="22" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="S114" s="22" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="T114" s="22" t="s">
         <v>44</v>
@@ -8248,15 +8254,15 @@
         <v>39</v>
       </c>
       <c r="Y114" s="42" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="115" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="115" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="20" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="B115" s="20" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="C115" s="21"/>
       <c r="D115" s="22" t="s">
@@ -8278,58 +8284,58 @@
         <v>39</v>
       </c>
       <c r="J115" s="22" t="s">
+        <v>217</v>
+      </c>
+      <c r="K115" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="L115" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="M115" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N115" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="O115" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="P115" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q115" s="22" t="s">
+        <v>217</v>
+      </c>
+      <c r="R115" s="22" t="s">
+        <v>218</v>
+      </c>
+      <c r="S115" s="22" t="s">
+        <v>217</v>
+      </c>
+      <c r="T115" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="U115" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="V115" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="W115" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="X115" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y115" s="42"/>
+    </row>
+    <row r="116" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A116" s="20" t="s">
         <v>221</v>
       </c>
-      <c r="K115" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="L115" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="M115" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="N115" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="O115" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="P115" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q115" s="22" t="s">
-        <v>221</v>
-      </c>
-      <c r="R115" s="22" t="s">
+      <c r="B116" s="20" t="s">
         <v>222</v>
-      </c>
-      <c r="S115" s="22" t="s">
-        <v>221</v>
-      </c>
-      <c r="T115" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="U115" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="V115" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="W115" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="X115" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y115" s="42"/>
-    </row>
-    <row r="116" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A116" s="20" t="s">
-        <v>225</v>
-      </c>
-      <c r="B116" s="20" t="s">
-        <v>226</v>
       </c>
       <c r="C116" s="21"/>
       <c r="D116" s="22" t="s">
@@ -8397,12 +8403,12 @@
       </c>
       <c r="Y116" s="12"/>
     </row>
-    <row r="117" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="117" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="20" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="B117" s="20" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="C117" s="21"/>
       <c r="D117" s="22" t="s">
@@ -8470,12 +8476,12 @@
       </c>
       <c r="Y117" s="13"/>
     </row>
-    <row r="118" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="118" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="20" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B118" s="20" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="C118" s="21"/>
       <c r="D118" s="22" t="s">
@@ -8502,15 +8508,15 @@
       <c r="W118" s="21"/>
       <c r="X118" s="21"/>
       <c r="Y118" s="32" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="119" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="119" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="20" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B119" s="20" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="C119" s="21"/>
       <c r="D119" s="22" t="s">
@@ -8550,12 +8556,12 @@
       <c r="X119" s="21"/>
       <c r="Y119" s="33"/>
     </row>
-    <row r="120" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="120" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="20" t="s">
+        <v>223</v>
+      </c>
+      <c r="B120" s="20" t="s">
         <v>227</v>
-      </c>
-      <c r="B120" s="20" t="s">
-        <v>231</v>
       </c>
       <c r="C120" s="21"/>
       <c r="D120" s="22" t="s">
@@ -8583,12 +8589,12 @@
       <c r="X120" s="21"/>
       <c r="Y120" s="12"/>
     </row>
-    <row r="121" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="121" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="20" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B121" s="20" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="C121" s="21"/>
       <c r="D121" s="22" t="s">
@@ -8616,12 +8622,12 @@
       <c r="X121" s="21"/>
       <c r="Y121" s="12"/>
     </row>
-    <row r="122" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="122" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="20" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B122" s="39" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="C122" s="21"/>
       <c r="D122" s="22" t="s">
@@ -8649,12 +8655,12 @@
       <c r="X122" s="21"/>
       <c r="Y122" s="12"/>
     </row>
-    <row r="123" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="123" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="20" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B123" s="20" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="C123" s="21"/>
       <c r="D123" s="22" t="s">
@@ -8682,12 +8688,12 @@
       <c r="X123" s="21"/>
       <c r="Y123" s="12"/>
     </row>
-    <row r="124" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="124" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="20" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B124" s="20" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="C124" s="21"/>
       <c r="D124" s="22" t="s">
@@ -8715,12 +8721,12 @@
       <c r="X124" s="21"/>
       <c r="Y124" s="12"/>
     </row>
-    <row r="125" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="125" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="20" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B125" s="20" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C125" s="21"/>
       <c r="D125" s="22" t="s">
@@ -8748,12 +8754,12 @@
       <c r="X125" s="21"/>
       <c r="Y125" s="12"/>
     </row>
-    <row r="126" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="126" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="20" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B126" s="20" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="C126" s="21"/>
       <c r="D126" s="22" t="s">
@@ -8781,12 +8787,12 @@
       <c r="X126" s="21"/>
       <c r="Y126" s="12"/>
     </row>
-    <row r="127" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="127" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="20" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B127" s="20" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="C127" s="21"/>
       <c r="D127" s="22" t="s">
@@ -8814,12 +8820,12 @@
       <c r="X127" s="21"/>
       <c r="Y127" s="12"/>
     </row>
-    <row r="128" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="128" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="20" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B128" s="20" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="C128" s="21"/>
       <c r="D128" s="22" t="s">
@@ -8847,12 +8853,12 @@
       <c r="X128" s="21"/>
       <c r="Y128" s="12"/>
     </row>
-    <row r="129" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="129" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="20" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B129" s="20" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="C129" s="21"/>
       <c r="D129" s="22" t="s">
@@ -8880,12 +8886,12 @@
       <c r="X129" s="21"/>
       <c r="Y129" s="12"/>
     </row>
-    <row r="130" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="130" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="20" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B130" s="20" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="C130" s="21"/>
       <c r="D130" s="22" t="s">
@@ -8913,12 +8919,12 @@
       <c r="X130" s="21"/>
       <c r="Y130" s="12"/>
     </row>
-    <row r="131" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="131" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="20" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B131" s="20" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="C131" s="21"/>
       <c r="D131" s="22" t="s">
@@ -8946,12 +8952,12 @@
       <c r="X131" s="21"/>
       <c r="Y131" s="12"/>
     </row>
-    <row r="132" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="132" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="20" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B132" s="20" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="C132" s="21"/>
       <c r="D132" s="22" t="s">
@@ -8979,12 +8985,12 @@
       <c r="X132" s="21"/>
       <c r="Y132" s="12"/>
     </row>
-    <row r="133" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="133" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="20" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B133" s="20" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="C133" s="21"/>
       <c r="D133" s="22" t="s">
@@ -9012,12 +9018,12 @@
       <c r="X133" s="21"/>
       <c r="Y133" s="12"/>
     </row>
-    <row r="134" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="134" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="20" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B134" s="20" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="C134" s="21"/>
       <c r="D134" s="22" t="s">
@@ -9045,12 +9051,12 @@
       <c r="X134" s="21"/>
       <c r="Y134" s="12"/>
     </row>
-    <row r="135" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="135" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="20" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B135" s="20" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="C135" s="21"/>
       <c r="D135" s="22" t="s">
@@ -9078,12 +9084,12 @@
       <c r="X135" s="21"/>
       <c r="Y135" s="12"/>
     </row>
-    <row r="136" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="136" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="20" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B136" s="20" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="C136" s="21"/>
       <c r="D136" s="22" t="s">
@@ -9111,12 +9117,12 @@
       <c r="X136" s="21"/>
       <c r="Y136" s="12"/>
     </row>
-    <row r="137" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="137" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="20" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B137" s="20" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C137" s="21"/>
       <c r="D137" s="22" t="s">
@@ -9144,16 +9150,16 @@
       <c r="X137" s="21"/>
       <c r="Y137" s="12"/>
     </row>
-    <row r="138" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="138" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="20" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B138" s="20" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="C138" s="21"/>
       <c r="D138" s="22" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E138" s="25"/>
       <c r="F138" s="21"/>
@@ -9177,12 +9183,12 @@
       <c r="X138" s="21"/>
       <c r="Y138" s="12"/>
     </row>
-    <row r="139" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="139" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="20" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B139" s="20" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="C139" s="21"/>
       <c r="D139" s="22" t="s">
@@ -9210,12 +9216,12 @@
       <c r="X139" s="21"/>
       <c r="Y139" s="12"/>
     </row>
-    <row r="140" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="140" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="20" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B140" s="39" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="C140" s="21"/>
       <c r="D140" s="22" t="s">
@@ -9243,12 +9249,12 @@
       <c r="X140" s="21"/>
       <c r="Y140" s="12"/>
     </row>
-    <row r="141" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="141" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="20" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="B141" s="20" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="C141" s="12"/>
       <c r="D141" s="22" t="s">
@@ -9276,67 +9282,67 @@
       <c r="X141" s="12"/>
       <c r="Y141" s="12"/>
     </row>
-    <row r="142" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="142" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="20" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="B142" s="20" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="C142" s="12"/>
       <c r="D142" s="22" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="E142" s="23" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="F142" s="21"/>
       <c r="G142" s="22" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="H142" s="21"/>
       <c r="I142" s="21"/>
       <c r="J142" s="22" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="K142" s="22" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="L142" s="23" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="M142" s="22" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="N142" s="22" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="O142" s="21"/>
       <c r="P142" s="21"/>
       <c r="Q142" s="22" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="R142" s="22" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="S142" s="22" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="T142" s="21"/>
       <c r="U142" s="22" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="V142" s="21"/>
       <c r="W142" s="21"/>
       <c r="X142" s="21"/>
       <c r="Y142" s="12"/>
     </row>
-    <row r="143" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="143" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="20" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="B143" s="20" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="C143" s="12"/>
       <c r="D143" s="22" t="s">
@@ -9391,7 +9397,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.6640625" customWidth="1"/>
     <col min="2" max="2" width="28.33203125" customWidth="1"/>
@@ -9399,26 +9405,26 @@
     <col min="5" max="5" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="35" t="s">
+        <v>253</v>
+      </c>
+      <c r="B1" s="35" t="s">
+        <v>254</v>
+      </c>
+      <c r="C1" s="35" t="s">
+        <v>255</v>
+      </c>
+      <c r="D1" s="35" t="s">
+        <v>256</v>
+      </c>
+      <c r="E1" s="35" t="s">
         <v>257</v>
       </c>
-      <c r="B1" s="35" t="s">
+    </row>
+    <row r="2" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="36" t="s">
         <v>258</v>
-      </c>
-      <c r="C1" s="35" t="s">
-        <v>259</v>
-      </c>
-      <c r="D1" s="35" t="s">
-        <v>260</v>
-      </c>
-      <c r="E1" s="35" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="36" t="s">
-        <v>262</v>
       </c>
       <c r="B2" s="36" t="s">
         <v>13</v>
@@ -9429,9 +9435,9 @@
       <c r="D2" s="37"/>
       <c r="E2" s="37"/>
     </row>
-    <row r="3" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="36" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="B3" s="36" t="s">
         <v>15</v>
@@ -9442,9 +9448,9 @@
       <c r="D3" s="37"/>
       <c r="E3" s="37"/>
     </row>
-    <row r="4" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="36" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="B4" s="36" t="s">
         <v>17</v>
@@ -9455,9 +9461,9 @@
       <c r="D4" s="37"/>
       <c r="E4" s="37"/>
     </row>
-    <row r="5" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="36" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="B5" s="36" t="s">
         <v>14</v>
@@ -9466,13 +9472,13 @@
         <v>4</v>
       </c>
       <c r="D5" s="38" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="E5" s="37"/>
     </row>
-    <row r="6" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="36" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="B6" s="36" t="s">
         <v>16</v>
@@ -9481,13 +9487,13 @@
         <v>4</v>
       </c>
       <c r="D6" s="38" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="E6" s="37"/>
     </row>
-    <row r="7" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="36" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="B7" s="36" t="s">
         <v>18</v>
@@ -9496,13 +9502,13 @@
         <v>4</v>
       </c>
       <c r="D7" s="38" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="E7" s="37"/>
     </row>
-    <row r="8" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="36" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="B8" s="36" t="s">
         <v>19</v>
@@ -9511,13 +9517,13 @@
         <v>4</v>
       </c>
       <c r="D8" s="38" t="s">
+        <v>262</v>
+      </c>
+      <c r="E8" s="37"/>
+    </row>
+    <row r="9" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="36" t="s">
         <v>266</v>
-      </c>
-      <c r="E8" s="37"/>
-    </row>
-    <row r="9" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="36" t="s">
-        <v>270</v>
       </c>
       <c r="B9" s="36" t="s">
         <v>27</v>
@@ -9526,13 +9532,13 @@
         <v>5</v>
       </c>
       <c r="D9" s="38" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="E9" s="37"/>
     </row>
-    <row r="10" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="36" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="B10" s="36" t="s">
         <v>20</v>
@@ -9543,9 +9549,9 @@
       <c r="D10" s="37"/>
       <c r="E10" s="37"/>
     </row>
-    <row r="11" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="36" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="B11" s="36" t="s">
         <v>23</v>
@@ -9556,9 +9562,9 @@
       <c r="D11" s="37"/>
       <c r="E11" s="37"/>
     </row>
-    <row r="12" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="36" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="B12" s="36" t="s">
         <v>24</v>
@@ -9569,9 +9575,9 @@
       <c r="D12" s="37"/>
       <c r="E12" s="37"/>
     </row>
-    <row r="13" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="36" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="B13" s="36" t="s">
         <v>21</v>
@@ -9580,13 +9586,13 @@
         <v>6</v>
       </c>
       <c r="D13" s="38" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="E13" s="37"/>
     </row>
-    <row r="14" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="36" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="B14" s="36" t="s">
         <v>22</v>
@@ -9595,13 +9601,13 @@
         <v>6</v>
       </c>
       <c r="D14" s="38" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="E14" s="37"/>
     </row>
-    <row r="15" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="36" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="B15" s="36" t="s">
         <v>25</v>
@@ -9610,13 +9616,13 @@
         <v>6</v>
       </c>
       <c r="D15" s="38" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="E15" s="37"/>
     </row>
-    <row r="16" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="36" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="B16" s="36" t="s">
         <v>26</v>
@@ -9625,13 +9631,13 @@
         <v>6</v>
       </c>
       <c r="D16" s="38" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="E16" s="37"/>
     </row>
-    <row r="17" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="36" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="B17" s="36" t="s">
         <v>29</v>
@@ -9640,13 +9646,13 @@
         <v>5</v>
       </c>
       <c r="D17" s="38" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="E17" s="37"/>
     </row>
-    <row r="18" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="36" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="B18" s="36" t="s">
         <v>31</v>
@@ -9655,13 +9661,13 @@
         <v>5</v>
       </c>
       <c r="D18" s="38" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="E18" s="37"/>
     </row>
-    <row r="19" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="36" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="B19" s="36" t="s">
         <v>28</v>
@@ -9670,13 +9676,13 @@
         <v>5</v>
       </c>
       <c r="D19" s="38" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="E19" s="37"/>
     </row>
-    <row r="20" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="36" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="B20" s="36" t="s">
         <v>30</v>
@@ -9685,11 +9691,11 @@
         <v>5</v>
       </c>
       <c r="D20" s="38" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="E20" s="37"/>
     </row>
-    <row r="21" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="36" t="s">
         <v>33</v>
       </c>
@@ -9700,13 +9706,13 @@
         <v>5</v>
       </c>
       <c r="D21" s="38" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="E21" s="37"/>
     </row>
-    <row r="22" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="36" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="B22" s="36" t="s">
         <v>32</v>
@@ -9715,7 +9721,7 @@
         <v>5</v>
       </c>
       <c r="D22" s="38" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="E22" s="37"/>
     </row>

</xml_diff>

<commit_message>
HARJA-2609: Päivitä kalustoresurssien lukuoikeudet laadunvalvojille
</commit_message>
<xml_diff>
--- a/resources/roolit.xlsx
+++ b/resources/roolit.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\henrikkorpi\harjaroot\harja\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elias.tahto/projects/harjaroot/harja/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9117453F-AF44-42BA-8AC5-D732D5D3CE8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4835EC2-C571-6E49-B0E2-59FF02070A99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-9060" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Oikeudet" sheetId="1" r:id="rId1"/>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2050" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2052" uniqueCount="292">
   <si>
     <t xml:space="preserve">Roolimääritysten selitykset: </t>
   </si>
@@ -1553,11 +1553,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Y143"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="31.6640625" customWidth="1"/>
-    <col min="3" max="3" width="14.109375" customWidth="1"/>
+    <col min="3" max="3" width="14.1640625" customWidth="1"/>
     <col min="4" max="4" width="30.33203125" customWidth="1"/>
     <col min="5" max="5" width="26.33203125" style="1" customWidth="1"/>
     <col min="6" max="6" width="12.6640625" customWidth="1"/>
@@ -1566,22 +1566,22 @@
     <col min="9" max="9" width="18.33203125" customWidth="1"/>
     <col min="10" max="10" width="25.33203125" customWidth="1"/>
     <col min="11" max="11" width="40.6640625" customWidth="1"/>
-    <col min="12" max="12" width="38.109375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="38.1640625" style="1" customWidth="1"/>
     <col min="13" max="13" width="12.33203125" customWidth="1"/>
     <col min="14" max="14" width="10.6640625" customWidth="1"/>
-    <col min="15" max="16" width="12.44140625" customWidth="1"/>
+    <col min="15" max="16" width="12.5" customWidth="1"/>
     <col min="17" max="17" width="21.6640625" customWidth="1"/>
     <col min="18" max="18" width="36" customWidth="1"/>
     <col min="19" max="19" width="29.6640625" customWidth="1"/>
     <col min="20" max="20" width="15" customWidth="1"/>
     <col min="21" max="21" width="17.6640625" customWidth="1"/>
-    <col min="22" max="22" width="11.44140625" customWidth="1"/>
+    <col min="22" max="22" width="11.5" customWidth="1"/>
     <col min="23" max="23" width="11.6640625" customWidth="1"/>
     <col min="24" max="24" width="11.33203125" customWidth="1"/>
     <col min="25" max="25" width="59" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" ht="24" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="2"/>
       <c r="B1" s="3" t="s">
         <v>0</v>
@@ -1612,7 +1612,7 @@
       <c r="X1" s="2"/>
       <c r="Y1" s="2"/>
     </row>
-    <row r="2" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="44" t="s">
@@ -1641,7 +1641,7 @@
       <c r="X2" s="2"/>
       <c r="Y2" s="2"/>
     </row>
-    <row r="3" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="2"/>
       <c r="B3" s="4" t="s">
         <v>3</v>
@@ -1676,7 +1676,7 @@
       <c r="X3" s="2"/>
       <c r="Y3" s="2"/>
     </row>
-    <row r="4" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="9"/>
@@ -1703,7 +1703,7 @@
       <c r="X4" s="2"/>
       <c r="Y4" s="2"/>
     </row>
-    <row r="5" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="12"/>
       <c r="B5" s="12"/>
       <c r="C5" s="45" t="s">
@@ -1738,7 +1738,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="14" t="s">
         <v>11</v>
       </c>
@@ -1811,7 +1811,7 @@
       </c>
       <c r="Y6" s="19"/>
     </row>
-    <row r="7" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="20" t="s">
         <v>34</v>
       </c>
@@ -1884,7 +1884,7 @@
       </c>
       <c r="Y7" s="12"/>
     </row>
-    <row r="8" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="20" t="s">
         <v>34</v>
       </c>
@@ -1943,7 +1943,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="20" t="s">
         <v>34</v>
       </c>
@@ -1996,7 +1996,7 @@
       <c r="X9" s="21"/>
       <c r="Y9" s="12"/>
     </row>
-    <row r="10" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="20" t="s">
         <v>34</v>
       </c>
@@ -2049,7 +2049,7 @@
       <c r="X10" s="21"/>
       <c r="Y10" s="12"/>
     </row>
-    <row r="11" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="20" t="s">
         <v>34</v>
       </c>
@@ -2108,7 +2108,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="12" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="20" t="s">
         <v>34</v>
       </c>
@@ -2161,7 +2161,7 @@
       <c r="X12" s="21"/>
       <c r="Y12" s="12"/>
     </row>
-    <row r="13" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="20" t="s">
         <v>34</v>
       </c>
@@ -2228,7 +2228,7 @@
       <c r="X13" s="21"/>
       <c r="Y13" s="12"/>
     </row>
-    <row r="14" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="20" t="s">
         <v>34</v>
       </c>
@@ -2295,7 +2295,7 @@
       <c r="X14" s="21"/>
       <c r="Y14" s="12"/>
     </row>
-    <row r="15" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="39" t="s">
         <v>34</v>
       </c>
@@ -2310,7 +2310,9 @@
         <v>37</v>
       </c>
       <c r="F15" s="22"/>
-      <c r="G15" s="22"/>
+      <c r="G15" s="41" t="s">
+        <v>39</v>
+      </c>
       <c r="H15" s="22"/>
       <c r="I15" s="22"/>
       <c r="J15" s="22"/>
@@ -2318,7 +2320,9 @@
       <c r="L15" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="M15" s="22"/>
+      <c r="M15" s="41" t="s">
+        <v>39</v>
+      </c>
       <c r="N15" s="22"/>
       <c r="O15" s="22"/>
       <c r="P15" s="21"/>
@@ -2332,7 +2336,7 @@
       <c r="X15" s="21"/>
       <c r="Y15" s="12"/>
     </row>
-    <row r="16" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="20" t="s">
         <v>34</v>
       </c>
@@ -2389,7 +2393,7 @@
       <c r="X16" s="21"/>
       <c r="Y16" s="12"/>
     </row>
-    <row r="17" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="20" t="s">
         <v>34</v>
       </c>
@@ -2446,7 +2450,7 @@
       <c r="X17" s="21"/>
       <c r="Y17" s="12"/>
     </row>
-    <row r="18" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="20" t="s">
         <v>34</v>
       </c>
@@ -2503,7 +2507,7 @@
       <c r="X18" s="21"/>
       <c r="Y18" s="12"/>
     </row>
-    <row r="19" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="20" t="s">
         <v>34</v>
       </c>
@@ -2570,7 +2574,7 @@
       <c r="X19" s="21"/>
       <c r="Y19" s="12"/>
     </row>
-    <row r="20" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="20" t="s">
         <v>34</v>
       </c>
@@ -2637,7 +2641,7 @@
       <c r="X20" s="21"/>
       <c r="Y20" s="12"/>
     </row>
-    <row r="21" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="20" t="s">
         <v>34</v>
       </c>
@@ -2692,7 +2696,7 @@
       <c r="X21" s="21"/>
       <c r="Y21" s="12"/>
     </row>
-    <row r="22" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="20" t="s">
         <v>34</v>
       </c>
@@ -2753,7 +2757,7 @@
       <c r="X22" s="21"/>
       <c r="Y22" s="12"/>
     </row>
-    <row r="23" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="20" t="s">
         <v>34</v>
       </c>
@@ -2820,7 +2824,7 @@
       <c r="X23" s="21"/>
       <c r="Y23" s="12"/>
     </row>
-    <row r="24" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="20" t="s">
         <v>34</v>
       </c>
@@ -2893,7 +2897,7 @@
       </c>
       <c r="Y24" s="12"/>
     </row>
-    <row r="25" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="20" t="s">
         <v>34</v>
       </c>
@@ -2956,7 +2960,7 @@
       <c r="X25" s="21"/>
       <c r="Y25" s="12"/>
     </row>
-    <row r="26" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="20" t="s">
         <v>34</v>
       </c>
@@ -3029,7 +3033,7 @@
       </c>
       <c r="Y26" s="12"/>
     </row>
-    <row r="27" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="20" t="s">
         <v>34</v>
       </c>
@@ -3100,7 +3104,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="28" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="20" t="s">
         <v>34</v>
       </c>
@@ -3169,7 +3173,7 @@
       <c r="X28" s="21"/>
       <c r="Y28" s="12"/>
     </row>
-    <row r="29" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="20" t="s">
         <v>34</v>
       </c>
@@ -3224,7 +3228,7 @@
       <c r="X29" s="2"/>
       <c r="Y29" s="12"/>
     </row>
-    <row r="30" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="20" t="s">
         <v>34</v>
       </c>
@@ -3293,7 +3297,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="31" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="20" t="s">
         <v>34</v>
       </c>
@@ -3362,7 +3366,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="32" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="20" t="s">
         <v>34</v>
       </c>
@@ -3423,7 +3427,7 @@
       <c r="X32" s="21"/>
       <c r="Y32" s="12"/>
     </row>
-    <row r="33" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="20" t="s">
         <v>34</v>
       </c>
@@ -3480,7 +3484,7 @@
       <c r="X33" s="21"/>
       <c r="Y33" s="12"/>
     </row>
-    <row r="34" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A34" s="20" t="s">
         <v>34</v>
       </c>
@@ -3533,7 +3537,7 @@
       <c r="X34" s="21"/>
       <c r="Y34" s="12"/>
     </row>
-    <row r="35" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A35" s="20" t="s">
         <v>34</v>
       </c>
@@ -3578,7 +3582,7 @@
       <c r="X35" s="21"/>
       <c r="Y35" s="12"/>
     </row>
-    <row r="36" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A36" s="20" t="s">
         <v>34</v>
       </c>
@@ -3623,7 +3627,7 @@
       <c r="X36" s="2"/>
       <c r="Y36" s="2"/>
     </row>
-    <row r="37" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A37" s="20" t="s">
         <v>34</v>
       </c>
@@ -3670,7 +3674,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="38" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A38" s="20" t="s">
         <v>34</v>
       </c>
@@ -3727,7 +3731,7 @@
       </c>
       <c r="Y38" s="12"/>
     </row>
-    <row r="39" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A39" s="20" t="s">
         <v>34</v>
       </c>
@@ -3790,7 +3794,7 @@
       <c r="X39" s="21"/>
       <c r="Y39" s="12"/>
     </row>
-    <row r="40" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A40" s="20" t="s">
         <v>34</v>
       </c>
@@ -3843,7 +3847,7 @@
       <c r="X40" s="21"/>
       <c r="Y40" s="12"/>
     </row>
-    <row r="41" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A41" s="20" t="s">
         <v>34</v>
       </c>
@@ -3912,7 +3916,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="42" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A42" s="20" t="s">
         <v>34</v>
       </c>
@@ -3975,7 +3979,7 @@
       <c r="X42" s="21"/>
       <c r="Y42" s="12"/>
     </row>
-    <row r="43" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A43" s="20" t="s">
         <v>34</v>
       </c>
@@ -4040,7 +4044,7 @@
       <c r="X43" s="21"/>
       <c r="Y43" s="12"/>
     </row>
-    <row r="44" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A44" s="20" t="s">
         <v>34</v>
       </c>
@@ -4103,7 +4107,7 @@
       <c r="X44" s="21"/>
       <c r="Y44" s="12"/>
     </row>
-    <row r="45" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A45" s="20" t="s">
         <v>34</v>
       </c>
@@ -4166,7 +4170,7 @@
       <c r="X45" s="21"/>
       <c r="Y45" s="12"/>
     </row>
-    <row r="46" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A46" s="20" t="s">
         <v>34</v>
       </c>
@@ -4229,7 +4233,7 @@
       <c r="X46" s="21"/>
       <c r="Y46" s="12"/>
     </row>
-    <row r="47" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A47" s="20" t="s">
         <v>34</v>
       </c>
@@ -4292,7 +4296,7 @@
       <c r="X47" s="21"/>
       <c r="Y47" s="12"/>
     </row>
-    <row r="48" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A48" s="20" t="s">
         <v>34</v>
       </c>
@@ -4355,7 +4359,7 @@
       <c r="X48" s="21"/>
       <c r="Y48" s="12"/>
     </row>
-    <row r="49" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A49" s="20" t="s">
         <v>34</v>
       </c>
@@ -4418,7 +4422,7 @@
       <c r="X49" s="21"/>
       <c r="Y49" s="12"/>
     </row>
-    <row r="50" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A50" s="20" t="s">
         <v>34</v>
       </c>
@@ -4491,7 +4495,7 @@
       </c>
       <c r="Y50" s="12"/>
     </row>
-    <row r="51" spans="1:25" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:25" ht="27.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A51" s="20" t="s">
         <v>34</v>
       </c>
@@ -4544,7 +4548,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="52" spans="1:25" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:25" ht="69.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A52" s="20" t="s">
         <v>34</v>
       </c>
@@ -4597,7 +4601,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="53" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A53" s="20" t="s">
         <v>34</v>
       </c>
@@ -4648,7 +4652,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="54" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A54" s="20" t="s">
         <v>34</v>
       </c>
@@ -4697,7 +4701,7 @@
       <c r="X54" s="21"/>
       <c r="Y54" s="12"/>
     </row>
-    <row r="55" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A55" s="20" t="s">
         <v>34</v>
       </c>
@@ -4750,7 +4754,7 @@
       <c r="X55" s="2"/>
       <c r="Y55" s="2"/>
     </row>
-    <row r="56" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A56" s="20" t="s">
         <v>34</v>
       </c>
@@ -4799,7 +4803,7 @@
       <c r="X56" s="21"/>
       <c r="Y56" s="12"/>
     </row>
-    <row r="57" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A57" s="20" t="s">
         <v>34</v>
       </c>
@@ -4832,7 +4836,7 @@
       <c r="X57" s="21"/>
       <c r="Y57" s="12"/>
     </row>
-    <row r="58" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A58" s="20" t="s">
         <v>34</v>
       </c>
@@ -4885,7 +4889,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="59" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A59" s="20" t="s">
         <v>34</v>
       </c>
@@ -4918,7 +4922,7 @@
       <c r="X59" s="21"/>
       <c r="Y59" s="12"/>
     </row>
-    <row r="60" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A60" s="20" t="s">
         <v>34</v>
       </c>
@@ -4969,7 +4973,7 @@
       <c r="X60" s="21"/>
       <c r="Y60" s="12"/>
     </row>
-    <row r="61" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A61" s="20" t="s">
         <v>34</v>
       </c>
@@ -5032,7 +5036,7 @@
       <c r="X61" s="21"/>
       <c r="Y61" s="12"/>
     </row>
-    <row r="62" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A62" s="20" t="s">
         <v>34</v>
       </c>
@@ -5091,7 +5095,7 @@
       <c r="X62" s="21"/>
       <c r="Y62" s="12"/>
     </row>
-    <row r="63" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A63" s="20" t="s">
         <v>34</v>
       </c>
@@ -5152,7 +5156,7 @@
       <c r="X63" s="21"/>
       <c r="Y63" s="12"/>
     </row>
-    <row r="64" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A64" s="20" t="s">
         <v>34</v>
       </c>
@@ -5207,7 +5211,7 @@
       <c r="X64" s="21"/>
       <c r="Y64" s="12"/>
     </row>
-    <row r="65" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A65" s="20" t="s">
         <v>34</v>
       </c>
@@ -5280,7 +5284,7 @@
       </c>
       <c r="Y65" s="12"/>
     </row>
-    <row r="66" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A66" s="20" t="s">
         <v>168</v>
       </c>
@@ -5333,7 +5337,7 @@
       <c r="X66" s="21"/>
       <c r="Y66" s="12"/>
     </row>
-    <row r="67" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A67" s="20" t="s">
         <v>168</v>
       </c>
@@ -5386,7 +5390,7 @@
       <c r="X67" s="21"/>
       <c r="Y67" s="12"/>
     </row>
-    <row r="68" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A68" s="20" t="s">
         <v>168</v>
       </c>
@@ -5439,7 +5443,7 @@
       <c r="X68" s="21"/>
       <c r="Y68" s="12"/>
     </row>
-    <row r="69" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A69" s="20" t="s">
         <v>168</v>
       </c>
@@ -5492,7 +5496,7 @@
       <c r="X69" s="21"/>
       <c r="Y69" s="12"/>
     </row>
-    <row r="70" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A70" s="20" t="s">
         <v>168</v>
       </c>
@@ -5539,7 +5543,7 @@
       <c r="X70" s="21"/>
       <c r="Y70" s="12"/>
     </row>
-    <row r="71" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A71" s="20" t="s">
         <v>168</v>
       </c>
@@ -5592,7 +5596,7 @@
       <c r="X71" s="21"/>
       <c r="Y71" s="12"/>
     </row>
-    <row r="72" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A72" s="20" t="s">
         <v>168</v>
       </c>
@@ -5645,7 +5649,7 @@
       <c r="X72" s="21"/>
       <c r="Y72" s="12"/>
     </row>
-    <row r="73" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A73" s="20" t="s">
         <v>168</v>
       </c>
@@ -5698,7 +5702,7 @@
       <c r="X73" s="21"/>
       <c r="Y73" s="12"/>
     </row>
-    <row r="74" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A74" s="20" t="s">
         <v>168</v>
       </c>
@@ -5751,7 +5755,7 @@
       <c r="X74" s="21"/>
       <c r="Y74" s="12"/>
     </row>
-    <row r="75" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A75" s="20" t="s">
         <v>168</v>
       </c>
@@ -5786,7 +5790,7 @@
       <c r="X75" s="21"/>
       <c r="Y75" s="12"/>
     </row>
-    <row r="76" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A76" s="20" t="s">
         <v>168</v>
       </c>
@@ -5857,7 +5861,7 @@
       </c>
       <c r="Y76" s="12"/>
     </row>
-    <row r="77" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A77" s="20" t="s">
         <v>168</v>
       </c>
@@ -5930,7 +5934,7 @@
       </c>
       <c r="Y77" s="12"/>
     </row>
-    <row r="78" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A78" s="20" t="s">
         <v>168</v>
       </c>
@@ -6001,7 +6005,7 @@
       </c>
       <c r="Y78" s="12"/>
     </row>
-    <row r="79" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A79" s="20" t="s">
         <v>168</v>
       </c>
@@ -6072,7 +6076,7 @@
       </c>
       <c r="Y79" s="12"/>
     </row>
-    <row r="80" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A80" s="20" t="s">
         <v>168</v>
       </c>
@@ -6125,7 +6129,7 @@
       <c r="X80" s="21"/>
       <c r="Y80" s="12"/>
     </row>
-    <row r="81" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A81" s="20" t="s">
         <v>168</v>
       </c>
@@ -6160,7 +6164,7 @@
       <c r="X81" s="21"/>
       <c r="Y81" s="12"/>
     </row>
-    <row r="82" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A82" s="20" t="s">
         <v>168</v>
       </c>
@@ -6231,7 +6235,7 @@
       </c>
       <c r="Y82" s="12"/>
     </row>
-    <row r="83" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A83" s="20" t="s">
         <v>168</v>
       </c>
@@ -6302,7 +6306,7 @@
       </c>
       <c r="Y83" s="12"/>
     </row>
-    <row r="84" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A84" s="20" t="s">
         <v>168</v>
       </c>
@@ -6371,7 +6375,7 @@
       </c>
       <c r="Y84" s="12"/>
     </row>
-    <row r="85" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A85" s="20" t="s">
         <v>168</v>
       </c>
@@ -6442,7 +6446,7 @@
       </c>
       <c r="Y85" s="12"/>
     </row>
-    <row r="86" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A86" s="20" t="s">
         <v>168</v>
       </c>
@@ -6505,7 +6509,7 @@
       </c>
       <c r="Y86" s="12"/>
     </row>
-    <row r="87" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A87" s="20" t="s">
         <v>168</v>
       </c>
@@ -6562,7 +6566,7 @@
       <c r="X87" s="21"/>
       <c r="Y87" s="12"/>
     </row>
-    <row r="88" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A88" s="20" t="s">
         <v>168</v>
       </c>
@@ -6597,7 +6601,7 @@
       <c r="X88" s="21"/>
       <c r="Y88" s="12"/>
     </row>
-    <row r="89" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A89" s="20" t="s">
         <v>168</v>
       </c>
@@ -6632,7 +6636,7 @@
       <c r="X89" s="21"/>
       <c r="Y89" s="12"/>
     </row>
-    <row r="90" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A90" s="20" t="s">
         <v>168</v>
       </c>
@@ -6667,7 +6671,7 @@
       <c r="X90" s="21"/>
       <c r="Y90" s="12"/>
     </row>
-    <row r="91" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A91" s="20" t="s">
         <v>168</v>
       </c>
@@ -6736,7 +6740,7 @@
       </c>
       <c r="Y91" s="12"/>
     </row>
-    <row r="92" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A92" s="20" t="s">
         <v>168</v>
       </c>
@@ -6805,7 +6809,7 @@
       </c>
       <c r="Y92" s="12"/>
     </row>
-    <row r="93" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A93" s="20" t="s">
         <v>168</v>
       </c>
@@ -6874,7 +6878,7 @@
       </c>
       <c r="Y93" s="12"/>
     </row>
-    <row r="94" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A94" s="20" t="s">
         <v>168</v>
       </c>
@@ -6943,7 +6947,7 @@
       </c>
       <c r="Y94" s="12"/>
     </row>
-    <row r="95" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A95" s="20" t="s">
         <v>168</v>
       </c>
@@ -7012,7 +7016,7 @@
       </c>
       <c r="Y95" s="12"/>
     </row>
-    <row r="96" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A96" s="20" t="s">
         <v>168</v>
       </c>
@@ -7083,7 +7087,7 @@
       </c>
       <c r="Y96" s="12"/>
     </row>
-    <row r="97" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A97" s="20" t="s">
         <v>168</v>
       </c>
@@ -7152,7 +7156,7 @@
       <c r="X97" s="21"/>
       <c r="Y97" s="12"/>
     </row>
-    <row r="98" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A98" s="20" t="s">
         <v>168</v>
       </c>
@@ -7221,7 +7225,7 @@
       <c r="X98" s="21"/>
       <c r="Y98" s="12"/>
     </row>
-    <row r="99" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A99" s="20" t="s">
         <v>168</v>
       </c>
@@ -7290,7 +7294,7 @@
       <c r="X99" s="21"/>
       <c r="Y99" s="12"/>
     </row>
-    <row r="100" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A100" s="20" t="s">
         <v>168</v>
       </c>
@@ -7359,7 +7363,7 @@
       <c r="X100" s="21"/>
       <c r="Y100" s="12"/>
     </row>
-    <row r="101" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A101" s="20" t="s">
         <v>168</v>
       </c>
@@ -7428,7 +7432,7 @@
       <c r="X101" s="21"/>
       <c r="Y101" s="12"/>
     </row>
-    <row r="102" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A102" s="20" t="s">
         <v>168</v>
       </c>
@@ -7463,7 +7467,7 @@
       <c r="X102" s="21"/>
       <c r="Y102" s="12"/>
     </row>
-    <row r="103" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A103" s="20" t="s">
         <v>168</v>
       </c>
@@ -7532,7 +7536,7 @@
       <c r="X103" s="21"/>
       <c r="Y103" s="12"/>
     </row>
-    <row r="104" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A104" s="20" t="s">
         <v>168</v>
       </c>
@@ -7585,7 +7589,7 @@
       <c r="X104" s="21"/>
       <c r="Y104" s="12"/>
     </row>
-    <row r="105" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A105" s="20" t="s">
         <v>168</v>
       </c>
@@ -7658,7 +7662,7 @@
       </c>
       <c r="Y105" s="12"/>
     </row>
-    <row r="106" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A106" s="20" t="s">
         <v>168</v>
       </c>
@@ -7731,7 +7735,7 @@
       </c>
       <c r="Y106" s="12"/>
     </row>
-    <row r="107" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A107" s="20" t="s">
         <v>168</v>
       </c>
@@ -7804,7 +7808,7 @@
       </c>
       <c r="Y107" s="12"/>
     </row>
-    <row r="108" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A108" s="20" t="s">
         <v>168</v>
       </c>
@@ -7875,7 +7879,7 @@
       </c>
       <c r="Y108" s="12"/>
     </row>
-    <row r="109" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A109" s="20" t="s">
         <v>168</v>
       </c>
@@ -7908,7 +7912,7 @@
       <c r="X109" s="21"/>
       <c r="Y109" s="12"/>
     </row>
-    <row r="110" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A110" s="20" t="s">
         <v>168</v>
       </c>
@@ -7979,7 +7983,7 @@
       </c>
       <c r="Y110" s="12"/>
     </row>
-    <row r="111" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A111" s="20" t="s">
         <v>168</v>
       </c>
@@ -8052,7 +8056,7 @@
       </c>
       <c r="Y111" s="12"/>
     </row>
-    <row r="112" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A112" s="20" t="s">
         <v>168</v>
       </c>
@@ -8125,7 +8129,7 @@
       </c>
       <c r="Y112" s="12"/>
     </row>
-    <row r="113" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A113" s="20" t="s">
         <v>168</v>
       </c>
@@ -8182,7 +8186,7 @@
       <c r="X113" s="21"/>
       <c r="Y113" s="12"/>
     </row>
-    <row r="114" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A114" s="20" t="s">
         <v>215</v>
       </c>
@@ -8257,7 +8261,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="115" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A115" s="20" t="s">
         <v>215</v>
       </c>
@@ -8330,7 +8334,7 @@
       </c>
       <c r="Y115" s="42"/>
     </row>
-    <row r="116" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A116" s="20" t="s">
         <v>221</v>
       </c>
@@ -8403,7 +8407,7 @@
       </c>
       <c r="Y116" s="12"/>
     </row>
-    <row r="117" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A117" s="20" t="s">
         <v>213</v>
       </c>
@@ -8476,7 +8480,7 @@
       </c>
       <c r="Y117" s="13"/>
     </row>
-    <row r="118" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A118" s="20" t="s">
         <v>223</v>
       </c>
@@ -8511,7 +8515,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="119" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A119" s="20" t="s">
         <v>223</v>
       </c>
@@ -8556,7 +8560,7 @@
       <c r="X119" s="21"/>
       <c r="Y119" s="33"/>
     </row>
-    <row r="120" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A120" s="20" t="s">
         <v>223</v>
       </c>
@@ -8589,7 +8593,7 @@
       <c r="X120" s="21"/>
       <c r="Y120" s="12"/>
     </row>
-    <row r="121" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A121" s="20" t="s">
         <v>223</v>
       </c>
@@ -8622,7 +8626,7 @@
       <c r="X121" s="21"/>
       <c r="Y121" s="12"/>
     </row>
-    <row r="122" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A122" s="20" t="s">
         <v>223</v>
       </c>
@@ -8655,7 +8659,7 @@
       <c r="X122" s="21"/>
       <c r="Y122" s="12"/>
     </row>
-    <row r="123" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A123" s="20" t="s">
         <v>223</v>
       </c>
@@ -8688,7 +8692,7 @@
       <c r="X123" s="21"/>
       <c r="Y123" s="12"/>
     </row>
-    <row r="124" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A124" s="20" t="s">
         <v>223</v>
       </c>
@@ -8721,7 +8725,7 @@
       <c r="X124" s="21"/>
       <c r="Y124" s="12"/>
     </row>
-    <row r="125" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A125" s="20" t="s">
         <v>223</v>
       </c>
@@ -8754,7 +8758,7 @@
       <c r="X125" s="21"/>
       <c r="Y125" s="12"/>
     </row>
-    <row r="126" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A126" s="20" t="s">
         <v>223</v>
       </c>
@@ -8787,7 +8791,7 @@
       <c r="X126" s="21"/>
       <c r="Y126" s="12"/>
     </row>
-    <row r="127" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A127" s="20" t="s">
         <v>223</v>
       </c>
@@ -8820,7 +8824,7 @@
       <c r="X127" s="21"/>
       <c r="Y127" s="12"/>
     </row>
-    <row r="128" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A128" s="20" t="s">
         <v>223</v>
       </c>
@@ -8853,7 +8857,7 @@
       <c r="X128" s="21"/>
       <c r="Y128" s="12"/>
     </row>
-    <row r="129" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A129" s="20" t="s">
         <v>223</v>
       </c>
@@ -8886,7 +8890,7 @@
       <c r="X129" s="21"/>
       <c r="Y129" s="12"/>
     </row>
-    <row r="130" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A130" s="20" t="s">
         <v>223</v>
       </c>
@@ -8919,7 +8923,7 @@
       <c r="X130" s="21"/>
       <c r="Y130" s="12"/>
     </row>
-    <row r="131" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A131" s="20" t="s">
         <v>223</v>
       </c>
@@ -8952,7 +8956,7 @@
       <c r="X131" s="21"/>
       <c r="Y131" s="12"/>
     </row>
-    <row r="132" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A132" s="20" t="s">
         <v>223</v>
       </c>
@@ -8985,7 +8989,7 @@
       <c r="X132" s="21"/>
       <c r="Y132" s="12"/>
     </row>
-    <row r="133" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A133" s="20" t="s">
         <v>223</v>
       </c>
@@ -9018,7 +9022,7 @@
       <c r="X133" s="21"/>
       <c r="Y133" s="12"/>
     </row>
-    <row r="134" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A134" s="20" t="s">
         <v>223</v>
       </c>
@@ -9051,7 +9055,7 @@
       <c r="X134" s="21"/>
       <c r="Y134" s="12"/>
     </row>
-    <row r="135" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A135" s="20" t="s">
         <v>223</v>
       </c>
@@ -9084,7 +9088,7 @@
       <c r="X135" s="21"/>
       <c r="Y135" s="12"/>
     </row>
-    <row r="136" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A136" s="20" t="s">
         <v>223</v>
       </c>
@@ -9117,7 +9121,7 @@
       <c r="X136" s="21"/>
       <c r="Y136" s="12"/>
     </row>
-    <row r="137" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A137" s="20" t="s">
         <v>223</v>
       </c>
@@ -9150,7 +9154,7 @@
       <c r="X137" s="21"/>
       <c r="Y137" s="12"/>
     </row>
-    <row r="138" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A138" s="20" t="s">
         <v>223</v>
       </c>
@@ -9183,7 +9187,7 @@
       <c r="X138" s="21"/>
       <c r="Y138" s="12"/>
     </row>
-    <row r="139" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A139" s="20" t="s">
         <v>223</v>
       </c>
@@ -9216,7 +9220,7 @@
       <c r="X139" s="21"/>
       <c r="Y139" s="12"/>
     </row>
-    <row r="140" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A140" s="20" t="s">
         <v>223</v>
       </c>
@@ -9249,7 +9253,7 @@
       <c r="X140" s="21"/>
       <c r="Y140" s="12"/>
     </row>
-    <row r="141" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A141" s="20" t="s">
         <v>245</v>
       </c>
@@ -9282,7 +9286,7 @@
       <c r="X141" s="12"/>
       <c r="Y141" s="12"/>
     </row>
-    <row r="142" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A142" s="20" t="s">
         <v>247</v>
       </c>
@@ -9337,7 +9341,7 @@
       <c r="X142" s="21"/>
       <c r="Y142" s="12"/>
     </row>
-    <row r="143" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A143" s="20" t="s">
         <v>252</v>
       </c>
@@ -9397,7 +9401,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E22"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="29.6640625" customWidth="1"/>
     <col min="2" max="2" width="28.33203125" customWidth="1"/>
@@ -9405,7 +9409,7 @@
     <col min="5" max="5" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="35" t="s">
         <v>253</v>
       </c>
@@ -9422,7 +9426,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="36" t="s">
         <v>258</v>
       </c>
@@ -9435,7 +9439,7 @@
       <c r="D2" s="37"/>
       <c r="E2" s="37"/>
     </row>
-    <row r="3" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="36" t="s">
         <v>259</v>
       </c>
@@ -9448,7 +9452,7 @@
       <c r="D3" s="37"/>
       <c r="E3" s="37"/>
     </row>
-    <row r="4" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="36" t="s">
         <v>260</v>
       </c>
@@ -9461,7 +9465,7 @@
       <c r="D4" s="37"/>
       <c r="E4" s="37"/>
     </row>
-    <row r="5" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="36" t="s">
         <v>261</v>
       </c>
@@ -9476,7 +9480,7 @@
       </c>
       <c r="E5" s="37"/>
     </row>
-    <row r="6" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="36" t="s">
         <v>263</v>
       </c>
@@ -9491,7 +9495,7 @@
       </c>
       <c r="E6" s="37"/>
     </row>
-    <row r="7" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="36" t="s">
         <v>264</v>
       </c>
@@ -9506,7 +9510,7 @@
       </c>
       <c r="E7" s="37"/>
     </row>
-    <row r="8" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="36" t="s">
         <v>265</v>
       </c>
@@ -9521,7 +9525,7 @@
       </c>
       <c r="E8" s="37"/>
     </row>
-    <row r="9" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="36" t="s">
         <v>266</v>
       </c>
@@ -9536,7 +9540,7 @@
       </c>
       <c r="E9" s="37"/>
     </row>
-    <row r="10" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="36" t="s">
         <v>268</v>
       </c>
@@ -9549,7 +9553,7 @@
       <c r="D10" s="37"/>
       <c r="E10" s="37"/>
     </row>
-    <row r="11" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="36" t="s">
         <v>269</v>
       </c>
@@ -9562,7 +9566,7 @@
       <c r="D11" s="37"/>
       <c r="E11" s="37"/>
     </row>
-    <row r="12" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="36" t="s">
         <v>270</v>
       </c>
@@ -9575,7 +9579,7 @@
       <c r="D12" s="37"/>
       <c r="E12" s="37"/>
     </row>
-    <row r="13" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="36" t="s">
         <v>271</v>
       </c>
@@ -9590,7 +9594,7 @@
       </c>
       <c r="E13" s="37"/>
     </row>
-    <row r="14" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="36" t="s">
         <v>272</v>
       </c>
@@ -9605,7 +9609,7 @@
       </c>
       <c r="E14" s="37"/>
     </row>
-    <row r="15" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="36" t="s">
         <v>273</v>
       </c>
@@ -9620,7 +9624,7 @@
       </c>
       <c r="E15" s="37"/>
     </row>
-    <row r="16" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="36" t="s">
         <v>274</v>
       </c>
@@ -9635,7 +9639,7 @@
       </c>
       <c r="E16" s="37"/>
     </row>
-    <row r="17" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="36" t="s">
         <v>275</v>
       </c>
@@ -9650,7 +9654,7 @@
       </c>
       <c r="E17" s="37"/>
     </row>
-    <row r="18" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="36" t="s">
         <v>276</v>
       </c>
@@ -9665,7 +9669,7 @@
       </c>
       <c r="E18" s="37"/>
     </row>
-    <row r="19" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="36" t="s">
         <v>277</v>
       </c>
@@ -9680,7 +9684,7 @@
       </c>
       <c r="E19" s="37"/>
     </row>
-    <row r="20" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="36" t="s">
         <v>278</v>
       </c>
@@ -9695,7 +9699,7 @@
       </c>
       <c r="E20" s="37"/>
     </row>
-    <row r="21" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="36" t="s">
         <v>33</v>
       </c>
@@ -9710,7 +9714,7 @@
       </c>
       <c r="E21" s="37"/>
     </row>
-    <row r="22" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="36" t="s">
         <v>279</v>
       </c>

</xml_diff>

<commit_message>
Uusi raportti roolit exceliin
</commit_message>
<xml_diff>
--- a/resources/roolit.xlsx
+++ b/resources/roolit.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elias.tahto/projects/harjaroot/harja/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/markusva/repos/Github/harja/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4835EC2-C571-6E49-B0E2-59FF02070A99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{395E9FDC-2890-D84A-A4EF-17F619C2C236}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="40160" yWindow="-5300" windowWidth="34560" windowHeight="21580" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Oikeudet" sheetId="1" r:id="rId1"/>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2052" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2065" uniqueCount="293">
   <si>
     <t xml:space="preserve">Roolimääritysten selitykset: </t>
   </si>
@@ -942,6 +942,9 @@
   </si>
   <si>
     <t>R*,W+,aseta-näkyviin-urakoitsijalle+,nakee-tilaajan-tarkastukset*</t>
+  </si>
+  <si>
+    <t>Välikatselmus</t>
   </si>
 </sst>
 </file>
@@ -1220,7 +1223,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normaali" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1236,7 +1239,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office-teema">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1552,7 +1555,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y143"/>
+  <dimension ref="A1:Y144"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -8188,10 +8191,10 @@
     </row>
     <row r="114" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A114" s="20" t="s">
-        <v>215</v>
-      </c>
-      <c r="B114" s="20" t="s">
-        <v>216</v>
+        <v>168</v>
+      </c>
+      <c r="B114" s="39" t="s">
+        <v>292</v>
       </c>
       <c r="C114" s="21"/>
       <c r="D114" s="22" t="s">
@@ -8203,17 +8206,11 @@
       <c r="F114" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="G114" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="H114" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="I114" s="22" t="s">
-        <v>39</v>
-      </c>
+      <c r="G114" s="21"/>
+      <c r="H114" s="21"/>
+      <c r="I114" s="21"/>
       <c r="J114" s="22" t="s">
-        <v>217</v>
+        <v>39</v>
       </c>
       <c r="K114" s="22" t="s">
         <v>38</v>
@@ -8221,52 +8218,36 @@
       <c r="L114" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="M114" s="22" t="s">
-        <v>39</v>
-      </c>
+      <c r="M114" s="21"/>
       <c r="N114" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="O114" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="P114" s="22" t="s">
-        <v>39</v>
-      </c>
+      <c r="O114" s="21"/>
+      <c r="P114" s="21"/>
       <c r="Q114" s="22" t="s">
-        <v>217</v>
+        <v>39</v>
       </c>
       <c r="R114" s="22" t="s">
-        <v>218</v>
+        <v>44</v>
       </c>
       <c r="S114" s="22" t="s">
-        <v>217</v>
-      </c>
-      <c r="T114" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="U114" s="22" t="s">
-        <v>39</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="T114" s="21"/>
+      <c r="U114" s="21"/>
       <c r="V114" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="W114" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="X114" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y114" s="42" t="s">
-        <v>219</v>
-      </c>
+      <c r="W114" s="21"/>
+      <c r="X114" s="21"/>
+      <c r="Y114" s="12"/>
     </row>
     <row r="115" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A115" s="20" t="s">
         <v>215</v>
       </c>
       <c r="B115" s="20" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="C115" s="21"/>
       <c r="D115" s="22" t="s">
@@ -8332,18 +8313,20 @@
       <c r="X115" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="Y115" s="42"/>
+      <c r="Y115" s="42" t="s">
+        <v>219</v>
+      </c>
     </row>
     <row r="116" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A116" s="20" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="B116" s="20" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C116" s="21"/>
       <c r="D116" s="22" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E116" s="23" t="s">
         <v>38</v>
@@ -8361,10 +8344,10 @@
         <v>39</v>
       </c>
       <c r="J116" s="22" t="s">
-        <v>39</v>
+        <v>217</v>
       </c>
       <c r="K116" s="22" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="L116" s="23" t="s">
         <v>38</v>
@@ -8382,37 +8365,37 @@
         <v>39</v>
       </c>
       <c r="Q116" s="22" t="s">
-        <v>39</v>
+        <v>217</v>
       </c>
       <c r="R116" s="22" t="s">
-        <v>42</v>
+        <v>218</v>
       </c>
       <c r="S116" s="22" t="s">
-        <v>40</v>
+        <v>217</v>
       </c>
       <c r="T116" s="22" t="s">
         <v>44</v>
       </c>
       <c r="U116" s="22" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="V116" s="22" t="s">
         <v>44</v>
       </c>
       <c r="W116" s="22" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="X116" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y116" s="12"/>
+        <v>39</v>
+      </c>
+      <c r="Y116" s="42"/>
     </row>
     <row r="117" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A117" s="20" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="B117" s="20" t="s">
-        <v>213</v>
+        <v>222</v>
       </c>
       <c r="C117" s="21"/>
       <c r="D117" s="22" t="s">
@@ -8478,77 +8461,103 @@
       <c r="X117" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="Y117" s="13"/>
+      <c r="Y117" s="12"/>
     </row>
     <row r="118" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A118" s="20" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="B118" s="20" t="s">
-        <v>224</v>
+        <v>213</v>
       </c>
       <c r="C118" s="21"/>
       <c r="D118" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="E118" s="25"/>
-      <c r="F118" s="21"/>
-      <c r="G118" s="21"/>
-      <c r="H118" s="21"/>
-      <c r="I118" s="21"/>
-      <c r="J118" s="21"/>
-      <c r="K118" s="21"/>
-      <c r="L118" s="25"/>
-      <c r="M118" s="21"/>
-      <c r="N118" s="21"/>
-      <c r="O118" s="21"/>
-      <c r="P118" s="21"/>
-      <c r="Q118" s="21"/>
-      <c r="R118" s="21"/>
-      <c r="S118" s="21"/>
-      <c r="T118" s="21"/>
-      <c r="U118" s="21"/>
-      <c r="V118" s="21"/>
-      <c r="W118" s="21"/>
-      <c r="X118" s="21"/>
-      <c r="Y118" s="32" t="s">
-        <v>225</v>
-      </c>
+      <c r="E118" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="F118" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="G118" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="H118" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="I118" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="J118" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="K118" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="L118" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="M118" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N118" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="O118" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="P118" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q118" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="R118" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="S118" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="T118" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="U118" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="V118" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="W118" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="X118" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="Y118" s="13"/>
     </row>
     <row r="119" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A119" s="20" t="s">
         <v>223</v>
       </c>
       <c r="B119" s="20" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C119" s="21"/>
       <c r="D119" s="22" t="s">
         <v>41</v>
       </c>
       <c r="E119" s="25"/>
-      <c r="F119" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="G119" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="H119" s="22" t="s">
-        <v>46</v>
-      </c>
+      <c r="F119" s="21"/>
+      <c r="G119" s="21"/>
+      <c r="H119" s="21"/>
       <c r="I119" s="21"/>
       <c r="J119" s="21"/>
       <c r="K119" s="21"/>
       <c r="L119" s="25"/>
-      <c r="M119" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="N119" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="O119" s="22" t="s">
-        <v>46</v>
-      </c>
+      <c r="M119" s="21"/>
+      <c r="N119" s="21"/>
+      <c r="O119" s="21"/>
       <c r="P119" s="21"/>
       <c r="Q119" s="21"/>
       <c r="R119" s="21"/>
@@ -8558,30 +8567,44 @@
       <c r="V119" s="21"/>
       <c r="W119" s="21"/>
       <c r="X119" s="21"/>
-      <c r="Y119" s="33"/>
+      <c r="Y119" s="32" t="s">
+        <v>225</v>
+      </c>
     </row>
     <row r="120" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A120" s="20" t="s">
         <v>223</v>
       </c>
       <c r="B120" s="20" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C120" s="21"/>
       <c r="D120" s="22" t="s">
         <v>41</v>
       </c>
       <c r="E120" s="25"/>
-      <c r="F120" s="21"/>
-      <c r="G120" s="21"/>
-      <c r="H120" s="21"/>
+      <c r="F120" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="G120" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="H120" s="22" t="s">
+        <v>46</v>
+      </c>
       <c r="I120" s="21"/>
       <c r="J120" s="21"/>
       <c r="K120" s="21"/>
       <c r="L120" s="25"/>
-      <c r="M120" s="21"/>
-      <c r="N120" s="21"/>
-      <c r="O120" s="21"/>
+      <c r="M120" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="N120" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="O120" s="22" t="s">
+        <v>46</v>
+      </c>
       <c r="P120" s="21"/>
       <c r="Q120" s="21"/>
       <c r="R120" s="21"/>
@@ -8591,14 +8614,14 @@
       <c r="V120" s="21"/>
       <c r="W120" s="21"/>
       <c r="X120" s="21"/>
-      <c r="Y120" s="12"/>
+      <c r="Y120" s="33"/>
     </row>
     <row r="121" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A121" s="20" t="s">
         <v>223</v>
       </c>
       <c r="B121" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C121" s="21"/>
       <c r="D121" s="22" t="s">
@@ -8630,8 +8653,8 @@
       <c r="A122" s="20" t="s">
         <v>223</v>
       </c>
-      <c r="B122" s="39" t="s">
-        <v>229</v>
+      <c r="B122" s="20" t="s">
+        <v>228</v>
       </c>
       <c r="C122" s="21"/>
       <c r="D122" s="22" t="s">
@@ -8663,8 +8686,8 @@
       <c r="A123" s="20" t="s">
         <v>223</v>
       </c>
-      <c r="B123" s="20" t="s">
-        <v>230</v>
+      <c r="B123" s="39" t="s">
+        <v>229</v>
       </c>
       <c r="C123" s="21"/>
       <c r="D123" s="22" t="s">
@@ -8697,7 +8720,7 @@
         <v>223</v>
       </c>
       <c r="B124" s="20" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C124" s="21"/>
       <c r="D124" s="22" t="s">
@@ -8730,7 +8753,7 @@
         <v>223</v>
       </c>
       <c r="B125" s="20" t="s">
-        <v>83</v>
+        <v>231</v>
       </c>
       <c r="C125" s="21"/>
       <c r="D125" s="22" t="s">
@@ -8763,7 +8786,7 @@
         <v>223</v>
       </c>
       <c r="B126" s="20" t="s">
-        <v>232</v>
+        <v>83</v>
       </c>
       <c r="C126" s="21"/>
       <c r="D126" s="22" t="s">
@@ -8796,7 +8819,7 @@
         <v>223</v>
       </c>
       <c r="B127" s="20" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C127" s="21"/>
       <c r="D127" s="22" t="s">
@@ -8829,7 +8852,7 @@
         <v>223</v>
       </c>
       <c r="B128" s="20" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C128" s="21"/>
       <c r="D128" s="22" t="s">
@@ -8862,7 +8885,7 @@
         <v>223</v>
       </c>
       <c r="B129" s="20" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C129" s="21"/>
       <c r="D129" s="22" t="s">
@@ -8895,7 +8918,7 @@
         <v>223</v>
       </c>
       <c r="B130" s="20" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C130" s="21"/>
       <c r="D130" s="22" t="s">
@@ -8928,7 +8951,7 @@
         <v>223</v>
       </c>
       <c r="B131" s="20" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C131" s="21"/>
       <c r="D131" s="22" t="s">
@@ -8956,12 +8979,12 @@
       <c r="X131" s="21"/>
       <c r="Y131" s="12"/>
     </row>
-    <row r="132" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="132" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A132" s="20" t="s">
         <v>223</v>
       </c>
       <c r="B132" s="20" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C132" s="21"/>
       <c r="D132" s="22" t="s">
@@ -8994,7 +9017,7 @@
         <v>223</v>
       </c>
       <c r="B133" s="20" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C133" s="21"/>
       <c r="D133" s="22" t="s">
@@ -9027,7 +9050,7 @@
         <v>223</v>
       </c>
       <c r="B134" s="20" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C134" s="21"/>
       <c r="D134" s="22" t="s">
@@ -9060,7 +9083,7 @@
         <v>223</v>
       </c>
       <c r="B135" s="20" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C135" s="21"/>
       <c r="D135" s="22" t="s">
@@ -9093,7 +9116,7 @@
         <v>223</v>
       </c>
       <c r="B136" s="20" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C136" s="21"/>
       <c r="D136" s="22" t="s">
@@ -9126,7 +9149,7 @@
         <v>223</v>
       </c>
       <c r="B137" s="20" t="s">
-        <v>76</v>
+        <v>242</v>
       </c>
       <c r="C137" s="21"/>
       <c r="D137" s="22" t="s">
@@ -9159,11 +9182,11 @@
         <v>223</v>
       </c>
       <c r="B138" s="20" t="s">
-        <v>243</v>
+        <v>76</v>
       </c>
       <c r="C138" s="21"/>
       <c r="D138" s="22" t="s">
-        <v>108</v>
+        <v>41</v>
       </c>
       <c r="E138" s="25"/>
       <c r="F138" s="21"/>
@@ -9192,11 +9215,11 @@
         <v>223</v>
       </c>
       <c r="B139" s="20" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C139" s="21"/>
       <c r="D139" s="22" t="s">
-        <v>41</v>
+        <v>108</v>
       </c>
       <c r="E139" s="25"/>
       <c r="F139" s="21"/>
@@ -9224,8 +9247,8 @@
       <c r="A140" s="20" t="s">
         <v>223</v>
       </c>
-      <c r="B140" s="39" t="s">
-        <v>280</v>
+      <c r="B140" s="20" t="s">
+        <v>244</v>
       </c>
       <c r="C140" s="21"/>
       <c r="D140" s="22" t="s">
@@ -9255,134 +9278,167 @@
     </row>
     <row r="141" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A141" s="20" t="s">
-        <v>245</v>
-      </c>
-      <c r="B141" s="20" t="s">
-        <v>246</v>
-      </c>
-      <c r="C141" s="12"/>
+        <v>223</v>
+      </c>
+      <c r="B141" s="39" t="s">
+        <v>280</v>
+      </c>
+      <c r="C141" s="21"/>
       <c r="D141" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="E141" s="34"/>
-      <c r="F141" s="12"/>
-      <c r="G141" s="12"/>
-      <c r="H141" s="12"/>
-      <c r="I141" s="12"/>
-      <c r="J141" s="12"/>
-      <c r="K141" s="12"/>
-      <c r="L141" s="34"/>
-      <c r="M141" s="12"/>
-      <c r="N141" s="12"/>
-      <c r="O141" s="12"/>
-      <c r="P141" s="12"/>
-      <c r="Q141" s="12"/>
-      <c r="R141" s="12"/>
-      <c r="S141" s="12"/>
-      <c r="T141" s="12"/>
-      <c r="U141" s="12"/>
-      <c r="V141" s="12"/>
-      <c r="W141" s="12"/>
-      <c r="X141" s="12"/>
+      <c r="E141" s="25"/>
+      <c r="F141" s="21"/>
+      <c r="G141" s="21"/>
+      <c r="H141" s="21"/>
+      <c r="I141" s="21"/>
+      <c r="J141" s="21"/>
+      <c r="K141" s="21"/>
+      <c r="L141" s="25"/>
+      <c r="M141" s="21"/>
+      <c r="N141" s="21"/>
+      <c r="O141" s="21"/>
+      <c r="P141" s="21"/>
+      <c r="Q141" s="21"/>
+      <c r="R141" s="21"/>
+      <c r="S141" s="21"/>
+      <c r="T141" s="21"/>
+      <c r="U141" s="21"/>
+      <c r="V141" s="21"/>
+      <c r="W141" s="21"/>
+      <c r="X141" s="21"/>
       <c r="Y141" s="12"/>
     </row>
     <row r="142" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A142" s="20" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B142" s="20" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C142" s="12"/>
       <c r="D142" s="22" t="s">
-        <v>249</v>
-      </c>
-      <c r="E142" s="23" t="s">
-        <v>249</v>
-      </c>
-      <c r="F142" s="21"/>
-      <c r="G142" s="22" t="s">
-        <v>249</v>
-      </c>
-      <c r="H142" s="21"/>
-      <c r="I142" s="21"/>
-      <c r="J142" s="22" t="s">
-        <v>250</v>
-      </c>
-      <c r="K142" s="22" t="s">
-        <v>249</v>
-      </c>
-      <c r="L142" s="23" t="s">
-        <v>249</v>
-      </c>
-      <c r="M142" s="22" t="s">
-        <v>249</v>
-      </c>
-      <c r="N142" s="22" t="s">
-        <v>249</v>
-      </c>
-      <c r="O142" s="21"/>
-      <c r="P142" s="21"/>
-      <c r="Q142" s="22" t="s">
-        <v>250</v>
-      </c>
-      <c r="R142" s="22" t="s">
-        <v>251</v>
-      </c>
-      <c r="S142" s="22" t="s">
-        <v>250</v>
-      </c>
-      <c r="T142" s="21"/>
-      <c r="U142" s="22" t="s">
-        <v>250</v>
-      </c>
-      <c r="V142" s="21"/>
-      <c r="W142" s="21"/>
-      <c r="X142" s="21"/>
+        <v>41</v>
+      </c>
+      <c r="E142" s="34"/>
+      <c r="F142" s="12"/>
+      <c r="G142" s="12"/>
+      <c r="H142" s="12"/>
+      <c r="I142" s="12"/>
+      <c r="J142" s="12"/>
+      <c r="K142" s="12"/>
+      <c r="L142" s="34"/>
+      <c r="M142" s="12"/>
+      <c r="N142" s="12"/>
+      <c r="O142" s="12"/>
+      <c r="P142" s="12"/>
+      <c r="Q142" s="12"/>
+      <c r="R142" s="12"/>
+      <c r="S142" s="12"/>
+      <c r="T142" s="12"/>
+      <c r="U142" s="12"/>
+      <c r="V142" s="12"/>
+      <c r="W142" s="12"/>
+      <c r="X142" s="12"/>
       <c r="Y142" s="12"/>
     </row>
     <row r="143" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A143" s="20" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="B143" s="20" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="C143" s="12"/>
       <c r="D143" s="22" t="s">
-        <v>38</v>
+        <v>249</v>
       </c>
       <c r="E143" s="23" t="s">
-        <v>38</v>
+        <v>249</v>
       </c>
       <c r="F143" s="21"/>
-      <c r="G143" s="21"/>
+      <c r="G143" s="22" t="s">
+        <v>249</v>
+      </c>
       <c r="H143" s="21"/>
       <c r="I143" s="21"/>
-      <c r="J143" s="21"/>
+      <c r="J143" s="22" t="s">
+        <v>250</v>
+      </c>
       <c r="K143" s="22" t="s">
-        <v>38</v>
+        <v>249</v>
       </c>
       <c r="L143" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="M143" s="21"/>
-      <c r="N143" s="21"/>
+        <v>249</v>
+      </c>
+      <c r="M143" s="22" t="s">
+        <v>249</v>
+      </c>
+      <c r="N143" s="22" t="s">
+        <v>249</v>
+      </c>
       <c r="O143" s="21"/>
       <c r="P143" s="21"/>
-      <c r="Q143" s="21"/>
-      <c r="R143" s="21"/>
-      <c r="S143" s="21"/>
+      <c r="Q143" s="22" t="s">
+        <v>250</v>
+      </c>
+      <c r="R143" s="22" t="s">
+        <v>251</v>
+      </c>
+      <c r="S143" s="22" t="s">
+        <v>250</v>
+      </c>
       <c r="T143" s="21"/>
-      <c r="U143" s="21"/>
+      <c r="U143" s="22" t="s">
+        <v>250</v>
+      </c>
       <c r="V143" s="21"/>
       <c r="W143" s="21"/>
       <c r="X143" s="21"/>
       <c r="Y143" s="12"/>
     </row>
+    <row r="144" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A144" s="20" t="s">
+        <v>252</v>
+      </c>
+      <c r="B144" s="20" t="s">
+        <v>252</v>
+      </c>
+      <c r="C144" s="12"/>
+      <c r="D144" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="E144" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="F144" s="21"/>
+      <c r="G144" s="21"/>
+      <c r="H144" s="21"/>
+      <c r="I144" s="21"/>
+      <c r="J144" s="21"/>
+      <c r="K144" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="L144" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="M144" s="21"/>
+      <c r="N144" s="21"/>
+      <c r="O144" s="21"/>
+      <c r="P144" s="21"/>
+      <c r="Q144" s="21"/>
+      <c r="R144" s="21"/>
+      <c r="S144" s="21"/>
+      <c r="T144" s="21"/>
+      <c r="U144" s="21"/>
+      <c r="V144" s="21"/>
+      <c r="W144" s="21"/>
+      <c r="X144" s="21"/>
+      <c r="Y144" s="12"/>
+    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="Y114:Y115"/>
+    <mergeCell ref="Y115:Y116"/>
     <mergeCell ref="C1:O1"/>
     <mergeCell ref="C2:O2"/>
     <mergeCell ref="C5:H5"/>

</xml_diff>